<commit_message>
Redesign as dark electrical-trade template with company/project drill-down
Replace the default Vite branding look with a dark, teenage.engineering-
inspired theme in the real Cassidy-Davies brand green, a real logo mark,
and self-hosted Inter font. Home page now drills down through service
category -> company -> project instead of a flat job list, with jobs
grouped into repeat companies with multiple projects each. Removed the
unused BPMN swimlane reference section.
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Swimlane Reference" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$J$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$K$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -99,7 +99,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -129,11 +129,44 @@
         <color rgb="001B365D"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -189,6 +222,7 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -580,62 +614,58 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Total Active Jobs</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n"/>
+      <c r="C4" s="25" t="n"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Automated AI Validations</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n"/>
+      <c r="F4" s="25" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="5">
         <f>COUNTA('Job Directory'!A5:A24)</f>
         <v/>
       </c>
-      <c r="C5" s="4" t="n"/>
+      <c r="C5" s="25" t="n"/>
       <c r="E5" s="5">
         <f>COUNTIF('Job Directory'!F5:F24, "Passed")</f>
         <v/>
       </c>
-      <c r="F5" s="4" t="n"/>
-    </row>
-    <row r="6"/>
+      <c r="F5" s="25" t="n"/>
+    </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Pending Manual Approval</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n"/>
+      <c r="C7" s="25" t="n"/>
       <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Total Revenue Pipeline</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n"/>
+      <c r="F7" s="25" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="5">
         <f>COUNTIF('Job Directory'!G5:G24, "Pending")</f>
         <v/>
       </c>
-      <c r="C8" s="4" t="n"/>
+      <c r="C8" s="25" t="n"/>
       <c r="E8" s="6">
         <f>SUM('Job Directory'!I5:I24)</f>
         <v/>
       </c>
-      <c r="F8" s="4" t="n"/>
-    </row>
-    <row r="9"/>
-    <row r="10"/>
+      <c r="F8" s="25" t="n"/>
+    </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -838,19 +868,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -863,11 +894,10 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tracking process flow across 6 standard Camunda BPMN swimlanes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Commercial, Residential &amp; Home Ventilation jobs across 6 BPMN swimlanes</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -881,40 +911,45 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
+          <t>Service Type</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
           <t>Job Category</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Current Swimlane</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>AI Check Status</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Approval Status</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>Assigned Tech</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>Est. Value ($)</t>
         </is>
       </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>BPMN Process ID</t>
         </is>
@@ -928,45 +963,50 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Canterbury Health Trust</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Commercial Inspection</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
+          <t>Riccarton Business Park</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>3-Phase Power Distribution</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>5. Electrical Technician</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G5" s="16" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>Mark Stevens</t>
         </is>
       </c>
-      <c r="I5" s="17" t="n">
-        <v>3450</v>
-      </c>
-      <c r="J5" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="J5" s="17" t="n">
+        <v>8200</v>
+      </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>PROC_COM_01</t>
         </is>
       </c>
     </row>
@@ -978,45 +1018,50 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Apex Retail Group</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
+          <t>Riccarton Business Park</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>Switchboard Upgrade</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>2. Service Coordinator</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="I6" s="19" t="inlineStr">
         <is>
           <t>Sarah Jenkins</t>
         </is>
       </c>
-      <c r="I6" s="20" t="n">
-        <v>8200</v>
-      </c>
-      <c r="J6" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_02</t>
+      <c r="J6" s="20" t="n">
+        <v>6400</v>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>PROC_COM_02</t>
         </is>
       </c>
     </row>
@@ -1028,45 +1073,50 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Riccarton Properties</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>HVAC Wiring &amp; Controls</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
+          <t>Papanui Auto Workshop</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Motor Control Centre Repair</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>6. Accounts &amp; Billing</t>
         </is>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>Mark Stevens</t>
         </is>
       </c>
-      <c r="I7" s="17" t="n">
-        <v>1250</v>
-      </c>
-      <c r="J7" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="J7" s="17" t="n">
+        <v>11200</v>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>PROC_COM_01</t>
         </is>
       </c>
     </row>
@@ -1078,45 +1128,50 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Christchurch Tech Park</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>Data &amp; Fiber Installation</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
+          <t>Papanui Auto Workshop</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Compliance Certification</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>4. AI Validation Layer</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>Flagged</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H8" s="19" t="inlineStr">
+      <c r="I8" s="19" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="I8" s="20" t="n">
-        <v>4600</v>
-      </c>
-      <c r="J8" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_03</t>
+      <c r="J8" s="20" t="n">
+        <v>3100</v>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
+        <is>
+          <t>PROC_COM_03</t>
         </is>
       </c>
     </row>
@@ -1128,45 +1183,50 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>High Street Cafe</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Emergency Lighting Maintenance</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
+          <t>Addington Cold Stores</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Refrigeration Wiring</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>5. Electrical Technician</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
         <is>
           <t>Dave Wilson</t>
         </is>
       </c>
-      <c r="I9" s="17" t="n">
-        <v>850</v>
-      </c>
-      <c r="J9" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="J9" s="17" t="n">
+        <v>5400</v>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>PROC_COM_01</t>
         </is>
       </c>
     </row>
@@ -1178,45 +1238,50 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Southern Logistics</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>Warehouse LED Retrofit</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
+          <t>Addington Cold Stores</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Emergency Lighting Maintenance</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>1. Client / Portal</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="G10" s="18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="H10" s="18" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="I10" s="19" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="I10" s="20" t="n">
-        <v>15400</v>
-      </c>
-      <c r="J10" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_02</t>
+      <c r="J10" s="20" t="n">
+        <v>850</v>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
+        <is>
+          <t>PROC_COM_02</t>
         </is>
       </c>
     </row>
@@ -1228,45 +1293,50 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Merivale Dental Clinic</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>UPS Backup Power Setup</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>3. Central Knowledge Repository</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
+          <t>Aidan &amp; Grace Family Home</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Full House Rewire</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>5. Electrical Technician</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G11" s="16" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>Sarah Jenkins</t>
-        </is>
-      </c>
-      <c r="I11" s="17" t="n">
-        <v>2900</v>
-      </c>
-      <c r="J11" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Mark Stevens</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="n">
+        <v>15400</v>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>PROC_RES_01</t>
         </is>
       </c>
     </row>
@@ -1278,45 +1348,50 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>University Student Housing</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>Compliance Certification</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>5. Electrical Technician</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
+          <t>Aidan &amp; Grace Family Home</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Switchboard Safety Upgrade</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>6. Accounts &amp; Billing</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
+      <c r="H12" s="18" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H12" s="19" t="inlineStr">
-        <is>
-          <t>Dave Wilson</t>
-        </is>
-      </c>
-      <c r="I12" s="20" t="n">
-        <v>6100</v>
-      </c>
-      <c r="J12" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_03</t>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>Mark Stevens</t>
+        </is>
+      </c>
+      <c r="J12" s="20" t="n">
+        <v>2150</v>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
+        <is>
+          <t>PROC_RES_02</t>
         </is>
       </c>
     </row>
@@ -1328,45 +1403,50 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Papanui Auto Workshop</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>3-Phase Power Distribution</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
+          <t>Halswell Family Home</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>EV Charger Installation</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>2. Service Coordinator</t>
         </is>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G13" s="16" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="I13" s="9" t="inlineStr">
         <is>
           <t>Sarah Jenkins</t>
         </is>
       </c>
-      <c r="I13" s="17" t="n">
-        <v>7300</v>
-      </c>
-      <c r="J13" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_02</t>
+      <c r="J13" s="17" t="n">
+        <v>3900</v>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>PROC_RES_01</t>
         </is>
       </c>
     </row>
@@ -1378,45 +1458,50 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Lyttelton Marine Services</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>Generator Control Automation</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>6. Accounts &amp; Billing</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
+          <t>Halswell Family Home</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Smart Lighting Setup</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>3. Central Knowledge Repository</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>Mark Stevens</t>
-        </is>
-      </c>
-      <c r="I14" s="20" t="n">
-        <v>9800</v>
-      </c>
-      <c r="J14" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="I14" s="19" t="inlineStr">
+        <is>
+          <t>Sarah Jenkins</t>
+        </is>
+      </c>
+      <c r="J14" s="20" t="n">
+        <v>2750</v>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>PROC_RES_02</t>
         </is>
       </c>
     </row>
@@ -1428,45 +1513,50 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Sydenham Warehousing</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Solar Inverter Maintenance</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
+          <t>Merivale Residence</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Solar Panel Wiring</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>4. AI Validation Layer</t>
         </is>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>Flagged</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="I15" s="9" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="I15" s="17" t="n">
-        <v>3100</v>
-      </c>
-      <c r="J15" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_03</t>
+      <c r="J15" s="17" t="n">
+        <v>8900</v>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>PROC_RES_01</t>
         </is>
       </c>
     </row>
@@ -1478,45 +1568,50 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Fendalton Medical Centre</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>Thermal Imaging Audit</t>
-        </is>
-      </c>
-      <c r="D16" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="E16" s="19" t="inlineStr">
+          <t>Merivale Residence</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Outdoor Security Lighting</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>5. Electrical Technician</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="G16" s="18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H16" s="19" t="inlineStr">
+      <c r="I16" s="19" t="inlineStr">
         <is>
           <t>Dave Wilson</t>
         </is>
       </c>
-      <c r="I16" s="20" t="n">
+      <c r="J16" s="20" t="n">
         <v>1850</v>
       </c>
-      <c r="J16" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>PROC_RES_02</t>
         </is>
       </c>
     </row>
@@ -1528,45 +1623,50 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Avonhead Shopping Centre</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Exterior Security Lighting</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>2. Service Coordinator</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
+          <t>Cashmere Residence</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Home Ventilation</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>5. Electrical Technician</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>Sarah Jenkins</t>
-        </is>
-      </c>
-      <c r="I17" s="17" t="n">
-        <v>4200</v>
-      </c>
-      <c r="J17" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_02</t>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>Dave Wilson</t>
+        </is>
+      </c>
+      <c r="J17" s="17" t="n">
+        <v>4600</v>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>PROC_VEN_01</t>
         </is>
       </c>
     </row>
@@ -1578,45 +1678,50 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Hornby Manufacturing</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="inlineStr">
-        <is>
-          <t>Motor Control Centre Repair</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>5. Electrical Technician</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
+          <t>Cashmere Residence</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Home Ventilation</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Ventilation System Service</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>1. Client / Portal</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>Mark Stevens</t>
-        </is>
-      </c>
-      <c r="I18" s="20" t="n">
-        <v>11200</v>
-      </c>
-      <c r="J18" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="J18" s="20" t="n">
+        <v>1250</v>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
+        <is>
+          <t>PROC_VEN_02</t>
         </is>
       </c>
     </row>
@@ -1628,45 +1733,50 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Addington Cold Stores</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Refrigeration Wiring</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>1. Client / Portal</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
+          <t>Hornby Residence</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Home Ventilation</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Whole-Home Ventilation System</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>2. Service Coordinator</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="I19" s="17" t="n">
-        <v>5400</v>
-      </c>
-      <c r="J19" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_02</t>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Sarah Jenkins</t>
+        </is>
+      </c>
+      <c r="J19" s="17" t="n">
+        <v>7300</v>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>PROC_VEN_01</t>
         </is>
       </c>
     </row>
@@ -1678,45 +1788,50 @@
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>St Albans Bakery</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="inlineStr">
-        <is>
-          <t>Oven Control Panel Upgrade</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="E20" s="19" t="inlineStr">
-        <is>
-          <t>3. Central Knowledge Repository</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
+          <t>Hornby Residence</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Home Ventilation</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Bathroom Extraction Fan Upgrade</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>6. Accounts &amp; Billing</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="H20" s="18" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="H20" s="19" t="inlineStr">
-        <is>
-          <t>Sarah Jenkins</t>
-        </is>
-      </c>
-      <c r="I20" s="20" t="n">
-        <v>2750</v>
-      </c>
-      <c r="J20" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="I20" s="19" t="inlineStr">
+        <is>
+          <t>Mark Stevens</t>
+        </is>
+      </c>
+      <c r="J20" s="20" t="n">
+        <v>950</v>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
+        <is>
+          <t>PROC_VEN_02</t>
         </is>
       </c>
     </row>
@@ -1728,45 +1843,50 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Cashmere Secondary School</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>PA System Power Integration</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>2. Service Coordinator</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
+          <t>Burnside Home</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Home Ventilation</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Heat Recovery Ventilation Install</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>5. Electrical Technician</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="I21" s="17" t="n">
-        <v>3900</v>
-      </c>
-      <c r="J21" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_03</t>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>Dave Wilson</t>
+        </is>
+      </c>
+      <c r="J21" s="17" t="n">
+        <v>6100</v>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>PROC_VEN_01</t>
         </is>
       </c>
     </row>
@@ -1778,169 +1898,75 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Burnside Fitness Centre</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="inlineStr">
-        <is>
-          <t>Sauna Heater Rewiring</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>5. Electrical Technician</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
+          <t>Burnside Home</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Home Ventilation</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Ducted Ventilation Maintenance</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>4. AI Validation Layer</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="G22" s="18" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="H22" s="19" t="inlineStr">
-        <is>
-          <t>Dave Wilson</t>
-        </is>
-      </c>
-      <c r="I22" s="20" t="n">
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="J22" s="20" t="n">
         <v>1600</v>
       </c>
-      <c r="J22" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>PROC_VEN_02</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>CDE-2026-019</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Linwood Community Hub</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>EV Charging Station Setup</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>4. AI Validation Layer</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G23" s="16" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="I23" s="17" t="n">
-        <v>8900</v>
-      </c>
-      <c r="J23" s="16" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_02</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>CDE-2026-020</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>Halswell Library</t>
-        </is>
-      </c>
-      <c r="C24" s="19" t="inlineStr">
-        <is>
-          <t>BMS Sensor Calibrations</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="E24" s="19" t="inlineStr">
-        <is>
-          <t>6. Accounts &amp; Billing</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="G24" s="18" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="H24" s="19" t="inlineStr">
-        <is>
-          <t>Mark Stevens</t>
-        </is>
-      </c>
-      <c r="I24" s="20" t="n">
-        <v>2150</v>
-      </c>
-      <c r="J24" s="18" t="inlineStr">
-        <is>
-          <t>PROC_ELEC_01</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>Total Pipeline Value</t>
         </is>
       </c>
-      <c r="B25" s="21" t="n"/>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="21" t="n"/>
-      <c r="E25" s="21" t="n"/>
-      <c r="F25" s="21" t="n"/>
-      <c r="G25" s="21" t="n"/>
-      <c r="H25" s="21" t="n"/>
-      <c r="I25" s="22">
-        <f>SUM(I5:I24)</f>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="21" t="n"/>
+      <c r="H23" s="21" t="n"/>
+      <c r="I23" s="21" t="n"/>
+      <c r="J23" s="22">
+        <f>SUM(J5:J22)</f>
         <v/>
       </c>
-      <c r="J25" s="21" t="n"/>
+      <c r="K23" s="21" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J24"/>
+  <autoFilter ref="A4:K22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1975,7 +2001,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update job data via upload form (2026-07-30T00:39:08.811Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixkwan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A45C8B5C-F46F-0947-BFC8-F9C9F3B5CC6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A65AB7-91F5-DC4F-8143-EBA45B9F2C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Executive Summary" sheetId="1" r:id="rId1"/>
@@ -139,9 +139,6 @@
     <t>CDE-2026-001</t>
   </si>
   <si>
-    <t>Riccarton Business Park</t>
-  </si>
-  <si>
     <t>Commercial</t>
   </si>
   <si>
@@ -473,6 +470,9 @@
   </si>
   <si>
     <t>Xero / MYOB API Integration</t>
+  </si>
+  <si>
+    <t>Riccarton Business Parks</t>
   </si>
 </sst>
 </file>
@@ -1284,634 +1284,634 @@
         <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="D5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="12" t="s">
         <v>35</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>36</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>16</v>
       </c>
       <c r="G5" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="I5" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="J5" s="13">
         <v>8200</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="15" t="s">
+      <c r="E6" s="14" t="s">
         <v>42</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>43</v>
       </c>
       <c r="F6" s="15" t="s">
         <v>13</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H6" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="15" t="s">
         <v>44</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>45</v>
       </c>
       <c r="J6" s="16">
         <v>6400</v>
       </c>
       <c r="K6" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="12" t="s">
         <v>49</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>50</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="I7" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="J7" s="13">
         <v>11200</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" s="15" t="s">
+      <c r="E8" s="14" t="s">
         <v>52</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>53</v>
       </c>
       <c r="F8" s="15" t="s">
         <v>15</v>
       </c>
       <c r="G8" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" s="15" t="s">
         <v>54</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="I8" s="15" t="s">
-        <v>55</v>
       </c>
       <c r="J8" s="16">
         <v>3100</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="12" t="s">
         <v>59</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>60</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>16</v>
       </c>
       <c r="G9" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="12" t="s">
-        <v>38</v>
-      </c>
       <c r="I9" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J9" s="13">
         <v>5400</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="15" t="s">
+      <c r="E10" s="14" t="s">
         <v>63</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>64</v>
       </c>
       <c r="F10" s="15" t="s">
         <v>12</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J10" s="16">
         <v>850</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="D11" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="12" t="s">
         <v>68</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>69</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>16</v>
       </c>
       <c r="G11" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="I11" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="J11" s="13">
         <v>15400</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D12" s="15" t="s">
+      <c r="E12" s="14" t="s">
         <v>72</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>73</v>
       </c>
       <c r="F12" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G12" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="H12" s="14" t="s">
+      <c r="I12" s="15" t="s">
         <v>38</v>
-      </c>
-      <c r="I12" s="15" t="s">
-        <v>39</v>
       </c>
       <c r="J12" s="16">
         <v>2150</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="12" t="s">
         <v>77</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>78</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H13" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="I13" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="J13" s="13">
         <v>3900</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D14" s="15" t="s">
+      <c r="E14" s="14" t="s">
         <v>80</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>81</v>
       </c>
       <c r="F14" s="15" t="s">
         <v>14</v>
       </c>
       <c r="G14" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="H14" s="14" t="s">
-        <v>38</v>
-      </c>
       <c r="I14" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J14" s="16">
         <v>2750</v>
       </c>
       <c r="K14" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="12" t="s">
         <v>84</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>85</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G15" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="H15" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>55</v>
       </c>
       <c r="J15" s="13">
         <v>8900</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B16" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D16" s="15" t="s">
+      <c r="E16" s="14" t="s">
         <v>87</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>88</v>
       </c>
       <c r="F16" s="15" t="s">
         <v>16</v>
       </c>
       <c r="G16" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="H16" s="14" t="s">
-        <v>38</v>
-      </c>
       <c r="I16" s="15" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J16" s="16">
         <v>1850</v>
       </c>
       <c r="K16" s="14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="D17" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="12" t="s">
         <v>92</v>
-      </c>
-      <c r="E17" s="12" t="s">
-        <v>93</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>16</v>
       </c>
       <c r="G17" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H17" s="12" t="s">
-        <v>38</v>
-      </c>
       <c r="I17" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J17" s="13">
         <v>4600</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B18" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D18" s="15" t="s">
+      <c r="E18" s="14" t="s">
         <v>96</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>97</v>
       </c>
       <c r="F18" s="15" t="s">
         <v>12</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J18" s="16">
         <v>1250</v>
       </c>
       <c r="K18" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="12" t="s">
         <v>101</v>
-      </c>
-      <c r="E19" s="12" t="s">
-        <v>102</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H19" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="I19" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="J19" s="13">
         <v>7300</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D20" s="15" t="s">
+      <c r="E20" s="14" t="s">
         <v>104</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>105</v>
       </c>
       <c r="F20" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G20" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H20" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="H20" s="14" t="s">
+      <c r="I20" s="15" t="s">
         <v>38</v>
-      </c>
-      <c r="I20" s="15" t="s">
-        <v>39</v>
       </c>
       <c r="J20" s="16">
         <v>950</v>
       </c>
       <c r="K20" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="12" t="s">
         <v>108</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>109</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>16</v>
       </c>
       <c r="G21" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H21" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H21" s="12" t="s">
-        <v>38</v>
-      </c>
       <c r="I21" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J21" s="13">
         <v>6100</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="B22" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D22" s="15" t="s">
+      <c r="E22" s="14" t="s">
         <v>111</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>112</v>
       </c>
       <c r="F22" s="15" t="s">
         <v>15</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J22" s="16">
         <v>1600</v>
       </c>
       <c r="K22" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B23" s="17"/>
       <c r="C23" s="17"/>
@@ -1947,29 +1947,29 @@
   <sheetData>
     <row r="1" spans="1:5" ht="23" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.2">
@@ -1977,16 +1977,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="E5" s="5" t="s">
         <v>123</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.2">
@@ -1994,16 +1994,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="D6" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="E6" s="15" t="s">
         <v>127</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.2">
@@ -2011,16 +2011,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="19" t="s">
         <v>130</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="E7" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.2">
@@ -2028,16 +2028,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="D8" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="E8" s="15" t="s">
         <v>135</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.2">
@@ -2045,16 +2045,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="E9" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.2">
@@ -2062,16 +2062,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="D10" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="E10" s="15" t="s">
         <v>143</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update job data via upload form (2026-08-03T23:54:24.490Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixkwan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EAF6DDE-EC7A-9E4D-AD97-65769184CE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A66620D0-EDA7-F449-B179-B032529BC379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Job Directory" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$K$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$K$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="103">
   <si>
     <t>Cassidy-Davies Electrical — Operations &amp; Workflow Dashboard</t>
   </si>
@@ -340,15 +340,6 @@
   </si>
   <si>
     <t>2026-07-13</t>
-  </si>
-  <si>
-    <t>CDE-2026-018</t>
-  </si>
-  <si>
-    <t>Ducted Ventilation Maintenance</t>
-  </si>
-  <si>
-    <t>2026-07-29</t>
   </si>
   <si>
     <t>Total Pipeline Value</t>
@@ -518,18 +509,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -844,59 +835,59 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="E3" s="18" t="s">
+      <c r="C3" s="17"/>
+      <c r="E3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="15"/>
+      <c r="F3" s="17"/>
     </row>
     <row r="4" spans="1:7" ht="21" x14ac:dyDescent="0.2">
-      <c r="B4" s="16">
-        <f>COUNTA('Job Directory'!A5:A24)</f>
-        <v>19</v>
-      </c>
-      <c r="C4" s="15"/>
-      <c r="E4" s="16">
-        <f>COUNTIF('Job Directory'!F5:F24, "Passed")</f>
+      <c r="B4" s="18">
+        <f>COUNTA('Job Directory'!A5:A23)</f>
+        <v>18</v>
+      </c>
+      <c r="C4" s="17"/>
+      <c r="E4" s="18">
+        <f>COUNTIF('Job Directory'!F5:F23, "Passed")</f>
         <v>0</v>
       </c>
-      <c r="F4" s="15"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="E6" s="18" t="s">
+      <c r="C6" s="17"/>
+      <c r="E6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="15"/>
+      <c r="F6" s="17"/>
     </row>
     <row r="7" spans="1:7" ht="21" x14ac:dyDescent="0.2">
-      <c r="B7" s="16">
-        <f>COUNTIF('Job Directory'!G5:G24, "Pending")</f>
+      <c r="B7" s="18">
+        <f>COUNTIF('Job Directory'!G5:G23, "Pending")</f>
         <v>0</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="E7" s="14">
-        <f>SUM('Job Directory'!I5:I24)</f>
+      <c r="C7" s="17"/>
+      <c r="E7" s="19">
+        <f>SUM('Job Directory'!I5:I23)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="15"/>
+      <c r="F7" s="17"/>
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
@@ -919,7 +910,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -984,7 +975,7 @@
         <v>24</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>25</v>
@@ -1019,7 +1010,7 @@
         <v>32</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>25</v>
@@ -1575,60 +1566,25 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="J22" s="11">
-        <v>1600</v>
-      </c>
-      <c r="K22" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A23" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="13">
-        <f>SUM(J5:J22)</f>
-        <v>91900</v>
-      </c>
-      <c r="K23" s="12"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="13">
+        <f>SUM(J5:J21)</f>
+        <v>90300</v>
+      </c>
+      <c r="K22" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K22" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A4:K21" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update job data via upload form (2026-08-04T00:07:13.359Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixkwan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A66620D0-EDA7-F449-B179-B032529BC379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD46AE67-0B40-6A4E-92A4-C95A91415942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Job Directory" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$K$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$I$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="88">
   <si>
     <t>Cassidy-Davies Electrical — Operations &amp; Workflow Dashboard</t>
   </si>
@@ -54,24 +54,6 @@
     <t>Total Revenue Pipeline</t>
   </si>
   <si>
-    <t>1. Client / Portal</t>
-  </si>
-  <si>
-    <t>2. Service Coordinator</t>
-  </si>
-  <si>
-    <t>3. Central Knowledge Repository</t>
-  </si>
-  <si>
-    <t>4. AI Validation Layer</t>
-  </si>
-  <si>
-    <t>5. Electrical Technician</t>
-  </si>
-  <si>
-    <t>6. Accounts &amp; Billing</t>
-  </si>
-  <si>
     <t>Cassidy-Davies Electrical — Active Job Log</t>
   </si>
   <si>
@@ -93,9 +75,6 @@
     <t>Creation Date</t>
   </si>
   <si>
-    <t>Current Swimlane</t>
-  </si>
-  <si>
     <t>AI Check Status</t>
   </si>
   <si>
@@ -108,9 +87,6 @@
     <t>Est. Value ($)</t>
   </si>
   <si>
-    <t>BPMN Process ID</t>
-  </si>
-  <si>
     <t>CDE-2026-001</t>
   </si>
   <si>
@@ -132,9 +108,6 @@
     <t>Mark Stevens</t>
   </si>
   <si>
-    <t>PROC_COM_01</t>
-  </si>
-  <si>
     <t>CDE-2026-002</t>
   </si>
   <si>
@@ -150,9 +123,6 @@
     <t>Sarah Jenkins</t>
   </si>
   <si>
-    <t>PROC_COM_02</t>
-  </si>
-  <si>
     <t>CDE-2026-003</t>
   </si>
   <si>
@@ -180,9 +150,6 @@
     <t>Unassigned</t>
   </si>
   <si>
-    <t>PROC_COM_03</t>
-  </si>
-  <si>
     <t>CDE-2026-005</t>
   </si>
   <si>
@@ -222,9 +189,6 @@
     <t>2026-07-05</t>
   </si>
   <si>
-    <t>PROC_RES_01</t>
-  </si>
-  <si>
     <t>CDE-2026-008</t>
   </si>
   <si>
@@ -234,9 +198,6 @@
     <t>2026-07-19</t>
   </si>
   <si>
-    <t>PROC_RES_02</t>
-  </si>
-  <si>
     <t>CDE-2026-009</t>
   </si>
   <si>
@@ -294,9 +255,6 @@
     <t>2026-07-11</t>
   </si>
   <si>
-    <t>PROC_VEN_01</t>
-  </si>
-  <si>
     <t>CDE-2026-014</t>
   </si>
   <si>
@@ -304,9 +262,6 @@
   </si>
   <si>
     <t>2026-07-23</t>
-  </si>
-  <si>
-    <t>PROC_VEN_02</t>
   </si>
   <si>
     <t>CDE-2026-015</t>
@@ -861,9 +816,9 @@
         <v>18</v>
       </c>
       <c r="C4" s="17"/>
-      <c r="E4" s="18">
-        <f>COUNTIF('Job Directory'!F5:F23, "Passed")</f>
-        <v>0</v>
+      <c r="E4" s="18" t="e">
+        <f>COUNTIF('Job Directory'!#REF!, "Passed")</f>
+        <v>#REF!</v>
       </c>
       <c r="F4" s="17"/>
     </row>
@@ -879,12 +834,12 @@
     </row>
     <row r="7" spans="1:7" ht="21" x14ac:dyDescent="0.2">
       <c r="B7" s="18">
-        <f>COUNTIF('Job Directory'!G5:G23, "Pending")</f>
+        <f>COUNTIF('Job Directory'!F5:F23, "Pending")</f>
         <v>0</v>
       </c>
       <c r="C7" s="17"/>
       <c r="E7" s="19">
-        <f>SUM('Job Directory'!I5:I23)</f>
+        <f>SUM('Job Directory'!H5:H23)</f>
         <v>0</v>
       </c>
       <c r="F7" s="17"/>
@@ -910,7 +865,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -918,656 +873,546 @@
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="37" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="35" customWidth="1"/>
-    <col min="7" max="8" width="19" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="19" customWidth="1"/>
+    <col min="6" max="7" width="19" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="23" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="4" t="s">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="B5" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="E5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="F5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="G5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="H5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="I5" s="8">
+        <v>8200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="B6" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C5" s="7" t="s">
+      <c r="E6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="F6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="H6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="7" t="s">
+      <c r="I6" s="11">
+        <v>6400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="C7" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="J5" s="8">
-        <v>8200</v>
-      </c>
-      <c r="K5" s="7" t="s">
+      <c r="E7" s="7" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="F7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="8">
+        <v>11200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="10" t="s">
+      <c r="B8" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="9" t="s">
+      <c r="F8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="G8" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="J6" s="11">
-        <v>6400</v>
-      </c>
-      <c r="K6" s="9" t="s">
+      <c r="I8" s="11">
+        <v>3100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E9" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="F9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J7" s="8">
-        <v>11200</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="I9" s="8">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="10" t="s">
+      <c r="B10" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E10" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="G8" s="9" t="s">
+      <c r="F10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I10" s="11">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="B11" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="8">
+        <v>15400</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I12" s="11">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I13" s="8">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="11">
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F15" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="I8" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="J8" s="11">
-        <v>3100</v>
-      </c>
-      <c r="K8" s="9" t="s">
+      <c r="G15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I15" s="8">
+        <v>8900</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J9" s="8">
-        <v>5400</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I10" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="J10" s="11">
-        <v>850</v>
-      </c>
-      <c r="K10" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J11" s="8">
-        <v>15400</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="I12" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="J12" s="11">
-        <v>2150</v>
-      </c>
-      <c r="K12" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="E16" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="F16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I16" s="11">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D13" s="5" t="s">
+      <c r="B17" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I13" s="5" t="s">
+      <c r="D17" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I17" s="8">
+        <v>4600</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H18" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="J13" s="8">
-        <v>3900</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="J14" s="11">
-        <v>2750</v>
-      </c>
-      <c r="K14" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D15" s="5" t="s">
+      <c r="I18" s="11">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="B19" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="J15" s="8">
-        <v>8900</v>
-      </c>
-      <c r="K15" s="7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="9" t="s">
+      <c r="C19" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="10" t="s">
+      <c r="E19" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="F19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I19" s="8">
+        <v>7300</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="J16" s="11">
-        <v>1850</v>
-      </c>
-      <c r="K16" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="7" t="s">
+      <c r="B20" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="E20" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="F20" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="11">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="B21" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="C21" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F17" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J17" s="8">
-        <v>4600</v>
-      </c>
-      <c r="K17" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="9" t="s">
+      <c r="F21" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I21" s="8">
+        <v>6100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
         <v>86</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I18" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="J18" s="11">
-        <v>1250</v>
-      </c>
-      <c r="K18" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J19" s="8">
-        <v>7300</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="J20" s="11">
-        <v>950</v>
-      </c>
-      <c r="K20" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J21" s="8">
-        <v>6100</v>
-      </c>
-      <c r="K21" s="7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A22" s="6" t="s">
-        <v>101</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -1576,15 +1421,13 @@
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
       <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="13">
-        <f>SUM(J5:J21)</f>
+      <c r="I22" s="13">
+        <f>SUM(I5:I21)</f>
         <v>90300</v>
       </c>
-      <c r="K22" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K21" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A4:I21" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update job data via upload form (2026-08-04T00:28:07.229Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixkwan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD46AE67-0B40-6A4E-92A4-C95A91415942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FADE0C7-5A79-594D-9DE7-60E0F05E64A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Job Directory" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$I$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="85">
   <si>
     <t>Cassidy-Davies Electrical — Operations &amp; Workflow Dashboard</t>
   </si>
@@ -174,19 +174,10 @@
     <t>2026-07-27</t>
   </si>
   <si>
-    <t>CDE-2026-007</t>
-  </si>
-  <si>
     <t>Aidan &amp; Grace Family Home</t>
   </si>
   <si>
     <t>Residential</t>
-  </si>
-  <si>
-    <t>Full House Rewire</t>
-  </si>
-  <si>
-    <t>2026-07-05</t>
   </si>
   <si>
     <t>CDE-2026-008</t>
@@ -812,8 +803,8 @@
     </row>
     <row r="4" spans="1:7" ht="21" x14ac:dyDescent="0.2">
       <c r="B4" s="18">
-        <f>COUNTA('Job Directory'!A5:A23)</f>
-        <v>18</v>
+        <f>COUNTA('Job Directory'!A5:A22)</f>
+        <v>17</v>
       </c>
       <c r="C4" s="17"/>
       <c r="E4" s="18" t="e">
@@ -834,12 +825,12 @@
     </row>
     <row r="7" spans="1:7" ht="21" x14ac:dyDescent="0.2">
       <c r="B7" s="18">
-        <f>COUNTIF('Job Directory'!F5:F23, "Pending")</f>
+        <f>COUNTIF('Job Directory'!F5:F22, "Pending")</f>
         <v>0</v>
       </c>
       <c r="C7" s="17"/>
       <c r="E7" s="19">
-        <f>SUM('Job Directory'!H5:H23)</f>
+        <f>SUM('Job Directory'!H5:H22)</f>
         <v>0</v>
       </c>
       <c r="F7" s="17"/>
@@ -865,7 +856,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -922,7 +913,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>17</v>
@@ -951,7 +942,7 @@
         <v>23</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>17</v>
@@ -1092,342 +1083,313 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I11" s="8">
-        <v>15400</v>
+      <c r="I11" s="11">
+        <v>2150</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12" s="8">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" s="9" t="s">
+      <c r="C13" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G13" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H13" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I13" s="11">
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I14" s="8">
+        <v>8900</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I15" s="11">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I16" s="8">
+        <v>4600</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" s="11">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I18" s="8">
+        <v>7300</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I12" s="11">
-        <v>2150</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="7" t="s">
+      <c r="I19" s="11">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I13" s="8">
-        <v>3900</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="9" t="s">
+      <c r="G20" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H14" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I14" s="11">
-        <v>2750</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I15" s="8">
-        <v>8900</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H16" s="10" t="s">
+      <c r="H20" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="I16" s="11">
-        <v>1850</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I17" s="8">
-        <v>4600</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="I18" s="11">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I19" s="8">
-        <v>7300</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I20" s="11">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="B21" s="5" t="s">
+      <c r="I20" s="8">
+        <v>6100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I21" s="8">
-        <v>6100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="13">
-        <f>SUM(I5:I21)</f>
-        <v>90300</v>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="13">
+        <f>SUM(I5:I20)</f>
+        <v>74900</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I21" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A4:I20" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update job data via upload form (2026-08-04T00:42:20.775Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixkwan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FADE0C7-5A79-594D-9DE7-60E0F05E64A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA587DB-0ACA-9048-B86F-54853822FD44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Job Directory" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$H$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="83">
   <si>
     <t>Cassidy-Davies Electrical — Operations &amp; Workflow Dashboard</t>
   </si>
@@ -78,9 +78,6 @@
     <t>AI Check Status</t>
   </si>
   <si>
-    <t>Approval Status</t>
-  </si>
-  <si>
     <t>Assigned Tech</t>
   </si>
   <si>
@@ -97,9 +94,6 @@
   </si>
   <si>
     <t>2026-07-10</t>
-  </si>
-  <si>
-    <t>Passed</t>
   </si>
   <si>
     <t>Approved</t>
@@ -826,11 +820,11 @@
     <row r="7" spans="1:7" ht="21" x14ac:dyDescent="0.2">
       <c r="B7" s="18">
         <f>COUNTIF('Job Directory'!F5:F22, "Pending")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C7" s="17"/>
       <c r="E7" s="19">
-        <f>SUM('Job Directory'!H5:H22)</f>
+        <f>SUM('Job Directory'!G5:G22)</f>
         <v>0</v>
       </c>
       <c r="F7" s="17"/>
@@ -856,7 +850,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -864,22 +858,22 @@
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="37" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="7" width="19" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="23" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
@@ -904,477 +898,426 @@
       <c r="H4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="4" t="s">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="B5" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="8">
+        <v>8200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="B6" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="8">
-        <v>8200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="10" t="s">
+      <c r="F6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="G6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="H6" s="11">
+        <v>6400</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="10" t="s">
+      <c r="H7" s="8">
+        <v>11200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="11">
-        <v>6400</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="7" t="s">
+      <c r="C8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="E8" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" s="11">
+        <v>3100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" s="8">
+        <v>5400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" s="11">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="8">
-        <v>11200</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="10" t="s">
+      <c r="H11" s="11">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="8">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="11">
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="G14" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="I8" s="11">
-        <v>3100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="H14" s="8">
+        <v>8900</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" s="7" t="s">
+      <c r="H15" s="11">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H16" s="8">
+        <v>4600</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="H17" s="11">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H18" s="8">
+        <v>7300</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I9" s="8">
-        <v>5400</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="I10" s="11">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I11" s="11">
-        <v>2150</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I12" s="8">
-        <v>3900</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I13" s="11">
-        <v>2750</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I14" s="8">
-        <v>8900</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="I15" s="11">
-        <v>1850</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
+      <c r="H19" s="11">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I16" s="8">
-        <v>4600</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="I17" s="11">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I18" s="8">
-        <v>7300</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="I19" s="11">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
+      <c r="D20" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="E20" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D20" s="5" t="s">
+      <c r="F20" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H20" s="8">
+        <v>6100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I20" s="8">
-        <v>6100</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -1382,14 +1325,14 @@
       <c r="E21" s="12"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
-      <c r="I21" s="13">
-        <f>SUM(I5:I20)</f>
+      <c r="H21" s="13">
+        <f>SUM(H5:H20)</f>
         <v>74900</v>
       </c>
     </row>
+    <row r="22" spans="1:8" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <autoFilter ref="A4:I20" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A4:H20" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update job data via upload form (2026-08-04T01:47:36.939Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixkwan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA587DB-0ACA-9048-B86F-54853822FD44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D110B8D4-753B-E144-A712-B57DEEE6ADF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,9 +75,6 @@
     <t>Creation Date</t>
   </si>
   <si>
-    <t>AI Check Status</t>
-  </si>
-  <si>
     <t>Assigned Tech</t>
   </si>
   <si>
@@ -286,6 +283,9 @@
   </si>
   <si>
     <t>Riccarton Business Parks</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -890,36 +890,36 @@
         <v>11</v>
       </c>
       <c r="F4" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="H5" s="8">
         <v>8200</v>
@@ -927,25 +927,25 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="10" t="s">
+      <c r="E6" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>25</v>
       </c>
       <c r="H6" s="11">
         <v>6400</v>
@@ -953,25 +953,25 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>29</v>
-      </c>
       <c r="F7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="H7" s="8">
         <v>11200</v>
@@ -979,25 +979,25 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="10" t="s">
+      <c r="E8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="F8" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="G8" s="10" t="s">
         <v>33</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>34</v>
       </c>
       <c r="H8" s="11">
         <v>3100</v>
@@ -1005,25 +1005,25 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="H9" s="8">
         <v>5400</v>
@@ -1031,25 +1031,25 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="10" t="s">
+      <c r="E10" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>42</v>
-      </c>
       <c r="F10" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H10" s="11">
         <v>850</v>
@@ -1057,25 +1057,25 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="10" t="s">
+      <c r="E11" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="9" t="s">
-        <v>47</v>
-      </c>
       <c r="F11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>19</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>20</v>
       </c>
       <c r="H11" s="11">
         <v>2150</v>
@@ -1083,25 +1083,25 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>51</v>
-      </c>
       <c r="F12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="H12" s="8">
         <v>3900</v>
@@ -1109,25 +1109,25 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="10" t="s">
+      <c r="E13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>54</v>
-      </c>
       <c r="F13" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H13" s="11">
         <v>2750</v>
@@ -1135,25 +1135,25 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>58</v>
-      </c>
       <c r="F14" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G14" s="5" t="s">
         <v>33</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>34</v>
       </c>
       <c r="H14" s="8">
         <v>8900</v>
@@ -1161,25 +1161,25 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="9" t="s">
-        <v>61</v>
-      </c>
       <c r="F15" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H15" s="11">
         <v>1850</v>
@@ -1187,25 +1187,25 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>66</v>
-      </c>
       <c r="F16" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H16" s="8">
         <v>4600</v>
@@ -1213,25 +1213,25 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B17" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D17" s="10" t="s">
+      <c r="E17" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E17" s="9" t="s">
-        <v>69</v>
-      </c>
       <c r="F17" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H17" s="11">
         <v>1250</v>
@@ -1239,25 +1239,25 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>73</v>
-      </c>
       <c r="F18" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="H18" s="8">
         <v>7300</v>
@@ -1265,25 +1265,25 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D19" s="10" t="s">
+      <c r="E19" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E19" s="9" t="s">
-        <v>76</v>
-      </c>
       <c r="F19" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="10" t="s">
         <v>19</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>20</v>
       </c>
       <c r="H19" s="11">
         <v>950</v>
@@ -1291,25 +1291,25 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="7" t="s">
-        <v>80</v>
-      </c>
       <c r="F20" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H20" s="8">
         <v>6100</v>
@@ -1317,7 +1317,7 @@
     </row>
     <row r="21" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>

</xml_diff>

<commit_message>
Update job data via upload form (2026-08-04T08:35:07.742Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixkwan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D110B8D4-753B-E144-A712-B57DEEE6ADF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86D82AD-8D60-3F49-A3DC-9CED32EB2782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Job Directory" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$H$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Job Directory'!$A$4:$H$19</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="80">
   <si>
     <t>Cassidy-Davies Electrical — Operations &amp; Workflow Dashboard</t>
   </si>
@@ -190,15 +190,6 @@
   </si>
   <si>
     <t>2026-07-12</t>
-  </si>
-  <si>
-    <t>CDE-2026-010</t>
-  </si>
-  <si>
-    <t>Smart Lighting Setup</t>
-  </si>
-  <si>
-    <t>2026-07-24</t>
   </si>
   <si>
     <t>CDE-2026-011</t>
@@ -797,8 +788,8 @@
     </row>
     <row r="4" spans="1:7" ht="21" x14ac:dyDescent="0.2">
       <c r="B4" s="18">
-        <f>COUNTA('Job Directory'!A5:A22)</f>
-        <v>17</v>
+        <f>COUNTA('Job Directory'!A5:A21)</f>
+        <v>16</v>
       </c>
       <c r="C4" s="17"/>
       <c r="E4" s="18" t="e">
@@ -819,12 +810,12 @@
     </row>
     <row r="7" spans="1:7" ht="21" x14ac:dyDescent="0.2">
       <c r="B7" s="18">
-        <f>COUNTIF('Job Directory'!F5:F22, "Pending")</f>
+        <f>COUNTIF('Job Directory'!F5:F21, "Pending")</f>
         <v>5</v>
       </c>
       <c r="C7" s="17"/>
       <c r="E7" s="19">
-        <f>SUM('Job Directory'!G5:G22)</f>
+        <f>SUM('Job Directory'!G5:G21)</f>
         <v>0</v>
       </c>
       <c r="F7" s="17"/>
@@ -850,7 +841,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -890,7 +881,7 @@
         <v>11</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>12</v>
@@ -904,7 +895,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>15</v>
@@ -930,7 +921,7 @@
         <v>20</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>15</v>
@@ -1108,231 +1099,205 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="9" t="s">
+      <c r="B13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="8">
+        <v>8900</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F13" s="9" t="s">
+      <c r="C14" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G14" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="H14" s="11">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H15" s="8">
+        <v>4600</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="H16" s="11">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="H13" s="11">
-        <v>2750</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H14" s="8">
-        <v>8900</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="E15" s="9" t="s">
+      <c r="H17" s="8">
+        <v>7300</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="D18" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F18" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="G18" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="11">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H15" s="11">
-        <v>1850</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H16" s="8">
-        <v>4600</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="H17" s="11">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H18" s="8">
-        <v>7300</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" s="11">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" s="5" t="s">
+      <c r="H19" s="8">
+        <v>6100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H20" s="8">
-        <v>6100</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="13">
-        <f>SUM(H5:H20)</f>
-        <v>74900</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="13">
+        <f>SUM(H5:H19)</f>
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="16" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <autoFilter ref="A4:H20" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A4:H19" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Process pending data updates (2026-08-18T01:41:04Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -11458,30 +11458,74 @@
       <c r="C41" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="53"/>
-      <c r="H41" s="52"/>
-      <c r="I41" s="52"/>
-      <c r="J41" s="52"/>
-      <c r="K41" s="52"/>
-      <c r="L41" s="52"/>
-      <c r="M41" s="53"/>
+      <c r="D41" s="52">
+        <v>128258.5</v>
+      </c>
+      <c r="E41" s="52">
+        <v>36398.39</v>
+      </c>
+      <c r="F41" s="52">
+        <v>91860.11</v>
+      </c>
+      <c r="G41" s="53">
+        <v>0.7162106994858041</v>
+      </c>
+      <c r="H41" s="52">
+        <v>94098.32</v>
+      </c>
+      <c r="I41" s="52">
+        <v>34659.62</v>
+      </c>
+      <c r="J41" s="52">
+        <v>69042.09000000001</v>
+      </c>
+      <c r="K41" s="52">
+        <v>28340.06</v>
+      </c>
+      <c r="L41" s="52">
+        <v>40702.03000000001</v>
+      </c>
+      <c r="M41" s="53">
+        <v>0.5895248825752524</v>
+      </c>
       <c r="N41" s="53"/>
-      <c r="O41" s="52"/>
-      <c r="P41" s="52"/>
-      <c r="Q41" s="52"/>
-      <c r="R41" s="53"/>
-      <c r="S41" s="54"/>
-      <c r="T41" s="54"/>
-      <c r="U41" s="54"/>
-      <c r="V41" s="53"/>
+      <c r="O41" s="52">
+        <v>25056.23</v>
+      </c>
+      <c r="P41" s="52">
+        <v>6319.56</v>
+      </c>
+      <c r="Q41" s="52">
+        <v>18736.67</v>
+      </c>
+      <c r="R41" s="53">
+        <v>0.7477848822428593</v>
+      </c>
+      <c r="S41" s="54">
+        <v>501.83</v>
+      </c>
+      <c r="T41" s="54">
+        <v>123.75</v>
+      </c>
+      <c r="U41" s="54">
+        <v>378.08</v>
+      </c>
+      <c r="V41" s="53">
+        <v>0.7534025466791543</v>
+      </c>
       <c r="W41" s="53"/>
-      <c r="X41" s="55"/>
-      <c r="Y41" s="55"/>
-      <c r="Z41" s="53"/>
-      <c r="AA41" s="56"/>
+      <c r="X41" s="55">
+        <v>14.050666666666666</v>
+      </c>
+      <c r="Y41" s="55">
+        <v>68.07122423898531</v>
+      </c>
+      <c r="Z41" s="53">
+        <v>0.0478</v>
+      </c>
+      <c r="AA41" s="56">
+        <v>0.2663</v>
+      </c>
       <c r="AB41" s="57"/>
       <c r="AD41" s="35"/>
       <c r="AE41" s="35"/>
@@ -11823,30 +11867,74 @@
       <c r="C48" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D48" s="52"/>
-      <c r="E48" s="52"/>
-      <c r="F48" s="52"/>
-      <c r="G48" s="53"/>
-      <c r="H48" s="52"/>
-      <c r="I48" s="52"/>
-      <c r="J48" s="52"/>
-      <c r="K48" s="52"/>
-      <c r="L48" s="52"/>
-      <c r="M48" s="53"/>
+      <c r="D48" s="52">
+        <v>65693.36</v>
+      </c>
+      <c r="E48" s="52">
+        <v>25322.07</v>
+      </c>
+      <c r="F48" s="52">
+        <v>40371.29</v>
+      </c>
+      <c r="G48" s="53">
+        <v>0.6145414087512041</v>
+      </c>
+      <c r="H48" s="52">
+        <v>50582.37</v>
+      </c>
+      <c r="I48" s="52">
+        <v>25131.9</v>
+      </c>
+      <c r="J48" s="52">
+        <v>39438.990000000005</v>
+      </c>
+      <c r="K48" s="52">
+        <v>20456.64</v>
+      </c>
+      <c r="L48" s="52">
+        <v>18982.350000000006</v>
+      </c>
+      <c r="M48" s="53">
+        <v>0.4813092323104624</v>
+      </c>
       <c r="N48" s="53"/>
-      <c r="O48" s="52"/>
-      <c r="P48" s="52"/>
-      <c r="Q48" s="52"/>
-      <c r="R48" s="53"/>
-      <c r="S48" s="54"/>
-      <c r="T48" s="54"/>
-      <c r="U48" s="54"/>
-      <c r="V48" s="53"/>
+      <c r="O48" s="52">
+        <v>11143.38</v>
+      </c>
+      <c r="P48" s="52">
+        <v>4675.26</v>
+      </c>
+      <c r="Q48" s="52">
+        <v>6468.119999999999</v>
+      </c>
+      <c r="R48" s="53">
+        <v>0.5804450714235716</v>
+      </c>
+      <c r="S48" s="54">
+        <v>223.22</v>
+      </c>
+      <c r="T48" s="54">
+        <v>102.25</v>
+      </c>
+      <c r="U48" s="54">
+        <v>120.97</v>
+      </c>
+      <c r="V48" s="53">
+        <v>0.5419317265478004</v>
+      </c>
       <c r="W48" s="53"/>
-      <c r="X48" s="55"/>
-      <c r="Y48" s="55"/>
-      <c r="Z48" s="53"/>
-      <c r="AA48" s="56"/>
+      <c r="X48" s="55">
+        <v>1.8598533007334963</v>
+      </c>
+      <c r="Y48" s="55">
+        <v>67.69550512136009</v>
+      </c>
+      <c r="Z48" s="53">
+        <v>0.0075</v>
+      </c>
+      <c r="AA48" s="56">
+        <v>0.23</v>
+      </c>
       <c r="AB48" s="57"/>
       <c r="AD48" s="35"/>
       <c r="AE48" s="35"/>
@@ -12186,30 +12274,74 @@
       <c r="C55" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="53"/>
-      <c r="H55" s="52"/>
-      <c r="I55" s="52"/>
-      <c r="J55" s="52"/>
-      <c r="K55" s="52"/>
-      <c r="L55" s="52"/>
-      <c r="M55" s="53"/>
+      <c r="D55" s="52">
+        <v>154527.79</v>
+      </c>
+      <c r="E55" s="52">
+        <v>98562.5</v>
+      </c>
+      <c r="F55" s="52">
+        <v>55965.29000000001</v>
+      </c>
+      <c r="G55" s="53">
+        <v>0.36216974306045535</v>
+      </c>
+      <c r="H55" s="52">
+        <v>108880.28</v>
+      </c>
+      <c r="I55" s="52">
+        <v>90918.83</v>
+      </c>
+      <c r="J55" s="52">
+        <v>74953.01000000001</v>
+      </c>
+      <c r="K55" s="52">
+        <v>71302.07</v>
+      </c>
+      <c r="L55" s="52">
+        <v>3650.9400000000023</v>
+      </c>
+      <c r="M55" s="53">
+        <v>0.04870971826214854</v>
+      </c>
       <c r="N55" s="53"/>
-      <c r="O55" s="52"/>
-      <c r="P55" s="52"/>
-      <c r="Q55" s="52"/>
-      <c r="R55" s="53"/>
-      <c r="S55" s="54"/>
-      <c r="T55" s="54"/>
-      <c r="U55" s="54"/>
-      <c r="V55" s="53"/>
+      <c r="O55" s="52">
+        <v>33927.27</v>
+      </c>
+      <c r="P55" s="52">
+        <v>19616.76</v>
+      </c>
+      <c r="Q55" s="52">
+        <v>14310.509999999998</v>
+      </c>
+      <c r="R55" s="53">
+        <v>0.4217996319774624</v>
+      </c>
+      <c r="S55" s="54">
+        <v>679.42</v>
+      </c>
+      <c r="T55" s="54">
+        <v>413</v>
+      </c>
+      <c r="U55" s="54">
+        <v>266.41999999999996</v>
+      </c>
+      <c r="V55" s="53">
+        <v>0.39212858025963315</v>
+      </c>
       <c r="W55" s="53"/>
-      <c r="X55" s="55"/>
-      <c r="Y55" s="55"/>
-      <c r="Z55" s="53"/>
-      <c r="AA55" s="56"/>
+      <c r="X55" s="55">
+        <v>18.50767554479419</v>
+      </c>
+      <c r="Y55" s="55">
+        <v>67.18600078134293</v>
+      </c>
+      <c r="Z55" s="53">
+        <v>0.0776</v>
+      </c>
+      <c r="AA55" s="56">
+        <v>0.2954</v>
+      </c>
       <c r="AB55" s="57"/>
       <c r="AD55" s="35"/>
       <c r="AE55" s="35"/>
@@ -12549,30 +12681,74 @@
       <c r="C62" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D62" s="52"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="53"/>
-      <c r="H62" s="52"/>
-      <c r="I62" s="52"/>
-      <c r="J62" s="52"/>
-      <c r="K62" s="52"/>
-      <c r="L62" s="52"/>
-      <c r="M62" s="53"/>
+      <c r="D62" s="52">
+        <v>20420.56</v>
+      </c>
+      <c r="E62" s="52">
+        <v>16358.37</v>
+      </c>
+      <c r="F62" s="52">
+        <v>4062.1900000000005</v>
+      </c>
+      <c r="G62" s="53">
+        <v>0.19892647410257114</v>
+      </c>
+      <c r="H62" s="52">
+        <v>15859.68</v>
+      </c>
+      <c r="I62" s="52">
+        <v>13601.05</v>
+      </c>
+      <c r="J62" s="52">
+        <v>12689.1</v>
+      </c>
+      <c r="K62" s="52">
+        <v>11685.13</v>
+      </c>
+      <c r="L62" s="52">
+        <v>1003.9700000000012</v>
+      </c>
+      <c r="M62" s="53">
+        <v>0.07912066261594605</v>
+      </c>
       <c r="N62" s="53"/>
-      <c r="O62" s="52"/>
-      <c r="P62" s="52"/>
-      <c r="Q62" s="52"/>
-      <c r="R62" s="53"/>
-      <c r="S62" s="54"/>
-      <c r="T62" s="54"/>
-      <c r="U62" s="54"/>
-      <c r="V62" s="53"/>
+      <c r="O62" s="52">
+        <v>3170.58</v>
+      </c>
+      <c r="P62" s="52">
+        <v>1915.92</v>
+      </c>
+      <c r="Q62" s="52">
+        <v>1254.6599999999999</v>
+      </c>
+      <c r="R62" s="53">
+        <v>0.39571939518952365</v>
+      </c>
+      <c r="S62" s="54">
+        <v>63.5</v>
+      </c>
+      <c r="T62" s="54">
+        <v>47.5</v>
+      </c>
+      <c r="U62" s="54">
+        <v>16</v>
+      </c>
+      <c r="V62" s="53">
+        <v>0.25196850393700787</v>
+      </c>
       <c r="W62" s="53"/>
-      <c r="X62" s="55"/>
-      <c r="Y62" s="55"/>
-      <c r="Z62" s="53"/>
-      <c r="AA62" s="56"/>
+      <c r="X62" s="55">
+        <v>58.04884210526316</v>
+      </c>
+      <c r="Y62" s="55">
+        <v>71.82495570677168</v>
+      </c>
+      <c r="Z62" s="53">
+        <v>0.1686</v>
+      </c>
+      <c r="AA62" s="56">
+        <v>0.2233</v>
+      </c>
       <c r="AB62" s="57"/>
       <c r="AD62" s="35"/>
       <c r="AE62" s="35"/>
@@ -13213,30 +13389,74 @@
       <c r="C76" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D76" s="52"/>
-      <c r="E76" s="52"/>
-      <c r="F76" s="52"/>
-      <c r="G76" s="53"/>
-      <c r="H76" s="52"/>
-      <c r="I76" s="52"/>
-      <c r="J76" s="52"/>
-      <c r="K76" s="52"/>
-      <c r="L76" s="52"/>
-      <c r="M76" s="53"/>
+      <c r="D76" s="52">
+        <v>77166.16</v>
+      </c>
+      <c r="E76" s="52">
+        <v>0</v>
+      </c>
+      <c r="F76" s="52">
+        <v>77166.16</v>
+      </c>
+      <c r="G76" s="53">
+        <v>1</v>
+      </c>
+      <c r="H76" s="52">
+        <v>54302.66</v>
+      </c>
+      <c r="I76" s="52">
+        <v>22353.17</v>
+      </c>
+      <c r="J76" s="52">
+        <v>31383.390000000003</v>
+      </c>
+      <c r="K76" s="52">
+        <v>22353.17</v>
+      </c>
+      <c r="L76" s="52">
+        <v>9030.220000000005</v>
+      </c>
+      <c r="M76" s="53">
+        <v>0.28773883254804544</v>
+      </c>
       <c r="N76" s="53"/>
-      <c r="O76" s="52"/>
-      <c r="P76" s="52"/>
-      <c r="Q76" s="52"/>
-      <c r="R76" s="53"/>
-      <c r="S76" s="54"/>
-      <c r="T76" s="54"/>
-      <c r="U76" s="54"/>
-      <c r="V76" s="53"/>
+      <c r="O76" s="52">
+        <v>22919.27</v>
+      </c>
+      <c r="P76" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="52">
+        <v>22919.27</v>
+      </c>
+      <c r="R76" s="53">
+        <v>1</v>
+      </c>
+      <c r="S76" s="54">
+        <v>470.62</v>
+      </c>
+      <c r="T76" s="54">
+        <v>0</v>
+      </c>
+      <c r="U76" s="54">
+        <v>470.62</v>
+      </c>
+      <c r="V76" s="53">
+        <v>1</v>
+      </c>
       <c r="W76" s="53"/>
-      <c r="X76" s="55"/>
-      <c r="Y76" s="55"/>
-      <c r="Z76" s="53"/>
-      <c r="AA76" s="56"/>
+      <c r="X76" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y76" s="55">
+        <v>48.58165977967362</v>
+      </c>
+      <c r="Z76" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="56">
+        <v>0.2963</v>
+      </c>
       <c r="AB76" s="57"/>
       <c r="AD76" s="35"/>
       <c r="AE76" s="35"/>
@@ -13935,30 +14155,74 @@
       <c r="C90" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D90" s="67"/>
-      <c r="E90" s="67"/>
-      <c r="F90" s="52"/>
-      <c r="G90" s="53"/>
-      <c r="H90" s="52"/>
-      <c r="I90" s="52"/>
-      <c r="J90" s="52"/>
-      <c r="K90" s="52"/>
-      <c r="L90" s="52"/>
-      <c r="M90" s="53"/>
+      <c r="D90" s="67">
+        <v>37083.03</v>
+      </c>
+      <c r="E90" s="67">
+        <v>33023.07</v>
+      </c>
+      <c r="F90" s="52">
+        <v>4059.959999999999</v>
+      </c>
+      <c r="G90" s="53">
+        <v>0.10948296296176444</v>
+      </c>
+      <c r="H90" s="52">
+        <v>27002.93</v>
+      </c>
+      <c r="I90" s="52">
+        <v>25996.77</v>
+      </c>
+      <c r="J90" s="52">
+        <v>15440.32</v>
+      </c>
+      <c r="K90" s="52">
+        <v>15990.78</v>
+      </c>
+      <c r="L90" s="52">
+        <v>-550.460000000001</v>
+      </c>
+      <c r="M90" s="53">
+        <v>-0.0356508155271394</v>
+      </c>
       <c r="N90" s="53"/>
-      <c r="O90" s="52"/>
-      <c r="P90" s="52"/>
-      <c r="Q90" s="52"/>
-      <c r="R90" s="53"/>
-      <c r="S90" s="68"/>
-      <c r="T90" s="68"/>
-      <c r="U90" s="54"/>
-      <c r="V90" s="53"/>
+      <c r="O90" s="52">
+        <v>11562.61</v>
+      </c>
+      <c r="P90" s="52">
+        <v>10005.99</v>
+      </c>
+      <c r="Q90" s="52">
+        <v>1556.6200000000008</v>
+      </c>
+      <c r="R90" s="53">
+        <v>0.13462531383485224</v>
+      </c>
+      <c r="S90" s="68">
+        <v>231.75</v>
+      </c>
+      <c r="T90" s="68">
+        <v>204.75</v>
+      </c>
+      <c r="U90" s="54">
+        <v>27</v>
+      </c>
+      <c r="V90" s="53">
+        <v>0.11650485436893204</v>
+      </c>
       <c r="W90" s="53"/>
-      <c r="X90" s="55"/>
-      <c r="Y90" s="55"/>
-      <c r="Z90" s="53"/>
-      <c r="AA90" s="56"/>
+      <c r="X90" s="55">
+        <v>34.316483516483515</v>
+      </c>
+      <c r="Y90" s="55">
+        <v>43.49557070636461</v>
+      </c>
+      <c r="Z90" s="53">
+        <v>0.21280000000000002</v>
+      </c>
+      <c r="AA90" s="56">
+        <v>0.2718</v>
+      </c>
       <c r="AB90" s="57"/>
       <c r="AD90" s="35"/>
       <c r="AE90" s="35"/>
@@ -14617,30 +14881,74 @@
       <c r="C104" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D104" s="52"/>
-      <c r="E104" s="69"/>
-      <c r="F104" s="52"/>
-      <c r="G104" s="53"/>
-      <c r="H104" s="52"/>
-      <c r="I104" s="52"/>
-      <c r="J104" s="52"/>
-      <c r="K104" s="52"/>
-      <c r="L104" s="52"/>
-      <c r="M104" s="53"/>
+      <c r="D104" s="52">
+        <v>32473.02</v>
+      </c>
+      <c r="E104" s="69">
+        <v>33188.03</v>
+      </c>
+      <c r="F104" s="52">
+        <v>-715.0099999999984</v>
+      </c>
+      <c r="G104" s="53">
+        <v>-0.022018586506582952</v>
+      </c>
+      <c r="H104" s="52">
+        <v>23075.07</v>
+      </c>
+      <c r="I104" s="52">
+        <v>31131.57</v>
+      </c>
+      <c r="J104" s="52">
+        <v>12691.21</v>
+      </c>
+      <c r="K104" s="52">
+        <v>15390.63</v>
+      </c>
+      <c r="L104" s="52">
+        <v>-2699.42</v>
+      </c>
+      <c r="M104" s="53">
+        <v>-0.21269997108234756</v>
+      </c>
       <c r="N104" s="53"/>
-      <c r="O104" s="52"/>
-      <c r="P104" s="52"/>
-      <c r="Q104" s="52"/>
-      <c r="R104" s="53"/>
-      <c r="S104" s="54"/>
-      <c r="T104" s="54"/>
-      <c r="U104" s="54"/>
-      <c r="V104" s="53"/>
+      <c r="O104" s="52">
+        <v>10383.86</v>
+      </c>
+      <c r="P104" s="52">
+        <v>15740.94</v>
+      </c>
+      <c r="Q104" s="52">
+        <v>-5357.08</v>
+      </c>
+      <c r="R104" s="53">
+        <v>-0.5159044902377343</v>
+      </c>
+      <c r="S104" s="54">
+        <v>208.2</v>
+      </c>
+      <c r="T104" s="54">
+        <v>317.25</v>
+      </c>
+      <c r="U104" s="54">
+        <v>-109.05000000000001</v>
+      </c>
+      <c r="V104" s="53">
+        <v>-0.5237752161383286</v>
+      </c>
       <c r="W104" s="53"/>
-      <c r="X104" s="55"/>
-      <c r="Y104" s="55"/>
-      <c r="Z104" s="53"/>
-      <c r="AA104" s="56"/>
+      <c r="X104" s="55">
+        <v>6.482143420015761</v>
+      </c>
+      <c r="Y104" s="55">
+        <v>45.139084580403456</v>
+      </c>
+      <c r="Z104" s="53">
+        <v>0.062</v>
+      </c>
+      <c r="AA104" s="56">
+        <v>0.2894</v>
+      </c>
       <c r="AB104" s="57"/>
       <c r="AD104" s="35"/>
       <c r="AE104" s="35"/>
@@ -14982,30 +15290,74 @@
       <c r="C111" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D111" s="52"/>
-      <c r="E111" s="52"/>
-      <c r="F111" s="52"/>
-      <c r="G111" s="53"/>
-      <c r="H111" s="52"/>
-      <c r="I111" s="52"/>
-      <c r="J111" s="52"/>
-      <c r="K111" s="52"/>
-      <c r="L111" s="52"/>
-      <c r="M111" s="53"/>
+      <c r="D111" s="52">
+        <v>58902.56</v>
+      </c>
+      <c r="E111" s="52">
+        <v>0</v>
+      </c>
+      <c r="F111" s="52">
+        <v>58902.56</v>
+      </c>
+      <c r="G111" s="53">
+        <v>1</v>
+      </c>
+      <c r="H111" s="52">
+        <v>37601.88</v>
+      </c>
+      <c r="I111" s="52">
+        <v>38195.76</v>
+      </c>
+      <c r="J111" s="52">
+        <v>21415.85</v>
+      </c>
+      <c r="K111" s="52">
+        <v>19158.27</v>
+      </c>
+      <c r="L111" s="52">
+        <v>2257.579999999998</v>
+      </c>
+      <c r="M111" s="53">
+        <v>0.10541631548596009</v>
+      </c>
       <c r="N111" s="53"/>
-      <c r="O111" s="52"/>
-      <c r="P111" s="52"/>
-      <c r="Q111" s="52"/>
-      <c r="R111" s="53"/>
-      <c r="S111" s="54"/>
-      <c r="T111" s="54"/>
-      <c r="U111" s="54"/>
-      <c r="V111" s="53"/>
+      <c r="O111" s="52">
+        <v>16186.03</v>
+      </c>
+      <c r="P111" s="52">
+        <v>19037.49</v>
+      </c>
+      <c r="Q111" s="52">
+        <v>-2851.460000000001</v>
+      </c>
+      <c r="R111" s="53">
+        <v>-0.1761679670678975</v>
+      </c>
+      <c r="S111" s="54">
+        <v>324.19</v>
+      </c>
+      <c r="T111" s="54">
+        <v>412.5</v>
+      </c>
+      <c r="U111" s="54">
+        <v>-88.31</v>
+      </c>
+      <c r="V111" s="53">
+        <v>-0.2724019864894044</v>
+      </c>
       <c r="W111" s="53"/>
-      <c r="X111" s="55"/>
-      <c r="Y111" s="55"/>
-      <c r="Z111" s="53"/>
-      <c r="AA111" s="56"/>
+      <c r="X111" s="55">
+        <v>-6.6456484848484845</v>
+      </c>
+      <c r="Y111" s="55">
+        <v>65.70431400737223</v>
+      </c>
+      <c r="Z111" s="53">
+        <v>-0.07730000000000001</v>
+      </c>
+      <c r="AA111" s="56">
+        <v>0.3616</v>
+      </c>
       <c r="AB111" s="57"/>
       <c r="AD111" s="35"/>
       <c r="AE111" s="35"/>
@@ -15670,32 +16022,74 @@
       <c r="C125" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D125" s="52"/>
-      <c r="E125" s="52"/>
+      <c r="D125" s="52">
+        <v>99768.39</v>
+      </c>
+      <c r="E125" s="52">
+        <v>15366.74</v>
+      </c>
       <c r="F125" s="52">
-        <v>0</v>
-      </c>
-      <c r="G125" s="53"/>
-      <c r="H125" s="52"/>
-      <c r="I125" s="52"/>
-      <c r="J125" s="52"/>
-      <c r="K125" s="52"/>
-      <c r="L125" s="52"/>
-      <c r="M125" s="53"/>
+        <v>84401.65</v>
+      </c>
+      <c r="G125" s="53">
+        <v>0.8459758647002321</v>
+      </c>
+      <c r="H125" s="52">
+        <v>81719.58</v>
+      </c>
+      <c r="I125" s="52">
+        <v>18551.86</v>
+      </c>
+      <c r="J125" s="52">
+        <v>67238.96</v>
+      </c>
+      <c r="K125" s="52">
+        <v>14369.1</v>
+      </c>
+      <c r="L125" s="52">
+        <v>52869.86000000001</v>
+      </c>
+      <c r="M125" s="53">
+        <v>0.7862980034194461</v>
+      </c>
       <c r="N125" s="53"/>
-      <c r="O125" s="52"/>
-      <c r="P125" s="52"/>
-      <c r="Q125" s="52"/>
-      <c r="R125" s="53"/>
-      <c r="S125" s="54"/>
-      <c r="T125" s="54"/>
-      <c r="U125" s="54"/>
-      <c r="V125" s="53"/>
+      <c r="O125" s="52">
+        <v>14480.62</v>
+      </c>
+      <c r="P125" s="52">
+        <v>4182.76</v>
+      </c>
+      <c r="Q125" s="52">
+        <v>10297.86</v>
+      </c>
+      <c r="R125" s="53">
+        <v>0.7111477271000828</v>
+      </c>
+      <c r="S125" s="54">
+        <v>290.15</v>
+      </c>
+      <c r="T125" s="54">
+        <v>91.75</v>
+      </c>
+      <c r="U125" s="54">
+        <v>198.39999999999998</v>
+      </c>
+      <c r="V125" s="53">
+        <v>0.6837842495261072</v>
+      </c>
       <c r="W125" s="53"/>
-      <c r="X125" s="55"/>
-      <c r="Y125" s="55"/>
-      <c r="Z125" s="53"/>
-      <c r="AA125" s="56"/>
+      <c r="X125" s="55">
+        <v>-34.715204359673024</v>
+      </c>
+      <c r="Y125" s="55">
+        <v>62.2051177714286</v>
+      </c>
+      <c r="Z125" s="53">
+        <v>-0.2073</v>
+      </c>
+      <c r="AA125" s="56">
+        <v>0.1809</v>
+      </c>
       <c r="AB125" s="57"/>
       <c r="AD125" s="35"/>
       <c r="AE125" s="35"/>
@@ -16357,30 +16751,74 @@
       <c r="C139" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D139" s="52"/>
-      <c r="E139" s="52"/>
-      <c r="F139" s="52"/>
-      <c r="G139" s="53"/>
-      <c r="H139" s="52"/>
-      <c r="I139" s="52"/>
-      <c r="J139" s="52"/>
-      <c r="K139" s="52"/>
-      <c r="L139" s="52"/>
-      <c r="M139" s="53"/>
+      <c r="D139" s="52">
+        <v>30749.24</v>
+      </c>
+      <c r="E139" s="52">
+        <v>30749.24</v>
+      </c>
+      <c r="F139" s="52">
+        <v>0</v>
+      </c>
+      <c r="G139" s="53">
+        <v>0</v>
+      </c>
+      <c r="H139" s="52">
+        <v>22587.89</v>
+      </c>
+      <c r="I139" s="52">
+        <v>25550.31</v>
+      </c>
+      <c r="J139" s="52">
+        <v>12565.06</v>
+      </c>
+      <c r="K139" s="52">
+        <v>11750.840000000002</v>
+      </c>
+      <c r="L139" s="52">
+        <v>814.2199999999975</v>
+      </c>
+      <c r="M139" s="53">
+        <v>0.06480032725669416</v>
+      </c>
       <c r="N139" s="53"/>
-      <c r="O139" s="52"/>
-      <c r="P139" s="52"/>
-      <c r="Q139" s="52"/>
-      <c r="R139" s="53"/>
-      <c r="S139" s="54"/>
-      <c r="T139" s="54"/>
-      <c r="U139" s="54"/>
-      <c r="V139" s="53"/>
+      <c r="O139" s="52">
+        <v>10022.83</v>
+      </c>
+      <c r="P139" s="52">
+        <v>13799.47</v>
+      </c>
+      <c r="Q139" s="52">
+        <v>-3776.6399999999994</v>
+      </c>
+      <c r="R139" s="53">
+        <v>-0.37680375702271707</v>
+      </c>
+      <c r="S139" s="54">
+        <v>200.82</v>
+      </c>
+      <c r="T139" s="54">
+        <v>278.25</v>
+      </c>
+      <c r="U139" s="54">
+        <v>-77.43</v>
+      </c>
+      <c r="V139" s="53">
+        <v>-0.3855691664176875</v>
+      </c>
       <c r="W139" s="53"/>
-      <c r="X139" s="55"/>
-      <c r="Y139" s="55"/>
-      <c r="Z139" s="53"/>
-      <c r="AA139" s="56"/>
+      <c r="X139" s="55">
+        <v>18.68438454627134</v>
+      </c>
+      <c r="Y139" s="55">
+        <v>40.64013272149188</v>
+      </c>
+      <c r="Z139" s="53">
+        <v>0.1691</v>
+      </c>
+      <c r="AA139" s="56">
+        <v>0.2654</v>
+      </c>
       <c r="AB139" s="57"/>
       <c r="AD139" s="35"/>
       <c r="AE139" s="35"/>
@@ -18014,32 +18452,74 @@
       <c r="C174" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D174" s="52"/>
-      <c r="E174" s="52"/>
-      <c r="F174" s="52"/>
-      <c r="G174" s="53"/>
-      <c r="H174" s="52"/>
-      <c r="I174" s="52"/>
-      <c r="J174" s="52"/>
+      <c r="D174" s="52">
+        <v>146237.11</v>
+      </c>
+      <c r="E174" s="52">
+        <v>94266.45</v>
+      </c>
+      <c r="F174" s="52">
+        <v>51970.65999999999</v>
+      </c>
+      <c r="G174" s="53">
+        <v>0.355386262761894</v>
+      </c>
+      <c r="H174" s="52">
+        <v>114651.87</v>
+      </c>
+      <c r="I174" s="52">
+        <v>95876.35</v>
+      </c>
+      <c r="J174" s="52">
+        <v>82888.07999999999</v>
+      </c>
       <c r="K174" s="52">
-        <v>0</v>
-      </c>
-      <c r="L174" s="52"/>
-      <c r="M174" s="53"/>
+        <v>74503.91</v>
+      </c>
+      <c r="L174" s="52">
+        <v>8384.169999999984</v>
+      </c>
+      <c r="M174" s="53">
+        <v>0.10115049112007402</v>
+      </c>
       <c r="N174" s="53"/>
-      <c r="O174" s="52"/>
-      <c r="P174" s="52"/>
-      <c r="Q174" s="52"/>
-      <c r="R174" s="53"/>
-      <c r="S174" s="54"/>
-      <c r="T174" s="54"/>
-      <c r="U174" s="54"/>
-      <c r="V174" s="53"/>
+      <c r="O174" s="52">
+        <v>31763.79</v>
+      </c>
+      <c r="P174" s="52">
+        <v>21372.44</v>
+      </c>
+      <c r="Q174" s="52">
+        <v>10391.350000000002</v>
+      </c>
+      <c r="R174" s="53">
+        <v>0.32714452525973764</v>
+      </c>
+      <c r="S174" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T174" s="54">
+        <v>430</v>
+      </c>
+      <c r="U174" s="54">
+        <v>229.73000000000002</v>
+      </c>
+      <c r="V174" s="53">
+        <v>0.34821821048004487</v>
+      </c>
       <c r="W174" s="53"/>
-      <c r="X174" s="55"/>
-      <c r="Y174" s="55"/>
-      <c r="Z174" s="53"/>
-      <c r="AA174" s="56"/>
+      <c r="X174" s="55">
+        <v>-3.7439534883720933</v>
+      </c>
+      <c r="Y174" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z174" s="53">
+        <v>-0.0171</v>
+      </c>
+      <c r="AA174" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB174" s="57"/>
       <c r="AD174" s="35"/>
       <c r="AE174" s="35"/>
@@ -20269,34 +20749,74 @@
       <c r="C222" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="D222" s="52"/>
-      <c r="E222" s="52"/>
-      <c r="F222" s="52"/>
-      <c r="G222" s="53"/>
-      <c r="H222" s="52"/>
-      <c r="I222" s="52"/>
+      <c r="D222" s="52">
+        <v>389318.35</v>
+      </c>
+      <c r="E222" s="52">
+        <v>271388.15</v>
+      </c>
+      <c r="F222" s="52">
+        <v>117930.19999999995</v>
+      </c>
+      <c r="G222" s="53">
+        <v>0.3029145685015874</v>
+      </c>
+      <c r="H222" s="52">
+        <v>289549.48</v>
+      </c>
+      <c r="I222" s="52">
+        <v>228314.4</v>
+      </c>
       <c r="J222" s="52">
-        <v>0</v>
+        <v>174279.97999999998</v>
       </c>
       <c r="K222" s="52">
-        <v>0</v>
-      </c>
-      <c r="L222" s="52"/>
-      <c r="M222" s="53"/>
+        <v>175133.49</v>
+      </c>
+      <c r="L222" s="52">
+        <v>-853.5100000000093</v>
+      </c>
+      <c r="M222" s="53">
+        <v>-0.004897349655422324</v>
+      </c>
       <c r="N222" s="53"/>
-      <c r="O222" s="52"/>
-      <c r="P222" s="52"/>
-      <c r="Q222" s="52"/>
-      <c r="R222" s="53"/>
-      <c r="S222" s="54"/>
-      <c r="T222" s="54"/>
-      <c r="U222" s="54"/>
-      <c r="V222" s="53"/>
+      <c r="O222" s="52">
+        <v>115269.5</v>
+      </c>
+      <c r="P222" s="52">
+        <v>53180.91</v>
+      </c>
+      <c r="Q222" s="52">
+        <v>62088.59</v>
+      </c>
+      <c r="R222" s="53">
+        <v>0.5386384950051835</v>
+      </c>
+      <c r="S222" s="54">
+        <v>2312.68</v>
+      </c>
+      <c r="T222" s="54">
+        <v>1120.5</v>
+      </c>
+      <c r="U222" s="54">
+        <v>1192.1799999999998</v>
+      </c>
+      <c r="V222" s="53">
+        <v>0.5154971721120085</v>
+      </c>
       <c r="W222" s="53"/>
-      <c r="X222" s="55"/>
-      <c r="Y222" s="55"/>
-      <c r="Z222" s="53"/>
-      <c r="AA222" s="56"/>
+      <c r="X222" s="55">
+        <v>38.441543953592145</v>
+      </c>
+      <c r="Y222" s="55">
+        <v>43.1399392286741</v>
+      </c>
+      <c r="Z222" s="53">
+        <v>0.15869999999999998</v>
+      </c>
+      <c r="AA222" s="56">
+        <v>0.2563</v>
+      </c>
       <c r="AB222" s="57"/>
       <c r="AD222" s="35" t="s">
         <v>93</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-18T21:26:41Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9721,30 +9721,74 @@
       <c r="C7" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="52"/>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="52"/>
-      <c r="L7" s="52"/>
-      <c r="M7" s="53"/>
+      <c r="D7" s="52">
+        <v>233882.27</v>
+      </c>
+      <c r="E7" s="52">
+        <v>205915.9</v>
+      </c>
+      <c r="F7" s="52">
+        <v>27966.369999999995</v>
+      </c>
+      <c r="G7" s="53">
+        <v>0.1195745620221661</v>
+      </c>
+      <c r="H7" s="52">
+        <v>199128.99</v>
+      </c>
+      <c r="I7" s="52">
+        <v>165210.04</v>
+      </c>
+      <c r="J7" s="52">
+        <v>172860.11</v>
+      </c>
+      <c r="K7" s="52">
+        <v>137410.69</v>
+      </c>
+      <c r="L7" s="52">
+        <v>35449.419999999984</v>
+      </c>
+      <c r="M7" s="53">
+        <v>0.20507576907130273</v>
+      </c>
       <c r="N7" s="53"/>
-      <c r="O7" s="52"/>
-      <c r="P7" s="52"/>
-      <c r="Q7" s="52"/>
-      <c r="R7" s="53"/>
-      <c r="S7" s="54"/>
-      <c r="T7" s="54"/>
-      <c r="U7" s="54"/>
-      <c r="V7" s="53"/>
+      <c r="O7" s="52">
+        <v>26268.88</v>
+      </c>
+      <c r="P7" s="52">
+        <v>27799.35</v>
+      </c>
+      <c r="Q7" s="52">
+        <v>-1530.4699999999975</v>
+      </c>
+      <c r="R7" s="53">
+        <v>-0.05826171500269511</v>
+      </c>
+      <c r="S7" s="54">
+        <v>530.95</v>
+      </c>
+      <c r="T7" s="54">
+        <v>556.5</v>
+      </c>
+      <c r="U7" s="54">
+        <v>-25.549999999999955</v>
+      </c>
+      <c r="V7" s="53">
+        <v>-0.04812129202373096</v>
+      </c>
       <c r="W7" s="53"/>
-      <c r="X7" s="55"/>
-      <c r="Y7" s="55"/>
-      <c r="Z7" s="53"/>
-      <c r="AA7" s="56"/>
+      <c r="X7" s="55">
+        <v>73.14619946091645</v>
+      </c>
+      <c r="Y7" s="55">
+        <v>65.45490166985587</v>
+      </c>
+      <c r="Z7" s="53">
+        <v>0.1977</v>
+      </c>
+      <c r="AA7" s="56">
+        <v>0.1486</v>
+      </c>
       <c r="AB7" s="57"/>
       <c r="AD7" s="35" t="s">
         <v>96</v>
@@ -21674,7 +21718,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="52">
-        <v>48113.58</v>
+        <v>51687.05</v>
       </c>
       <c r="E4" s="52">
         <f>C4-D4</f>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-18T21:30:19Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9737,54 +9737,54 @@
         <v>199128.99</v>
       </c>
       <c r="I7" s="52">
-        <v>165210.04</v>
+        <v>164808.35</v>
       </c>
       <c r="J7" s="52">
         <v>172860.11</v>
       </c>
       <c r="K7" s="52">
-        <v>137410.69</v>
+        <v>137510.76</v>
       </c>
       <c r="L7" s="52">
-        <v>35449.419999999984</v>
+        <v>35349.34999999998</v>
       </c>
       <c r="M7" s="53">
-        <v>0.20507576907130273</v>
+        <v>0.20449686165304407</v>
       </c>
       <c r="N7" s="53"/>
       <c r="O7" s="52">
         <v>26268.88</v>
       </c>
       <c r="P7" s="52">
-        <v>27799.35</v>
+        <v>27297.59</v>
       </c>
       <c r="Q7" s="52">
-        <v>-1530.4699999999975</v>
+        <v>-1028.7099999999991</v>
       </c>
       <c r="R7" s="53">
-        <v>-0.05826171500269511</v>
+        <v>-0.03916078645149695</v>
       </c>
       <c r="S7" s="54">
         <v>530.95</v>
       </c>
       <c r="T7" s="54">
-        <v>556.5</v>
+        <v>548</v>
       </c>
       <c r="U7" s="54">
-        <v>-25.549999999999955</v>
+        <v>-17.049999999999955</v>
       </c>
       <c r="V7" s="53">
-        <v>-0.04812129202373096</v>
+        <v>-0.032112251624446655</v>
       </c>
       <c r="W7" s="53"/>
       <c r="X7" s="55">
-        <v>73.14619946091645</v>
+        <v>75.01377737226278</v>
       </c>
       <c r="Y7" s="55">
         <v>65.45490166985587</v>
       </c>
       <c r="Z7" s="53">
-        <v>0.1977</v>
+        <v>0.1996</v>
       </c>
       <c r="AA7" s="56">
         <v>0.1486</v>
@@ -10128,30 +10128,74 @@
       <c r="C14" s="63" t="s">
         <v>95</v>
       </c>
-      <c r="D14" s="52"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="52"/>
-      <c r="G14" s="53"/>
-      <c r="H14" s="52"/>
-      <c r="I14" s="52"/>
-      <c r="J14" s="52"/>
-      <c r="K14" s="52"/>
-      <c r="L14" s="52"/>
-      <c r="M14" s="53"/>
+      <c r="D14" s="52">
+        <v>129074.86</v>
+      </c>
+      <c r="E14" s="62">
+        <v>55068.11</v>
+      </c>
+      <c r="F14" s="52">
+        <v>74006.75</v>
+      </c>
+      <c r="G14" s="53">
+        <v>0.5733630081024299</v>
+      </c>
+      <c r="H14" s="52">
+        <v>101420.72</v>
+      </c>
+      <c r="I14" s="52">
+        <v>55851.96</v>
+      </c>
+      <c r="J14" s="52">
+        <v>83645.65</v>
+      </c>
+      <c r="K14" s="52">
+        <v>51392.88</v>
+      </c>
+      <c r="L14" s="52">
+        <v>32252.769999999997</v>
+      </c>
+      <c r="M14" s="53">
+        <v>0.3855881327959075</v>
+      </c>
       <c r="N14" s="53"/>
-      <c r="O14" s="52"/>
-      <c r="P14" s="52"/>
-      <c r="Q14" s="52"/>
-      <c r="R14" s="53"/>
-      <c r="S14" s="54"/>
-      <c r="T14" s="54"/>
-      <c r="U14" s="54"/>
-      <c r="V14" s="53"/>
+      <c r="O14" s="52">
+        <v>17775.07</v>
+      </c>
+      <c r="P14" s="52">
+        <v>4459.08</v>
+      </c>
+      <c r="Q14" s="52">
+        <v>13315.99</v>
+      </c>
+      <c r="R14" s="53">
+        <v>0.7491385406639749</v>
+      </c>
+      <c r="S14" s="54">
+        <v>356.07</v>
+      </c>
+      <c r="T14" s="54">
+        <v>90.75</v>
+      </c>
+      <c r="U14" s="54">
+        <v>265.32</v>
+      </c>
+      <c r="V14" s="53">
+        <v>0.7451343836886005</v>
+      </c>
       <c r="W14" s="53"/>
-      <c r="X14" s="55"/>
-      <c r="Y14" s="55"/>
-      <c r="Z14" s="53"/>
-      <c r="AA14" s="56"/>
+      <c r="X14" s="55">
+        <v>-8.637465564738292</v>
+      </c>
+      <c r="Y14" s="55">
+        <v>77.66490997775718</v>
+      </c>
+      <c r="Z14" s="53">
+        <v>-0.014199999999999999</v>
+      </c>
+      <c r="AA14" s="56">
+        <v>0.2142</v>
+      </c>
       <c r="AB14" s="57"/>
       <c r="AD14" s="35" t="s">
         <v>96</v>
@@ -10447,30 +10491,74 @@
       <c r="C21" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D21" s="52"/>
-      <c r="E21" s="52"/>
-      <c r="F21" s="52"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="52"/>
-      <c r="I21" s="52"/>
-      <c r="J21" s="52"/>
-      <c r="K21" s="52"/>
-      <c r="L21" s="52"/>
-      <c r="M21" s="53"/>
+      <c r="D21" s="52">
+        <v>27500.32</v>
+      </c>
+      <c r="E21" s="52">
+        <v>6999.08</v>
+      </c>
+      <c r="F21" s="52">
+        <v>20501.239999999998</v>
+      </c>
+      <c r="G21" s="53">
+        <v>0.74549096155972</v>
+      </c>
+      <c r="H21" s="52">
+        <v>19565.83</v>
+      </c>
+      <c r="I21" s="52">
+        <v>7621.92</v>
+      </c>
+      <c r="J21" s="52">
+        <v>13767.340000000002</v>
+      </c>
+      <c r="K21" s="52">
+        <v>5911.24</v>
+      </c>
+      <c r="L21" s="52">
+        <v>7856.100000000002</v>
+      </c>
+      <c r="M21" s="53">
+        <v>0.5706331070490016</v>
+      </c>
       <c r="N21" s="53"/>
-      <c r="O21" s="52"/>
-      <c r="P21" s="52"/>
-      <c r="Q21" s="52"/>
-      <c r="R21" s="53"/>
-      <c r="S21" s="54"/>
-      <c r="T21" s="54"/>
-      <c r="U21" s="54"/>
-      <c r="V21" s="53"/>
+      <c r="O21" s="52">
+        <v>5798.49</v>
+      </c>
+      <c r="P21" s="52">
+        <v>1710.68</v>
+      </c>
+      <c r="Q21" s="52">
+        <v>4087.8099999999995</v>
+      </c>
+      <c r="R21" s="53">
+        <v>0.7049783650571096</v>
+      </c>
+      <c r="S21" s="54">
+        <v>125.39</v>
+      </c>
+      <c r="T21" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U21" s="54">
+        <v>90.64</v>
+      </c>
+      <c r="V21" s="53">
+        <v>0.7228646622537682</v>
+      </c>
       <c r="W21" s="53"/>
-      <c r="X21" s="55"/>
-      <c r="Y21" s="55"/>
-      <c r="Z21" s="53"/>
-      <c r="AA21" s="56"/>
+      <c r="X21" s="55">
+        <v>-17.923453237410072</v>
+      </c>
+      <c r="Y21" s="55">
+        <v>63.27846478985563</v>
+      </c>
+      <c r="Z21" s="53">
+        <v>-0.08900000000000001</v>
+      </c>
+      <c r="AA21" s="56">
+        <v>0.2885</v>
+      </c>
       <c r="AB21" s="57"/>
       <c r="AD21" s="35" t="s">
         <v>96</v>
@@ -10812,30 +10900,74 @@
       <c r="C28" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D28" s="55"/>
-      <c r="E28" s="55"/>
-      <c r="F28" s="52"/>
-      <c r="G28" s="53"/>
-      <c r="H28" s="52"/>
-      <c r="I28" s="52"/>
-      <c r="J28" s="52"/>
-      <c r="K28" s="52"/>
-      <c r="L28" s="52"/>
-      <c r="M28" s="53"/>
+      <c r="D28" s="55">
+        <v>150850.82</v>
+      </c>
+      <c r="E28" s="55">
+        <v>111983.72</v>
+      </c>
+      <c r="F28" s="52">
+        <v>38867.100000000006</v>
+      </c>
+      <c r="G28" s="53">
+        <v>0.25765256032416667</v>
+      </c>
+      <c r="H28" s="52">
+        <v>102178.42</v>
+      </c>
+      <c r="I28" s="52">
+        <v>84545.62</v>
+      </c>
+      <c r="J28" s="52">
+        <v>62464.86</v>
+      </c>
+      <c r="K28" s="52">
+        <v>58627.5</v>
+      </c>
+      <c r="L28" s="52">
+        <v>3837.3600000000006</v>
+      </c>
+      <c r="M28" s="53">
+        <v>0.06143229969618119</v>
+      </c>
       <c r="N28" s="53"/>
-      <c r="O28" s="52"/>
-      <c r="P28" s="52"/>
-      <c r="Q28" s="52"/>
-      <c r="R28" s="53"/>
-      <c r="S28" s="54"/>
-      <c r="T28" s="54"/>
-      <c r="U28" s="54"/>
-      <c r="V28" s="53"/>
+      <c r="O28" s="52">
+        <v>39713.56</v>
+      </c>
+      <c r="P28" s="52">
+        <v>25918.12</v>
+      </c>
+      <c r="Q28" s="52">
+        <v>13795.439999999999</v>
+      </c>
+      <c r="R28" s="53">
+        <v>0.34737354193378783</v>
+      </c>
+      <c r="S28" s="54">
+        <v>795.22</v>
+      </c>
+      <c r="T28" s="54">
+        <v>531.25</v>
+      </c>
+      <c r="U28" s="54">
+        <v>263.97</v>
+      </c>
+      <c r="V28" s="53">
+        <v>0.33194587661276126</v>
+      </c>
       <c r="W28" s="53"/>
-      <c r="X28" s="55"/>
-      <c r="Y28" s="55"/>
-      <c r="Z28" s="53"/>
-      <c r="AA28" s="56"/>
+      <c r="X28" s="55">
+        <v>51.648188235294114</v>
+      </c>
+      <c r="Y28" s="55">
+        <v>61.20621468124544</v>
+      </c>
+      <c r="Z28" s="53">
+        <v>0.245</v>
+      </c>
+      <c r="AA28" s="56">
+        <v>0.3227</v>
+      </c>
       <c r="AB28" s="57"/>
       <c r="AD28" s="35" t="s">
         <v>96</v>
@@ -11175,30 +11307,74 @@
       <c r="C35" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="53"/>
-      <c r="H35" s="52"/>
-      <c r="I35" s="65"/>
-      <c r="J35" s="52"/>
-      <c r="K35" s="52"/>
-      <c r="L35" s="52"/>
-      <c r="M35" s="53"/>
+      <c r="D35" s="52">
+        <v>396422.03</v>
+      </c>
+      <c r="E35" s="52">
+        <v>176161.65</v>
+      </c>
+      <c r="F35" s="52">
+        <v>220260.38000000003</v>
+      </c>
+      <c r="G35" s="53">
+        <v>0.5556209376153994</v>
+      </c>
+      <c r="H35" s="52">
+        <v>327431.12</v>
+      </c>
+      <c r="I35" s="65">
+        <v>150094.16</v>
+      </c>
+      <c r="J35" s="52">
+        <v>271519.78</v>
+      </c>
+      <c r="K35" s="52">
+        <v>132259.14</v>
+      </c>
+      <c r="L35" s="52">
+        <v>139260.64</v>
+      </c>
+      <c r="M35" s="53">
+        <v>0.5128931674885712</v>
+      </c>
       <c r="N35" s="53"/>
-      <c r="O35" s="52"/>
-      <c r="P35" s="52"/>
-      <c r="Q35" s="52"/>
-      <c r="R35" s="53"/>
-      <c r="S35" s="54"/>
-      <c r="T35" s="54"/>
-      <c r="U35" s="54"/>
-      <c r="V35" s="53"/>
+      <c r="O35" s="52">
+        <v>55911.34</v>
+      </c>
+      <c r="P35" s="52">
+        <v>17835.02</v>
+      </c>
+      <c r="Q35" s="52">
+        <v>38076.31999999999</v>
+      </c>
+      <c r="R35" s="53">
+        <v>0.6810124743924935</v>
+      </c>
+      <c r="S35" s="54">
+        <v>1120.27</v>
+      </c>
+      <c r="T35" s="54">
+        <v>416.25</v>
+      </c>
+      <c r="U35" s="54">
+        <v>704.02</v>
+      </c>
+      <c r="V35" s="53">
+        <v>0.6284377873191285</v>
+      </c>
       <c r="W35" s="53"/>
-      <c r="X35" s="55"/>
-      <c r="Y35" s="55"/>
-      <c r="Z35" s="53"/>
-      <c r="AA35" s="56"/>
+      <c r="X35" s="55">
+        <v>62.6246006006006</v>
+      </c>
+      <c r="Y35" s="55">
+        <v>61.5841822414239</v>
+      </c>
+      <c r="Z35" s="53">
+        <v>0.14800000000000002</v>
+      </c>
+      <c r="AA35" s="56">
+        <v>0.174</v>
+      </c>
       <c r="AB35" s="57"/>
       <c r="AD35" s="35" t="s">
         <v>96</v>
@@ -11582,30 +11758,74 @@
       <c r="C42" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D42" s="52"/>
-      <c r="E42" s="52"/>
-      <c r="F42" s="52"/>
-      <c r="G42" s="53"/>
-      <c r="H42" s="52"/>
-      <c r="I42" s="52"/>
-      <c r="J42" s="52"/>
-      <c r="K42" s="52"/>
-      <c r="L42" s="52"/>
-      <c r="M42" s="53"/>
+      <c r="D42" s="52">
+        <v>128258.5</v>
+      </c>
+      <c r="E42" s="52">
+        <v>36398.39</v>
+      </c>
+      <c r="F42" s="52">
+        <v>91860.11</v>
+      </c>
+      <c r="G42" s="53">
+        <v>0.7162106994858041</v>
+      </c>
+      <c r="H42" s="52">
+        <v>94098.32</v>
+      </c>
+      <c r="I42" s="52">
+        <v>34659.62</v>
+      </c>
+      <c r="J42" s="52">
+        <v>69042.09000000001</v>
+      </c>
+      <c r="K42" s="52">
+        <v>28340.06</v>
+      </c>
+      <c r="L42" s="52">
+        <v>40702.03000000001</v>
+      </c>
+      <c r="M42" s="53">
+        <v>0.5895248825752524</v>
+      </c>
       <c r="N42" s="53"/>
-      <c r="O42" s="52"/>
-      <c r="P42" s="52"/>
-      <c r="Q42" s="52"/>
-      <c r="R42" s="53"/>
-      <c r="S42" s="54"/>
-      <c r="T42" s="54"/>
-      <c r="U42" s="54"/>
-      <c r="V42" s="53"/>
+      <c r="O42" s="52">
+        <v>25056.23</v>
+      </c>
+      <c r="P42" s="52">
+        <v>6319.56</v>
+      </c>
+      <c r="Q42" s="52">
+        <v>18736.67</v>
+      </c>
+      <c r="R42" s="53">
+        <v>0.7477848822428593</v>
+      </c>
+      <c r="S42" s="54">
+        <v>501.83</v>
+      </c>
+      <c r="T42" s="54">
+        <v>123.75</v>
+      </c>
+      <c r="U42" s="54">
+        <v>378.08</v>
+      </c>
+      <c r="V42" s="53">
+        <v>0.7534025466791543</v>
+      </c>
       <c r="W42" s="53"/>
-      <c r="X42" s="55"/>
-      <c r="Y42" s="55"/>
-      <c r="Z42" s="53"/>
-      <c r="AA42" s="56"/>
+      <c r="X42" s="55">
+        <v>14.050666666666666</v>
+      </c>
+      <c r="Y42" s="55">
+        <v>68.07122423898531</v>
+      </c>
+      <c r="Z42" s="53">
+        <v>0.0478</v>
+      </c>
+      <c r="AA42" s="56">
+        <v>0.2663</v>
+      </c>
       <c r="AB42" s="57"/>
       <c r="AD42" s="35" t="s">
         <v>96</v>
@@ -11991,30 +12211,74 @@
       <c r="C49" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D49" s="52"/>
-      <c r="E49" s="52"/>
-      <c r="F49" s="52"/>
-      <c r="G49" s="53"/>
-      <c r="H49" s="52"/>
-      <c r="I49" s="52"/>
-      <c r="J49" s="52"/>
-      <c r="K49" s="52"/>
-      <c r="L49" s="52"/>
-      <c r="M49" s="53"/>
+      <c r="D49" s="52">
+        <v>65693.36</v>
+      </c>
+      <c r="E49" s="52">
+        <v>25322.07</v>
+      </c>
+      <c r="F49" s="52">
+        <v>40371.29</v>
+      </c>
+      <c r="G49" s="53">
+        <v>0.6145414087512041</v>
+      </c>
+      <c r="H49" s="52">
+        <v>50582.37</v>
+      </c>
+      <c r="I49" s="52">
+        <v>25131.9</v>
+      </c>
+      <c r="J49" s="52">
+        <v>39438.990000000005</v>
+      </c>
+      <c r="K49" s="52">
+        <v>20456.64</v>
+      </c>
+      <c r="L49" s="52">
+        <v>18982.350000000006</v>
+      </c>
+      <c r="M49" s="53">
+        <v>0.4813092323104624</v>
+      </c>
       <c r="N49" s="53"/>
-      <c r="O49" s="52"/>
-      <c r="P49" s="52"/>
-      <c r="Q49" s="52"/>
-      <c r="R49" s="53"/>
-      <c r="S49" s="54"/>
-      <c r="T49" s="54"/>
-      <c r="U49" s="54"/>
-      <c r="V49" s="53"/>
+      <c r="O49" s="52">
+        <v>11143.38</v>
+      </c>
+      <c r="P49" s="52">
+        <v>4675.26</v>
+      </c>
+      <c r="Q49" s="52">
+        <v>6468.119999999999</v>
+      </c>
+      <c r="R49" s="53">
+        <v>0.5804450714235716</v>
+      </c>
+      <c r="S49" s="54">
+        <v>223.22</v>
+      </c>
+      <c r="T49" s="54">
+        <v>102.25</v>
+      </c>
+      <c r="U49" s="54">
+        <v>120.97</v>
+      </c>
+      <c r="V49" s="53">
+        <v>0.5419317265478004</v>
+      </c>
       <c r="W49" s="53"/>
-      <c r="X49" s="55"/>
-      <c r="Y49" s="55"/>
-      <c r="Z49" s="53"/>
-      <c r="AA49" s="56"/>
+      <c r="X49" s="55">
+        <v>1.8598533007334963</v>
+      </c>
+      <c r="Y49" s="55">
+        <v>67.69550512136009</v>
+      </c>
+      <c r="Z49" s="53">
+        <v>0.0075</v>
+      </c>
+      <c r="AA49" s="56">
+        <v>0.23</v>
+      </c>
       <c r="AB49" s="57"/>
       <c r="AD49" s="35" t="s">
         <v>96</v>
@@ -12398,30 +12662,74 @@
       <c r="C56" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D56" s="52"/>
-      <c r="E56" s="52"/>
-      <c r="F56" s="52"/>
-      <c r="G56" s="53"/>
-      <c r="H56" s="52"/>
-      <c r="I56" s="52"/>
-      <c r="J56" s="52"/>
-      <c r="K56" s="52"/>
-      <c r="L56" s="52"/>
-      <c r="M56" s="53"/>
+      <c r="D56" s="52">
+        <v>154527.79</v>
+      </c>
+      <c r="E56" s="52">
+        <v>98562.5</v>
+      </c>
+      <c r="F56" s="52">
+        <v>55965.29000000001</v>
+      </c>
+      <c r="G56" s="53">
+        <v>0.36216974306045535</v>
+      </c>
+      <c r="H56" s="52">
+        <v>108880.28</v>
+      </c>
+      <c r="I56" s="52">
+        <v>90918.83</v>
+      </c>
+      <c r="J56" s="52">
+        <v>74953.01000000001</v>
+      </c>
+      <c r="K56" s="52">
+        <v>71302.07</v>
+      </c>
+      <c r="L56" s="52">
+        <v>3650.9400000000023</v>
+      </c>
+      <c r="M56" s="53">
+        <v>0.04870971826214854</v>
+      </c>
       <c r="N56" s="53"/>
-      <c r="O56" s="52"/>
-      <c r="P56" s="52"/>
-      <c r="Q56" s="52"/>
-      <c r="R56" s="53"/>
-      <c r="S56" s="54"/>
-      <c r="T56" s="54"/>
-      <c r="U56" s="54"/>
-      <c r="V56" s="53"/>
+      <c r="O56" s="52">
+        <v>33927.27</v>
+      </c>
+      <c r="P56" s="52">
+        <v>19616.76</v>
+      </c>
+      <c r="Q56" s="52">
+        <v>14310.509999999998</v>
+      </c>
+      <c r="R56" s="53">
+        <v>0.4217996319774624</v>
+      </c>
+      <c r="S56" s="54">
+        <v>679.42</v>
+      </c>
+      <c r="T56" s="54">
+        <v>413</v>
+      </c>
+      <c r="U56" s="54">
+        <v>266.41999999999996</v>
+      </c>
+      <c r="V56" s="53">
+        <v>0.39212858025963315</v>
+      </c>
       <c r="W56" s="53"/>
-      <c r="X56" s="55"/>
-      <c r="Y56" s="55"/>
-      <c r="Z56" s="53"/>
-      <c r="AA56" s="56"/>
+      <c r="X56" s="55">
+        <v>18.50767554479419</v>
+      </c>
+      <c r="Y56" s="55">
+        <v>67.18600078134293</v>
+      </c>
+      <c r="Z56" s="53">
+        <v>0.0776</v>
+      </c>
+      <c r="AA56" s="56">
+        <v>0.2954</v>
+      </c>
       <c r="AB56" s="57"/>
       <c r="AD56" s="35" t="s">
         <v>96</v>
@@ -12805,30 +13113,74 @@
       <c r="C63" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D63" s="52"/>
-      <c r="E63" s="52"/>
-      <c r="F63" s="52"/>
-      <c r="G63" s="53"/>
-      <c r="H63" s="52"/>
-      <c r="I63" s="52"/>
-      <c r="J63" s="52"/>
-      <c r="K63" s="52"/>
-      <c r="L63" s="52"/>
-      <c r="M63" s="53"/>
+      <c r="D63" s="52">
+        <v>20420.56</v>
+      </c>
+      <c r="E63" s="52">
+        <v>16358.37</v>
+      </c>
+      <c r="F63" s="52">
+        <v>4062.1900000000005</v>
+      </c>
+      <c r="G63" s="53">
+        <v>0.19892647410257114</v>
+      </c>
+      <c r="H63" s="52">
+        <v>15859.68</v>
+      </c>
+      <c r="I63" s="52">
+        <v>13601.05</v>
+      </c>
+      <c r="J63" s="52">
+        <v>12689.1</v>
+      </c>
+      <c r="K63" s="52">
+        <v>11685.13</v>
+      </c>
+      <c r="L63" s="52">
+        <v>1003.9700000000012</v>
+      </c>
+      <c r="M63" s="53">
+        <v>0.07912066261594605</v>
+      </c>
       <c r="N63" s="53"/>
-      <c r="O63" s="52"/>
-      <c r="P63" s="52"/>
-      <c r="Q63" s="52"/>
-      <c r="R63" s="53"/>
-      <c r="S63" s="54"/>
-      <c r="T63" s="54"/>
-      <c r="U63" s="54"/>
-      <c r="V63" s="53"/>
+      <c r="O63" s="52">
+        <v>3170.58</v>
+      </c>
+      <c r="P63" s="52">
+        <v>1915.92</v>
+      </c>
+      <c r="Q63" s="52">
+        <v>1254.6599999999999</v>
+      </c>
+      <c r="R63" s="53">
+        <v>0.39571939518952365</v>
+      </c>
+      <c r="S63" s="54">
+        <v>63.5</v>
+      </c>
+      <c r="T63" s="54">
+        <v>47.5</v>
+      </c>
+      <c r="U63" s="54">
+        <v>16</v>
+      </c>
+      <c r="V63" s="53">
+        <v>0.25196850393700787</v>
+      </c>
       <c r="W63" s="53"/>
-      <c r="X63" s="55"/>
-      <c r="Y63" s="55"/>
-      <c r="Z63" s="53"/>
-      <c r="AA63" s="56"/>
+      <c r="X63" s="55">
+        <v>58.04884210526316</v>
+      </c>
+      <c r="Y63" s="55">
+        <v>71.82495570677168</v>
+      </c>
+      <c r="Z63" s="53">
+        <v>0.1686</v>
+      </c>
+      <c r="AA63" s="56">
+        <v>0.2233</v>
+      </c>
       <c r="AB63" s="57"/>
       <c r="AD63" s="35" t="s">
         <v>96</v>
@@ -13160,30 +13512,74 @@
       <c r="C70" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D70" s="52"/>
-      <c r="E70" s="52"/>
-      <c r="F70" s="52"/>
-      <c r="G70" s="53"/>
-      <c r="H70" s="52"/>
-      <c r="I70" s="52"/>
-      <c r="J70" s="52"/>
-      <c r="K70" s="52"/>
-      <c r="L70" s="52"/>
-      <c r="M70" s="53"/>
+      <c r="D70" s="52">
+        <v>46303.5</v>
+      </c>
+      <c r="E70" s="52">
+        <v>6131.46</v>
+      </c>
+      <c r="F70" s="52">
+        <v>40172.04</v>
+      </c>
+      <c r="G70" s="53">
+        <v>0.8675810683857592</v>
+      </c>
+      <c r="H70" s="52">
+        <v>34612.41</v>
+      </c>
+      <c r="I70" s="52">
+        <v>9981.43</v>
+      </c>
+      <c r="J70" s="52">
+        <v>26584.530000000002</v>
+      </c>
+      <c r="K70" s="52">
+        <v>9832.65</v>
+      </c>
+      <c r="L70" s="52">
+        <v>16751.880000000005</v>
+      </c>
+      <c r="M70" s="53">
+        <v>0.6301363988755868</v>
+      </c>
       <c r="N70" s="53"/>
-      <c r="O70" s="52"/>
-      <c r="P70" s="52"/>
-      <c r="Q70" s="52"/>
-      <c r="R70" s="53"/>
-      <c r="S70" s="54"/>
-      <c r="T70" s="54"/>
-      <c r="U70" s="54"/>
-      <c r="V70" s="53"/>
+      <c r="O70" s="52">
+        <v>8027.88</v>
+      </c>
+      <c r="P70" s="52">
+        <v>148.78</v>
+      </c>
+      <c r="Q70" s="52">
+        <v>7879.1</v>
+      </c>
+      <c r="R70" s="53">
+        <v>0.9814670872011042</v>
+      </c>
+      <c r="S70" s="54">
+        <v>160.82</v>
+      </c>
+      <c r="T70" s="54">
+        <v>2.75</v>
+      </c>
+      <c r="U70" s="54">
+        <v>158.07</v>
+      </c>
+      <c r="V70" s="53">
+        <v>0.9829001367989056</v>
+      </c>
       <c r="W70" s="53"/>
-      <c r="X70" s="55"/>
-      <c r="Y70" s="55"/>
-      <c r="Z70" s="53"/>
-      <c r="AA70" s="56"/>
+      <c r="X70" s="55">
+        <v>-1399.989090909091</v>
+      </c>
+      <c r="Y70" s="55">
+        <v>72.69676349334662</v>
+      </c>
+      <c r="Z70" s="53">
+        <v>-0.6279</v>
+      </c>
+      <c r="AA70" s="56">
+        <v>0.2525</v>
+      </c>
       <c r="AB70" s="57"/>
       <c r="AD70" s="35" t="s">
         <v>96</v>
@@ -13513,30 +13909,74 @@
       <c r="C77" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D77" s="52"/>
-      <c r="E77" s="52"/>
-      <c r="F77" s="52"/>
-      <c r="G77" s="53"/>
-      <c r="H77" s="52"/>
-      <c r="I77" s="52"/>
-      <c r="J77" s="52"/>
-      <c r="K77" s="52"/>
-      <c r="L77" s="52"/>
-      <c r="M77" s="53"/>
+      <c r="D77" s="52">
+        <v>77166.16</v>
+      </c>
+      <c r="E77" s="52">
+        <v>0</v>
+      </c>
+      <c r="F77" s="52">
+        <v>77166.16</v>
+      </c>
+      <c r="G77" s="53">
+        <v>1</v>
+      </c>
+      <c r="H77" s="52">
+        <v>54302.66</v>
+      </c>
+      <c r="I77" s="52">
+        <v>22353.17</v>
+      </c>
+      <c r="J77" s="52">
+        <v>31383.390000000003</v>
+      </c>
+      <c r="K77" s="52">
+        <v>22353.17</v>
+      </c>
+      <c r="L77" s="52">
+        <v>9030.220000000005</v>
+      </c>
+      <c r="M77" s="53">
+        <v>0.28773883254804544</v>
+      </c>
       <c r="N77" s="53"/>
-      <c r="O77" s="52"/>
-      <c r="P77" s="52"/>
-      <c r="Q77" s="52"/>
-      <c r="R77" s="53"/>
-      <c r="S77" s="54"/>
-      <c r="T77" s="54"/>
-      <c r="U77" s="54"/>
-      <c r="V77" s="53"/>
+      <c r="O77" s="52">
+        <v>22919.27</v>
+      </c>
+      <c r="P77" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q77" s="52">
+        <v>22919.27</v>
+      </c>
+      <c r="R77" s="53">
+        <v>1</v>
+      </c>
+      <c r="S77" s="54">
+        <v>470.62</v>
+      </c>
+      <c r="T77" s="54">
+        <v>0</v>
+      </c>
+      <c r="U77" s="54">
+        <v>470.62</v>
+      </c>
+      <c r="V77" s="53">
+        <v>1</v>
+      </c>
       <c r="W77" s="53"/>
-      <c r="X77" s="55"/>
-      <c r="Y77" s="55"/>
-      <c r="Z77" s="53"/>
-      <c r="AA77" s="56"/>
+      <c r="X77" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y77" s="55">
+        <v>48.58165977967362</v>
+      </c>
+      <c r="Z77" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="56">
+        <v>0.2963</v>
+      </c>
       <c r="AB77" s="57"/>
       <c r="AD77" s="35" t="s">
         <v>96</v>
@@ -13872,30 +14312,74 @@
       <c r="C84" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D84" s="52"/>
-      <c r="E84" s="52"/>
-      <c r="F84" s="52"/>
-      <c r="G84" s="53"/>
-      <c r="H84" s="52"/>
-      <c r="I84" s="52"/>
-      <c r="J84" s="52"/>
-      <c r="K84" s="52"/>
-      <c r="L84" s="52"/>
-      <c r="M84" s="53"/>
+      <c r="D84" s="52">
+        <v>25467.84</v>
+      </c>
+      <c r="E84" s="52">
+        <v>19598.41</v>
+      </c>
+      <c r="F84" s="52">
+        <v>5869.43</v>
+      </c>
+      <c r="G84" s="53">
+        <v>0.2304643817457625</v>
+      </c>
+      <c r="H84" s="52">
+        <v>16606.83</v>
+      </c>
+      <c r="I84" s="52">
+        <v>12729.14</v>
+      </c>
+      <c r="J84" s="52">
+        <v>9659.990000000002</v>
+      </c>
+      <c r="K84" s="52">
+        <v>5354.119999999999</v>
+      </c>
+      <c r="L84" s="52">
+        <v>4305.870000000003</v>
+      </c>
+      <c r="M84" s="53">
+        <v>0.44574269745620876</v>
+      </c>
       <c r="N84" s="53"/>
-      <c r="O84" s="52"/>
-      <c r="P84" s="52"/>
-      <c r="Q84" s="52"/>
-      <c r="R84" s="53"/>
-      <c r="S84" s="54"/>
-      <c r="T84" s="54"/>
-      <c r="U84" s="54"/>
-      <c r="V84" s="53"/>
+      <c r="O84" s="52">
+        <v>6946.84</v>
+      </c>
+      <c r="P84" s="52">
+        <v>7375.02</v>
+      </c>
+      <c r="Q84" s="52">
+        <v>-428.1800000000003</v>
+      </c>
+      <c r="R84" s="53">
+        <v>-0.061636657818518965</v>
+      </c>
+      <c r="S84" s="54">
+        <v>139.07</v>
+      </c>
+      <c r="T84" s="54">
+        <v>143.25</v>
+      </c>
+      <c r="U84" s="54">
+        <v>-4.180000000000007</v>
+      </c>
+      <c r="V84" s="53">
+        <v>-0.030056805925073756</v>
+      </c>
       <c r="W84" s="53"/>
-      <c r="X84" s="55"/>
-      <c r="Y84" s="55"/>
-      <c r="Z84" s="53"/>
-      <c r="AA84" s="56"/>
+      <c r="X84" s="55">
+        <v>47.95301919720768</v>
+      </c>
+      <c r="Y84" s="55">
+        <v>63.7162162306752</v>
+      </c>
+      <c r="Z84" s="53">
+        <v>0.3505</v>
+      </c>
+      <c r="AA84" s="56">
+        <v>0.3479</v>
+      </c>
       <c r="AB84" s="57"/>
       <c r="AD84" s="35" t="s">
         <v>96</v>
@@ -14279,30 +14763,74 @@
       <c r="C91" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D91" s="67"/>
-      <c r="E91" s="67"/>
-      <c r="F91" s="52"/>
-      <c r="G91" s="53"/>
-      <c r="H91" s="52"/>
-      <c r="I91" s="52"/>
-      <c r="J91" s="52"/>
-      <c r="K91" s="52"/>
-      <c r="L91" s="52"/>
-      <c r="M91" s="53"/>
+      <c r="D91" s="67">
+        <v>37083.03</v>
+      </c>
+      <c r="E91" s="67">
+        <v>33023.07</v>
+      </c>
+      <c r="F91" s="52">
+        <v>4059.959999999999</v>
+      </c>
+      <c r="G91" s="53">
+        <v>0.10948296296176444</v>
+      </c>
+      <c r="H91" s="52">
+        <v>27002.93</v>
+      </c>
+      <c r="I91" s="52">
+        <v>25996.77</v>
+      </c>
+      <c r="J91" s="52">
+        <v>15440.32</v>
+      </c>
+      <c r="K91" s="52">
+        <v>15990.78</v>
+      </c>
+      <c r="L91" s="52">
+        <v>-550.460000000001</v>
+      </c>
+      <c r="M91" s="53">
+        <v>-0.0356508155271394</v>
+      </c>
       <c r="N91" s="53"/>
-      <c r="O91" s="52"/>
-      <c r="P91" s="52"/>
-      <c r="Q91" s="52"/>
-      <c r="R91" s="53"/>
-      <c r="S91" s="68"/>
-      <c r="T91" s="68"/>
-      <c r="U91" s="54"/>
-      <c r="V91" s="53"/>
+      <c r="O91" s="52">
+        <v>11562.61</v>
+      </c>
+      <c r="P91" s="52">
+        <v>10005.99</v>
+      </c>
+      <c r="Q91" s="52">
+        <v>1556.6200000000008</v>
+      </c>
+      <c r="R91" s="53">
+        <v>0.13462531383485224</v>
+      </c>
+      <c r="S91" s="68">
+        <v>231.75</v>
+      </c>
+      <c r="T91" s="68">
+        <v>204.75</v>
+      </c>
+      <c r="U91" s="54">
+        <v>27</v>
+      </c>
+      <c r="V91" s="53">
+        <v>0.11650485436893204</v>
+      </c>
       <c r="W91" s="53"/>
-      <c r="X91" s="55"/>
-      <c r="Y91" s="55"/>
-      <c r="Z91" s="53"/>
-      <c r="AA91" s="56"/>
+      <c r="X91" s="55">
+        <v>34.316483516483515</v>
+      </c>
+      <c r="Y91" s="55">
+        <v>43.49557070636461</v>
+      </c>
+      <c r="Z91" s="53">
+        <v>0.21280000000000002</v>
+      </c>
+      <c r="AA91" s="56">
+        <v>0.2718</v>
+      </c>
       <c r="AB91" s="57"/>
       <c r="AD91" s="35" t="s">
         <v>96</v>
@@ -14598,30 +15126,74 @@
       <c r="C98" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D98" s="52"/>
-      <c r="E98" s="52"/>
-      <c r="F98" s="52"/>
-      <c r="G98" s="53"/>
-      <c r="H98" s="52"/>
-      <c r="I98" s="52"/>
-      <c r="J98" s="52"/>
-      <c r="K98" s="52"/>
-      <c r="L98" s="52"/>
-      <c r="M98" s="53"/>
+      <c r="D98" s="52">
+        <v>26186.14</v>
+      </c>
+      <c r="E98" s="52">
+        <v>5762.27</v>
+      </c>
+      <c r="F98" s="52">
+        <v>20423.87</v>
+      </c>
+      <c r="G98" s="53">
+        <v>0.7799496222047235</v>
+      </c>
+      <c r="H98" s="52">
+        <v>19428.98</v>
+      </c>
+      <c r="I98" s="52">
+        <v>7925.81</v>
+      </c>
+      <c r="J98" s="52">
+        <v>12051.32</v>
+      </c>
+      <c r="K98" s="52">
+        <v>7679.910000000001</v>
+      </c>
+      <c r="L98" s="52">
+        <v>4371.409999999999</v>
+      </c>
+      <c r="M98" s="53">
+        <v>0.36273287905391266</v>
+      </c>
       <c r="N98" s="53"/>
-      <c r="O98" s="52"/>
-      <c r="P98" s="52"/>
-      <c r="Q98" s="52"/>
-      <c r="R98" s="53"/>
-      <c r="S98" s="54"/>
-      <c r="T98" s="54"/>
-      <c r="U98" s="54"/>
-      <c r="V98" s="53"/>
+      <c r="O98" s="52">
+        <v>7377.66</v>
+      </c>
+      <c r="P98" s="52">
+        <v>245.9</v>
+      </c>
+      <c r="Q98" s="52">
+        <v>7131.76</v>
+      </c>
+      <c r="R98" s="53">
+        <v>0.9666696486419813</v>
+      </c>
+      <c r="S98" s="54">
+        <v>147.9</v>
+      </c>
+      <c r="T98" s="54">
+        <v>5</v>
+      </c>
+      <c r="U98" s="54">
+        <v>142.9</v>
+      </c>
+      <c r="V98" s="53">
+        <v>0.9661933739012847</v>
+      </c>
       <c r="W98" s="53"/>
-      <c r="X98" s="55"/>
-      <c r="Y98" s="55"/>
-      <c r="Z98" s="53"/>
-      <c r="AA98" s="56"/>
+      <c r="X98" s="55">
+        <v>-432.70799999999997</v>
+      </c>
+      <c r="Y98" s="55">
+        <v>45.687352144692355</v>
+      </c>
+      <c r="Z98" s="53">
+        <v>-0.37549999999999994</v>
+      </c>
+      <c r="AA98" s="56">
+        <v>0.258</v>
+      </c>
       <c r="AB98" s="57"/>
       <c r="AD98" s="35" t="s">
         <v>96</v>
@@ -15005,30 +15577,74 @@
       <c r="C105" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D105" s="52"/>
-      <c r="E105" s="69"/>
-      <c r="F105" s="52"/>
-      <c r="G105" s="53"/>
-      <c r="H105" s="52"/>
-      <c r="I105" s="52"/>
-      <c r="J105" s="52"/>
-      <c r="K105" s="52"/>
-      <c r="L105" s="52"/>
-      <c r="M105" s="53"/>
+      <c r="D105" s="52">
+        <v>32473.02</v>
+      </c>
+      <c r="E105" s="69">
+        <v>33188.03</v>
+      </c>
+      <c r="F105" s="52">
+        <v>-715.0099999999984</v>
+      </c>
+      <c r="G105" s="53">
+        <v>-0.022018586506582952</v>
+      </c>
+      <c r="H105" s="52">
+        <v>23075.07</v>
+      </c>
+      <c r="I105" s="52">
+        <v>31131.57</v>
+      </c>
+      <c r="J105" s="52">
+        <v>12691.21</v>
+      </c>
+      <c r="K105" s="52">
+        <v>15390.63</v>
+      </c>
+      <c r="L105" s="52">
+        <v>-2699.42</v>
+      </c>
+      <c r="M105" s="53">
+        <v>-0.21269997108234756</v>
+      </c>
       <c r="N105" s="53"/>
-      <c r="O105" s="52"/>
-      <c r="P105" s="52"/>
-      <c r="Q105" s="52"/>
-      <c r="R105" s="53"/>
-      <c r="S105" s="54"/>
-      <c r="T105" s="54"/>
-      <c r="U105" s="54"/>
-      <c r="V105" s="53"/>
+      <c r="O105" s="52">
+        <v>10383.86</v>
+      </c>
+      <c r="P105" s="52">
+        <v>15740.94</v>
+      </c>
+      <c r="Q105" s="52">
+        <v>-5357.08</v>
+      </c>
+      <c r="R105" s="53">
+        <v>-0.5159044902377343</v>
+      </c>
+      <c r="S105" s="54">
+        <v>208.2</v>
+      </c>
+      <c r="T105" s="54">
+        <v>317.25</v>
+      </c>
+      <c r="U105" s="54">
+        <v>-109.05000000000001</v>
+      </c>
+      <c r="V105" s="53">
+        <v>-0.5237752161383286</v>
+      </c>
       <c r="W105" s="53"/>
-      <c r="X105" s="55"/>
-      <c r="Y105" s="55"/>
-      <c r="Z105" s="53"/>
-      <c r="AA105" s="56"/>
+      <c r="X105" s="55">
+        <v>6.482143420015761</v>
+      </c>
+      <c r="Y105" s="55">
+        <v>45.139084580403456</v>
+      </c>
+      <c r="Z105" s="53">
+        <v>0.062</v>
+      </c>
+      <c r="AA105" s="56">
+        <v>0.2894</v>
+      </c>
       <c r="AB105" s="57"/>
       <c r="AD105" s="35" t="s">
         <v>96</v>
@@ -15414,30 +16030,74 @@
       <c r="C112" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D112" s="52"/>
-      <c r="E112" s="52"/>
-      <c r="F112" s="52"/>
-      <c r="G112" s="53"/>
-      <c r="H112" s="52"/>
-      <c r="I112" s="52"/>
-      <c r="J112" s="52"/>
-      <c r="K112" s="52"/>
-      <c r="L112" s="52"/>
-      <c r="M112" s="53"/>
+      <c r="D112" s="52">
+        <v>58902.56</v>
+      </c>
+      <c r="E112" s="52">
+        <v>0</v>
+      </c>
+      <c r="F112" s="52">
+        <v>58902.56</v>
+      </c>
+      <c r="G112" s="53">
+        <v>1</v>
+      </c>
+      <c r="H112" s="52">
+        <v>37601.88</v>
+      </c>
+      <c r="I112" s="52">
+        <v>38195.76</v>
+      </c>
+      <c r="J112" s="52">
+        <v>21415.85</v>
+      </c>
+      <c r="K112" s="52">
+        <v>19158.27</v>
+      </c>
+      <c r="L112" s="52">
+        <v>2257.579999999998</v>
+      </c>
+      <c r="M112" s="53">
+        <v>0.10541631548596009</v>
+      </c>
       <c r="N112" s="53"/>
-      <c r="O112" s="52"/>
-      <c r="P112" s="52"/>
-      <c r="Q112" s="52"/>
-      <c r="R112" s="53"/>
-      <c r="S112" s="54"/>
-      <c r="T112" s="54"/>
-      <c r="U112" s="54"/>
-      <c r="V112" s="53"/>
+      <c r="O112" s="52">
+        <v>16186.03</v>
+      </c>
+      <c r="P112" s="52">
+        <v>19037.49</v>
+      </c>
+      <c r="Q112" s="52">
+        <v>-2851.460000000001</v>
+      </c>
+      <c r="R112" s="53">
+        <v>-0.1761679670678975</v>
+      </c>
+      <c r="S112" s="54">
+        <v>324.19</v>
+      </c>
+      <c r="T112" s="54">
+        <v>412.5</v>
+      </c>
+      <c r="U112" s="54">
+        <v>-88.31</v>
+      </c>
+      <c r="V112" s="53">
+        <v>-0.2724019864894044</v>
+      </c>
       <c r="W112" s="53"/>
-      <c r="X112" s="55"/>
-      <c r="Y112" s="55"/>
-      <c r="Z112" s="53"/>
-      <c r="AA112" s="56"/>
+      <c r="X112" s="55">
+        <v>-6.6456484848484845</v>
+      </c>
+      <c r="Y112" s="55">
+        <v>65.70431400737223</v>
+      </c>
+      <c r="Z112" s="53">
+        <v>-0.07730000000000001</v>
+      </c>
+      <c r="AA112" s="56">
+        <v>0.3616</v>
+      </c>
       <c r="AB112" s="57"/>
       <c r="AD112" s="35" t="s">
         <v>96</v>
@@ -15747,32 +16407,74 @@
       <c r="C119" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D119" s="52"/>
-      <c r="E119" s="52"/>
+      <c r="D119" s="52">
+        <v>21404.82</v>
+      </c>
+      <c r="E119" s="52">
+        <v>0</v>
+      </c>
       <c r="F119" s="52">
-        <v>0</v>
-      </c>
-      <c r="G119" s="53"/>
-      <c r="H119" s="52"/>
-      <c r="I119" s="52"/>
-      <c r="J119" s="52"/>
-      <c r="K119" s="52"/>
-      <c r="L119" s="52"/>
-      <c r="M119" s="53"/>
+        <v>21404.82</v>
+      </c>
+      <c r="G119" s="53">
+        <v>1</v>
+      </c>
+      <c r="H119" s="52">
+        <v>17514.09</v>
+      </c>
+      <c r="I119" s="52">
+        <v>0</v>
+      </c>
+      <c r="J119" s="52">
+        <v>13318.880000000001</v>
+      </c>
+      <c r="K119" s="52">
+        <v>0</v>
+      </c>
+      <c r="L119" s="52">
+        <v>13318.880000000001</v>
+      </c>
+      <c r="M119" s="53">
+        <v>1</v>
+      </c>
       <c r="N119" s="53"/>
-      <c r="O119" s="52"/>
-      <c r="P119" s="52"/>
-      <c r="Q119" s="52"/>
-      <c r="R119" s="53"/>
-      <c r="S119" s="54"/>
-      <c r="T119" s="54"/>
-      <c r="U119" s="54"/>
-      <c r="V119" s="53"/>
+      <c r="O119" s="52">
+        <v>4195.21</v>
+      </c>
+      <c r="P119" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q119" s="52">
+        <v>4195.21</v>
+      </c>
+      <c r="R119" s="53">
+        <v>1</v>
+      </c>
+      <c r="S119" s="54">
+        <v>84.05</v>
+      </c>
+      <c r="T119" s="54">
+        <v>0</v>
+      </c>
+      <c r="U119" s="54">
+        <v>84.05</v>
+      </c>
+      <c r="V119" s="53">
+        <v>1</v>
+      </c>
       <c r="W119" s="53"/>
-      <c r="X119" s="55"/>
-      <c r="Y119" s="55"/>
-      <c r="Z119" s="53"/>
-      <c r="AA119" s="56"/>
+      <c r="X119" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y119" s="55">
+        <v>46.29062162403328</v>
+      </c>
+      <c r="Z119" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA119" s="56">
+        <v>0.1818</v>
+      </c>
       <c r="AB119" s="57"/>
       <c r="AD119" s="35" t="s">
         <v>96</v>
@@ -16146,32 +16848,74 @@
       <c r="C126" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D126" s="52"/>
-      <c r="E126" s="52"/>
+      <c r="D126" s="52">
+        <v>99768.39</v>
+      </c>
+      <c r="E126" s="52">
+        <v>15366.74</v>
+      </c>
       <c r="F126" s="52">
-        <v>0</v>
-      </c>
-      <c r="G126" s="53"/>
-      <c r="H126" s="52"/>
-      <c r="I126" s="52"/>
-      <c r="J126" s="52"/>
-      <c r="K126" s="52"/>
-      <c r="L126" s="52"/>
-      <c r="M126" s="53"/>
+        <v>84401.65</v>
+      </c>
+      <c r="G126" s="53">
+        <v>0.8459758647002321</v>
+      </c>
+      <c r="H126" s="52">
+        <v>81719.58</v>
+      </c>
+      <c r="I126" s="52">
+        <v>18551.86</v>
+      </c>
+      <c r="J126" s="52">
+        <v>67238.96</v>
+      </c>
+      <c r="K126" s="52">
+        <v>14369.1</v>
+      </c>
+      <c r="L126" s="52">
+        <v>52869.86000000001</v>
+      </c>
+      <c r="M126" s="53">
+        <v>0.7862980034194461</v>
+      </c>
       <c r="N126" s="53"/>
-      <c r="O126" s="52"/>
-      <c r="P126" s="52"/>
-      <c r="Q126" s="52"/>
-      <c r="R126" s="53"/>
-      <c r="S126" s="54"/>
-      <c r="T126" s="54"/>
-      <c r="U126" s="54"/>
-      <c r="V126" s="53"/>
+      <c r="O126" s="52">
+        <v>14480.62</v>
+      </c>
+      <c r="P126" s="52">
+        <v>4182.76</v>
+      </c>
+      <c r="Q126" s="52">
+        <v>10297.86</v>
+      </c>
+      <c r="R126" s="53">
+        <v>0.7111477271000828</v>
+      </c>
+      <c r="S126" s="54">
+        <v>290.15</v>
+      </c>
+      <c r="T126" s="54">
+        <v>91.75</v>
+      </c>
+      <c r="U126" s="54">
+        <v>198.39999999999998</v>
+      </c>
+      <c r="V126" s="53">
+        <v>0.6837842495261072</v>
+      </c>
       <c r="W126" s="53"/>
-      <c r="X126" s="55"/>
-      <c r="Y126" s="55"/>
-      <c r="Z126" s="53"/>
-      <c r="AA126" s="56"/>
+      <c r="X126" s="55">
+        <v>-34.715204359673024</v>
+      </c>
+      <c r="Y126" s="55">
+        <v>62.2051177714286</v>
+      </c>
+      <c r="Z126" s="53">
+        <v>-0.2073</v>
+      </c>
+      <c r="AA126" s="56">
+        <v>0.1809</v>
+      </c>
       <c r="AB126" s="57"/>
       <c r="AD126" s="35" t="s">
         <v>96</v>
@@ -16468,30 +17212,74 @@
       <c r="C133" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D133" s="52"/>
-      <c r="E133" s="52"/>
-      <c r="F133" s="52"/>
-      <c r="G133" s="53"/>
-      <c r="H133" s="52"/>
-      <c r="I133" s="52"/>
-      <c r="J133" s="52"/>
-      <c r="K133" s="52"/>
-      <c r="L133" s="52"/>
-      <c r="M133" s="53"/>
+      <c r="D133" s="52">
+        <v>31802.41</v>
+      </c>
+      <c r="E133" s="52">
+        <v>14370.83</v>
+      </c>
+      <c r="F133" s="52">
+        <v>17431.58</v>
+      </c>
+      <c r="G133" s="53">
+        <v>0.5481213530672676</v>
+      </c>
+      <c r="H133" s="52">
+        <v>23448.14</v>
+      </c>
+      <c r="I133" s="52">
+        <v>11238.62</v>
+      </c>
+      <c r="J133" s="52">
+        <v>15632.029999999999</v>
+      </c>
+      <c r="K133" s="52">
+        <v>11154.51</v>
+      </c>
+      <c r="L133" s="52">
+        <v>4477.519999999999</v>
+      </c>
+      <c r="M133" s="53">
+        <v>0.2864324083308437</v>
+      </c>
       <c r="N133" s="53"/>
-      <c r="O133" s="52"/>
-      <c r="P133" s="52"/>
-      <c r="Q133" s="52"/>
-      <c r="R133" s="53"/>
-      <c r="S133" s="54"/>
-      <c r="T133" s="54"/>
-      <c r="U133" s="54"/>
-      <c r="V133" s="53"/>
+      <c r="O133" s="52">
+        <v>7816.11</v>
+      </c>
+      <c r="P133" s="52">
+        <v>84.11</v>
+      </c>
+      <c r="Q133" s="52">
+        <v>7732</v>
+      </c>
+      <c r="R133" s="53">
+        <v>0.989238892492557</v>
+      </c>
+      <c r="S133" s="54">
+        <v>156.69</v>
+      </c>
+      <c r="T133" s="54">
+        <v>2</v>
+      </c>
+      <c r="U133" s="54">
+        <v>154.69</v>
+      </c>
+      <c r="V133" s="53">
+        <v>0.9872359435828706</v>
+      </c>
       <c r="W133" s="53"/>
-      <c r="X133" s="55"/>
-      <c r="Y133" s="55"/>
-      <c r="Z133" s="53"/>
-      <c r="AA133" s="56"/>
+      <c r="X133" s="55">
+        <v>1566.105</v>
+      </c>
+      <c r="Y133" s="55">
+        <v>53.31719360265494</v>
+      </c>
+      <c r="Z133" s="53">
+        <v>0.218</v>
+      </c>
+      <c r="AA133" s="56">
+        <v>0.2627</v>
+      </c>
       <c r="AB133" s="57"/>
       <c r="AD133" s="35" t="s">
         <v>96</v>
@@ -16875,30 +17663,74 @@
       <c r="C140" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D140" s="52"/>
-      <c r="E140" s="52"/>
-      <c r="F140" s="52"/>
-      <c r="G140" s="53"/>
-      <c r="H140" s="52"/>
-      <c r="I140" s="52"/>
-      <c r="J140" s="52"/>
-      <c r="K140" s="52"/>
-      <c r="L140" s="52"/>
-      <c r="M140" s="53"/>
+      <c r="D140" s="52">
+        <v>30749.24</v>
+      </c>
+      <c r="E140" s="52">
+        <v>30749.24</v>
+      </c>
+      <c r="F140" s="52">
+        <v>0</v>
+      </c>
+      <c r="G140" s="53">
+        <v>0</v>
+      </c>
+      <c r="H140" s="52">
+        <v>22587.89</v>
+      </c>
+      <c r="I140" s="52">
+        <v>25550.31</v>
+      </c>
+      <c r="J140" s="52">
+        <v>12565.06</v>
+      </c>
+      <c r="K140" s="52">
+        <v>11750.840000000002</v>
+      </c>
+      <c r="L140" s="52">
+        <v>814.2199999999975</v>
+      </c>
+      <c r="M140" s="53">
+        <v>0.06480032725669416</v>
+      </c>
       <c r="N140" s="53"/>
-      <c r="O140" s="52"/>
-      <c r="P140" s="52"/>
-      <c r="Q140" s="52"/>
-      <c r="R140" s="53"/>
-      <c r="S140" s="54"/>
-      <c r="T140" s="54"/>
-      <c r="U140" s="54"/>
-      <c r="V140" s="53"/>
+      <c r="O140" s="52">
+        <v>10022.83</v>
+      </c>
+      <c r="P140" s="52">
+        <v>13799.47</v>
+      </c>
+      <c r="Q140" s="52">
+        <v>-3776.6399999999994</v>
+      </c>
+      <c r="R140" s="53">
+        <v>-0.37680375702271707</v>
+      </c>
+      <c r="S140" s="54">
+        <v>200.82</v>
+      </c>
+      <c r="T140" s="54">
+        <v>278.25</v>
+      </c>
+      <c r="U140" s="54">
+        <v>-77.43</v>
+      </c>
+      <c r="V140" s="53">
+        <v>-0.3855691664176875</v>
+      </c>
       <c r="W140" s="53"/>
-      <c r="X140" s="55"/>
-      <c r="Y140" s="55"/>
-      <c r="Z140" s="53"/>
-      <c r="AA140" s="56"/>
+      <c r="X140" s="55">
+        <v>18.68438454627134</v>
+      </c>
+      <c r="Y140" s="55">
+        <v>40.64013272149188</v>
+      </c>
+      <c r="Z140" s="53">
+        <v>0.1691</v>
+      </c>
+      <c r="AA140" s="56">
+        <v>0.2654</v>
+      </c>
       <c r="AB140" s="57"/>
       <c r="AD140" s="35" t="s">
         <v>96</v>
@@ -17196,30 +18028,74 @@
       <c r="C147" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D147" s="52"/>
-      <c r="E147" s="52"/>
-      <c r="F147" s="52"/>
-      <c r="G147" s="53"/>
-      <c r="H147" s="52"/>
-      <c r="I147" s="52"/>
-      <c r="J147" s="52"/>
-      <c r="K147" s="52"/>
-      <c r="L147" s="52"/>
-      <c r="M147" s="53"/>
+      <c r="D147" s="52">
+        <v>268228.26</v>
+      </c>
+      <c r="E147" s="52">
+        <v>9034.53</v>
+      </c>
+      <c r="F147" s="52">
+        <v>259193.73</v>
+      </c>
+      <c r="G147" s="53">
+        <v>0.9663177548853353</v>
+      </c>
+      <c r="H147" s="52">
+        <v>238611.58</v>
+      </c>
+      <c r="I147" s="52">
+        <v>6362.08</v>
+      </c>
+      <c r="J147" s="52">
+        <v>214154.25</v>
+      </c>
+      <c r="K147" s="52">
+        <v>3465.35</v>
+      </c>
+      <c r="L147" s="52">
+        <v>210688.9</v>
+      </c>
+      <c r="M147" s="53">
+        <v>0.9838184392791645</v>
+      </c>
       <c r="N147" s="53"/>
-      <c r="O147" s="52"/>
-      <c r="P147" s="52"/>
-      <c r="Q147" s="52"/>
-      <c r="R147" s="53"/>
-      <c r="S147" s="54"/>
-      <c r="T147" s="54"/>
-      <c r="U147" s="54"/>
-      <c r="V147" s="53"/>
+      <c r="O147" s="52">
+        <v>24457.33</v>
+      </c>
+      <c r="P147" s="52">
+        <v>2896.73</v>
+      </c>
+      <c r="Q147" s="52">
+        <v>21560.600000000002</v>
+      </c>
+      <c r="R147" s="53">
+        <v>0.8815598432044708</v>
+      </c>
+      <c r="S147" s="54">
+        <v>497.55</v>
+      </c>
+      <c r="T147" s="54">
+        <v>58.25</v>
+      </c>
+      <c r="U147" s="54">
+        <v>439.3</v>
+      </c>
+      <c r="V147" s="53">
+        <v>0.8829263390614008</v>
+      </c>
       <c r="W147" s="53"/>
-      <c r="X147" s="55"/>
-      <c r="Y147" s="55"/>
-      <c r="Z147" s="53"/>
-      <c r="AA147" s="56"/>
+      <c r="X147" s="55">
+        <v>45.878969957081544</v>
+      </c>
+      <c r="Y147" s="55">
+        <v>59.525035875791396</v>
+      </c>
+      <c r="Z147" s="53">
+        <v>0.2958</v>
+      </c>
+      <c r="AA147" s="56">
+        <v>0.1104</v>
+      </c>
       <c r="AB147" s="57"/>
       <c r="AD147" s="35" t="s">
         <v>96</v>
@@ -17549,30 +18425,74 @@
       <c r="C154" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D154" s="52"/>
-      <c r="E154" s="52"/>
-      <c r="F154" s="52"/>
-      <c r="G154" s="53"/>
-      <c r="H154" s="52"/>
-      <c r="I154" s="52"/>
-      <c r="J154" s="52"/>
-      <c r="K154" s="52"/>
-      <c r="L154" s="52"/>
-      <c r="M154" s="53"/>
+      <c r="D154" s="52">
+        <v>32773.41</v>
+      </c>
+      <c r="E154" s="52">
+        <v>32773.41</v>
+      </c>
+      <c r="F154" s="52">
+        <v>0</v>
+      </c>
+      <c r="G154" s="53">
+        <v>0</v>
+      </c>
+      <c r="H154" s="52">
+        <v>22750.99</v>
+      </c>
+      <c r="I154" s="52">
+        <v>22254.11</v>
+      </c>
+      <c r="J154" s="52">
+        <v>12243.410000000002</v>
+      </c>
+      <c r="K154" s="52">
+        <v>9324.41</v>
+      </c>
+      <c r="L154" s="52">
+        <v>2919.000000000002</v>
+      </c>
+      <c r="M154" s="53">
+        <v>0.23841397127107575</v>
+      </c>
       <c r="N154" s="53"/>
-      <c r="O154" s="52"/>
-      <c r="P154" s="52"/>
-      <c r="Q154" s="52"/>
-      <c r="R154" s="53"/>
-      <c r="S154" s="54"/>
-      <c r="T154" s="54"/>
-      <c r="U154" s="54"/>
-      <c r="V154" s="53"/>
+      <c r="O154" s="52">
+        <v>10507.58</v>
+      </c>
+      <c r="P154" s="52">
+        <v>12929.7</v>
+      </c>
+      <c r="Q154" s="52">
+        <v>-2422.120000000001</v>
+      </c>
+      <c r="R154" s="53">
+        <v>-0.23051168775303169</v>
+      </c>
+      <c r="S154" s="54">
+        <v>210.6</v>
+      </c>
+      <c r="T154" s="54">
+        <v>260.75</v>
+      </c>
+      <c r="U154" s="54">
+        <v>-50.150000000000006</v>
+      </c>
+      <c r="V154" s="53">
+        <v>-0.2381291547958215</v>
+      </c>
       <c r="W154" s="53"/>
-      <c r="X154" s="55"/>
-      <c r="Y154" s="55"/>
-      <c r="Z154" s="53"/>
-      <c r="AA154" s="56"/>
+      <c r="X154" s="55">
+        <v>40.342473633748796</v>
+      </c>
+      <c r="Y154" s="55">
+        <v>47.58984852136751</v>
+      </c>
+      <c r="Z154" s="53">
+        <v>0.321</v>
+      </c>
+      <c r="AA154" s="56">
+        <v>0.3058</v>
+      </c>
       <c r="AB154" s="57"/>
       <c r="AD154" s="35" t="s">
         <v>96</v>
@@ -17904,34 +18824,74 @@
       <c r="C161" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D161" s="52"/>
-      <c r="E161" s="52"/>
-      <c r="F161" s="52"/>
-      <c r="G161" s="53"/>
-      <c r="H161" s="52"/>
-      <c r="I161" s="52"/>
+      <c r="D161" s="52">
+        <v>17899.33</v>
+      </c>
+      <c r="E161" s="52">
+        <v>13424.5</v>
+      </c>
+      <c r="F161" s="52">
+        <v>4474.830000000002</v>
+      </c>
+      <c r="G161" s="53">
+        <v>0.24999986032996774</v>
+      </c>
+      <c r="H161" s="52">
+        <v>13919.4</v>
+      </c>
+      <c r="I161" s="52">
+        <v>10424.13</v>
+      </c>
       <c r="J161" s="52">
-        <v>0</v>
+        <v>8410.93</v>
       </c>
       <c r="K161" s="52">
-        <v>0</v>
-      </c>
-      <c r="L161" s="52"/>
-      <c r="M161" s="53"/>
+        <v>7300.139999999999</v>
+      </c>
+      <c r="L161" s="52">
+        <v>1110.7900000000009</v>
+      </c>
+      <c r="M161" s="53">
+        <v>0.13206506295974416</v>
+      </c>
       <c r="N161" s="53"/>
-      <c r="O161" s="52"/>
-      <c r="P161" s="52"/>
-      <c r="Q161" s="52"/>
-      <c r="R161" s="53"/>
-      <c r="S161" s="54"/>
-      <c r="T161" s="54"/>
-      <c r="U161" s="54"/>
-      <c r="V161" s="53"/>
+      <c r="O161" s="52">
+        <v>5508.47</v>
+      </c>
+      <c r="P161" s="52">
+        <v>3123.99</v>
+      </c>
+      <c r="Q161" s="52">
+        <v>2384.4800000000005</v>
+      </c>
+      <c r="R161" s="53">
+        <v>0.43287519038861977</v>
+      </c>
+      <c r="S161" s="54">
+        <v>110.44</v>
+      </c>
+      <c r="T161" s="54">
+        <v>60.75</v>
+      </c>
+      <c r="U161" s="54">
+        <v>49.69</v>
+      </c>
+      <c r="V161" s="53">
+        <v>0.44992756247736326</v>
+      </c>
       <c r="W161" s="53"/>
-      <c r="X161" s="55"/>
-      <c r="Y161" s="55"/>
-      <c r="Z161" s="53"/>
-      <c r="AA161" s="56"/>
+      <c r="X161" s="55">
+        <v>49.388806584362136</v>
+      </c>
+      <c r="Y161" s="55">
+        <v>36.03704967040926</v>
+      </c>
+      <c r="Z161" s="53">
+        <v>0.2235</v>
+      </c>
+      <c r="AA161" s="56">
+        <v>0.2224</v>
+      </c>
       <c r="AB161" s="57"/>
       <c r="AD161" s="35" t="s">
         <v>96</v>
@@ -18941,30 +19901,74 @@
       <c r="C182" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D182" s="52"/>
-      <c r="E182" s="52"/>
-      <c r="F182" s="52"/>
-      <c r="G182" s="53"/>
-      <c r="H182" s="52"/>
-      <c r="I182" s="52"/>
-      <c r="J182" s="52"/>
-      <c r="K182" s="52"/>
-      <c r="L182" s="52"/>
-      <c r="M182" s="53"/>
+      <c r="D182" s="52">
+        <v>16897.53</v>
+      </c>
+      <c r="E182" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F182" s="52">
+        <v>11405.829999999998</v>
+      </c>
+      <c r="G182" s="53">
+        <v>0.6749998372543206</v>
+      </c>
+      <c r="H182" s="52">
+        <v>9226.27</v>
+      </c>
+      <c r="I182" s="52">
+        <v>3702.78</v>
+      </c>
+      <c r="J182" s="52">
+        <v>2977.1100000000006</v>
+      </c>
+      <c r="K182" s="52">
+        <v>2335.9700000000003</v>
+      </c>
+      <c r="L182" s="52">
+        <v>641.1400000000003</v>
+      </c>
+      <c r="M182" s="53">
+        <v>0.2153565034546927</v>
+      </c>
       <c r="N182" s="53"/>
-      <c r="O182" s="52"/>
-      <c r="P182" s="52"/>
-      <c r="Q182" s="52"/>
-      <c r="R182" s="53"/>
-      <c r="S182" s="54"/>
-      <c r="T182" s="54"/>
-      <c r="U182" s="54"/>
-      <c r="V182" s="53"/>
+      <c r="O182" s="52">
+        <v>6249.16</v>
+      </c>
+      <c r="P182" s="52">
+        <v>1366.81</v>
+      </c>
+      <c r="Q182" s="52">
+        <v>4882.35</v>
+      </c>
+      <c r="R182" s="53">
+        <v>0.7812810041669601</v>
+      </c>
+      <c r="S182" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T182" s="54">
+        <v>23.75</v>
+      </c>
+      <c r="U182" s="54">
+        <v>101.42</v>
+      </c>
+      <c r="V182" s="53">
+        <v>0.8102580490532876</v>
+      </c>
       <c r="W182" s="53"/>
-      <c r="X182" s="55"/>
-      <c r="Y182" s="55"/>
-      <c r="Z182" s="53"/>
-      <c r="AA182" s="56"/>
+      <c r="X182" s="55">
+        <v>75.32294736842105</v>
+      </c>
+      <c r="Y182" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z182" s="53">
+        <v>0.3257</v>
+      </c>
+      <c r="AA182" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB182" s="57"/>
       <c r="AD182" s="35" t="s">
         <v>96</v>
@@ -21718,7 +22722,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="52">
-        <v>51687.05</v>
+        <v>51285.36</v>
       </c>
       <c r="E4" s="52">
         <f>C4-D4</f>
@@ -21790,7 +22794,7 @@
         <v>3912</v>
       </c>
       <c r="D6" s="52">
-        <v>6513.389999999999</v>
+        <v>7555.1500000000015</v>
       </c>
       <c r="E6" s="52">
         <f>C6-D6</f>
@@ -21937,7 +22941,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="52">
-        <v>5315.239999999991</v>
+        <v>8827.48999999999</v>
       </c>
       <c r="E10" s="52">
         <f>C10-D10</f>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-18T21:40:22Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9737,54 +9737,54 @@
         <v>199128.99</v>
       </c>
       <c r="I7" s="52">
-        <v>164808.35</v>
+        <v>165210.04</v>
       </c>
       <c r="J7" s="52">
         <v>172860.11</v>
       </c>
       <c r="K7" s="52">
-        <v>137510.76</v>
+        <v>137410.69</v>
       </c>
       <c r="L7" s="52">
-        <v>35349.34999999998</v>
+        <v>35449.419999999984</v>
       </c>
       <c r="M7" s="53">
-        <v>0.20449686165304407</v>
+        <v>0.20507576907130273</v>
       </c>
       <c r="N7" s="53"/>
       <c r="O7" s="52">
         <v>26268.88</v>
       </c>
       <c r="P7" s="52">
-        <v>27297.59</v>
+        <v>27799.35</v>
       </c>
       <c r="Q7" s="52">
-        <v>-1028.7099999999991</v>
+        <v>-1530.4699999999975</v>
       </c>
       <c r="R7" s="53">
-        <v>-0.03916078645149695</v>
+        <v>-0.05826171500269511</v>
       </c>
       <c r="S7" s="54">
         <v>530.95</v>
       </c>
       <c r="T7" s="54">
-        <v>548</v>
+        <v>556.5</v>
       </c>
       <c r="U7" s="54">
-        <v>-17.049999999999955</v>
+        <v>-25.549999999999955</v>
       </c>
       <c r="V7" s="53">
-        <v>-0.032112251624446655</v>
+        <v>-0.04812129202373096</v>
       </c>
       <c r="W7" s="53"/>
       <c r="X7" s="55">
-        <v>75.01377737226278</v>
+        <v>73.14619946091645</v>
       </c>
       <c r="Y7" s="55">
         <v>65.45490166985587</v>
       </c>
       <c r="Z7" s="53">
-        <v>0.1996</v>
+        <v>0.1977</v>
       </c>
       <c r="AA7" s="56">
         <v>0.1486</v>
@@ -19536,32 +19536,74 @@
       <c r="C175" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D175" s="52"/>
-      <c r="E175" s="52"/>
-      <c r="F175" s="52"/>
-      <c r="G175" s="53"/>
-      <c r="H175" s="52"/>
-      <c r="I175" s="52"/>
-      <c r="J175" s="52"/>
+      <c r="D175" s="52">
+        <v>146237.11</v>
+      </c>
+      <c r="E175" s="52">
+        <v>94266.45</v>
+      </c>
+      <c r="F175" s="52">
+        <v>51970.65999999999</v>
+      </c>
+      <c r="G175" s="53">
+        <v>0.355386262761894</v>
+      </c>
+      <c r="H175" s="52">
+        <v>114651.87</v>
+      </c>
+      <c r="I175" s="52">
+        <v>95876.35</v>
+      </c>
+      <c r="J175" s="52">
+        <v>82888.07999999999</v>
+      </c>
       <c r="K175" s="52">
-        <v>0</v>
-      </c>
-      <c r="L175" s="52"/>
-      <c r="M175" s="53"/>
+        <v>74503.91</v>
+      </c>
+      <c r="L175" s="52">
+        <v>8384.169999999984</v>
+      </c>
+      <c r="M175" s="53">
+        <v>0.10115049112007402</v>
+      </c>
       <c r="N175" s="53"/>
-      <c r="O175" s="52"/>
-      <c r="P175" s="52"/>
-      <c r="Q175" s="52"/>
-      <c r="R175" s="53"/>
-      <c r="S175" s="54"/>
-      <c r="T175" s="54"/>
-      <c r="U175" s="54"/>
-      <c r="V175" s="53"/>
+      <c r="O175" s="52">
+        <v>31763.79</v>
+      </c>
+      <c r="P175" s="52">
+        <v>21372.44</v>
+      </c>
+      <c r="Q175" s="52">
+        <v>10391.350000000002</v>
+      </c>
+      <c r="R175" s="53">
+        <v>0.32714452525973764</v>
+      </c>
+      <c r="S175" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T175" s="54">
+        <v>430</v>
+      </c>
+      <c r="U175" s="54">
+        <v>229.73000000000002</v>
+      </c>
+      <c r="V175" s="53">
+        <v>0.34821821048004487</v>
+      </c>
       <c r="W175" s="53"/>
-      <c r="X175" s="55"/>
-      <c r="Y175" s="55"/>
-      <c r="Z175" s="53"/>
-      <c r="AA175" s="56"/>
+      <c r="X175" s="55">
+        <v>-3.7439534883720933</v>
+      </c>
+      <c r="Y175" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z175" s="53">
+        <v>-0.0171</v>
+      </c>
+      <c r="AA175" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB175" s="57"/>
       <c r="AD175" s="35" t="s">
         <v>96</v>
@@ -20637,32 +20679,74 @@
       <c r="C196" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D196" s="52"/>
-      <c r="E196" s="52"/>
-      <c r="F196" s="52"/>
-      <c r="G196" s="53"/>
-      <c r="H196" s="52"/>
-      <c r="I196" s="52"/>
-      <c r="J196" s="52"/>
+      <c r="D196" s="52">
+        <v>23770.95</v>
+      </c>
+      <c r="E196" s="52">
+        <v>0</v>
+      </c>
+      <c r="F196" s="52">
+        <v>23770.95</v>
+      </c>
+      <c r="G196" s="53">
+        <v>1</v>
+      </c>
+      <c r="H196" s="52">
+        <v>14310.96</v>
+      </c>
+      <c r="I196" s="52">
+        <v>7180.07</v>
+      </c>
+      <c r="J196" s="52">
+        <v>7389.339999999999</v>
+      </c>
       <c r="K196" s="52">
-        <v>0</v>
-      </c>
-      <c r="L196" s="52"/>
-      <c r="M196" s="53"/>
+        <v>6849.16</v>
+      </c>
+      <c r="L196" s="52">
+        <v>540.1799999999994</v>
+      </c>
+      <c r="M196" s="53">
+        <v>0.07310260456278903</v>
+      </c>
       <c r="N196" s="53"/>
-      <c r="O196" s="52"/>
-      <c r="P196" s="52"/>
-      <c r="Q196" s="52"/>
-      <c r="R196" s="53"/>
-      <c r="S196" s="54"/>
-      <c r="T196" s="54"/>
-      <c r="U196" s="54"/>
-      <c r="V196" s="53"/>
+      <c r="O196" s="52">
+        <v>6921.62</v>
+      </c>
+      <c r="P196" s="52">
+        <v>330.91</v>
+      </c>
+      <c r="Q196" s="52">
+        <v>6590.71</v>
+      </c>
+      <c r="R196" s="53">
+        <v>0.9521918279246766</v>
+      </c>
+      <c r="S196" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T196" s="54">
+        <v>5.75</v>
+      </c>
+      <c r="U196" s="54">
+        <v>134.4</v>
+      </c>
+      <c r="V196" s="53">
+        <v>0.9589725294327506</v>
+      </c>
       <c r="W196" s="53"/>
-      <c r="X196" s="55"/>
-      <c r="Y196" s="55"/>
-      <c r="Z196" s="53"/>
-      <c r="AA196" s="56"/>
+      <c r="X196" s="55">
+        <v>-1248.7078260869564</v>
+      </c>
+      <c r="Y196" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z196" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA196" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB196" s="57"/>
       <c r="AD196" s="35" t="s">
         <v>96</v>
@@ -21566,30 +21650,74 @@
       <c r="C217" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D217" s="52"/>
-      <c r="E217" s="52"/>
-      <c r="F217" s="52"/>
-      <c r="G217" s="53"/>
-      <c r="H217" s="52"/>
-      <c r="I217" s="52"/>
-      <c r="J217" s="52"/>
-      <c r="K217" s="52"/>
-      <c r="L217" s="52"/>
-      <c r="M217" s="53"/>
+      <c r="D217" s="52">
+        <v>137109.56</v>
+      </c>
+      <c r="E217" s="52">
+        <v>0</v>
+      </c>
+      <c r="F217" s="52">
+        <v>137109.56</v>
+      </c>
+      <c r="G217" s="53">
+        <v>1</v>
+      </c>
+      <c r="H217" s="52">
+        <v>117394.57</v>
+      </c>
+      <c r="I217" s="52">
+        <v>1749.8</v>
+      </c>
+      <c r="J217" s="52">
+        <v>99479.62000000001</v>
+      </c>
+      <c r="K217" s="52">
+        <v>1749.8</v>
+      </c>
+      <c r="L217" s="52">
+        <v>97729.82</v>
+      </c>
+      <c r="M217" s="53">
+        <v>0.9824104675912513</v>
+      </c>
       <c r="N217" s="53"/>
-      <c r="O217" s="52"/>
-      <c r="P217" s="52"/>
-      <c r="Q217" s="52"/>
-      <c r="R217" s="53"/>
-      <c r="S217" s="54"/>
-      <c r="T217" s="54"/>
-      <c r="U217" s="54"/>
-      <c r="V217" s="53"/>
+      <c r="O217" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="P217" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q217" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="R217" s="53">
+        <v>1</v>
+      </c>
+      <c r="S217" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T217" s="54">
+        <v>0</v>
+      </c>
+      <c r="U217" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V217" s="53">
+        <v>1</v>
+      </c>
       <c r="W217" s="53"/>
-      <c r="X217" s="55"/>
-      <c r="Y217" s="55"/>
-      <c r="Z217" s="53"/>
-      <c r="AA217" s="56"/>
+      <c r="X217" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y217" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z217" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA217" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB217" s="57"/>
       <c r="AD217" s="35" t="s">
         <v>96</v>
@@ -21919,34 +22047,74 @@
       <c r="C224" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D224" s="52"/>
-      <c r="E224" s="52"/>
-      <c r="F224" s="52"/>
-      <c r="G224" s="53"/>
-      <c r="H224" s="52"/>
-      <c r="I224" s="52"/>
+      <c r="D224" s="52">
+        <v>389318.35</v>
+      </c>
+      <c r="E224" s="52">
+        <v>271388.15</v>
+      </c>
+      <c r="F224" s="52">
+        <v>117930.19999999995</v>
+      </c>
+      <c r="G224" s="53">
+        <v>0.3029145685015874</v>
+      </c>
+      <c r="H224" s="52">
+        <v>289549.48</v>
+      </c>
+      <c r="I224" s="52">
+        <v>227043.56</v>
+      </c>
       <c r="J224" s="52">
-        <v>0</v>
+        <v>174279.97999999998</v>
       </c>
       <c r="K224" s="52">
-        <v>0</v>
-      </c>
-      <c r="L224" s="52"/>
-      <c r="M224" s="53"/>
+        <v>173862.65</v>
+      </c>
+      <c r="L224" s="52">
+        <v>417.3299999999872</v>
+      </c>
+      <c r="M224" s="53">
+        <v>0.0023945951795495226</v>
+      </c>
       <c r="N224" s="53"/>
-      <c r="O224" s="52"/>
-      <c r="P224" s="52"/>
-      <c r="Q224" s="52"/>
-      <c r="R224" s="53"/>
-      <c r="S224" s="54"/>
-      <c r="T224" s="54"/>
-      <c r="U224" s="54"/>
-      <c r="V224" s="53"/>
+      <c r="O224" s="52">
+        <v>115269.5</v>
+      </c>
+      <c r="P224" s="52">
+        <v>53180.91</v>
+      </c>
+      <c r="Q224" s="52">
+        <v>62088.59</v>
+      </c>
+      <c r="R224" s="53">
+        <v>0.5386384950051835</v>
+      </c>
+      <c r="S224" s="54">
+        <v>2312.68</v>
+      </c>
+      <c r="T224" s="54">
+        <v>1120.5</v>
+      </c>
+      <c r="U224" s="54">
+        <v>1192.1799999999998</v>
+      </c>
+      <c r="V224" s="53">
+        <v>0.5154971721120085</v>
+      </c>
       <c r="W224" s="53"/>
-      <c r="X224" s="55"/>
-      <c r="Y224" s="55"/>
-      <c r="Z224" s="53"/>
-      <c r="AA224" s="56"/>
+      <c r="X224" s="55">
+        <v>39.57571619812583</v>
+      </c>
+      <c r="Y224" s="55">
+        <v>43.1399392286741</v>
+      </c>
+      <c r="Z224" s="53">
+        <v>0.1634</v>
+      </c>
+      <c r="AA224" s="56">
+        <v>0.2563</v>
+      </c>
       <c r="AB224" s="57"/>
       <c r="AD224" s="35" t="s">
         <v>96</v>
@@ -22722,7 +22890,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="52">
-        <v>51285.36</v>
+        <v>51687.05</v>
       </c>
       <c r="E4" s="52">
         <f>C4-D4</f>
@@ -24917,7 +25085,7 @@
         <v>0</v>
       </c>
       <c r="D66" s="99">
-        <v>3855.079999999987</v>
+        <v>2584.2399999999907</v>
       </c>
       <c r="E66" s="99">
         <f>C66-D66</f>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-18T22:05:51Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10144,19 +10144,19 @@
         <v>101420.72</v>
       </c>
       <c r="I14" s="52">
-        <v>55851.96</v>
+        <v>54087.96</v>
       </c>
       <c r="J14" s="52">
         <v>83645.65</v>
       </c>
       <c r="K14" s="52">
-        <v>51392.88</v>
+        <v>49628.88</v>
       </c>
       <c r="L14" s="52">
-        <v>32252.769999999997</v>
+        <v>34016.77</v>
       </c>
       <c r="M14" s="53">
-        <v>0.3855881327959075</v>
+        <v>0.4066770955811808</v>
       </c>
       <c r="N14" s="53"/>
       <c r="O14" s="52">
@@ -10185,13 +10185,13 @@
       </c>
       <c r="W14" s="53"/>
       <c r="X14" s="55">
-        <v>-8.637465564738292</v>
+        <v>10.800550964187327</v>
       </c>
       <c r="Y14" s="55">
         <v>77.66490997775718</v>
       </c>
       <c r="Z14" s="53">
-        <v>-0.014199999999999999</v>
+        <v>0.0178</v>
       </c>
       <c r="AA14" s="56">
         <v>0.2142</v>
@@ -22962,7 +22962,7 @@
         <v>3912</v>
       </c>
       <c r="D6" s="52">
-        <v>7555.1500000000015</v>
+        <v>5791.1500000000015</v>
       </c>
       <c r="E6" s="52">
         <f>C6-D6</f>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-18T22:07:15Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -20346,32 +20346,74 @@
       <c r="C189" s="51" t="s">
         <v>95</v>
       </c>
-      <c r="D189" s="52"/>
-      <c r="E189" s="52"/>
-      <c r="F189" s="52"/>
-      <c r="G189" s="53"/>
-      <c r="H189" s="52"/>
-      <c r="I189" s="52"/>
-      <c r="J189" s="52"/>
+      <c r="D189" s="52">
+        <v>20992.12</v>
+      </c>
+      <c r="E189" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F189" s="52">
+        <v>6822.439999999999</v>
+      </c>
+      <c r="G189" s="53">
+        <v>0.32500004763692275</v>
+      </c>
+      <c r="H189" s="52">
+        <v>16299.09</v>
+      </c>
+      <c r="I189" s="52">
+        <v>9755.47</v>
+      </c>
+      <c r="J189" s="52">
+        <v>9784.33</v>
+      </c>
       <c r="K189" s="52">
-        <v>0</v>
-      </c>
-      <c r="L189" s="52"/>
-      <c r="M189" s="53"/>
+        <v>8193.84</v>
+      </c>
+      <c r="L189" s="52">
+        <v>1590.4899999999998</v>
+      </c>
+      <c r="M189" s="53">
+        <v>0.16255481979859632</v>
+      </c>
       <c r="N189" s="53"/>
-      <c r="O189" s="52"/>
-      <c r="P189" s="52"/>
-      <c r="Q189" s="52"/>
-      <c r="R189" s="53"/>
-      <c r="S189" s="54"/>
-      <c r="T189" s="54"/>
-      <c r="U189" s="54"/>
-      <c r="V189" s="53"/>
+      <c r="O189" s="52">
+        <v>6514.76</v>
+      </c>
+      <c r="P189" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q189" s="52">
+        <v>4953.13</v>
+      </c>
+      <c r="R189" s="53">
+        <v>0.7602935488030257</v>
+      </c>
+      <c r="S189" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T189" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U189" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V189" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W189" s="53"/>
-      <c r="X189" s="55"/>
-      <c r="Y189" s="55"/>
-      <c r="Z189" s="53"/>
-      <c r="AA189" s="56"/>
+      <c r="X189" s="55">
+        <v>127.02762589928058</v>
+      </c>
+      <c r="Y189" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z189" s="53">
+        <v>0.3115</v>
+      </c>
+      <c r="AA189" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB189" s="57"/>
       <c r="AD189" s="35" t="s">
         <v>96</v>

</xml_diff>

<commit_message>
Fix stale Quoted/Used/Remaining Hours on Upcoming Work Calculator
Same root cause as the Claim Calculator Profit/Margin bug fixed
earlier: these three columns are LOOKUP formulas reading the last
non-zero value off the Deliverables Sheet's Start-of-month-through-
Week-5 range for that job, and ExcelJS never recalculates a formula's
cached result just because the cells it references changed. Confirmed
directly: 7429's Used Hours read 32.25 (last month's figure) even
though this week's export had already updated actual hours to 34.75.

Recomputed from the exact same range the formula itself reads,
written as plain values — every one of the 20 jobs with real hours
movement this month was affected, some by 100+ hours. Backfilled the
currently-committed workbook the same way, verified against a copy
first.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17207,7 +17207,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -22817,7 +22817,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -22831,7 +22831,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -22853,7 +22853,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>99</v>
       </c>
@@ -22901,7 +22901,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -22919,7 +22919,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <f>'Main Sheet'!A4</f>
         <v>7658</v>
@@ -22968,7 +22968,7 @@
         <v>-2588.8525</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -22985,7 +22985,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <f>'Main Sheet'!A6</f>
         <v>8142</v>
@@ -23039,7 +23039,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23056,7 +23056,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <f>'Main Sheet'!A8</f>
         <v>8824</v>
@@ -23103,7 +23103,7 @@
         <v>34.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23120,7 +23120,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <f>'Main Sheet'!A10</f>
         <v>8127</v>
@@ -23171,7 +23171,7 @@
         <v>40.40408523144744</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23188,7 +23188,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23237,7 +23237,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23254,7 +23254,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <f>'Main Sheet'!A14</f>
         <v>8886</v>
@@ -23305,7 +23305,7 @@
         <v>45.876428571428605</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23322,7 +23322,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <f>'Main Sheet'!A16</f>
         <v>8887</v>
@@ -23371,7 +23371,7 @@
         <v>98.73233429394816</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23388,7 +23388,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <f>'Main Sheet'!A18</f>
         <v>8670</v>
@@ -23442,7 +23442,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23459,7 +23459,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <f>'Main Sheet'!A20</f>
         <v>8907</v>
@@ -23501,7 +23501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23518,7 +23518,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <f>'Main Sheet'!A22</f>
         <v>9065</v>
@@ -23565,7 +23565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23582,7 +23582,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <f>'Main Sheet'!A24</f>
         <v>9259</v>
@@ -23627,7 +23627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -23644,7 +23644,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <f>'Main Sheet'!A26</f>
         <v>8352</v>
@@ -23693,7 +23693,7 @@
         <v>-1.343804537521815</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -23710,7 +23710,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <f>'Main Sheet'!A28</f>
         <v>8234</v>
@@ -23757,7 +23757,7 @@
         <v>30.14242424242425</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -23774,7 +23774,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <f>'Main Sheet'!A30</f>
         <v>8214</v>
@@ -23821,7 +23821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -23838,7 +23838,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <f>'Main Sheet'!A32</f>
         <v>6792</v>
@@ -23889,7 +23889,7 @@
         <v>5.481184600197436</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -23906,7 +23906,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <f>'Main Sheet'!A34</f>
         <v>8840</v>
@@ -23955,7 +23955,7 @@
         <v>252.9351404151404</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -23972,7 +23972,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <f>'Main Sheet'!A36</f>
         <v>8769</v>
@@ -24023,7 +24023,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24040,7 +24040,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <f>'Main Sheet'!A38</f>
         <v>7901</v>
@@ -24087,7 +24087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24104,7 +24104,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <f>'Main Sheet'!A40</f>
         <v>8923</v>
@@ -24153,7 +24153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24170,7 +24170,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <f>'Main Sheet'!A42</f>
         <v>7864</v>
@@ -24217,7 +24217,7 @@
         <v>-11.131808809746953</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24234,7 +24234,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <f>'Main Sheet'!A44</f>
         <v>7912</v>
@@ -24279,7 +24279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24296,7 +24296,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <f>'Main Sheet'!A46</f>
         <v>8360</v>
@@ -24341,7 +24341,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24358,7 +24358,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <f>'Main Sheet'!A48</f>
         <v>8337</v>
@@ -24405,7 +24405,7 @@
         <v>-179.4969832402235</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24422,7 +24422,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <f>'Main Sheet'!A50</f>
         <v>9240</v>
@@ -24472,7 +24472,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24489,7 +24489,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <f>'Main Sheet'!A52</f>
         <v>7428</v>
@@ -24538,7 +24538,7 @@
         <v>79.30441796516956</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24555,7 +24555,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <f>'Main Sheet'!A54</f>
         <v>9351</v>
@@ -24604,7 +24604,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24621,7 +24621,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <f>'Main Sheet'!A56</f>
         <v>7429</v>
@@ -24670,7 +24670,7 @@
         <v>-120.76000000000003</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -24687,7 +24687,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <f>'Main Sheet'!A58</f>
         <v>9508</v>
@@ -24732,7 +24732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -24749,7 +24749,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59">
         <f>'Main Sheet'!A60</f>
         <v>0</v>
@@ -24796,7 +24796,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -24813,7 +24813,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59">
         <f>'Main Sheet'!A62</f>
         <v>0</v>
@@ -24862,7 +24862,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -24879,7 +24879,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <f>'Main Sheet'!A64</f>
         <v>8946</v>
@@ -24926,7 +24926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -24943,7 +24943,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -24991,7 +24991,7 @@
         <v>6.191319240032102</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -25008,7 +25008,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -25025,7 +25025,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>119</v>
       </c>
@@ -25060,7 +25060,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>123</v>
@@ -25445,7 +25445,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25456,7 +25456,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25477,7 +25477,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>124</v>
@@ -25539,7 +25539,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>140</v>
       </c>
@@ -25597,7 +25597,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <f>'Main Sheet'!A4</f>
         <v>7658</v>
@@ -25607,16 +25607,13 @@
         <v>Charity Hospital</v>
       </c>
       <c r="C4" s="54">
-        <f t="array" ref="C4:C4">LOOKUP(2,1/('Deliverables Sheet'!S4:S9&lt;&gt;0),'Deliverables Sheet'!S4:S9)</f>
         <v>530.95</v>
       </c>
       <c r="D4" s="54">
-        <f t="array" ref="D4:D4">LOOKUP(2,1/('Deliverables Sheet'!T4:T9&lt;&gt;0),'Deliverables Sheet'!T4:T9)</f>
-        <v>418</v>
+        <v>556.5</v>
       </c>
       <c r="E4" s="54">
-        <f t="array" ref="E4:E4">LOOKUP(2,1/('Deliverables Sheet'!U4:U9&lt;&gt;0),'Deliverables Sheet'!U4:U9)</f>
-        <v>112.95</v>
+        <v>-25.549999999999955</v>
       </c>
       <c r="F4" s="54"/>
       <c r="G4" s="54"/>
@@ -25636,7 +25633,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25655,7 +25652,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <f>'Main Sheet'!A6</f>
         <v>8142</v>
@@ -25665,16 +25662,13 @@
         <v>Fisher Developements</v>
       </c>
       <c r="C6" s="54">
-        <f t="array" ref="C6:C6">LOOKUP(2,1/('Deliverables Sheet'!S11:S16&lt;&gt;0),'Deliverables Sheet'!S11:S16)</f>
-        <v>311.89</v>
+        <v>356.07</v>
       </c>
       <c r="D6" s="54">
-        <f t="array" ref="D6:D6">LOOKUP(2,1/('Deliverables Sheet'!T11:T16&lt;&gt;0),'Deliverables Sheet'!T11:T16)</f>
-        <v>52.5</v>
+        <v>90.75</v>
       </c>
       <c r="E6" s="54">
-        <f t="array" ref="E6:E6">LOOKUP(2,1/('Deliverables Sheet'!U11:U16&lt;&gt;0),'Deliverables Sheet'!U11:U16)</f>
-        <v>259.39</v>
+        <v>265.32</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -25694,7 +25688,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25713,7 +25707,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <f>'Main Sheet'!A8</f>
         <v>8824</v>
@@ -25723,15 +25717,12 @@
         <v>3 Innovation Road</v>
       </c>
       <c r="C8" s="54">
-        <f t="array" ref="C8:C8">LOOKUP(2,1/('Deliverables Sheet'!S18:S23&lt;&gt;0),'Deliverables Sheet'!S18:S23)</f>
         <v>125.39</v>
       </c>
       <c r="D8" s="54">
-        <f t="array" ref="D8:D8">LOOKUP(2,1/('Deliverables Sheet'!T18:T23&lt;&gt;0),'Deliverables Sheet'!T18:T23)</f>
         <v>34.75</v>
       </c>
       <c r="E8" s="54">
-        <f t="array" ref="E8:E8">LOOKUP(2,1/('Deliverables Sheet'!U18:U23&lt;&gt;0),'Deliverables Sheet'!U18:U23)</f>
         <v>90.64</v>
       </c>
       <c r="F8" s="54"/>
@@ -25752,7 +25743,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -25771,7 +25762,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <f>'Main Sheet'!A10</f>
         <v>8127</v>
@@ -25781,16 +25772,13 @@
         <v>Rolly Autowash</v>
       </c>
       <c r="C10" s="54">
-        <f t="array" ref="C10:C10">LOOKUP(2,1/('Deliverables Sheet'!S25:S30&lt;&gt;0),'Deliverables Sheet'!S25:S30)</f>
         <v>795.22</v>
       </c>
       <c r="D10" s="54">
-        <f t="array" ref="D10:D10">LOOKUP(2,1/('Deliverables Sheet'!T25:T30&lt;&gt;0),'Deliverables Sheet'!T25:T30)</f>
-        <v>388.25</v>
+        <v>531.25</v>
       </c>
       <c r="E10" s="54">
-        <f t="array" ref="E10:E10">LOOKUP(2,1/('Deliverables Sheet'!U25:U30&lt;&gt;0),'Deliverables Sheet'!U25:U30)</f>
-        <v>406.97</v>
+        <v>263.97</v>
       </c>
       <c r="F10" s="54"/>
       <c r="G10" s="54"/>
@@ -25812,7 +25800,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -25831,7 +25819,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -25839,16 +25827,13 @@
         <v>115</v>
       </c>
       <c r="C12" s="54">
-        <f>'Deliverables Sheet'!S32</f>
         <v>1120.27</v>
       </c>
       <c r="D12" s="54">
-        <f>'Deliverables Sheet'!T32</f>
-        <v>387.5</v>
+        <v>416.25</v>
       </c>
       <c r="E12" s="54">
-        <f t="array" ref="E12:E12">LOOKUP(2,1/('Deliverables Sheet'!U32:U37&lt;&gt;0),'Deliverables Sheet'!U32:U37)</f>
-        <v>732.77</v>
+        <v>704.02</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -25872,7 +25857,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -25891,7 +25876,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <f>'Main Sheet'!A14</f>
         <v>8886</v>
@@ -25901,16 +25886,13 @@
         <v>Monkey Toe - Fisher fit out</v>
       </c>
       <c r="C14" s="54">
-        <f>'Deliverables Sheet'!S39</f>
-        <v>501</v>
+        <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <f>'Deliverables Sheet'!T39</f>
-        <v>112</v>
+        <v>123.75</v>
       </c>
       <c r="E14" s="54">
-        <f t="array" ref="E14:E14">LOOKUP(2,1/('Deliverables Sheet'!U39:U44&lt;&gt;0),'Deliverables Sheet'!U39:U44)</f>
-        <v>389</v>
+        <v>378.08</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -25934,7 +25916,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -25953,7 +25935,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <f>'Main Sheet'!A16</f>
         <v>8887</v>
@@ -25963,16 +25945,13 @@
         <v>Tenancy 2 - Fisher Fit out</v>
       </c>
       <c r="C16" s="54">
-        <f t="array" ref="C16:C16">LOOKUP(2,1/('Deliverables Sheet'!S46:S51&lt;&gt;0),'Deliverables Sheet'!S46:S51)</f>
-        <v>212.3</v>
+        <v>223.22</v>
       </c>
       <c r="D16" s="54">
-        <f t="array" ref="D16:D16">LOOKUP(2,1/('Deliverables Sheet'!T46:T51&lt;&gt;0),'Deliverables Sheet'!T46:T51)</f>
-        <v>86.75</v>
+        <v>102.25</v>
       </c>
       <c r="E16" s="54">
-        <f t="array" ref="E16:E16">LOOKUP(2,1/('Deliverables Sheet'!U46:U51&lt;&gt;0),'Deliverables Sheet'!U46:U51)</f>
-        <v>125.55</v>
+        <v>120.97</v>
       </c>
       <c r="F16" s="54"/>
       <c r="G16" s="54"/>
@@ -25991,7 +25970,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26010,7 +25989,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <f>'Main Sheet'!A18</f>
         <v>8670</v>
@@ -26020,16 +25999,13 @@
         <v>Studio DB - tautara fit out</v>
       </c>
       <c r="C18" s="54">
-        <f t="array" ref="C18:C18">LOOKUP(2,1/('Deliverables Sheet'!S53:S58&lt;&gt;0),'Deliverables Sheet'!S53:S58)</f>
-        <v>668.92</v>
+        <v>679.42</v>
       </c>
       <c r="D18" s="54">
-        <f t="array" ref="D18:D18">LOOKUP(2,1/('Deliverables Sheet'!T53:T58&lt;&gt;0),'Deliverables Sheet'!T53:T58)</f>
-        <v>269</v>
+        <v>413</v>
       </c>
       <c r="E18" s="54">
-        <f t="array" ref="E18:E18">LOOKUP(2,1/('Deliverables Sheet'!U53:U58&lt;&gt;0),'Deliverables Sheet'!U53:U58)</f>
-        <v>399.92</v>
+        <v>266.41999999999996</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -26048,7 +26024,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -26067,7 +26043,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <f>'Main Sheet'!A20</f>
         <v>8907</v>
@@ -26077,16 +26053,13 @@
         <v>35 Mania</v>
       </c>
       <c r="C20" s="54">
-        <f t="array" ref="C20:C20">LOOKUP(2,1/('Deliverables Sheet'!S60:S65&lt;&gt;0),'Deliverables Sheet'!S60:S65)</f>
         <v>63.5</v>
       </c>
       <c r="D20" s="54">
-        <f t="array" ref="D20:D20">LOOKUP(2,1/('Deliverables Sheet'!T60:T65&lt;&gt;0),'Deliverables Sheet'!T60:T65)</f>
-        <v>26.75</v>
+        <v>47.5</v>
       </c>
       <c r="E20" s="54">
-        <f t="array" ref="E20:E20">LOOKUP(2,1/('Deliverables Sheet'!U60:U65&lt;&gt;0),'Deliverables Sheet'!U60:U65)</f>
-        <v>36.75</v>
+        <v>16</v>
       </c>
       <c r="F20" s="54"/>
       <c r="G20" s="54"/>
@@ -26103,7 +26076,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26122,7 +26095,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <f>'Main Sheet'!A22</f>
         <v>9065</v>
@@ -26132,16 +26105,13 @@
         <v>Cooltranz stage 4</v>
       </c>
       <c r="C22" s="54">
-        <f t="array" ref="C22:C22">LOOKUP(2,1/('Deliverables Sheet'!S67:S72&lt;&gt;0),'Deliverables Sheet'!S67:S72)</f>
         <v>160.82</v>
       </c>
-      <c r="D22" s="54" t="e">
-        <f t="array" ref="D22:D22">LOOKUP(2,1/('Deliverables Sheet'!T67:T72&lt;&gt;0),'Deliverables Sheet'!T67:T72)</f>
-        <v>#N/A</v>
+      <c r="D22" s="54">
+        <v>2.75</v>
       </c>
       <c r="E22" s="54">
-        <f t="array" ref="E22:E22">LOOKUP(2,1/('Deliverables Sheet'!U67:U72&lt;&gt;0),'Deliverables Sheet'!U67:U72)</f>
-        <v>160.82</v>
+        <v>158.07</v>
       </c>
       <c r="F22" s="54"/>
       <c r="G22" s="54"/>
@@ -26162,7 +26132,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26181,7 +26151,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <f>'Main Sheet'!A24</f>
         <v>9259</v>
@@ -26190,11 +26160,14 @@
         <f>'Main Sheet'!B24</f>
         <v>Andrew Reeve Stage 2</v>
       </c>
-      <c r="C24" s="54"/>
-      <c r="D24" s="54"/>
-      <c r="E24" s="54" t="e">
-        <f t="array" ref="E24:E24">LOOKUP(2,1/('Deliverables Sheet'!U69:U74&lt;&gt;0),'Deliverables Sheet'!U69:U74)</f>
-        <v>#N/A</v>
+      <c r="C24" s="54">
+        <v>470.62</v>
+      </c>
+      <c r="D24" s="54">
+        <v>0</v>
+      </c>
+      <c r="E24" s="54">
+        <v>470.62</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>
@@ -26213,7 +26186,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26232,7 +26205,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <f>'Main Sheet'!A26</f>
         <v>8352</v>
@@ -26242,16 +26215,13 @@
         <v>5 Sanscrit Place</v>
       </c>
       <c r="C26" s="54">
-        <f t="array" ref="C26:C26">LOOKUP(2,1/('Deliverables Sheet'!S81:S86&lt;&gt;0),'Deliverables Sheet'!S81:S86)</f>
         <v>139.07</v>
       </c>
       <c r="D26" s="54">
-        <f t="array" ref="D26:D26">LOOKUP(2,1/('Deliverables Sheet'!T81:T86&lt;&gt;0),'Deliverables Sheet'!T81:T86)</f>
         <v>143.25</v>
       </c>
       <c r="E26" s="54">
-        <f t="array" ref="E26:E26">LOOKUP(2,1/('Deliverables Sheet'!U81:U86&lt;&gt;0),'Deliverables Sheet'!U81:U86)</f>
-        <v>-4.18000000000001</v>
+        <v>-4.180000000000007</v>
       </c>
       <c r="F26" s="54"/>
       <c r="G26" s="54"/>
@@ -26268,7 +26238,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26287,7 +26257,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <f>'Main Sheet'!A28</f>
         <v>8234</v>
@@ -26297,16 +26267,13 @@
         <v>Melhuish House</v>
       </c>
       <c r="C28" s="54">
-        <f t="array" ref="C28:C28">LOOKUP(2,1/('Deliverables Sheet'!S88:S93&lt;&gt;0),'Deliverables Sheet'!S88:S93)</f>
         <v>231.75</v>
       </c>
       <c r="D28" s="54">
-        <f t="array" ref="D28:D28">LOOKUP(2,1/('Deliverables Sheet'!T88:T93&lt;&gt;0),'Deliverables Sheet'!T88:T93)</f>
-        <v>148.5</v>
+        <v>204.75</v>
       </c>
       <c r="E28" s="54">
-        <f t="array" ref="E28:E28">LOOKUP(2,1/('Deliverables Sheet'!U88:U93&lt;&gt;0),'Deliverables Sheet'!U88:U93)</f>
-        <v>83.25</v>
+        <v>27</v>
       </c>
       <c r="F28" s="54"/>
       <c r="G28" s="54"/>
@@ -26324,7 +26291,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26343,7 +26310,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <f>'Main Sheet'!A30</f>
         <v>8214</v>
@@ -26353,15 +26320,12 @@
         <v>6 Tiroroa Lane</v>
       </c>
       <c r="C30" s="54">
-        <f t="array" ref="C30:C30">LOOKUP(2,1/('Deliverables Sheet'!S95:S100&lt;&gt;0),'Deliverables Sheet'!S95:S100)</f>
         <v>147.9</v>
       </c>
       <c r="D30" s="54">
-        <f t="array" ref="D30:D30">LOOKUP(2,1/('Deliverables Sheet'!T95:T100&lt;&gt;0),'Deliverables Sheet'!T95:T100)</f>
         <v>5</v>
       </c>
       <c r="E30" s="54">
-        <f t="array" ref="E30:E30">LOOKUP(2,1/('Deliverables Sheet'!U95:U100&lt;&gt;0),'Deliverables Sheet'!U95:U100)</f>
         <v>142.9</v>
       </c>
       <c r="F30" s="54"/>
@@ -26384,7 +26348,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26403,7 +26367,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <f>'Main Sheet'!A32</f>
         <v>6792</v>
@@ -26413,16 +26377,13 @@
         <v>Major Hornbrook </v>
       </c>
       <c r="C32" s="54">
-        <f t="array" ref="C32:C32">LOOKUP(2,1/('Deliverables Sheet'!S102:S107&lt;&gt;0),'Deliverables Sheet'!S102:S107)</f>
         <v>208.2</v>
       </c>
       <c r="D32" s="54">
-        <f t="array" ref="D32:D32">LOOKUP(2,1/('Deliverables Sheet'!T102:T107&lt;&gt;0),'Deliverables Sheet'!T102:T107)</f>
         <v>317.25</v>
       </c>
       <c r="E32" s="54">
-        <f t="array" ref="E32:E32">LOOKUP(2,1/('Deliverables Sheet'!U102:U107&lt;&gt;0),'Deliverables Sheet'!U102:U107)</f>
-        <v>-109.05</v>
+        <v>-109.05000000000001</v>
       </c>
       <c r="F32" s="54"/>
       <c r="G32" s="54"/>
@@ -26437,7 +26398,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26456,7 +26417,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <f>'Main Sheet'!A34</f>
         <v>8840</v>
@@ -26466,16 +26427,13 @@
         <v>Inline Architecture</v>
       </c>
       <c r="C34" s="54">
-        <f t="array" ref="C34:C34">LOOKUP(2,1/('Deliverables Sheet'!S109:S114&lt;&gt;0),'Deliverables Sheet'!S109:S114)</f>
-        <v>316.34</v>
+        <v>324.19</v>
       </c>
       <c r="D34" s="54">
-        <f t="array" ref="D34:D34">LOOKUP(2,1/('Deliverables Sheet'!T109:T114&lt;&gt;0),'Deliverables Sheet'!T109:T114)</f>
-        <v>204.75</v>
+        <v>412.5</v>
       </c>
       <c r="E34" s="54">
-        <f t="array" ref="E34:E34">LOOKUP(2,1/('Deliverables Sheet'!U109:U114&lt;&gt;0),'Deliverables Sheet'!U109:U114)</f>
-        <v>111.59</v>
+        <v>-88.31</v>
       </c>
       <c r="F34" s="54"/>
       <c r="G34" s="54"/>
@@ -26492,7 +26450,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26511,7 +26469,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <f>'Main Sheet'!A36</f>
         <v>8769</v>
@@ -26520,17 +26478,14 @@
         <f>'Main Sheet'!B36</f>
         <v>Percival Bach</v>
       </c>
-      <c r="C36" s="54" t="e">
-        <f t="array" ref="C36:C36">LOOKUP(2,1/('Deliverables Sheet'!S116:S121&lt;&gt;0),'Deliverables Sheet'!S116:S121)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D36" s="54" t="e">
-        <f t="array" ref="D36:D36">LOOKUP(2,1/('Deliverables Sheet'!T116:T121&lt;&gt;0),'Deliverables Sheet'!T116:T121)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E36" s="54" t="e">
-        <f t="array" ref="E36:E36">LOOKUP(2,1/('Deliverables Sheet'!U116:U121&lt;&gt;0),'Deliverables Sheet'!U116:U121)</f>
-        <v>#N/A</v>
+      <c r="C36" s="54">
+        <v>84.05</v>
+      </c>
+      <c r="D36" s="54">
+        <v>0</v>
+      </c>
+      <c r="E36" s="54">
+        <v>84.05</v>
       </c>
       <c r="F36" s="54"/>
       <c r="G36" s="54"/>
@@ -26549,7 +26504,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26568,7 +26523,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <f>'Main Sheet'!A38</f>
         <v>7901</v>
@@ -26578,16 +26533,13 @@
         <v>St Albans Street</v>
       </c>
       <c r="C38" s="54">
-        <f t="array" ref="C38:C38">LOOKUP(2,1/('Deliverables Sheet'!S123:S128&lt;&gt;0),'Deliverables Sheet'!S123:S128)</f>
-        <v>273.37</v>
-      </c>
-      <c r="D38" s="54" t="e">
-        <f t="array" ref="D38:D38">LOOKUP(2,1/('Deliverables Sheet'!T123:T128&lt;&gt;0),'Deliverables Sheet'!T123:T128)</f>
-        <v>#N/A</v>
+        <v>290.15</v>
+      </c>
+      <c r="D38" s="54">
+        <v>91.75</v>
       </c>
       <c r="E38" s="54">
-        <f t="array" ref="E38:E38">LOOKUP(2,1/('Deliverables Sheet'!U123:U128&lt;&gt;0),'Deliverables Sheet'!U123:U128)</f>
-        <v>273.37</v>
+        <v>198.39999999999998</v>
       </c>
       <c r="F38" s="54"/>
       <c r="G38" s="54"/>
@@ -26609,7 +26561,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26628,7 +26580,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <f>'Main Sheet'!A40</f>
         <v>8923</v>
@@ -26638,16 +26590,13 @@
         <v>4 Perry St</v>
       </c>
       <c r="C40" s="54">
-        <f t="array" ref="C40:C40">LOOKUP(2,1/('Deliverables Sheet'!S130:S135&lt;&gt;0),'Deliverables Sheet'!S130:S135)</f>
-        <v>157</v>
+        <v>156.69</v>
       </c>
       <c r="D40" s="54">
-        <f t="array" ref="D40:D40">LOOKUP(2,1/('Deliverables Sheet'!T130:T135&lt;&gt;0),'Deliverables Sheet'!T130:T135)</f>
         <v>2</v>
       </c>
       <c r="E40" s="54">
-        <f t="array" ref="E40:E40">LOOKUP(2,1/('Deliverables Sheet'!U130:U135&lt;&gt;0),'Deliverables Sheet'!U130:U135)</f>
-        <v>155</v>
+        <v>154.69</v>
       </c>
       <c r="F40" s="54">
         <v>60</v>
@@ -26668,7 +26617,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26687,7 +26636,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <f>'Main Sheet'!A42</f>
         <v>7864</v>
@@ -26697,16 +26646,13 @@
         <v>Ryans House</v>
       </c>
       <c r="C42" s="54">
-        <f t="array" ref="C42:C42">LOOKUP(2,1/('Deliverables Sheet'!S137:S142&lt;&gt;0),'Deliverables Sheet'!S137:S142)</f>
-        <v>193.82</v>
+        <v>200.82</v>
       </c>
       <c r="D42" s="54">
-        <f t="array" ref="D42:D42">LOOKUP(2,1/('Deliverables Sheet'!T137:T142&lt;&gt;0),'Deliverables Sheet'!T137:T142)</f>
-        <v>266.75</v>
+        <v>278.25</v>
       </c>
       <c r="E42" s="54">
-        <f t="array" ref="E42:E42">LOOKUP(2,1/('Deliverables Sheet'!U137:U142&lt;&gt;0),'Deliverables Sheet'!U137:U142)</f>
-        <v>-72.93</v>
+        <v>-77.43</v>
       </c>
       <c r="F42" s="54"/>
       <c r="G42" s="54"/>
@@ -26722,7 +26668,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26741,7 +26687,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <f>'Main Sheet'!A44</f>
         <v>7912</v>
@@ -26750,17 +26696,14 @@
         <f>'Main Sheet'!B44</f>
         <v>71A Fendalton Road </v>
       </c>
-      <c r="C44" s="54" t="e">
-        <f t="array" ref="C44:C44">LOOKUP(2,1/('Deliverables Sheet'!S144:S149&lt;&gt;0),'Deliverables Sheet'!S144:S149)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D44" s="54" t="e">
-        <f t="array" ref="D44:D44">LOOKUP(2,1/('Deliverables Sheet'!T144:T149&lt;&gt;0),'Deliverables Sheet'!T144:T149)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E44" s="54" t="e">
-        <f t="array" ref="E44:E44">LOOKUP(2,1/('Deliverables Sheet'!U144:U149&lt;&gt;0),'Deliverables Sheet'!U144:U149)</f>
-        <v>#N/A</v>
+      <c r="C44" s="54">
+        <v>497.55</v>
+      </c>
+      <c r="D44" s="54">
+        <v>58.25</v>
+      </c>
+      <c r="E44" s="54">
+        <v>439.3</v>
       </c>
       <c r="F44" s="54">
         <v>80</v>
@@ -26786,7 +26729,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26805,7 +26748,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <f>'Main Sheet'!A46</f>
         <v>8360</v>
@@ -26815,16 +26758,13 @@
         <v>Dixon House</v>
       </c>
       <c r="C46" s="54">
-        <f t="array" ref="C46:C46">LOOKUP(2,1/('Deliverables Sheet'!S151:S156&lt;&gt;0),'Deliverables Sheet'!S151:S156)</f>
         <v>210.6</v>
       </c>
       <c r="D46" s="54">
-        <f t="array" ref="D46:D46">LOOKUP(2,1/('Deliverables Sheet'!T151:T156&lt;&gt;0),'Deliverables Sheet'!T151:T156)</f>
         <v>260.75</v>
       </c>
       <c r="E46" s="54">
-        <f t="array" ref="E46:E46">LOOKUP(2,1/('Deliverables Sheet'!U151:U156&lt;&gt;0),'Deliverables Sheet'!U151:U156)</f>
-        <v>-50.15</v>
+        <v>-50.150000000000006</v>
       </c>
       <c r="F46" s="98"/>
       <c r="G46" s="98"/>
@@ -26839,7 +26779,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -26858,7 +26798,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <f>'Main Sheet'!A48</f>
         <v>8337</v>
@@ -26868,16 +26808,13 @@
         <v>Waimak Dairys </v>
       </c>
       <c r="C48" s="54">
-        <f t="array" ref="C48:C48">LOOKUP(2,1/('Deliverables Sheet'!S158:S163&lt;&gt;0),'Deliverables Sheet'!S158:S163)</f>
         <v>110.44</v>
       </c>
       <c r="D48" s="54">
-        <f t="array" ref="D48:D48">LOOKUP(2,1/('Deliverables Sheet'!T158:T163&lt;&gt;0),'Deliverables Sheet'!T158:T163)</f>
-        <v>44.75</v>
+        <v>60.75</v>
       </c>
       <c r="E48" s="54">
-        <f t="array" ref="E48:E48">LOOKUP(2,1/('Deliverables Sheet'!U158:U163&lt;&gt;0),'Deliverables Sheet'!U158:U163)</f>
-        <v>65.69</v>
+        <v>49.69</v>
       </c>
       <c r="F48" s="54"/>
       <c r="G48" s="54"/>
@@ -26896,7 +26833,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -26915,7 +26852,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <f>'Main Sheet'!A50</f>
         <v>9240</v>
@@ -26924,17 +26861,14 @@
         <f>'Main Sheet'!B50</f>
         <v>Daves Twizel Shack</v>
       </c>
-      <c r="C50" s="54" t="e">
-        <f t="array" ref="C50:C50">LOOKUP(2,1/('Deliverables Sheet'!S165:S170&lt;&gt;0),'Deliverables Sheet'!S165:S170)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D50" s="54" t="e">
-        <f t="array" ref="D50:D50">LOOKUP(2,1/('Deliverables Sheet'!T165:T170&lt;&gt;0),'Deliverables Sheet'!T165:T170)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E50" s="54" t="e">
-        <f t="array" ref="E50:E50">LOOKUP(2,1/('Deliverables Sheet'!U165:U170&lt;&gt;0),'Deliverables Sheet'!U165:U170)</f>
-        <v>#N/A</v>
+      <c r="C50" s="54">
+        <v>0</v>
+      </c>
+      <c r="D50" s="54">
+        <v>0</v>
+      </c>
+      <c r="E50" s="54">
+        <v>0</v>
       </c>
       <c r="F50" s="54"/>
       <c r="G50" s="54"/>
@@ -26953,7 +26887,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -26972,7 +26906,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <f>'Main Sheet'!A52</f>
         <v>7428</v>
@@ -26982,16 +26916,13 @@
         <v>FAB Pegasus Lakeside</v>
       </c>
       <c r="C52" s="54">
-        <f t="array" ref="C52:C52">LOOKUP(2,1/('Deliverables Sheet'!S172:S177&lt;&gt;0),'Deliverables Sheet'!S172:S177)</f>
         <v>659.73</v>
       </c>
       <c r="D52" s="54">
-        <f t="array" ref="D52:D52">LOOKUP(2,1/('Deliverables Sheet'!T172:T177&lt;&gt;0),'Deliverables Sheet'!T172:T177)</f>
-        <v>304.75</v>
+        <v>430</v>
       </c>
       <c r="E52" s="54">
-        <f t="array" ref="E52:E52">LOOKUP(2,1/('Deliverables Sheet'!U172:U177&lt;&gt;0),'Deliverables Sheet'!U172:U177)</f>
-        <v>354.98</v>
+        <v>229.73000000000002</v>
       </c>
       <c r="F52" s="54"/>
       <c r="G52" s="54"/>
@@ -27013,7 +26944,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -27032,7 +26963,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <f>'Main Sheet'!A54</f>
         <v>9351</v>
@@ -27042,16 +26973,13 @@
         <v>Harewood Golf Club</v>
       </c>
       <c r="C54" s="54">
-        <f t="array" ref="C54:C54">LOOKUP(2,1/('Deliverables Sheet'!S179:S184&lt;&gt;0),'Deliverables Sheet'!S179:S184)</f>
         <v>125.17</v>
       </c>
       <c r="D54" s="54">
-        <f t="array" ref="D54:D54">LOOKUP(2,1/('Deliverables Sheet'!T179:T184&lt;&gt;0),'Deliverables Sheet'!T179:T184)</f>
-        <v>11.25</v>
+        <v>23.75</v>
       </c>
       <c r="E54" s="54">
-        <f t="array" ref="E54:E54">LOOKUP(2,1/('Deliverables Sheet'!U179:U184&lt;&gt;0),'Deliverables Sheet'!U179:U184)</f>
-        <v>113.92</v>
+        <v>101.42</v>
       </c>
       <c r="F54" s="54"/>
       <c r="G54" s="54"/>
@@ -27073,7 +27001,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -27092,7 +27020,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <f>'Main Sheet'!A56</f>
         <v>7429</v>
@@ -27102,16 +27030,13 @@
         <v>Taggart House</v>
       </c>
       <c r="C56" s="54">
-        <f t="array" ref="C56:C56">LOOKUP(2,1/('Deliverables Sheet'!S186:S191&lt;&gt;0),'Deliverables Sheet'!S186:S191)</f>
         <v>130.62</v>
       </c>
       <c r="D56" s="54">
-        <f t="array" ref="D56:D56">LOOKUP(2,1/('Deliverables Sheet'!T186:T191&lt;&gt;0),'Deliverables Sheet'!T186:T191)</f>
-        <v>32.25</v>
+        <v>34.75</v>
       </c>
       <c r="E56" s="54">
-        <f t="array" ref="E56:E56">LOOKUP(2,1/('Deliverables Sheet'!U186:U191&lt;&gt;0),'Deliverables Sheet'!U186:U191)</f>
-        <v>98.37</v>
+        <v>95.87</v>
       </c>
       <c r="F56" s="54"/>
       <c r="G56" s="54"/>
@@ -27131,7 +27056,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -27150,7 +27075,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <f>'Main Sheet'!A58</f>
         <v>9508</v>
@@ -27159,17 +27084,14 @@
         <f>'Main Sheet'!B58</f>
         <v>St Barnabas Church</v>
       </c>
-      <c r="C58" s="54" t="e">
-        <f t="array" ref="C58:C58">LOOKUP(2,1/('Deliverables Sheet'!S193:S198&lt;&gt;0),'Deliverables Sheet'!S193:S198)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D58" s="54" t="e">
-        <f t="array" ref="D58:D58">LOOKUP(2,1/('Deliverables Sheet'!T193:T198&lt;&gt;0),'Deliverables Sheet'!T193:T198)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E58" s="54" t="e">
-        <f t="array" ref="E58:E58">LOOKUP(2,1/('Deliverables Sheet'!U193:U198&lt;&gt;0),'Deliverables Sheet'!U193:U198)</f>
-        <v>#N/A</v>
+      <c r="C58" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="D58" s="54">
+        <v>5.75</v>
+      </c>
+      <c r="E58" s="54">
+        <v>134.4</v>
       </c>
       <c r="F58" s="54"/>
       <c r="G58" s="54"/>
@@ -27190,7 +27112,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27209,7 +27131,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19">
         <f>'Main Sheet'!A60</f>
         <v>0</v>
@@ -27243,7 +27165,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27262,7 +27184,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19">
         <f>'Main Sheet'!A62</f>
         <v>0</v>
@@ -27296,7 +27218,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27315,7 +27237,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <f>'Main Sheet'!A64</f>
         <v>8946</v>
@@ -27325,15 +27247,12 @@
         <v>Westcoast Vaults</v>
       </c>
       <c r="C64" s="54">
-        <f t="array" ref="C64:C64">LOOKUP(2,1/('Deliverables Sheet'!S214:S219&lt;&gt;0),'Deliverables Sheet'!S214:S219)</f>
         <v>358.86</v>
       </c>
-      <c r="D64" s="54" t="e">
-        <f t="array" ref="D64:D64">LOOKUP(2,1/('Deliverables Sheet'!T214:T219&lt;&gt;0),'Deliverables Sheet'!T214:T219)</f>
-        <v>#N/A</v>
+      <c r="D64" s="54">
+        <v>0</v>
       </c>
       <c r="E64" s="54">
-        <f t="array" ref="E64:E64">LOOKUP(2,1/('Deliverables Sheet'!U214:U219&lt;&gt;0),'Deliverables Sheet'!U214:U219)</f>
         <v>358.86</v>
       </c>
       <c r="F64" s="54"/>
@@ -27353,7 +27272,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27372,7 +27291,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <f>'Main Sheet'!A66</f>
         <v>8308</v>
@@ -27382,16 +27301,13 @@
         <v>Roydvale</v>
       </c>
       <c r="C66" s="54">
-        <f t="array" ref="C66:C66">LOOKUP(2,1/('Deliverables Sheet'!S221:S226&lt;&gt;0),'Deliverables Sheet'!S221:S226)</f>
         <v>2312.68</v>
       </c>
       <c r="D66" s="54">
-        <f t="array" ref="D66:D66">LOOKUP(2,1/('Deliverables Sheet'!T221:T226&lt;&gt;0),'Deliverables Sheet'!T221:T226)</f>
-        <v>1014.25</v>
+        <v>1120.5</v>
       </c>
       <c r="E66" s="54">
-        <f t="array" ref="E66:E66">LOOKUP(2,1/('Deliverables Sheet'!U221:U226&lt;&gt;0),'Deliverables Sheet'!U221:U226)</f>
-        <v>1298.43</v>
+        <v>1192.1799999999998</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>
@@ -27416,7 +27332,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -27435,7 +27351,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27454,7 +27370,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -27473,7 +27389,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>144</v>
@@ -27539,7 +27455,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>145</v>
@@ -27605,7 +27521,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>146</v>
@@ -27671,7 +27587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>147</v>
@@ -27728,7 +27644,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>148</v>
@@ -27785,7 +27701,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -27804,7 +27720,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>149</v>
@@ -27851,7 +27767,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>151</v>
@@ -27896,7 +27812,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -27915,7 +27831,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>152</v>
@@ -27938,7 +27854,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>154</v>
@@ -27961,7 +27877,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>155</v>
@@ -27984,7 +27900,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>156</v>
@@ -28007,7 +27923,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>157</v>
@@ -28030,7 +27946,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>158</v>
@@ -28053,7 +27969,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>159</v>
@@ -28076,7 +27992,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>160</v>
@@ -28099,7 +28015,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>161</v>
@@ -28122,7 +28038,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>162</v>
@@ -28145,7 +28061,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>163</v>
@@ -28168,7 +28084,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>164</v>
@@ -28191,7 +28107,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -28212,7 +28128,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -28233,7 +28149,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -28254,7 +28170,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -28275,7 +28191,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -28296,7 +28212,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -28317,7 +28233,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28338,7 +28254,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>165</v>
@@ -28361,7 +28277,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>166</v>
@@ -28384,7 +28300,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>167</v>
@@ -28407,7 +28323,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>168</v>
@@ -28430,7 +28346,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>169</v>
@@ -28453,7 +28369,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>170</v>
@@ -28476,7 +28392,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>171</v>
@@ -28499,7 +28415,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -28518,7 +28434,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28537,7 +28453,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28556,7 +28472,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -28575,7 +28491,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>172</v>
@@ -28650,10 +28566,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>173</v>
       </c>
@@ -28685,7 +28602,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>174</v>
       </c>
@@ -28718,7 +28635,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>175</v>
       </c>
@@ -28751,7 +28668,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>176</v>
       </c>
@@ -28784,7 +28701,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>177</v>
       </c>
@@ -28817,7 +28734,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>178</v>
       </c>
@@ -28850,7 +28767,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>179</v>
       </c>
@@ -28883,7 +28800,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>180</v>
       </c>
@@ -28916,7 +28833,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28947,7 +28864,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -28978,7 +28895,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>181</v>
       </c>
@@ -29011,7 +28928,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>182</v>
       </c>
@@ -29044,7 +28961,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>183</v>
       </c>
@@ -29077,7 +28994,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>184</v>
       </c>
@@ -29110,7 +29027,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>185</v>
       </c>
@@ -29143,7 +29060,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>186</v>
       </c>
@@ -29176,7 +29093,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>187</v>
       </c>
@@ -29209,7 +29126,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>188</v>
       </c>
@@ -29242,7 +29159,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>189</v>
       </c>
@@ -29275,7 +29192,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>190</v>
       </c>
@@ -29308,7 +29225,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>191</v>
       </c>
@@ -29341,7 +29258,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>192</v>
       </c>
@@ -29374,7 +29291,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>193</v>
       </c>
@@ -29407,7 +29324,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>194</v>
       </c>
@@ -29440,7 +29357,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>195</v>
       </c>
@@ -29473,7 +29390,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>196</v>
       </c>
@@ -29506,7 +29423,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>197</v>
       </c>
@@ -29538,7 +29455,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>198</v>
       </c>
@@ -29570,7 +29487,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>199</v>
       </c>
@@ -29602,7 +29519,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>200</v>
       </c>
@@ -29634,7 +29551,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>201</v>
       </c>
@@ -29666,7 +29583,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29696,7 +29613,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29726,7 +29643,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>202</v>
       </c>
@@ -29758,7 +29675,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>203</v>
       </c>
@@ -29790,7 +29707,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>204</v>
       </c>
@@ -29822,7 +29739,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>205</v>
       </c>
@@ -29854,7 +29771,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>206</v>
       </c>
@@ -29886,7 +29803,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29916,7 +29833,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>207</v>
       </c>
@@ -29948,7 +29865,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>208</v>
       </c>
@@ -29980,7 +29897,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>209</v>
       </c>
@@ -30012,7 +29929,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>210</v>
       </c>
@@ -30044,7 +29961,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -30074,7 +29991,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -30104,7 +30021,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -30134,7 +30051,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -30164,7 +30081,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>211</v>
       </c>
@@ -30196,7 +30113,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>212</v>
       </c>
@@ -30228,7 +30145,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -30258,7 +30175,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -30288,7 +30205,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -30318,7 +30235,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30348,7 +30265,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30378,7 +30295,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30473,10 +30390,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>213</v>
       </c>
@@ -30508,7 +30426,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30539,7 +30457,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30570,7 +30488,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30601,7 +30519,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30632,7 +30550,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30663,7 +30581,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30694,7 +30612,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30725,7 +30643,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30756,7 +30674,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30787,7 +30705,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30818,7 +30736,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30849,7 +30767,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30880,7 +30798,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30911,7 +30829,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30942,7 +30860,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -30973,7 +30891,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31004,7 +30922,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31035,7 +30953,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31066,7 +30984,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -31097,7 +31015,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -31127,7 +31045,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -31157,7 +31075,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -31187,7 +31105,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -31217,7 +31135,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -31247,7 +31165,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -31277,7 +31195,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -31307,7 +31225,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31337,7 +31255,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31367,7 +31285,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31397,7 +31315,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31427,7 +31345,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31457,7 +31375,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31487,7 +31405,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31517,7 +31435,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31547,7 +31465,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31577,7 +31495,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>211</v>
       </c>
@@ -31609,7 +31527,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>212</v>
       </c>
@@ -31641,7 +31559,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31671,7 +31589,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31701,7 +31619,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31731,7 +31649,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31761,7 +31679,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31791,7 +31709,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53534,19 +53452,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53560,7 +53478,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>220</v>
       </c>
@@ -53572,7 +53490,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>221</v>
       </c>
@@ -53583,7 +53501,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>222</v>
       </c>
@@ -53594,7 +53512,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>223</v>
       </c>
@@ -53605,13 +53523,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-18T23:50:32Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -6719,7 +6719,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F32" s="13" t="s">
         <v>27</v>
@@ -17252,7 +17252,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -22964,7 +22964,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -22978,7 +22978,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23000,7 +23000,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -23048,7 +23048,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23066,7 +23066,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23113,7 +23113,7 @@
         <v>-2588.8525</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23130,7 +23130,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23180,7 +23180,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23197,7 +23197,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23240,7 +23240,7 @@
         <v>34.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23257,7 +23257,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23304,7 +23304,7 @@
         <v>40.40408523144744</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23321,7 +23321,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23369,7 +23369,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23386,7 +23386,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23433,7 +23433,7 @@
         <v>45.876428571428605</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23450,7 +23450,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23495,7 +23495,7 @@
         <v>98.73233429394816</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23512,7 +23512,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23562,7 +23562,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23579,7 +23579,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23618,7 +23618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23635,7 +23635,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23676,7 +23676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23693,7 +23693,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -23730,7 +23730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -23747,7 +23747,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -23792,7 +23792,7 @@
         <v>-1.343804537521815</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -23809,7 +23809,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -23852,7 +23852,7 @@
         <v>30.14242424242425</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -23869,7 +23869,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -23912,7 +23912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -23929,7 +23929,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -23976,7 +23976,7 @@
         <v>5.481184600197436</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -23993,7 +23993,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24038,7 +24038,7 @@
         <v>252.9351404151404</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24055,7 +24055,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24098,7 +24098,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24115,7 +24115,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24156,7 +24156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24173,7 +24173,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24218,7 +24218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24235,7 +24235,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24278,7 +24278,7 @@
         <v>-11.131808809746953</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24295,7 +24295,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24332,7 +24332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24349,7 +24349,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24390,7 +24390,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24407,7 +24407,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24450,7 +24450,7 @@
         <v>-179.4969832402235</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24467,7 +24467,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24509,7 +24509,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24526,7 +24526,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24571,7 +24571,7 @@
         <v>79.30441796516956</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24588,7 +24588,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24633,7 +24633,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24650,7 +24650,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24695,7 +24695,7 @@
         <v>-120.76000000000003</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -24712,7 +24712,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -24749,7 +24749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -24766,7 +24766,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -24783,7 +24783,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -24800,7 +24800,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -24821,7 +24821,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -24838,7 +24838,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -24941,7 +24941,7 @@
         <v>6.191319240032102</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -24958,7 +24958,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -24975,7 +24975,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -25010,7 +25010,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -25393,7 +25393,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25404,7 +25404,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25425,7 +25425,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -25487,7 +25487,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -25545,7 +25545,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25579,7 +25579,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25598,7 +25598,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25632,7 +25632,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25651,7 +25651,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -25685,7 +25685,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -25704,7 +25704,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -25740,7 +25740,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -25759,7 +25759,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -25797,7 +25797,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -25816,7 +25816,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -25854,7 +25854,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -25873,7 +25873,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -25906,7 +25906,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -25925,7 +25925,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -25958,7 +25958,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -25977,7 +25977,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -26008,7 +26008,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26027,7 +26027,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26062,7 +26062,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26081,7 +26081,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26114,7 +26114,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26133,7 +26133,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26164,7 +26164,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26183,7 +26183,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -26215,7 +26215,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26234,7 +26234,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26270,7 +26270,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26289,7 +26289,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26318,7 +26318,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26337,7 +26337,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26368,7 +26368,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26387,7 +26387,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26420,7 +26420,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26439,7 +26439,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26475,7 +26475,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26494,7 +26494,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26529,7 +26529,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26548,7 +26548,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26578,7 +26578,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26597,7 +26597,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26637,7 +26637,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26656,7 +26656,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -26685,7 +26685,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -26704,7 +26704,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -26737,7 +26737,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -26756,7 +26756,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -26789,7 +26789,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -26808,7 +26808,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -26844,7 +26844,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -26863,7 +26863,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -26899,7 +26899,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -26918,7 +26918,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -26952,7 +26952,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -26971,7 +26971,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -27006,7 +27006,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27025,7 +27025,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -27044,7 +27044,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27063,7 +27063,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -27084,7 +27084,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27103,7 +27103,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -27136,7 +27136,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27155,7 +27155,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -27194,7 +27194,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -27213,7 +27213,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27232,7 +27232,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -27251,7 +27251,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -27296,7 +27296,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -27335,7 +27335,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -27364,7 +27364,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -27409,7 +27409,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -27454,7 +27454,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -27473,7 +27473,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -27520,7 +27520,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -27565,7 +27565,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -27584,7 +27584,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -27607,7 +27607,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -27630,7 +27630,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -27653,7 +27653,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -27676,7 +27676,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -27699,7 +27699,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -27722,7 +27722,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -27745,7 +27745,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -27768,7 +27768,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -27791,7 +27791,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -27814,7 +27814,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -27837,7 +27837,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -27860,7 +27860,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -27881,7 +27881,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -27902,7 +27902,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -27923,7 +27923,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -27944,7 +27944,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -27965,7 +27965,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -27986,7 +27986,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28007,7 +28007,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -28030,7 +28030,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -28053,7 +28053,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -28076,7 +28076,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -28099,7 +28099,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -28122,7 +28122,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -28145,7 +28145,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -28168,7 +28168,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -28187,7 +28187,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28206,7 +28206,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28225,7 +28225,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -28244,7 +28244,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -28318,11 +28318,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -28354,7 +28353,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -28387,7 +28386,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -28420,7 +28419,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -28453,7 +28452,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -28486,7 +28485,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -28519,7 +28518,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -28552,7 +28551,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -28585,7 +28584,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28616,7 +28615,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -28647,7 +28646,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -28680,7 +28679,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -28713,7 +28712,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -28746,7 +28745,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -28779,7 +28778,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -28812,7 +28811,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -28845,7 +28844,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -28878,7 +28877,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -28911,7 +28910,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -28944,7 +28943,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -28977,7 +28976,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -29010,7 +29009,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -29043,7 +29042,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -29076,7 +29075,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -29109,7 +29108,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -29142,7 +29141,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -29175,7 +29174,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -29207,7 +29206,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -29239,7 +29238,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -29271,7 +29270,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -29303,7 +29302,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -29335,7 +29334,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29365,7 +29364,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29395,7 +29394,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -29427,7 +29426,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -29459,7 +29458,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -29491,7 +29490,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -29523,7 +29522,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -29555,7 +29554,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29585,7 +29584,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -29617,7 +29616,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -29649,7 +29648,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -29681,7 +29680,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -29713,7 +29712,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -29743,7 +29742,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -29773,7 +29772,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -29803,7 +29802,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -29833,7 +29832,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -29865,7 +29864,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -29897,7 +29896,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -29927,7 +29926,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -29957,7 +29956,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -29987,7 +29986,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30017,7 +30016,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30047,7 +30046,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30142,11 +30141,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -30178,7 +30176,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30209,7 +30207,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30240,7 +30238,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30271,7 +30269,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30302,7 +30300,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30333,7 +30331,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30364,7 +30362,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30395,7 +30393,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30426,7 +30424,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30457,7 +30455,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30488,7 +30486,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30519,7 +30517,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30550,7 +30548,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30581,7 +30579,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30612,7 +30610,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -30643,7 +30641,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -30674,7 +30672,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -30705,7 +30703,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -30736,7 +30734,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -30767,7 +30765,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -30797,7 +30795,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -30827,7 +30825,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -30857,7 +30855,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -30887,7 +30885,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -30917,7 +30915,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -30947,7 +30945,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -30977,7 +30975,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31007,7 +31005,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31037,7 +31035,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31067,7 +31065,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31097,7 +31095,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31127,7 +31125,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31157,7 +31155,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31187,7 +31185,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31217,7 +31215,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31247,7 +31245,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -31279,7 +31277,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -31311,7 +31309,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31341,7 +31339,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31371,7 +31369,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31401,7 +31399,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31431,7 +31429,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31461,7 +31459,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53204,19 +53202,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53230,7 +53228,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -53242,7 +53240,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -53253,7 +53251,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -53264,7 +53262,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -53275,13 +53273,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-19T00:19:24Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -11777,54 +11777,54 @@
         <v>94098.32</v>
       </c>
       <c r="I42" s="52">
-        <v>34659.62</v>
+        <v>34818.98</v>
       </c>
       <c r="J42" s="52">
         <v>69042.09000000001</v>
       </c>
       <c r="K42" s="52">
-        <v>28340.06</v>
+        <v>28340.060000000005</v>
       </c>
       <c r="L42" s="52">
-        <v>40702.03000000001</v>
+        <v>40702.030000000006</v>
       </c>
       <c r="M42" s="53">
-        <v>0.5895248825752524</v>
+        <v>0.5895248825752523</v>
       </c>
       <c r="N42" s="53"/>
       <c r="O42" s="52">
         <v>25056.23</v>
       </c>
       <c r="P42" s="52">
-        <v>6319.56</v>
+        <v>6478.92</v>
       </c>
       <c r="Q42" s="52">
-        <v>18736.67</v>
+        <v>18577.309999999998</v>
       </c>
       <c r="R42" s="53">
-        <v>0.7477848822428593</v>
+        <v>0.7414247873682512</v>
       </c>
       <c r="S42" s="54">
         <v>501.83</v>
       </c>
       <c r="T42" s="54">
-        <v>123.75</v>
+        <v>127.75</v>
       </c>
       <c r="U42" s="54">
-        <v>378.08</v>
+        <v>374.08</v>
       </c>
       <c r="V42" s="53">
-        <v>0.7534025466791543</v>
+        <v>0.7454317199051471</v>
       </c>
       <c r="W42" s="53"/>
       <c r="X42" s="55">
-        <v>14.050666666666666</v>
+        <v>12.363287671232877</v>
       </c>
       <c r="Y42" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z42" s="53">
-        <v>0.0478</v>
+        <v>0.0434</v>
       </c>
       <c r="AA42" s="56">
         <v>0.2663</v>
@@ -12230,54 +12230,54 @@
         <v>50582.37</v>
       </c>
       <c r="I49" s="52">
-        <v>25131.9</v>
+        <v>25211.58</v>
       </c>
       <c r="J49" s="52">
         <v>39438.990000000005</v>
       </c>
       <c r="K49" s="52">
-        <v>20456.64</v>
+        <v>20456.640000000003</v>
       </c>
       <c r="L49" s="52">
-        <v>18982.350000000006</v>
+        <v>18982.350000000002</v>
       </c>
       <c r="M49" s="53">
-        <v>0.4813092323104624</v>
+        <v>0.4813092323104623</v>
       </c>
       <c r="N49" s="53"/>
       <c r="O49" s="52">
         <v>11143.38</v>
       </c>
       <c r="P49" s="52">
-        <v>4675.26</v>
+        <v>4754.94</v>
       </c>
       <c r="Q49" s="52">
-        <v>6468.119999999999</v>
+        <v>6388.44</v>
       </c>
       <c r="R49" s="53">
-        <v>0.5804450714235716</v>
+        <v>0.5732946377131535</v>
       </c>
       <c r="S49" s="54">
         <v>223.22</v>
       </c>
       <c r="T49" s="54">
-        <v>102.25</v>
+        <v>104.25</v>
       </c>
       <c r="U49" s="54">
-        <v>120.97</v>
+        <v>118.97</v>
       </c>
       <c r="V49" s="53">
-        <v>0.5419317265478004</v>
+        <v>0.5329719559179285</v>
       </c>
       <c r="W49" s="53"/>
       <c r="X49" s="55">
-        <v>1.8598533007334963</v>
+        <v>1.0598561151079136</v>
       </c>
       <c r="Y49" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z49" s="53">
-        <v>0.0075</v>
+        <v>0.0044</v>
       </c>
       <c r="AA49" s="56">
         <v>0.23</v>
@@ -12681,54 +12681,54 @@
         <v>108880.28</v>
       </c>
       <c r="I56" s="52">
-        <v>90918.83</v>
+        <v>91257.87</v>
       </c>
       <c r="J56" s="52">
         <v>74953.01000000001</v>
       </c>
       <c r="K56" s="52">
-        <v>71302.07</v>
+        <v>71042.06999999999</v>
       </c>
       <c r="L56" s="52">
-        <v>3650.9400000000023</v>
+        <v>3910.940000000017</v>
       </c>
       <c r="M56" s="53">
-        <v>0.04870971826214854</v>
+        <v>0.052178558272710014</v>
       </c>
       <c r="N56" s="53"/>
       <c r="O56" s="52">
         <v>33927.27</v>
       </c>
       <c r="P56" s="52">
-        <v>19616.76</v>
+        <v>20215.8</v>
       </c>
       <c r="Q56" s="52">
-        <v>14310.509999999998</v>
+        <v>13711.469999999998</v>
       </c>
       <c r="R56" s="53">
-        <v>0.4217996319774624</v>
+        <v>0.4041430389182507</v>
       </c>
       <c r="S56" s="54">
         <v>679.42</v>
       </c>
       <c r="T56" s="54">
-        <v>413</v>
+        <v>427</v>
       </c>
       <c r="U56" s="54">
-        <v>266.41999999999996</v>
+        <v>252.41999999999996</v>
       </c>
       <c r="V56" s="53">
-        <v>0.39212858025963315</v>
+        <v>0.3715227694209767</v>
       </c>
       <c r="W56" s="53"/>
       <c r="X56" s="55">
-        <v>18.50767554479419</v>
+        <v>17.10686182669789</v>
       </c>
       <c r="Y56" s="55">
         <v>67.18600078134293</v>
       </c>
       <c r="Z56" s="53">
-        <v>0.0776</v>
+        <v>0.0741</v>
       </c>
       <c r="AA56" s="56">
         <v>0.2954</v>
@@ -13132,54 +13132,54 @@
         <v>15859.68</v>
       </c>
       <c r="I63" s="52">
-        <v>13601.05</v>
+        <v>13642</v>
       </c>
       <c r="J63" s="52">
         <v>12689.1</v>
       </c>
       <c r="K63" s="52">
-        <v>11685.13</v>
+        <v>11685.130000000001</v>
       </c>
       <c r="L63" s="52">
-        <v>1003.9700000000012</v>
+        <v>1003.9699999999993</v>
       </c>
       <c r="M63" s="53">
-        <v>0.07912066261594605</v>
+        <v>0.07912066261594591</v>
       </c>
       <c r="N63" s="53"/>
       <c r="O63" s="52">
         <v>3170.58</v>
       </c>
       <c r="P63" s="52">
-        <v>1915.92</v>
+        <v>1956.87</v>
       </c>
       <c r="Q63" s="52">
-        <v>1254.6599999999999</v>
+        <v>1213.71</v>
       </c>
       <c r="R63" s="53">
-        <v>0.39571939518952365</v>
+        <v>0.38280377722687964</v>
       </c>
       <c r="S63" s="54">
         <v>63.5</v>
       </c>
       <c r="T63" s="54">
-        <v>47.5</v>
+        <v>48.25</v>
       </c>
       <c r="U63" s="54">
-        <v>16</v>
+        <v>15.25</v>
       </c>
       <c r="V63" s="53">
-        <v>0.25196850393700787</v>
+        <v>0.24015748031496062</v>
       </c>
       <c r="W63" s="53"/>
       <c r="X63" s="55">
-        <v>58.04884210526316</v>
+        <v>56.29782383419689</v>
       </c>
       <c r="Y63" s="55">
         <v>71.82495570677168</v>
       </c>
       <c r="Z63" s="53">
-        <v>0.1686</v>
+        <v>0.1661</v>
       </c>
       <c r="AA63" s="56">
         <v>0.2233</v>
@@ -13946,19 +13946,19 @@
         <v>54302.66</v>
       </c>
       <c r="I77" s="52">
-        <v>22353.17</v>
+        <v>25724.04</v>
       </c>
       <c r="J77" s="52">
         <v>31383.390000000003</v>
       </c>
       <c r="K77" s="52">
-        <v>22353.17</v>
+        <v>25724.04</v>
       </c>
       <c r="L77" s="52">
-        <v>9030.220000000005</v>
+        <v>5659.350000000002</v>
       </c>
       <c r="M77" s="53">
-        <v>0.28773883254804544</v>
+        <v>0.18032946727552382</v>
       </c>
       <c r="N77" s="53"/>
       <c r="O77" s="52">
@@ -14800,54 +14800,54 @@
         <v>27002.93</v>
       </c>
       <c r="I91" s="52">
-        <v>25996.77</v>
+        <v>26156.33</v>
       </c>
       <c r="J91" s="52">
         <v>15440.32</v>
       </c>
       <c r="K91" s="52">
-        <v>15990.78</v>
+        <v>16043.360000000002</v>
       </c>
       <c r="L91" s="52">
-        <v>-550.460000000001</v>
+        <v>-603.0400000000027</v>
       </c>
       <c r="M91" s="53">
-        <v>-0.0356508155271394</v>
+        <v>-0.03905618536403408</v>
       </c>
       <c r="N91" s="53"/>
       <c r="O91" s="52">
         <v>11562.61</v>
       </c>
       <c r="P91" s="52">
-        <v>10005.99</v>
+        <v>10112.97</v>
       </c>
       <c r="Q91" s="52">
-        <v>1556.6200000000008</v>
+        <v>1449.6400000000012</v>
       </c>
       <c r="R91" s="53">
-        <v>0.13462531383485224</v>
+        <v>0.12537307753180305</v>
       </c>
       <c r="S91" s="68">
         <v>231.75</v>
       </c>
       <c r="T91" s="68">
-        <v>204.75</v>
+        <v>207.25</v>
       </c>
       <c r="U91" s="54">
-        <v>27</v>
+        <v>24.5</v>
       </c>
       <c r="V91" s="53">
-        <v>0.11650485436893204</v>
+        <v>0.10571736785329018</v>
       </c>
       <c r="W91" s="53"/>
       <c r="X91" s="55">
-        <v>34.316483516483515</v>
+        <v>33.13264173703257</v>
       </c>
       <c r="Y91" s="55">
         <v>43.49557070636461</v>
       </c>
       <c r="Z91" s="53">
-        <v>0.21280000000000002</v>
+        <v>0.2079</v>
       </c>
       <c r="AA91" s="56">
         <v>0.2718</v>
@@ -16067,54 +16067,54 @@
         <v>37601.88</v>
       </c>
       <c r="I112" s="52">
-        <v>38195.76</v>
+        <v>39781.27</v>
       </c>
       <c r="J112" s="52">
         <v>21415.85</v>
       </c>
       <c r="K112" s="52">
-        <v>19158.27</v>
+        <v>20554.529999999995</v>
       </c>
       <c r="L112" s="52">
-        <v>2257.579999999998</v>
+        <v>861.3200000000033</v>
       </c>
       <c r="M112" s="53">
-        <v>0.10541631548596009</v>
+        <v>0.04021880990014421</v>
       </c>
       <c r="N112" s="53"/>
       <c r="O112" s="52">
         <v>16186.03</v>
       </c>
       <c r="P112" s="52">
-        <v>19037.49</v>
+        <v>19226.74</v>
       </c>
       <c r="Q112" s="52">
-        <v>-2851.460000000001</v>
+        <v>-3040.710000000001</v>
       </c>
       <c r="R112" s="53">
-        <v>-0.1761679670678975</v>
+        <v>-0.1878601485354964</v>
       </c>
       <c r="S112" s="54">
         <v>324.19</v>
       </c>
       <c r="T112" s="54">
-        <v>412.5</v>
+        <v>417</v>
       </c>
       <c r="U112" s="54">
-        <v>-88.31</v>
+        <v>-92.81</v>
       </c>
       <c r="V112" s="53">
-        <v>-0.2724019864894044</v>
+        <v>-0.28628273543292515</v>
       </c>
       <c r="W112" s="53"/>
       <c r="X112" s="55">
-        <v>-6.6456484848484845</v>
+        <v>-10.37611510791367</v>
       </c>
       <c r="Y112" s="55">
         <v>65.70431400737223</v>
       </c>
       <c r="Z112" s="53">
-        <v>-0.07730000000000001</v>
+        <v>-0.122</v>
       </c>
       <c r="AA112" s="56">
         <v>0.3616</v>
@@ -16894,34 +16894,34 @@
         <v>95</v>
       </c>
       <c r="D126" s="52">
-        <v>99768.39</v>
+        <v>100987.51</v>
       </c>
       <c r="E126" s="52">
         <v>15366.74</v>
       </c>
       <c r="F126" s="52">
-        <v>84401.65</v>
+        <v>85620.76999999999</v>
       </c>
       <c r="G126" s="53">
-        <v>0.8459758647002321</v>
+        <v>0.8478352421997531</v>
       </c>
       <c r="H126" s="52">
-        <v>81719.58</v>
+        <v>82694.87</v>
       </c>
       <c r="I126" s="52">
         <v>18551.86</v>
       </c>
       <c r="J126" s="52">
-        <v>67238.96</v>
+        <v>68214.25</v>
       </c>
       <c r="K126" s="52">
         <v>14369.1</v>
       </c>
       <c r="L126" s="52">
-        <v>52869.86000000001</v>
+        <v>53845.15</v>
       </c>
       <c r="M126" s="53">
-        <v>0.7862980034194461</v>
+        <v>0.7893533975672239</v>
       </c>
       <c r="N126" s="53"/>
       <c r="O126" s="52">
@@ -16953,13 +16953,13 @@
         <v>-34.715204359673024</v>
       </c>
       <c r="Y126" s="55">
-        <v>62.2051177714286</v>
+        <v>63.04545035767707</v>
       </c>
       <c r="Z126" s="53">
         <v>-0.2073</v>
       </c>
       <c r="AA126" s="56">
-        <v>0.1809</v>
+        <v>0.1811</v>
       </c>
       <c r="AB126" s="57"/>
       <c r="AD126" s="35" t="s">
@@ -17252,7 +17252,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -17724,19 +17724,19 @@
         <v>22587.89</v>
       </c>
       <c r="I140" s="52">
-        <v>25550.31</v>
+        <v>25625.28</v>
       </c>
       <c r="J140" s="52">
         <v>12565.06</v>
       </c>
       <c r="K140" s="52">
-        <v>11750.840000000002</v>
+        <v>11825.81</v>
       </c>
       <c r="L140" s="52">
-        <v>814.2199999999975</v>
+        <v>739.25</v>
       </c>
       <c r="M140" s="53">
-        <v>0.06480032725669416</v>
+        <v>0.05883378193180136</v>
       </c>
       <c r="N140" s="53"/>
       <c r="O140" s="52">
@@ -17765,13 +17765,13 @@
       </c>
       <c r="W140" s="53"/>
       <c r="X140" s="55">
-        <v>18.68438454627134</v>
+        <v>18.414950584007187</v>
       </c>
       <c r="Y140" s="55">
         <v>40.64013272149188</v>
       </c>
       <c r="Z140" s="53">
-        <v>0.1691</v>
+        <v>0.1666</v>
       </c>
       <c r="AA140" s="56">
         <v>0.2654</v>
@@ -22964,7 +22964,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -22978,7 +22978,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23000,7 +23000,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -23048,7 +23048,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23066,7 +23066,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23113,7 +23113,7 @@
         <v>-2588.8525</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23130,7 +23130,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23180,7 +23180,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23197,7 +23197,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23240,7 +23240,7 @@
         <v>34.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23257,7 +23257,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23304,7 +23304,7 @@
         <v>40.40408523144744</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23321,7 +23321,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23369,7 +23369,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23386,7 +23386,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23397,10 +23397,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>2138.1600000000035</v>
+        <v>2297.520000000004</v>
       </c>
       <c r="E14" s="52">
-        <v>-2138.1600000000035</v>
+        <v>-2297.520000000004</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -23424,16 +23424,16 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-5138.1600000000035</v>
+        <v>-5297.520000000004</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>45.876428571428605</v>
-      </c>
-    </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>47.29928571428575</v>
+      </c>
+    </row>
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23450,7 +23450,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23461,10 +23461,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>5565.0300000000025</v>
+        <v>5644.710000000003</v>
       </c>
       <c r="E16" s="52">
-        <v>-5565.0300000000025</v>
+        <v>-5644.710000000003</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -23486,16 +23486,16 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-8565.030000000002</v>
+        <v>-8644.710000000003</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>98.73233429394816</v>
-      </c>
-    </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>99.65083573487036</v>
+      </c>
+    </row>
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23512,7 +23512,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23523,10 +23523,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>10982.64</v>
+        <v>11321.679999999993</v>
       </c>
       <c r="E18" s="52">
-        <v>-10982.64</v>
+        <v>-11321.679999999993</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -23550,19 +23550,19 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-19182.64</v>
+        <v>-19521.679999999993</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>101.49544973544974</v>
+        <v>103.28931216931213</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23579,7 +23579,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23590,10 +23590,10 @@
         <v>0</v>
       </c>
       <c r="D20" s="52">
-        <v>1407.8799999999992</v>
+        <v>1448.83</v>
       </c>
       <c r="E20" s="52">
-        <v>-1407.8799999999992</v>
+        <v>-1448.83</v>
       </c>
       <c r="F20" s="52"/>
       <c r="G20" s="53">
@@ -23611,14 +23611,14 @@
         <v>0</v>
       </c>
       <c r="M20" s="52">
-        <v>-1407.8799999999992</v>
+        <v>-1448.83</v>
       </c>
       <c r="N20" s="54"/>
       <c r="O20" s="58">
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23635,7 +23635,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23676,7 +23676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23693,7 +23693,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -23704,10 +23704,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>22353.17</v>
+        <v>25724.04</v>
       </c>
       <c r="E24" s="52">
-        <v>-22353.17</v>
+        <v>-25724.04</v>
       </c>
       <c r="F24" s="52"/>
       <c r="G24" s="53">
@@ -23723,14 +23723,14 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>-22353.17</v>
+        <v>-25724.04</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -23747,7 +23747,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -23792,7 +23792,7 @@
         <v>-1.343804537521815</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -23809,7 +23809,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -23820,10 +23820,10 @@
         <v>0</v>
       </c>
       <c r="D28" s="52">
-        <v>4476.1500000000015</v>
+        <v>4635.710000000003</v>
       </c>
       <c r="E28" s="52">
-        <v>-4476.1500000000015</v>
+        <v>-4635.710000000003</v>
       </c>
       <c r="F28" s="52">
         <v>0</v>
@@ -23843,16 +23843,16 @@
         <v>0</v>
       </c>
       <c r="M28" s="52">
-        <v>-4476.1500000000015</v>
+        <v>-4635.710000000003</v>
       </c>
       <c r="N28" s="54">
         <v>-148.5</v>
       </c>
       <c r="O28" s="58">
-        <v>30.14242424242425</v>
-      </c>
-    </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>31.216902356902377</v>
+      </c>
+    </row>
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -23869,7 +23869,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -23912,7 +23912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -23929,7 +23929,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -23976,7 +23976,7 @@
         <v>5.481184600197436</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -23993,7 +23993,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24004,16 +24004,16 @@
         <v>-35454.43</v>
       </c>
       <c r="D34" s="52">
-        <v>16334.04</v>
+        <v>17919.549999999996</v>
       </c>
       <c r="E34" s="52">
-        <v>-51788.47</v>
+        <v>-53373.979999999996</v>
       </c>
       <c r="F34" s="52">
         <v>0</v>
       </c>
       <c r="G34" s="53">
-        <v>1.4607051925528065</v>
+        <v>1.5054248509988737</v>
       </c>
       <c r="H34" s="53">
         <v>0.364182044343228</v>
@@ -24026,19 +24026,19 @@
         <v>0</v>
       </c>
       <c r="L34" s="53">
-        <v>1.4607051925528065</v>
+        <v>1.5054248509988737</v>
       </c>
       <c r="M34" s="52">
-        <v>-51788.47</v>
+        <v>-53373.979999999996</v>
       </c>
       <c r="N34" s="54">
         <v>-204.75</v>
       </c>
       <c r="O34" s="58">
-        <v>252.9351404151404</v>
-      </c>
-    </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>260.67877899877897</v>
+      </c>
+    </row>
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24055,7 +24055,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24098,7 +24098,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24115,7 +24115,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24156,7 +24156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24173,7 +24173,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24218,7 +24218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24235,7 +24235,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24246,14 +24246,14 @@
         <v>3554.300000000003</v>
       </c>
       <c r="D42" s="52">
-        <v>584.890000000003</v>
+        <v>659.8600000000006</v>
       </c>
       <c r="E42" s="52">
-        <v>2969.41</v>
+        <v>2894.4400000000023</v>
       </c>
       <c r="F42" s="52"/>
       <c r="G42" s="53">
-        <v>0.8354415778071624</v>
+        <v>0.8143488169259769</v>
       </c>
       <c r="H42" s="53">
         <v>0.257245709794332</v>
@@ -24266,19 +24266,19 @@
         <v>0</v>
       </c>
       <c r="L42" s="53">
-        <v>0.8354415778071624</v>
+        <v>0.8143488169259769</v>
       </c>
       <c r="M42" s="52">
-        <v>2969.41</v>
+        <v>2894.4400000000023</v>
       </c>
       <c r="N42" s="54">
         <v>-266.75</v>
       </c>
       <c r="O42" s="58">
-        <v>-11.131808809746953</v>
-      </c>
-    </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-10.850759137769456</v>
+      </c>
+    </row>
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24295,7 +24295,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24332,7 +24332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24349,7 +24349,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24390,7 +24390,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24407,7 +24407,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24450,7 +24450,7 @@
         <v>-179.4969832402235</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24467,7 +24467,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24509,7 +24509,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24526,7 +24526,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24571,7 +24571,7 @@
         <v>79.30441796516956</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24588,7 +24588,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24633,7 +24633,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24650,7 +24650,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24695,7 +24695,7 @@
         <v>-120.76000000000003</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -24712,7 +24712,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -24749,7 +24749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -24766,7 +24766,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -24783,7 +24783,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -24800,7 +24800,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -24821,7 +24821,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -24838,7 +24838,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -24941,7 +24941,7 @@
         <v>6.191319240032102</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -24958,7 +24958,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -24975,7 +24975,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -24986,22 +24986,22 @@
         <v>3865.1700000000037</v>
       </c>
       <c r="D69" s="104">
-        <v>180905.65</v>
+        <v>186715.58999999997</v>
       </c>
       <c r="E69" s="105">
-        <v>-177040.47999999995</v>
+        <v>-182850.41999999998</v>
       </c>
       <c r="F69" s="106" t="s">
         <v>122</v>
       </c>
       <c r="G69" s="107">
-        <v>-45.80406036474457</v>
+        <v>-47.30721287808811</v>
       </c>
       <c r="H69" s="108" t="s">
         <v>123</v>
       </c>
       <c r="I69" s="109">
-        <v>-57.17810083385718</v>
+        <v>-58.68125334720071</v>
       </c>
       <c r="J69" s="36"/>
       <c r="K69" s="36"/>
@@ -25010,7 +25010,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -25393,7 +25393,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25404,7 +25404,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25425,7 +25425,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -25487,7 +25487,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -25545,7 +25545,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25579,7 +25579,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25598,7 +25598,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25632,7 +25632,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25651,7 +25651,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -25685,7 +25685,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -25704,7 +25704,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -25740,7 +25740,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -25759,7 +25759,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -25797,7 +25797,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -25816,7 +25816,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -25827,10 +25827,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>123.75</v>
+        <v>127.75</v>
       </c>
       <c r="E14" s="54">
-        <v>378.08</v>
+        <v>374.08</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -25854,7 +25854,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -25873,7 +25873,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -25884,10 +25884,10 @@
         <v>223.22</v>
       </c>
       <c r="D16" s="54">
-        <v>102.25</v>
+        <v>104.25</v>
       </c>
       <c r="E16" s="54">
-        <v>120.97</v>
+        <v>118.97</v>
       </c>
       <c r="F16" s="54"/>
       <c r="G16" s="54"/>
@@ -25906,7 +25906,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -25925,7 +25925,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -25936,10 +25936,10 @@
         <v>679.42</v>
       </c>
       <c r="D18" s="54">
-        <v>413</v>
+        <v>427</v>
       </c>
       <c r="E18" s="54">
-        <v>266.41999999999996</v>
+        <v>252.41999999999996</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -25958,7 +25958,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -25977,7 +25977,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -25988,10 +25988,10 @@
         <v>63.5</v>
       </c>
       <c r="D20" s="54">
-        <v>47.5</v>
+        <v>48.25</v>
       </c>
       <c r="E20" s="54">
-        <v>16</v>
+        <v>15.25</v>
       </c>
       <c r="F20" s="54"/>
       <c r="G20" s="54"/>
@@ -26008,7 +26008,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26027,7 +26027,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26062,7 +26062,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26081,7 +26081,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26114,7 +26114,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26133,7 +26133,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26164,7 +26164,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26183,7 +26183,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -26194,10 +26194,10 @@
         <v>231.75</v>
       </c>
       <c r="D28" s="54">
-        <v>204.75</v>
+        <v>207.25</v>
       </c>
       <c r="E28" s="54">
-        <v>27</v>
+        <v>24.5</v>
       </c>
       <c r="F28" s="54"/>
       <c r="G28" s="54"/>
@@ -26215,7 +26215,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26234,7 +26234,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26270,7 +26270,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26289,7 +26289,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26318,7 +26318,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26337,7 +26337,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26348,10 +26348,10 @@
         <v>324.19</v>
       </c>
       <c r="D34" s="54">
-        <v>412.5</v>
+        <v>417</v>
       </c>
       <c r="E34" s="54">
-        <v>-88.31</v>
+        <v>-92.81</v>
       </c>
       <c r="F34" s="54"/>
       <c r="G34" s="54"/>
@@ -26368,7 +26368,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26387,7 +26387,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26420,7 +26420,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26439,7 +26439,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26475,7 +26475,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26494,7 +26494,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26529,7 +26529,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26548,7 +26548,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26578,7 +26578,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26597,7 +26597,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26637,7 +26637,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26656,7 +26656,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -26685,7 +26685,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -26704,7 +26704,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -26737,7 +26737,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -26756,7 +26756,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -26789,7 +26789,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -26808,7 +26808,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -26844,7 +26844,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -26863,7 +26863,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -26899,7 +26899,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -26918,7 +26918,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -26952,7 +26952,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -26971,7 +26971,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -27006,7 +27006,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27025,7 +27025,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -27044,7 +27044,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27063,7 +27063,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -27084,7 +27084,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27103,7 +27103,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -27136,7 +27136,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27155,7 +27155,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -27194,7 +27194,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -27213,7 +27213,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27232,7 +27232,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -27251,7 +27251,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -27296,7 +27296,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -27335,7 +27335,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -27364,7 +27364,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -27409,7 +27409,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -27454,7 +27454,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -27473,7 +27473,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -27520,7 +27520,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -27565,7 +27565,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -27584,7 +27584,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -27607,7 +27607,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -27630,7 +27630,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -27653,7 +27653,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -27676,7 +27676,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -27699,7 +27699,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -27722,7 +27722,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -27745,7 +27745,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -27768,7 +27768,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -27791,7 +27791,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -27814,7 +27814,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -27837,7 +27837,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -27860,7 +27860,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -27881,7 +27881,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -27902,7 +27902,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -27923,7 +27923,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -27944,7 +27944,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -27965,7 +27965,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -27986,7 +27986,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28007,7 +28007,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -28030,7 +28030,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -28053,7 +28053,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -28076,7 +28076,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -28099,7 +28099,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -28122,7 +28122,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -28145,7 +28145,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -28168,7 +28168,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -28187,7 +28187,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28206,7 +28206,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28225,7 +28225,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -28244,7 +28244,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -28318,10 +28318,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -28353,7 +28354,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -28386,7 +28387,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -28419,7 +28420,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -28452,7 +28453,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -28485,7 +28486,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -28518,7 +28519,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -28551,7 +28552,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -28584,7 +28585,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28615,7 +28616,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -28646,7 +28647,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -28679,7 +28680,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -28712,7 +28713,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -28745,7 +28746,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -28778,7 +28779,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -28811,7 +28812,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -28844,7 +28845,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -28877,7 +28878,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -28910,7 +28911,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -28943,7 +28944,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -28976,7 +28977,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -29009,7 +29010,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -29042,7 +29043,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -29075,7 +29076,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -29108,7 +29109,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -29141,7 +29142,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -29174,7 +29175,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -29206,7 +29207,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -29238,7 +29239,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -29270,7 +29271,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -29302,7 +29303,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -29334,7 +29335,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29364,7 +29365,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29394,7 +29395,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -29426,7 +29427,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -29458,7 +29459,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -29490,7 +29491,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -29522,7 +29523,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -29554,7 +29555,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29584,7 +29585,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -29616,7 +29617,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -29648,7 +29649,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -29680,7 +29681,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -29712,7 +29713,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -29742,7 +29743,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -29772,7 +29773,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -29802,7 +29803,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -29832,7 +29833,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -29864,7 +29865,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -29896,7 +29897,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -29926,7 +29927,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -29956,7 +29957,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -29986,7 +29987,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30016,7 +30017,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30046,7 +30047,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30141,10 +30142,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -30176,7 +30178,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30207,7 +30209,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30238,7 +30240,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30269,7 +30271,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30300,7 +30302,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30331,7 +30333,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30362,7 +30364,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30393,7 +30395,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30424,7 +30426,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30455,7 +30457,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30486,7 +30488,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30517,7 +30519,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30548,7 +30550,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30579,7 +30581,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30610,7 +30612,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -30641,7 +30643,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -30672,7 +30674,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -30703,7 +30705,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -30734,7 +30736,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -30765,7 +30767,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -30795,7 +30797,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -30825,7 +30827,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -30855,7 +30857,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -30885,7 +30887,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -30915,7 +30917,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -30945,7 +30947,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -30975,7 +30977,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31005,7 +31007,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31035,7 +31037,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31065,7 +31067,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31095,7 +31097,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31125,7 +31127,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31155,7 +31157,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31185,7 +31187,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31215,7 +31217,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31245,7 +31247,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -31277,7 +31279,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -31309,7 +31311,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31339,7 +31341,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31369,7 +31371,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31399,7 +31401,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31429,7 +31431,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31459,7 +31461,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53202,19 +53204,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53228,7 +53230,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -53240,7 +53242,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -53251,7 +53253,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -53262,7 +53264,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -53273,13 +53275,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-25T03:53:52Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17252,7 +17252,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -22964,7 +22964,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -22978,7 +22978,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23000,7 +23000,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -23048,7 +23048,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23066,7 +23066,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23092,10 +23092,10 @@
         <v>0.2149</v>
       </c>
       <c r="I4" s="86">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J4" s="87">
-        <v>90</v>
+        <v>5000</v>
       </c>
       <c r="K4" s="52">
         <v>90</v>
@@ -23113,7 +23113,7 @@
         <v>-2588.8525</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23130,7 +23130,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23180,7 +23180,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23197,7 +23197,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23240,7 +23240,7 @@
         <v>34.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23257,7 +23257,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23304,7 +23304,7 @@
         <v>40.40408523144744</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23321,7 +23321,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23369,7 +23369,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23386,7 +23386,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23433,7 +23433,7 @@
         <v>47.29928571428575</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23450,7 +23450,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23495,7 +23495,7 @@
         <v>99.65083573487036</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23512,7 +23512,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23562,7 +23562,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23579,7 +23579,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23618,7 +23618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23635,7 +23635,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23676,7 +23676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23693,7 +23693,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -23730,7 +23730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -23747,7 +23747,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -23792,7 +23792,7 @@
         <v>-1.343804537521815</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -23809,7 +23809,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -23852,7 +23852,7 @@
         <v>31.216902356902377</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -23869,7 +23869,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -23912,7 +23912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -23929,7 +23929,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -23976,7 +23976,7 @@
         <v>5.481184600197436</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -23993,7 +23993,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24038,7 +24038,7 @@
         <v>260.67877899877897</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24055,7 +24055,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24098,7 +24098,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24115,7 +24115,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24156,7 +24156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24173,7 +24173,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24218,7 +24218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24235,7 +24235,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24278,7 +24278,7 @@
         <v>-10.850759137769456</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24295,7 +24295,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24332,7 +24332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24349,7 +24349,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24390,7 +24390,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24407,7 +24407,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24450,7 +24450,7 @@
         <v>-179.4969832402235</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24467,7 +24467,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24509,7 +24509,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24526,7 +24526,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24571,7 +24571,7 @@
         <v>79.30441796516956</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24588,7 +24588,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24633,7 +24633,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24650,7 +24650,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24695,7 +24695,7 @@
         <v>-120.76000000000003</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -24712,7 +24712,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -24749,7 +24749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -24766,7 +24766,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -24783,7 +24783,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -24800,7 +24800,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -24821,7 +24821,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -24838,7 +24838,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -24941,7 +24941,7 @@
         <v>6.191319240032102</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -24958,7 +24958,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -24975,7 +24975,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -25010,7 +25010,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -25393,7 +25393,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25404,7 +25404,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25425,7 +25425,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -25487,7 +25487,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -25545,7 +25545,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25579,7 +25579,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25598,7 +25598,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25632,7 +25632,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25651,7 +25651,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -25685,7 +25685,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -25704,7 +25704,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -25740,7 +25740,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -25759,7 +25759,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -25797,7 +25797,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -25816,7 +25816,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -25854,7 +25854,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -25873,7 +25873,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -25906,7 +25906,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -25925,7 +25925,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -25958,7 +25958,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -25977,7 +25977,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -26008,7 +26008,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26027,7 +26027,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26062,7 +26062,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26081,7 +26081,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26114,7 +26114,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26133,7 +26133,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26164,7 +26164,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26183,7 +26183,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -26215,7 +26215,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26234,7 +26234,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26270,7 +26270,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26289,7 +26289,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26318,7 +26318,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26337,7 +26337,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26368,7 +26368,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26387,7 +26387,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26420,7 +26420,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26439,7 +26439,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26475,7 +26475,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26494,7 +26494,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26529,7 +26529,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26548,7 +26548,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26578,7 +26578,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26597,7 +26597,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26637,7 +26637,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26656,7 +26656,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -26685,7 +26685,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -26704,7 +26704,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -26737,7 +26737,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -26756,7 +26756,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -26789,7 +26789,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -26808,7 +26808,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -26844,7 +26844,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -26863,7 +26863,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -26899,7 +26899,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -26918,7 +26918,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -26952,7 +26952,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -26971,7 +26971,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -27006,7 +27006,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27025,7 +27025,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -27044,7 +27044,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27063,7 +27063,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -27084,7 +27084,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27103,7 +27103,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -27136,7 +27136,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27155,7 +27155,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -27194,7 +27194,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -27213,7 +27213,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27232,7 +27232,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -27251,7 +27251,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -27296,7 +27296,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -27335,7 +27335,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -27364,7 +27364,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -27409,7 +27409,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -27454,7 +27454,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -27473,7 +27473,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -27520,7 +27520,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -27565,7 +27565,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -27584,7 +27584,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -27607,7 +27607,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -27630,7 +27630,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -27653,7 +27653,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -27676,7 +27676,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -27699,7 +27699,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -27722,7 +27722,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -27745,7 +27745,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -27768,7 +27768,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -27791,7 +27791,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -27814,7 +27814,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -27837,7 +27837,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -27860,7 +27860,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -27881,7 +27881,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -27902,7 +27902,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -27923,7 +27923,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -27944,7 +27944,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -27965,7 +27965,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -27986,7 +27986,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28007,7 +28007,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -28030,7 +28030,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -28053,7 +28053,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -28076,7 +28076,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -28099,7 +28099,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -28122,7 +28122,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -28145,7 +28145,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -28168,7 +28168,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -28187,7 +28187,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28206,7 +28206,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28225,7 +28225,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -28244,7 +28244,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -28318,11 +28318,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -28354,7 +28353,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -28387,7 +28386,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -28420,7 +28419,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -28453,7 +28452,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -28486,7 +28485,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -28519,7 +28518,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -28552,7 +28551,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -28585,7 +28584,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28616,7 +28615,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -28647,7 +28646,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -28680,7 +28679,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -28713,7 +28712,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -28746,7 +28745,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -28779,7 +28778,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -28812,7 +28811,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -28845,7 +28844,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -28878,7 +28877,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -28911,7 +28910,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -28944,7 +28943,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -28977,7 +28976,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -29010,7 +29009,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -29043,7 +29042,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -29076,7 +29075,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -29109,7 +29108,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -29142,7 +29141,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -29175,7 +29174,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -29207,7 +29206,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -29239,7 +29238,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -29271,7 +29270,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -29303,7 +29302,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -29335,7 +29334,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29365,7 +29364,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29395,7 +29394,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -29427,7 +29426,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -29459,7 +29458,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -29491,7 +29490,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -29523,7 +29522,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -29555,7 +29554,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29585,7 +29584,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -29617,7 +29616,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -29649,7 +29648,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -29681,7 +29680,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -29713,7 +29712,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -29743,7 +29742,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -29773,7 +29772,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -29803,7 +29802,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -29833,7 +29832,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -29865,7 +29864,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -29897,7 +29896,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -29927,7 +29926,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -29957,7 +29956,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -29987,7 +29986,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30017,7 +30016,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30047,7 +30046,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30142,11 +30141,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -30178,7 +30176,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30209,7 +30207,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30240,7 +30238,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30271,7 +30269,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30302,7 +30300,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30333,7 +30331,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30364,7 +30362,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30395,7 +30393,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30426,7 +30424,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30457,7 +30455,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30488,7 +30486,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30519,7 +30517,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30550,7 +30548,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30581,7 +30579,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30612,7 +30610,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -30643,7 +30641,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -30674,7 +30672,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -30705,7 +30703,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -30736,7 +30734,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -30767,7 +30765,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -30797,7 +30795,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -30827,7 +30825,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -30857,7 +30855,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -30887,7 +30885,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -30917,7 +30915,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -30947,7 +30945,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -30977,7 +30975,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31007,7 +31005,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31037,7 +31035,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31067,7 +31065,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31097,7 +31095,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31127,7 +31125,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31157,7 +31155,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31187,7 +31185,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31217,7 +31215,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31247,7 +31245,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -31279,7 +31277,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -31311,7 +31309,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31341,7 +31339,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31371,7 +31369,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31401,7 +31399,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31431,7 +31429,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31461,7 +31459,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53204,19 +53202,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53230,7 +53228,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -53242,7 +53240,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -53253,7 +53251,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -53264,7 +53262,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -53275,13 +53273,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-25T04:08:30Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6724,8 +6724,8 @@
       <c r="F32" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G32" s="14">
-        <v>45979</v>
+      <c r="G32" s="14" t="s">
+        <v>27</v>
       </c>
       <c r="H32" s="13" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-25T05:07:44Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -6725,7 +6725,7 @@
         <v>27</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H32" s="13" t="s">
         <v>27</v>
@@ -23946,7 +23946,7 @@
         <v>1171.8899999999994</v>
       </c>
       <c r="F32" s="52">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G32" s="53">
         <v>0</v>

</xml_diff>

<commit_message>
Sync data files (2026-08-26T21:04:36Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18043,7 +18043,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -21193,30 +21193,74 @@
       <c r="C183" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D183" s="52"/>
-      <c r="E183" s="52"/>
-      <c r="F183" s="52"/>
-      <c r="G183" s="53"/>
-      <c r="H183" s="52"/>
-      <c r="I183" s="52"/>
-      <c r="J183" s="52"/>
-      <c r="K183" s="52"/>
-      <c r="L183" s="52"/>
-      <c r="M183" s="53"/>
+      <c r="D183" s="52">
+        <v>16897.53</v>
+      </c>
+      <c r="E183" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F183" s="52">
+        <v>11405.829999999998</v>
+      </c>
+      <c r="G183" s="53">
+        <v>0.6749998372543206</v>
+      </c>
+      <c r="H183" s="52">
+        <v>9226.27</v>
+      </c>
+      <c r="I183" s="52">
+        <v>3702.78</v>
+      </c>
+      <c r="J183" s="52">
+        <v>2977.1100000000006</v>
+      </c>
+      <c r="K183" s="52">
+        <v>2335.9700000000003</v>
+      </c>
+      <c r="L183" s="52">
+        <v>641.1400000000003</v>
+      </c>
+      <c r="M183" s="53">
+        <v>0.2153565034546927</v>
+      </c>
       <c r="N183" s="53"/>
-      <c r="O183" s="52"/>
-      <c r="P183" s="52"/>
-      <c r="Q183" s="52"/>
-      <c r="R183" s="53"/>
-      <c r="S183" s="54"/>
-      <c r="T183" s="54"/>
-      <c r="U183" s="54"/>
-      <c r="V183" s="53"/>
+      <c r="O183" s="52">
+        <v>6249.16</v>
+      </c>
+      <c r="P183" s="52">
+        <v>1366.81</v>
+      </c>
+      <c r="Q183" s="52">
+        <v>4882.35</v>
+      </c>
+      <c r="R183" s="53">
+        <v>0.7812810041669601</v>
+      </c>
+      <c r="S183" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T183" s="54">
+        <v>23.75</v>
+      </c>
+      <c r="U183" s="54">
+        <v>101.42</v>
+      </c>
+      <c r="V183" s="53">
+        <v>0.8102580490532876</v>
+      </c>
       <c r="W183" s="53"/>
-      <c r="X183" s="55"/>
-      <c r="Y183" s="55"/>
-      <c r="Z183" s="53"/>
-      <c r="AA183" s="56"/>
+      <c r="X183" s="55">
+        <v>75.32294736842105</v>
+      </c>
+      <c r="Y183" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z183" s="53">
+        <v>0.3257</v>
+      </c>
+      <c r="AA183" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB183" s="57"/>
       <c r="AD183" s="35"/>
       <c r="AE183" s="35"/>
@@ -21596,32 +21640,74 @@
       <c r="C190" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D190" s="52"/>
-      <c r="E190" s="52"/>
-      <c r="F190" s="52"/>
-      <c r="G190" s="53"/>
-      <c r="H190" s="52"/>
-      <c r="I190" s="52"/>
-      <c r="J190" s="52"/>
+      <c r="D190" s="52">
+        <v>20992.12</v>
+      </c>
+      <c r="E190" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F190" s="52">
+        <v>6822.439999999999</v>
+      </c>
+      <c r="G190" s="53">
+        <v>0.32500004763692275</v>
+      </c>
+      <c r="H190" s="52">
+        <v>16299.09</v>
+      </c>
+      <c r="I190" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J190" s="52">
+        <v>9784.33</v>
+      </c>
       <c r="K190" s="52">
-        <v>0</v>
-      </c>
-      <c r="L190" s="52"/>
-      <c r="M190" s="53"/>
+        <v>8137.88</v>
+      </c>
+      <c r="L190" s="52">
+        <v>1646.4499999999998</v>
+      </c>
+      <c r="M190" s="53">
+        <v>0.16827416900288522</v>
+      </c>
       <c r="N190" s="53"/>
-      <c r="O190" s="52"/>
-      <c r="P190" s="52"/>
-      <c r="Q190" s="52"/>
-      <c r="R190" s="53"/>
-      <c r="S190" s="54"/>
-      <c r="T190" s="54"/>
-      <c r="U190" s="54"/>
-      <c r="V190" s="53"/>
+      <c r="O190" s="52">
+        <v>6514.76</v>
+      </c>
+      <c r="P190" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q190" s="52">
+        <v>4953.13</v>
+      </c>
+      <c r="R190" s="53">
+        <v>0.7602935488030257</v>
+      </c>
+      <c r="S190" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T190" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U190" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V190" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W190" s="53"/>
-      <c r="X190" s="55"/>
-      <c r="Y190" s="55"/>
-      <c r="Z190" s="53"/>
-      <c r="AA190" s="56"/>
+      <c r="X190" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y190" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z190" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA190" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB190" s="57"/>
       <c r="AD190" s="35"/>
       <c r="AE190" s="35"/>
@@ -21995,32 +22081,74 @@
       <c r="C197" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D197" s="52"/>
-      <c r="E197" s="52"/>
-      <c r="F197" s="52"/>
-      <c r="G197" s="53"/>
-      <c r="H197" s="52"/>
-      <c r="I197" s="52"/>
-      <c r="J197" s="52"/>
+      <c r="D197" s="52">
+        <v>23770.95</v>
+      </c>
+      <c r="E197" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F197" s="52">
+        <v>13566.41</v>
+      </c>
+      <c r="G197" s="53">
+        <v>0.5707138334816235</v>
+      </c>
+      <c r="H197" s="52">
+        <v>14310.96</v>
+      </c>
+      <c r="I197" s="52">
+        <v>6935.96</v>
+      </c>
+      <c r="J197" s="52">
+        <v>7389.339999999999</v>
+      </c>
       <c r="K197" s="52">
-        <v>0</v>
-      </c>
-      <c r="L197" s="52"/>
-      <c r="M197" s="53"/>
+        <v>6605.05</v>
+      </c>
+      <c r="L197" s="52">
+        <v>784.289999999999</v>
+      </c>
+      <c r="M197" s="53">
+        <v>0.1061380312720756</v>
+      </c>
       <c r="N197" s="53"/>
-      <c r="O197" s="52"/>
-      <c r="P197" s="52"/>
-      <c r="Q197" s="52"/>
-      <c r="R197" s="53"/>
-      <c r="S197" s="54"/>
-      <c r="T197" s="54"/>
-      <c r="U197" s="54"/>
-      <c r="V197" s="53"/>
+      <c r="O197" s="52">
+        <v>6921.62</v>
+      </c>
+      <c r="P197" s="52">
+        <v>330.91</v>
+      </c>
+      <c r="Q197" s="52">
+        <v>6590.71</v>
+      </c>
+      <c r="R197" s="53">
+        <v>0.9521918279246766</v>
+      </c>
+      <c r="S197" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T197" s="54">
+        <v>5.75</v>
+      </c>
+      <c r="U197" s="54">
+        <v>134.4</v>
+      </c>
+      <c r="V197" s="53">
+        <v>0.9589725294327506</v>
+      </c>
       <c r="W197" s="53"/>
-      <c r="X197" s="55"/>
-      <c r="Y197" s="55"/>
-      <c r="Z197" s="53"/>
-      <c r="AA197" s="56"/>
+      <c r="X197" s="55">
+        <v>568.4486956521739</v>
+      </c>
+      <c r="Y197" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z197" s="53">
+        <v>0.32030000000000003</v>
+      </c>
+      <c r="AA197" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB197" s="57"/>
       <c r="AD197" s="35"/>
       <c r="AE197" s="35"/>
@@ -22968,30 +23096,74 @@
       <c r="C218" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D218" s="52"/>
-      <c r="E218" s="52"/>
-      <c r="F218" s="52"/>
-      <c r="G218" s="53"/>
-      <c r="H218" s="52"/>
-      <c r="I218" s="52"/>
-      <c r="J218" s="52"/>
-      <c r="K218" s="52"/>
-      <c r="L218" s="52"/>
-      <c r="M218" s="53"/>
+      <c r="D218" s="52">
+        <v>137109.56</v>
+      </c>
+      <c r="E218" s="52">
+        <v>30174.75</v>
+      </c>
+      <c r="F218" s="52">
+        <v>106934.81</v>
+      </c>
+      <c r="G218" s="53">
+        <v>0.7799223482301307</v>
+      </c>
+      <c r="H218" s="52">
+        <v>117394.57</v>
+      </c>
+      <c r="I218" s="52">
+        <v>26124</v>
+      </c>
+      <c r="J218" s="52">
+        <v>99479.62000000001</v>
+      </c>
+      <c r="K218" s="52">
+        <v>26124</v>
+      </c>
+      <c r="L218" s="52">
+        <v>73355.62000000001</v>
+      </c>
+      <c r="M218" s="53">
+        <v>0.7373934480248316</v>
+      </c>
       <c r="N218" s="53"/>
-      <c r="O218" s="52"/>
-      <c r="P218" s="52"/>
-      <c r="Q218" s="52"/>
-      <c r="R218" s="53"/>
-      <c r="S218" s="54"/>
-      <c r="T218" s="54"/>
-      <c r="U218" s="54"/>
-      <c r="V218" s="53"/>
+      <c r="O218" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="P218" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q218" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="R218" s="53">
+        <v>1</v>
+      </c>
+      <c r="S218" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T218" s="54">
+        <v>0</v>
+      </c>
+      <c r="U218" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V218" s="53">
+        <v>1</v>
+      </c>
       <c r="W218" s="53"/>
-      <c r="X218" s="55"/>
-      <c r="Y218" s="55"/>
-      <c r="Z218" s="53"/>
-      <c r="AA218" s="56"/>
+      <c r="X218" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y218" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z218" s="53">
+        <v>0.13419999999999999</v>
+      </c>
+      <c r="AA218" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB218" s="57"/>
       <c r="AD218" s="35"/>
       <c r="AE218" s="35"/>
@@ -23369,34 +23541,74 @@
       <c r="C225" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D225" s="52"/>
-      <c r="E225" s="52"/>
-      <c r="F225" s="52"/>
-      <c r="G225" s="53"/>
-      <c r="H225" s="52"/>
-      <c r="I225" s="52"/>
+      <c r="D225" s="52">
+        <v>396453.46</v>
+      </c>
+      <c r="E225" s="52">
+        <v>271388.15</v>
+      </c>
+      <c r="F225" s="52">
+        <v>125065.31</v>
+      </c>
+      <c r="G225" s="53">
+        <v>0.3154602560411504</v>
+      </c>
+      <c r="H225" s="52">
+        <v>295569.99</v>
+      </c>
+      <c r="I225" s="52">
+        <v>234322.81</v>
+      </c>
       <c r="J225" s="52">
-        <v>0</v>
+        <v>178700.37</v>
       </c>
       <c r="K225" s="52">
-        <v>0</v>
-      </c>
-      <c r="L225" s="52"/>
-      <c r="M225" s="53"/>
+        <v>177071.47999999998</v>
+      </c>
+      <c r="L225" s="52">
+        <v>1628.890000000014</v>
+      </c>
+      <c r="M225" s="53">
+        <v>0.009115202167740415</v>
+      </c>
       <c r="N225" s="53"/>
-      <c r="O225" s="52"/>
-      <c r="P225" s="52"/>
-      <c r="Q225" s="52"/>
-      <c r="R225" s="53"/>
-      <c r="S225" s="54"/>
-      <c r="T225" s="54"/>
-      <c r="U225" s="54"/>
-      <c r="V225" s="53"/>
+      <c r="O225" s="52">
+        <v>116869.62</v>
+      </c>
+      <c r="P225" s="52">
+        <v>57251.33</v>
+      </c>
+      <c r="Q225" s="52">
+        <v>59618.28999999999</v>
+      </c>
+      <c r="R225" s="53">
+        <v>0.5101264982293944</v>
+      </c>
+      <c r="S225" s="54">
+        <v>2344.68</v>
+      </c>
+      <c r="T225" s="54">
+        <v>1212</v>
+      </c>
+      <c r="U225" s="54">
+        <v>1132.6799999999998</v>
+      </c>
+      <c r="V225" s="53">
+        <v>0.48308511182762676</v>
+      </c>
       <c r="W225" s="53"/>
-      <c r="X225" s="55"/>
-      <c r="Y225" s="55"/>
-      <c r="Z225" s="53"/>
-      <c r="AA225" s="56"/>
+      <c r="X225" s="55">
+        <v>30.581963696369634</v>
+      </c>
+      <c r="Y225" s="55">
+        <v>43.0265399367206</v>
+      </c>
+      <c r="Z225" s="53">
+        <v>0.1366</v>
+      </c>
+      <c r="AA225" s="56">
+        <v>0.2545</v>
+      </c>
       <c r="AB225" s="57"/>
       <c r="AD225" s="35"/>
       <c r="AE225" s="35"/>
@@ -24013,7 +24225,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -24027,7 +24239,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -24049,7 +24261,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -24097,7 +24309,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -24115,7 +24327,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -24162,7 +24374,7 @@
         <v>-726.0072857142857</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -24179,7 +24391,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -24199,7 +24411,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="53">
-        <v>0.2556317756411565</v>
+        <v>0.25548771651006935</v>
       </c>
       <c r="H6" s="53">
         <v>0.239214585617637</v>
@@ -24214,22 +24426,22 @@
         <v>1872.6</v>
       </c>
       <c r="L6" s="53">
-        <v>0.2016787498663849</v>
+        <v>0.20153469073529773</v>
       </c>
       <c r="M6" s="52">
-        <v>6999.8599999999915</v>
+        <v>6994.8599999999915</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>-559.9887999999993</v>
+        <v>-559.5887999999993</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -24246,7 +24458,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -24289,7 +24501,7 @@
         <v>-232.53333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -24306,7 +24518,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -24353,7 +24565,7 @@
         <v>-50.95312270389416</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -24370,7 +24582,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -24418,7 +24630,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -24435,7 +24647,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -24482,7 +24694,7 @@
         <v>-42.80544642857142</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -24499,7 +24711,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -24544,7 +24756,7 @@
         <v>7.380864553314173</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -24561,7 +24773,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -24611,7 +24823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -24628,7 +24840,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -24667,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -24684,7 +24896,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -24725,7 +24937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -24742,7 +24954,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24779,7 +24991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -24796,7 +25008,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24841,7 +25053,7 @@
         <v>0.2554973821989554</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -24858,7 +25070,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24901,7 +25113,7 @@
         <v>7.589966329966334</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -24918,7 +25130,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24961,7 +25173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -24978,7 +25190,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25025,7 +25237,7 @@
         <v>4.666337611056268</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -25042,7 +25254,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25087,7 +25299,7 @@
         <v>285.64884004884004</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -25104,7 +25316,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25147,7 +25359,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -25164,7 +25376,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25205,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -25222,7 +25434,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25267,7 +25479,7 @@
         <v>561.1049999999996</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -25284,7 +25496,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25327,7 +25539,7 @@
         <v>-9.801274601686979</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -25344,7 +25556,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25381,7 +25593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -25398,7 +25610,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25439,7 +25651,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -25456,7 +25668,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -25499,7 +25711,7 @@
         <v>-179.9832402234637</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -25516,7 +25728,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -25558,7 +25770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -25575,7 +25787,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -25620,7 +25832,7 @@
         <v>-9.106177818515201</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -25637,7 +25849,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -25682,7 +25894,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -25699,7 +25911,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -25710,14 +25922,14 @@
         <v>12937.1</v>
       </c>
       <c r="D56" s="99">
-        <v>4850.19</v>
+        <v>4794.2300000000005</v>
       </c>
       <c r="E56" s="99">
-        <v>8086.910000000001</v>
+        <v>8142.87</v>
       </c>
       <c r="F56" s="99"/>
       <c r="G56" s="100">
-        <v>0.6250944956752287</v>
+        <v>0.6294200400398853</v>
       </c>
       <c r="H56" s="100">
         <v>0.22356150784199</v>
@@ -25732,19 +25944,19 @@
         <v>5400</v>
       </c>
       <c r="L56" s="100">
-        <v>0.20769028607647777</v>
+        <v>0.2120158304411344</v>
       </c>
       <c r="M56" s="99">
-        <v>2686.9100000000008</v>
+        <v>2742.87</v>
       </c>
       <c r="N56" s="98">
         <v>-32.25</v>
       </c>
       <c r="O56" s="60">
-        <v>-120.76000000000003</v>
-      </c>
-    </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-123.27505617977528</v>
+      </c>
+    </row>
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25761,7 +25973,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -25769,17 +25981,17 @@
         <v>60</v>
       </c>
       <c r="C58" s="99">
-        <v>0</v>
+        <v>10204.54</v>
       </c>
       <c r="D58" s="99">
-        <v>6849.16</v>
+        <v>6605.05</v>
       </c>
       <c r="E58" s="99">
-        <v>-6849.16</v>
+        <v>3599.4900000000007</v>
       </c>
       <c r="F58" s="99"/>
       <c r="G58" s="100">
-        <v>0</v>
+        <v>0.35273417518085093</v>
       </c>
       <c r="H58" s="100"/>
       <c r="I58" s="98"/>
@@ -25788,17 +26000,17 @@
         <v>0</v>
       </c>
       <c r="L58" s="100">
-        <v>0</v>
+        <v>0.35273417518085093</v>
       </c>
       <c r="M58" s="99">
-        <v>-6849.16</v>
+        <v>3599.4900000000007</v>
       </c>
       <c r="N58" s="98"/>
       <c r="O58" s="60">
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -25815,7 +26027,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -25832,7 +26044,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -25849,7 +26061,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -25870,7 +26082,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -25887,7 +26099,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -25895,17 +26107,17 @@
         <v>62</v>
       </c>
       <c r="C64" s="99">
-        <v>0</v>
+        <v>30174.75</v>
       </c>
       <c r="D64" s="99">
-        <v>1749.8</v>
+        <v>26124</v>
       </c>
       <c r="E64" s="99">
-        <v>-1749.8</v>
+        <v>4050.75</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
-        <v>0</v>
+        <v>0.13424303432505655</v>
       </c>
       <c r="H64" s="100">
         <v>0.143790046441692</v>
@@ -25918,17 +26130,17 @@
         <v>1750</v>
       </c>
       <c r="L64" s="100">
-        <v>0</v>
+        <v>0.07624752483450567</v>
       </c>
       <c r="M64" s="99">
-        <v>-3499.8</v>
+        <v>2300.75</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -25945,7 +26157,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -25956,10 +26168,10 @@
         <v>0</v>
       </c>
       <c r="D66" s="99">
-        <v>2584.2399999999907</v>
+        <v>9863.48999999999</v>
       </c>
       <c r="E66" s="99">
-        <v>-2584.2399999999907</v>
+        <v>-9863.48999999999</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
@@ -25981,16 +26193,16 @@
         <v>0</v>
       </c>
       <c r="M66" s="99">
-        <v>-5784.239999999991</v>
+        <v>-13063.48999999999</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>6.191319240032102</v>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>13.982863259298894</v>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -26007,7 +26219,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -26024,7 +26236,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>121</v>
       </c>
@@ -26032,25 +26244,25 @@
         <v>122</v>
       </c>
       <c r="C69" s="104">
-        <v>308475.47</v>
+        <v>348854.75999999995</v>
       </c>
       <c r="D69" s="104">
-        <v>345627.75999999995</v>
+        <v>376981.13999999996</v>
       </c>
       <c r="E69" s="105">
-        <v>-37152.289999999986</v>
+        <v>-28126.379999999983</v>
       </c>
       <c r="F69" s="106" t="s">
         <v>123</v>
       </c>
       <c r="G69" s="107">
-        <v>-0.12043839336722621</v>
+        <v>-0.08062489960005129</v>
       </c>
       <c r="H69" s="108" t="s">
         <v>124</v>
       </c>
       <c r="I69" s="109">
-        <v>-0.2884666647886135</v>
+        <v>-0.2292042109444056</v>
       </c>
       <c r="J69" s="36"/>
       <c r="K69" s="36"/>
@@ -26059,7 +26271,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>125</v>
@@ -26442,7 +26654,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -26453,7 +26665,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -26474,7 +26686,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -26536,7 +26748,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -26594,7 +26806,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -26628,7 +26840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -26647,7 +26859,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -26681,7 +26893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -26700,7 +26912,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26734,7 +26946,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26753,7 +26965,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26789,7 +27001,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -26808,7 +27020,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -26846,7 +27058,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -26865,7 +27077,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -26903,7 +27115,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -26922,7 +27134,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -26955,7 +27167,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26974,7 +27186,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -27007,7 +27219,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -27026,7 +27238,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -27057,7 +27269,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -27076,7 +27288,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -27111,7 +27323,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -27130,7 +27342,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -27163,7 +27375,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -27182,7 +27394,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -27213,7 +27425,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -27232,7 +27444,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27264,7 +27476,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -27283,7 +27495,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27319,7 +27531,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -27338,7 +27550,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27367,7 +27579,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -27386,7 +27598,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27417,7 +27629,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -27436,7 +27648,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27469,7 +27681,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -27488,7 +27700,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27524,7 +27736,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -27543,7 +27755,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27578,7 +27790,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -27597,7 +27809,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27627,7 +27839,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -27646,7 +27858,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27686,7 +27898,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27705,7 +27917,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27734,7 +27946,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27753,7 +27965,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27786,7 +27998,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -27805,7 +28017,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -27838,7 +28050,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -27857,7 +28069,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -27893,7 +28105,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -27912,7 +28124,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -27948,7 +28160,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -27967,7 +28179,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -28001,7 +28213,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -28020,7 +28232,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -28055,7 +28267,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -28074,7 +28286,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -28093,7 +28305,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -28112,7 +28324,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -28133,7 +28345,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -28152,7 +28364,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -28185,7 +28397,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -28204,7 +28416,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -28212,13 +28424,13 @@
         <v>63</v>
       </c>
       <c r="C66" s="54">
-        <v>2312.68</v>
+        <v>2344.68</v>
       </c>
       <c r="D66" s="54">
-        <v>1120.5</v>
+        <v>1212</v>
       </c>
       <c r="E66" s="54">
-        <v>1192.1799999999998</v>
+        <v>1132.6799999999998</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>
@@ -28243,7 +28455,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -28262,7 +28474,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -28281,7 +28493,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -28300,7 +28512,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>146</v>
@@ -28345,7 +28557,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>147</v>
@@ -28384,7 +28596,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -28413,7 +28625,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>149</v>
@@ -28458,7 +28670,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>150</v>
@@ -28503,7 +28715,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -28522,7 +28734,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>151</v>
@@ -28569,7 +28781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>153</v>
@@ -28614,7 +28826,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -28633,7 +28845,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>154</v>
@@ -28656,7 +28868,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>156</v>
@@ -28679,7 +28891,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>157</v>
@@ -28702,7 +28914,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28725,7 +28937,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28748,7 +28960,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28771,7 +28983,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -28794,7 +29006,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -28817,7 +29029,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -28840,7 +29052,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -28863,7 +29075,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -28886,7 +29098,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -28909,7 +29121,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -28930,7 +29142,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -28951,7 +29163,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -28972,7 +29184,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -28993,7 +29205,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -29014,7 +29226,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -29035,7 +29247,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -29056,7 +29268,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>167</v>
@@ -29079,7 +29291,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -29102,7 +29314,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -29125,7 +29337,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -29148,7 +29360,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -29171,7 +29383,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -29194,7 +29406,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -29217,7 +29429,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -29236,7 +29448,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -29255,7 +29467,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -29274,7 +29486,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -29293,7 +29505,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>174</v>
@@ -29367,10 +29579,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>175</v>
       </c>
@@ -29402,7 +29615,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>176</v>
       </c>
@@ -29435,7 +29648,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>177</v>
       </c>
@@ -29468,7 +29681,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>178</v>
       </c>
@@ -29501,7 +29714,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>179</v>
       </c>
@@ -29534,7 +29747,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>180</v>
       </c>
@@ -29567,7 +29780,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>181</v>
       </c>
@@ -29600,7 +29813,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>182</v>
       </c>
@@ -29633,7 +29846,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -29664,7 +29877,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29695,7 +29908,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>183</v>
       </c>
@@ -29728,7 +29941,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>184</v>
       </c>
@@ -29761,7 +29974,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>185</v>
       </c>
@@ -29794,7 +30007,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>186</v>
       </c>
@@ -29827,7 +30040,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>187</v>
       </c>
@@ -29860,7 +30073,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>188</v>
       </c>
@@ -29893,7 +30106,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>189</v>
       </c>
@@ -29926,7 +30139,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>190</v>
       </c>
@@ -29959,7 +30172,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>191</v>
       </c>
@@ -29992,7 +30205,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>192</v>
       </c>
@@ -30025,7 +30238,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>193</v>
       </c>
@@ -30058,7 +30271,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>194</v>
       </c>
@@ -30091,7 +30304,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>195</v>
       </c>
@@ -30124,7 +30337,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>196</v>
       </c>
@@ -30157,7 +30370,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>197</v>
       </c>
@@ -30190,7 +30403,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>198</v>
       </c>
@@ -30223,7 +30436,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>199</v>
       </c>
@@ -30255,7 +30468,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>200</v>
       </c>
@@ -30287,7 +30500,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>201</v>
       </c>
@@ -30319,7 +30532,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>202</v>
       </c>
@@ -30351,7 +30564,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>203</v>
       </c>
@@ -30383,7 +30596,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -30413,7 +30626,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -30443,7 +30656,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>204</v>
       </c>
@@ -30475,7 +30688,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>205</v>
       </c>
@@ -30507,7 +30720,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>206</v>
       </c>
@@ -30539,7 +30752,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>207</v>
       </c>
@@ -30571,7 +30784,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>208</v>
       </c>
@@ -30603,7 +30816,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -30633,7 +30846,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>209</v>
       </c>
@@ -30665,7 +30878,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>210</v>
       </c>
@@ -30697,7 +30910,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>211</v>
       </c>
@@ -30729,7 +30942,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>212</v>
       </c>
@@ -30761,7 +30974,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -30791,7 +31004,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -30821,7 +31034,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -30851,7 +31064,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -30881,7 +31094,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>213</v>
       </c>
@@ -30913,7 +31126,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>214</v>
       </c>
@@ -30945,7 +31158,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -30975,7 +31188,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -31005,7 +31218,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -31035,7 +31248,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -31065,7 +31278,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -31095,7 +31308,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -31190,10 +31403,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>215</v>
       </c>
@@ -31225,7 +31439,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -31256,7 +31470,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -31287,7 +31501,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -31318,7 +31532,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -31349,7 +31563,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -31380,7 +31594,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -31411,7 +31625,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -31442,7 +31656,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -31473,7 +31687,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -31504,7 +31718,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -31535,7 +31749,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -31566,7 +31780,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -31597,7 +31811,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -31628,7 +31842,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -31659,7 +31873,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31690,7 +31904,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31721,7 +31935,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31752,7 +31966,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31783,7 +31997,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -31814,7 +32028,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -31844,7 +32058,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -31874,7 +32088,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -31904,7 +32118,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -31934,7 +32148,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -31964,7 +32178,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -31994,7 +32208,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -32024,7 +32238,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -32054,7 +32268,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -32084,7 +32298,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -32114,7 +32328,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -32144,7 +32358,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -32174,7 +32388,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -32204,7 +32418,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -32234,7 +32448,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -32264,7 +32478,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -32294,7 +32508,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>213</v>
       </c>
@@ -32326,7 +32540,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>214</v>
       </c>
@@ -32358,7 +32572,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -32388,7 +32602,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -32418,7 +32632,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -32448,7 +32662,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -32478,7 +32692,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -32508,7 +32722,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -54251,19 +54465,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -54277,7 +54491,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>222</v>
       </c>
@@ -54289,7 +54503,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>223</v>
       </c>
@@ -54300,7 +54514,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>224</v>
       </c>
@@ -54311,7 +54525,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>225</v>
       </c>
@@ -54322,13 +54536,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-08-26T21:15:55Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18043,7 +18043,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -24225,7 +24225,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -24239,7 +24239,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -24261,7 +24261,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -24309,7 +24309,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -24327,7 +24327,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -24374,7 +24374,7 @@
         <v>-726.0072857142857</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -24391,7 +24391,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -24441,7 +24441,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -24458,7 +24458,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -24501,7 +24501,7 @@
         <v>-232.53333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -24518,7 +24518,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -24565,7 +24565,7 @@
         <v>-50.95312270389416</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -24582,7 +24582,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -24630,7 +24630,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -24647,7 +24647,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -24694,7 +24694,7 @@
         <v>-42.80544642857142</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -24711,7 +24711,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -24756,7 +24756,7 @@
         <v>7.380864553314173</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -24773,7 +24773,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -24823,7 +24823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -24840,7 +24840,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -24937,7 +24937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -24954,7 +24954,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24991,7 +24991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -25008,7 +25008,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25053,7 +25053,7 @@
         <v>0.2554973821989554</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -25070,7 +25070,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25113,7 +25113,7 @@
         <v>7.589966329966334</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -25130,7 +25130,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25173,7 +25173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -25190,7 +25190,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25237,7 +25237,7 @@
         <v>4.666337611056268</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -25254,7 +25254,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25299,7 +25299,7 @@
         <v>285.64884004884004</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -25316,7 +25316,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25359,7 +25359,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -25376,7 +25376,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25417,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -25434,7 +25434,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25479,7 +25479,7 @@
         <v>561.1049999999996</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -25496,7 +25496,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25539,7 +25539,7 @@
         <v>-9.801274601686979</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -25556,7 +25556,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25593,7 +25593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -25610,7 +25610,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25651,7 +25651,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -25668,7 +25668,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -25711,7 +25711,7 @@
         <v>-179.9832402234637</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -25728,7 +25728,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -25770,7 +25770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -25787,7 +25787,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -25832,7 +25832,7 @@
         <v>-9.106177818515201</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -25849,7 +25849,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -25894,7 +25894,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -25911,7 +25911,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -25956,7 +25956,7 @@
         <v>-123.27505617977528</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25973,7 +25973,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -26010,7 +26010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -26027,7 +26027,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -26044,7 +26044,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -26061,7 +26061,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -26082,7 +26082,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -26099,7 +26099,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -26140,7 +26140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -26157,7 +26157,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -26202,7 +26202,7 @@
         <v>13.982863259298894</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -26219,7 +26219,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -26236,7 +26236,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>121</v>
       </c>
@@ -26271,7 +26271,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>125</v>
@@ -26654,7 +26654,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -26665,7 +26665,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -26686,7 +26686,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -26748,7 +26748,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -26806,7 +26806,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -26840,7 +26840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -26859,7 +26859,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -26893,7 +26893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -26912,7 +26912,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26946,7 +26946,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26965,7 +26965,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -27001,7 +27001,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -27020,7 +27020,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -27058,7 +27058,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -27077,7 +27077,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -27115,7 +27115,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -27134,7 +27134,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -27167,7 +27167,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -27186,7 +27186,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -27219,7 +27219,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -27238,7 +27238,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -27269,7 +27269,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -27288,7 +27288,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -27323,7 +27323,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -27342,7 +27342,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -27375,7 +27375,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -27394,7 +27394,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -27425,7 +27425,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -27444,7 +27444,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27476,7 +27476,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -27495,7 +27495,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27531,7 +27531,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -27550,7 +27550,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27579,7 +27579,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -27598,7 +27598,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27629,7 +27629,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -27648,7 +27648,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27681,7 +27681,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -27700,7 +27700,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27736,7 +27736,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -27755,7 +27755,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27790,7 +27790,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -27809,7 +27809,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27839,7 +27839,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -27858,7 +27858,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27898,7 +27898,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27917,7 +27917,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27946,7 +27946,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27965,7 +27965,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27998,7 +27998,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -28017,7 +28017,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -28050,7 +28050,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -28069,7 +28069,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -28105,7 +28105,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -28124,7 +28124,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -28160,7 +28160,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -28179,7 +28179,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -28213,7 +28213,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -28232,7 +28232,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -28267,7 +28267,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -28286,7 +28286,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -28305,7 +28305,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -28324,7 +28324,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -28345,7 +28345,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -28364,7 +28364,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -28397,7 +28397,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -28416,7 +28416,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -28455,7 +28455,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -28474,7 +28474,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -28493,7 +28493,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -28512,7 +28512,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>146</v>
@@ -28557,7 +28557,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>147</v>
@@ -28596,7 +28596,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -28625,7 +28625,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>149</v>
@@ -28670,7 +28670,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>150</v>
@@ -28715,7 +28715,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -28734,7 +28734,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>151</v>
@@ -28781,7 +28781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>153</v>
@@ -28826,7 +28826,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -28845,7 +28845,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>154</v>
@@ -28868,7 +28868,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>156</v>
@@ -28891,7 +28891,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>157</v>
@@ -28914,7 +28914,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28937,7 +28937,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28960,7 +28960,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28983,7 +28983,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -29006,7 +29006,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -29029,7 +29029,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -29052,7 +29052,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -29075,7 +29075,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -29098,7 +29098,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -29121,7 +29121,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -29142,7 +29142,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -29163,7 +29163,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -29184,7 +29184,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -29205,7 +29205,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -29226,7 +29226,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -29247,7 +29247,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -29268,7 +29268,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>167</v>
@@ -29291,7 +29291,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -29314,7 +29314,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -29337,7 +29337,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -29360,7 +29360,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -29383,7 +29383,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -29406,7 +29406,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -29429,7 +29429,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -29448,7 +29448,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -29467,7 +29467,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -29486,7 +29486,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -29505,7 +29505,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>174</v>
@@ -29579,11 +29579,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>175</v>
       </c>
@@ -29615,7 +29614,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>176</v>
       </c>
@@ -29648,7 +29647,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>177</v>
       </c>
@@ -29681,7 +29680,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>178</v>
       </c>
@@ -29714,7 +29713,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>179</v>
       </c>
@@ -29747,7 +29746,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>180</v>
       </c>
@@ -29780,7 +29779,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>181</v>
       </c>
@@ -29813,7 +29812,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>182</v>
       </c>
@@ -29846,7 +29845,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -29877,7 +29876,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29908,7 +29907,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>183</v>
       </c>
@@ -29941,7 +29940,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>184</v>
       </c>
@@ -29974,7 +29973,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>185</v>
       </c>
@@ -30007,7 +30006,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>186</v>
       </c>
@@ -30040,7 +30039,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>187</v>
       </c>
@@ -30073,7 +30072,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>188</v>
       </c>
@@ -30106,7 +30105,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>189</v>
       </c>
@@ -30139,7 +30138,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>190</v>
       </c>
@@ -30172,7 +30171,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>191</v>
       </c>
@@ -30205,7 +30204,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>192</v>
       </c>
@@ -30238,7 +30237,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>193</v>
       </c>
@@ -30271,7 +30270,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>194</v>
       </c>
@@ -30304,7 +30303,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>195</v>
       </c>
@@ -30337,7 +30336,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>196</v>
       </c>
@@ -30370,7 +30369,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>197</v>
       </c>
@@ -30403,7 +30402,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>198</v>
       </c>
@@ -30436,7 +30435,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>199</v>
       </c>
@@ -30468,7 +30467,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>200</v>
       </c>
@@ -30500,7 +30499,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>201</v>
       </c>
@@ -30532,7 +30531,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>202</v>
       </c>
@@ -30564,7 +30563,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>203</v>
       </c>
@@ -30596,7 +30595,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -30626,7 +30625,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -30656,7 +30655,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>204</v>
       </c>
@@ -30688,7 +30687,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>205</v>
       </c>
@@ -30720,7 +30719,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>206</v>
       </c>
@@ -30752,7 +30751,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>207</v>
       </c>
@@ -30784,7 +30783,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>208</v>
       </c>
@@ -30816,7 +30815,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -30846,7 +30845,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>209</v>
       </c>
@@ -30878,7 +30877,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>210</v>
       </c>
@@ -30910,7 +30909,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>211</v>
       </c>
@@ -30942,7 +30941,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>212</v>
       </c>
@@ -30974,7 +30973,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -31004,7 +31003,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -31034,7 +31033,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -31064,7 +31063,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -31094,7 +31093,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>213</v>
       </c>
@@ -31126,7 +31125,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>214</v>
       </c>
@@ -31158,7 +31157,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -31188,7 +31187,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -31218,7 +31217,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -31248,7 +31247,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -31278,7 +31277,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -31308,7 +31307,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -31403,11 +31402,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>215</v>
       </c>
@@ -31439,7 +31437,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -31470,7 +31468,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -31501,7 +31499,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -31532,7 +31530,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -31563,7 +31561,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -31594,7 +31592,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -31625,7 +31623,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -31656,7 +31654,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -31687,7 +31685,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -31718,7 +31716,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -31749,7 +31747,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -31780,7 +31778,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -31811,7 +31809,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -31842,7 +31840,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -31873,7 +31871,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31904,7 +31902,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31935,7 +31933,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31966,7 +31964,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31997,7 +31995,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -32028,7 +32026,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -32058,7 +32056,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -32088,7 +32086,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -32118,7 +32116,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -32148,7 +32146,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -32178,7 +32176,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -32208,7 +32206,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -32238,7 +32236,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -32268,7 +32266,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -32298,7 +32296,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -32328,7 +32326,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -32358,7 +32356,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -32388,7 +32386,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -32418,7 +32416,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -32448,7 +32446,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -32478,7 +32476,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -32508,7 +32506,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>213</v>
       </c>
@@ -32540,7 +32538,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>214</v>
       </c>
@@ -32572,7 +32570,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -32602,7 +32600,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -32632,7 +32630,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -32662,7 +32660,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -32692,7 +32690,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -32722,7 +32720,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -54465,19 +54463,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -54491,7 +54489,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>222</v>
       </c>
@@ -54503,7 +54501,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>223</v>
       </c>
@@ -54514,7 +54512,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>224</v>
       </c>
@@ -54525,7 +54523,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>225</v>
       </c>
@@ -54536,13 +54534,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-08-26T23:20:17Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18043,7 +18043,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -24225,7 +24225,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -24239,7 +24239,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -24261,7 +24261,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -24309,7 +24309,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -24327,7 +24327,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -24374,7 +24374,7 @@
         <v>-726.0072857142857</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -24391,7 +24391,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -24441,7 +24441,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -24458,7 +24458,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -24501,7 +24501,7 @@
         <v>-232.53333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -24518,7 +24518,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -24565,7 +24565,7 @@
         <v>-50.95312270389416</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -24582,7 +24582,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -24630,7 +24630,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -24647,7 +24647,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -24694,7 +24694,7 @@
         <v>-42.80544642857142</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -24711,7 +24711,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -24756,7 +24756,7 @@
         <v>7.380864553314173</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -24773,7 +24773,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -24823,7 +24823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -24840,7 +24840,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -24937,7 +24937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -24954,7 +24954,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24991,7 +24991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -25008,7 +25008,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25053,7 +25053,7 @@
         <v>0.2554973821989554</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -25070,7 +25070,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25113,7 +25113,7 @@
         <v>7.589966329966334</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -25130,7 +25130,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25173,7 +25173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -25190,7 +25190,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25237,7 +25237,7 @@
         <v>4.666337611056268</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -25254,7 +25254,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25299,7 +25299,7 @@
         <v>285.64884004884004</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -25316,7 +25316,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25359,7 +25359,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -25376,7 +25376,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25417,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -25434,7 +25434,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25479,7 +25479,7 @@
         <v>561.1049999999996</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -25496,7 +25496,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25539,7 +25539,7 @@
         <v>-9.801274601686979</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -25556,7 +25556,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25593,7 +25593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -25610,7 +25610,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25651,7 +25651,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -25668,7 +25668,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -25711,7 +25711,7 @@
         <v>-179.9832402234637</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -25728,7 +25728,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -25770,7 +25770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -25787,7 +25787,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -25832,7 +25832,7 @@
         <v>-9.106177818515201</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -25849,7 +25849,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -25894,7 +25894,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -25911,7 +25911,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -25956,7 +25956,7 @@
         <v>-123.27505617977528</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25973,7 +25973,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -26010,7 +26010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -26027,7 +26027,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -26044,7 +26044,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -26061,7 +26061,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -26082,7 +26082,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -26099,7 +26099,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -26140,7 +26140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -26157,7 +26157,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -26202,7 +26202,7 @@
         <v>13.982863259298894</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -26219,7 +26219,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -26236,7 +26236,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>121</v>
       </c>
@@ -26271,7 +26271,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>125</v>
@@ -26654,7 +26654,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -26665,7 +26665,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -26686,7 +26686,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -26748,7 +26748,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -26806,7 +26806,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -26840,7 +26840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -26859,7 +26859,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -26893,7 +26893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -26912,7 +26912,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26946,7 +26946,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26965,7 +26965,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -27001,7 +27001,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -27020,7 +27020,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -27058,7 +27058,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -27077,7 +27077,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -27115,7 +27115,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -27134,7 +27134,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -27167,7 +27167,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -27186,7 +27186,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -27219,7 +27219,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -27238,7 +27238,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -27269,7 +27269,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -27288,7 +27288,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -27323,7 +27323,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -27342,7 +27342,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -27375,7 +27375,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -27394,7 +27394,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -27425,7 +27425,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -27444,7 +27444,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27476,7 +27476,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -27495,7 +27495,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27531,7 +27531,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -27550,7 +27550,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27579,7 +27579,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -27598,7 +27598,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27629,7 +27629,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -27648,7 +27648,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27681,7 +27681,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -27700,7 +27700,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27736,7 +27736,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -27755,7 +27755,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27790,7 +27790,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -27809,7 +27809,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27839,7 +27839,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -27858,7 +27858,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27898,7 +27898,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27917,7 +27917,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27946,7 +27946,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27965,7 +27965,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27998,7 +27998,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -28017,7 +28017,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -28050,7 +28050,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -28069,7 +28069,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -28105,7 +28105,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -28124,7 +28124,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -28160,7 +28160,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -28179,7 +28179,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -28213,7 +28213,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -28232,7 +28232,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -28267,7 +28267,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -28286,7 +28286,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -28305,7 +28305,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -28324,7 +28324,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -28345,7 +28345,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -28364,7 +28364,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -28397,7 +28397,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -28416,7 +28416,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -28455,7 +28455,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -28474,7 +28474,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -28493,7 +28493,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -28512,7 +28512,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>146</v>
@@ -28557,7 +28557,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>147</v>
@@ -28596,7 +28596,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -28625,7 +28625,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>149</v>
@@ -28670,7 +28670,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>150</v>
@@ -28715,7 +28715,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -28734,7 +28734,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>151</v>
@@ -28781,7 +28781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>153</v>
@@ -28826,7 +28826,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -28845,7 +28845,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>154</v>
@@ -28868,7 +28868,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>156</v>
@@ -28891,7 +28891,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>157</v>
@@ -28914,7 +28914,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28937,7 +28937,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28960,7 +28960,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28983,7 +28983,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -29006,7 +29006,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -29029,7 +29029,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -29052,7 +29052,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -29075,7 +29075,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -29098,7 +29098,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -29121,7 +29121,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -29142,7 +29142,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -29163,7 +29163,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -29184,7 +29184,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -29205,7 +29205,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -29226,7 +29226,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -29247,7 +29247,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -29268,7 +29268,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>167</v>
@@ -29291,7 +29291,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -29314,7 +29314,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -29337,7 +29337,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -29360,7 +29360,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -29383,7 +29383,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -29406,7 +29406,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -29429,7 +29429,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -29448,7 +29448,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -29467,7 +29467,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -29486,7 +29486,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -29505,7 +29505,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>174</v>
@@ -29579,10 +29579,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>175</v>
       </c>
@@ -29614,7 +29615,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>176</v>
       </c>
@@ -29647,7 +29648,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>177</v>
       </c>
@@ -29680,7 +29681,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>178</v>
       </c>
@@ -29713,7 +29714,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>179</v>
       </c>
@@ -29746,7 +29747,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>180</v>
       </c>
@@ -29779,7 +29780,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>181</v>
       </c>
@@ -29812,7 +29813,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>182</v>
       </c>
@@ -29845,7 +29846,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -29876,7 +29877,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29907,7 +29908,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>183</v>
       </c>
@@ -29940,7 +29941,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>184</v>
       </c>
@@ -29973,7 +29974,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>185</v>
       </c>
@@ -30006,7 +30007,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>186</v>
       </c>
@@ -30039,7 +30040,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>187</v>
       </c>
@@ -30072,7 +30073,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>188</v>
       </c>
@@ -30105,7 +30106,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>189</v>
       </c>
@@ -30138,7 +30139,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>190</v>
       </c>
@@ -30171,7 +30172,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>191</v>
       </c>
@@ -30204,7 +30205,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>192</v>
       </c>
@@ -30237,7 +30238,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>193</v>
       </c>
@@ -30270,7 +30271,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>194</v>
       </c>
@@ -30303,7 +30304,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>195</v>
       </c>
@@ -30336,7 +30337,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>196</v>
       </c>
@@ -30369,7 +30370,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>197</v>
       </c>
@@ -30402,7 +30403,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>198</v>
       </c>
@@ -30435,7 +30436,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>199</v>
       </c>
@@ -30467,7 +30468,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>200</v>
       </c>
@@ -30499,7 +30500,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>201</v>
       </c>
@@ -30531,7 +30532,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>202</v>
       </c>
@@ -30563,7 +30564,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>203</v>
       </c>
@@ -30595,7 +30596,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -30625,7 +30626,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -30655,7 +30656,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>204</v>
       </c>
@@ -30687,7 +30688,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>205</v>
       </c>
@@ -30719,7 +30720,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>206</v>
       </c>
@@ -30751,7 +30752,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>207</v>
       </c>
@@ -30783,7 +30784,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>208</v>
       </c>
@@ -30815,7 +30816,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -30845,7 +30846,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>209</v>
       </c>
@@ -30877,7 +30878,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>210</v>
       </c>
@@ -30909,7 +30910,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>211</v>
       </c>
@@ -30941,7 +30942,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>212</v>
       </c>
@@ -30973,7 +30974,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -31003,7 +31004,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -31033,7 +31034,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -31063,7 +31064,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -31093,7 +31094,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>213</v>
       </c>
@@ -31125,7 +31126,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>214</v>
       </c>
@@ -31157,7 +31158,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -31187,7 +31188,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -31217,7 +31218,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -31247,7 +31248,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -31277,7 +31278,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -31307,7 +31308,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -31402,10 +31403,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>215</v>
       </c>
@@ -31437,7 +31439,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -31468,7 +31470,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -31499,7 +31501,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -31530,7 +31532,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -31561,7 +31563,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -31592,7 +31594,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -31623,7 +31625,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -31654,7 +31656,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -31685,7 +31687,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -31716,7 +31718,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -31747,7 +31749,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -31778,7 +31780,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -31809,7 +31811,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -31840,7 +31842,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -31871,7 +31873,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31902,7 +31904,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31933,7 +31935,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31964,7 +31966,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31995,7 +31997,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -32026,7 +32028,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -32056,7 +32058,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -32086,7 +32088,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -32116,7 +32118,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -32146,7 +32148,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -32176,7 +32178,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -32206,7 +32208,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -32236,7 +32238,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -32266,7 +32268,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -32296,7 +32298,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -32326,7 +32328,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -32356,7 +32358,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -32386,7 +32388,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -32416,7 +32418,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -32446,7 +32448,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -32476,7 +32478,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -32506,7 +32508,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>213</v>
       </c>
@@ -32538,7 +32540,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>214</v>
       </c>
@@ -32570,7 +32572,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -32600,7 +32602,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -32630,7 +32632,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -32660,7 +32662,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -32690,7 +32692,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -32720,7 +32722,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -54463,19 +54465,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -54489,7 +54491,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>222</v>
       </c>
@@ -54501,7 +54503,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>223</v>
       </c>
@@ -54512,7 +54514,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>224</v>
       </c>
@@ -54523,7 +54525,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>225</v>
       </c>
@@ -54534,13 +54536,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-08-26T23:24:20Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18043,7 +18043,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -24225,7 +24225,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -24239,7 +24239,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -24261,7 +24261,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -24309,7 +24309,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -24327,7 +24327,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -24374,7 +24374,7 @@
         <v>-726.0072857142857</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -24391,7 +24391,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -24441,7 +24441,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -24458,7 +24458,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -24501,7 +24501,7 @@
         <v>-232.53333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -24518,7 +24518,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -24565,7 +24565,7 @@
         <v>-50.95312270389416</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -24582,7 +24582,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -24630,7 +24630,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -24647,7 +24647,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -24694,7 +24694,7 @@
         <v>-42.80544642857142</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -24711,7 +24711,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -24756,7 +24756,7 @@
         <v>7.380864553314173</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -24773,7 +24773,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -24823,7 +24823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -24840,7 +24840,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -24937,7 +24937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -24954,7 +24954,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24991,7 +24991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -25008,7 +25008,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25053,7 +25053,7 @@
         <v>0.2554973821989554</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -25070,7 +25070,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25113,7 +25113,7 @@
         <v>7.589966329966334</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -25130,7 +25130,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25173,7 +25173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -25190,7 +25190,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25237,7 +25237,7 @@
         <v>4.666337611056268</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -25254,7 +25254,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25299,7 +25299,7 @@
         <v>285.64884004884004</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -25316,7 +25316,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25359,7 +25359,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -25376,7 +25376,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25417,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -25434,7 +25434,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25479,7 +25479,7 @@
         <v>561.1049999999996</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -25496,7 +25496,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25539,7 +25539,7 @@
         <v>-9.801274601686979</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -25556,7 +25556,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25593,7 +25593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -25610,7 +25610,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25651,7 +25651,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -25668,7 +25668,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -25711,7 +25711,7 @@
         <v>-179.9832402234637</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -25728,7 +25728,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -25770,7 +25770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -25787,7 +25787,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -25832,7 +25832,7 @@
         <v>-9.106177818515201</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -25849,7 +25849,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -25894,7 +25894,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -25911,7 +25911,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -25956,7 +25956,7 @@
         <v>-123.27505617977528</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25973,7 +25973,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -26010,7 +26010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -26027,7 +26027,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -26044,7 +26044,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -26061,7 +26061,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -26082,7 +26082,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -26099,7 +26099,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -26140,7 +26140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -26157,7 +26157,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -26202,7 +26202,7 @@
         <v>13.982863259298894</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -26219,7 +26219,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -26236,7 +26236,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>121</v>
       </c>
@@ -26271,7 +26271,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>125</v>
@@ -26654,7 +26654,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -26665,7 +26665,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -26686,7 +26686,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -26748,7 +26748,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -26806,7 +26806,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -26840,7 +26840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -26859,7 +26859,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -26893,7 +26893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -26912,7 +26912,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26946,7 +26946,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26965,7 +26965,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26994,14 +26994,16 @@
       <c r="N10" s="54">
         <v>80</v>
       </c>
-      <c r="O10" s="54"/>
+      <c r="O10" s="54">
+        <v>0</v>
+      </c>
       <c r="P10" s="54"/>
       <c r="Q10" s="131"/>
       <c r="S10" s="35" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -27020,7 +27022,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -27058,7 +27060,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -27077,7 +27079,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -27115,7 +27117,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -27134,7 +27136,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -27167,7 +27169,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -27186,7 +27188,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -27219,7 +27221,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -27238,7 +27240,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -27269,7 +27271,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -27288,7 +27290,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -27323,7 +27325,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -27342,7 +27344,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -27375,7 +27377,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -27394,7 +27396,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -27425,7 +27427,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -27444,7 +27446,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27476,7 +27478,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -27495,7 +27497,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27531,7 +27533,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -27550,7 +27552,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27579,7 +27581,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -27598,7 +27600,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27629,7 +27631,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -27648,7 +27650,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27681,7 +27683,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -27700,7 +27702,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27736,7 +27738,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -27755,7 +27757,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27790,7 +27792,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -27809,7 +27811,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27839,7 +27841,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -27858,7 +27860,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27898,7 +27900,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27917,7 +27919,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27946,7 +27948,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27965,7 +27967,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27998,7 +28000,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -28017,7 +28019,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -28050,7 +28052,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -28069,7 +28071,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -28105,7 +28107,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -28124,7 +28126,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -28160,7 +28162,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -28179,7 +28181,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -28213,7 +28215,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -28232,7 +28234,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -28267,7 +28269,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -28286,7 +28288,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -28305,7 +28307,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -28324,7 +28326,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -28345,7 +28347,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -28364,7 +28366,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -28397,7 +28399,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -28416,7 +28418,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -28455,7 +28457,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -28474,7 +28476,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -28493,7 +28495,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -28512,7 +28514,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>146</v>
@@ -28557,7 +28559,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>147</v>
@@ -28596,7 +28598,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -28625,7 +28627,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>149</v>
@@ -28670,7 +28672,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>150</v>
@@ -28715,7 +28717,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -28734,7 +28736,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>151</v>
@@ -28781,7 +28783,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>153</v>
@@ -28826,7 +28828,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -28845,7 +28847,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>154</v>
@@ -28868,7 +28870,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>156</v>
@@ -28891,7 +28893,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>157</v>
@@ -28914,7 +28916,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28937,7 +28939,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28960,7 +28962,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28983,7 +28985,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -29006,7 +29008,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -29029,7 +29031,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -29052,7 +29054,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -29075,7 +29077,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -29098,7 +29100,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -29121,7 +29123,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -29142,7 +29144,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -29163,7 +29165,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -29184,7 +29186,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -29205,7 +29207,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -29226,7 +29228,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -29247,7 +29249,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -29268,7 +29270,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>167</v>
@@ -29291,7 +29293,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -29314,7 +29316,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -29337,7 +29339,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -29360,7 +29362,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -29383,7 +29385,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -29406,7 +29408,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -29429,7 +29431,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -29448,7 +29450,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -29467,7 +29469,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -29486,7 +29488,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -29505,7 +29507,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>174</v>
@@ -29579,11 +29581,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>175</v>
       </c>
@@ -29615,7 +29616,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>176</v>
       </c>
@@ -29648,7 +29649,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>177</v>
       </c>
@@ -29681,7 +29682,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>178</v>
       </c>
@@ -29714,7 +29715,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>179</v>
       </c>
@@ -29747,7 +29748,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>180</v>
       </c>
@@ -29780,7 +29781,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>181</v>
       </c>
@@ -29813,7 +29814,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>182</v>
       </c>
@@ -29846,7 +29847,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -29877,7 +29878,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29908,7 +29909,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>183</v>
       </c>
@@ -29941,7 +29942,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>184</v>
       </c>
@@ -29974,7 +29975,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>185</v>
       </c>
@@ -30007,7 +30008,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>186</v>
       </c>
@@ -30040,7 +30041,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>187</v>
       </c>
@@ -30073,7 +30074,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>188</v>
       </c>
@@ -30106,7 +30107,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>189</v>
       </c>
@@ -30139,7 +30140,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>190</v>
       </c>
@@ -30172,7 +30173,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>191</v>
       </c>
@@ -30205,7 +30206,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>192</v>
       </c>
@@ -30238,7 +30239,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>193</v>
       </c>
@@ -30271,7 +30272,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>194</v>
       </c>
@@ -30304,7 +30305,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>195</v>
       </c>
@@ -30337,7 +30338,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>196</v>
       </c>
@@ -30370,7 +30371,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>197</v>
       </c>
@@ -30403,7 +30404,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>198</v>
       </c>
@@ -30436,7 +30437,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>199</v>
       </c>
@@ -30468,7 +30469,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>200</v>
       </c>
@@ -30500,7 +30501,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>201</v>
       </c>
@@ -30532,7 +30533,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>202</v>
       </c>
@@ -30564,7 +30565,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>203</v>
       </c>
@@ -30596,7 +30597,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -30626,7 +30627,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -30656,7 +30657,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>204</v>
       </c>
@@ -30688,7 +30689,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>205</v>
       </c>
@@ -30720,7 +30721,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>206</v>
       </c>
@@ -30752,7 +30753,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>207</v>
       </c>
@@ -30784,7 +30785,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>208</v>
       </c>
@@ -30816,7 +30817,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -30846,7 +30847,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>209</v>
       </c>
@@ -30878,7 +30879,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>210</v>
       </c>
@@ -30910,7 +30911,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>211</v>
       </c>
@@ -30942,7 +30943,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>212</v>
       </c>
@@ -30974,7 +30975,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -31004,7 +31005,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -31034,7 +31035,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -31064,7 +31065,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -31094,7 +31095,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>213</v>
       </c>
@@ -31126,7 +31127,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>214</v>
       </c>
@@ -31158,7 +31159,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -31188,7 +31189,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -31218,7 +31219,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -31248,7 +31249,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -31278,7 +31279,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -31308,7 +31309,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -31403,11 +31404,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>215</v>
       </c>
@@ -31439,7 +31439,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -31470,7 +31470,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -31501,7 +31501,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -31532,7 +31532,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -31563,7 +31563,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -31594,7 +31594,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -31625,7 +31625,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -31656,7 +31656,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -31687,7 +31687,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -31718,7 +31718,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -31749,7 +31749,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -31780,7 +31780,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -31811,7 +31811,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -31842,7 +31842,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -31873,7 +31873,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31904,7 +31904,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31935,7 +31935,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31966,7 +31966,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31997,7 +31997,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -32028,7 +32028,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -32058,7 +32058,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -32088,7 +32088,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -32118,7 +32118,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -32148,7 +32148,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -32178,7 +32178,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -32208,7 +32208,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -32238,7 +32238,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -32268,7 +32268,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -32298,7 +32298,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -32328,7 +32328,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -32358,7 +32358,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -32388,7 +32388,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -32418,7 +32418,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -32448,7 +32448,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -32478,7 +32478,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -32508,7 +32508,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>213</v>
       </c>
@@ -32540,7 +32540,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>214</v>
       </c>
@@ -32572,7 +32572,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -32602,7 +32602,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -32632,7 +32632,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -32662,7 +32662,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -32692,7 +32692,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -32722,7 +32722,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -54465,19 +54465,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -54491,7 +54491,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>222</v>
       </c>
@@ -54503,7 +54503,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>223</v>
       </c>
@@ -54514,7 +54514,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>224</v>
       </c>
@@ -54525,7 +54525,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>225</v>
       </c>
@@ -54536,13 +54536,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T00:21:42Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9939,54 +9939,54 @@
         <v>101420.72</v>
       </c>
       <c r="I12" s="52">
-        <v>75109.37</v>
+        <v>76488.35</v>
       </c>
       <c r="J12" s="52">
         <v>83645.65</v>
       </c>
       <c r="K12" s="52">
-        <v>70211.29</v>
+        <v>70758.46</v>
       </c>
       <c r="L12" s="52">
-        <v>13434.36</v>
+        <v>12887.189999999988</v>
       </c>
       <c r="M12" s="53">
-        <v>0.16061038440134068</v>
+        <v>0.1540688607237793</v>
       </c>
       <c r="N12" s="53"/>
       <c r="O12" s="52">
         <v>17775.07</v>
       </c>
       <c r="P12" s="52">
-        <v>4898.08</v>
+        <v>5729.89</v>
       </c>
       <c r="Q12" s="52">
-        <v>12876.99</v>
+        <v>12045.18</v>
       </c>
       <c r="R12" s="53">
-        <v>0.724441028924218</v>
+        <v>0.6776445887414227</v>
       </c>
       <c r="S12" s="54">
         <v>356.07</v>
       </c>
       <c r="T12" s="54">
-        <v>100.75</v>
+        <v>117.75</v>
       </c>
       <c r="U12" s="54">
-        <v>255.32</v>
+        <v>238.32</v>
       </c>
       <c r="V12" s="53">
-        <v>0.7170500182548375</v>
+        <v>0.6693065970174403</v>
       </c>
       <c r="W12" s="53"/>
       <c r="X12" s="55">
-        <v>106.74650124069478</v>
+        <v>79.624033970276</v>
       </c>
       <c r="Y12" s="55">
         <v>77.66490997775718</v>
       </c>
       <c r="Z12" s="53">
-        <v>0.1253</v>
+        <v>0.1092</v>
       </c>
       <c r="AA12" s="56">
         <v>0.2142</v>
@@ -10302,19 +10302,19 @@
         <v>19565.83</v>
       </c>
       <c r="I19" s="52">
-        <v>7621.92</v>
+        <v>7921.92</v>
       </c>
       <c r="J19" s="52">
         <v>13767.340000000002</v>
       </c>
       <c r="K19" s="52">
-        <v>5911.24</v>
+        <v>6211.24</v>
       </c>
       <c r="L19" s="52">
-        <v>7856.100000000002</v>
+        <v>7556.100000000002</v>
       </c>
       <c r="M19" s="53">
-        <v>0.5706331070490016</v>
+        <v>0.5488424052867149</v>
       </c>
       <c r="N19" s="53"/>
       <c r="O19" s="52">
@@ -10343,13 +10343,13 @@
       </c>
       <c r="W19" s="53"/>
       <c r="X19" s="55">
-        <v>125.96143884892086</v>
+        <v>117.328345323741</v>
       </c>
       <c r="Y19" s="55">
         <v>63.27846478985563</v>
       </c>
       <c r="Z19" s="53">
-        <v>0.36479999999999996</v>
+        <v>0.3398</v>
       </c>
       <c r="AA19" s="56">
         <v>0.2885</v>
@@ -10667,19 +10667,19 @@
         <v>102178.42</v>
       </c>
       <c r="I26" s="52">
-        <v>87230.67</v>
+        <v>87101.11</v>
       </c>
       <c r="J26" s="52">
         <v>62464.86</v>
       </c>
       <c r="K26" s="52">
-        <v>58028.31</v>
+        <v>57898.75</v>
       </c>
       <c r="L26" s="52">
-        <v>4436.550000000003</v>
+        <v>4566.110000000001</v>
       </c>
       <c r="M26" s="53">
-        <v>0.07102473294585152</v>
+        <v>0.07309885910254182</v>
       </c>
       <c r="N26" s="53"/>
       <c r="O26" s="52">
@@ -10708,13 +10708,13 @@
       </c>
       <c r="W26" s="53"/>
       <c r="X26" s="55">
-        <v>96.11460050462573</v>
+        <v>96.3325315391085</v>
       </c>
       <c r="Y26" s="55">
         <v>61.20621468124544</v>
       </c>
       <c r="Z26" s="53">
-        <v>0.3958</v>
+        <v>0.3967</v>
       </c>
       <c r="AA26" s="56">
         <v>0.3227</v>
@@ -11030,54 +11030,54 @@
         <v>327431.12</v>
       </c>
       <c r="I33" s="65">
-        <v>219182.25</v>
+        <v>220187.84</v>
       </c>
       <c r="J33" s="52">
         <v>271519.78</v>
       </c>
       <c r="K33" s="52">
-        <v>196853</v>
+        <v>196879.33</v>
       </c>
       <c r="L33" s="52">
-        <v>74666.78000000003</v>
+        <v>74640.45000000004</v>
       </c>
       <c r="M33" s="53">
-        <v>0.2749957295928865</v>
+        <v>0.27489875691561044</v>
       </c>
       <c r="N33" s="53"/>
       <c r="O33" s="52">
         <v>55911.34</v>
       </c>
       <c r="P33" s="52">
-        <v>22329.25</v>
+        <v>23308.51</v>
       </c>
       <c r="Q33" s="52">
-        <v>33582.09</v>
+        <v>32602.829999999998</v>
       </c>
       <c r="R33" s="53">
-        <v>0.6006311063193978</v>
+        <v>0.5831165913748445</v>
       </c>
       <c r="S33" s="54">
         <v>1120.27</v>
       </c>
       <c r="T33" s="54">
-        <v>522.25</v>
+        <v>543.5</v>
       </c>
       <c r="U33" s="54">
-        <v>598.02</v>
+        <v>576.77</v>
       </c>
       <c r="V33" s="53">
-        <v>0.5338177403661617</v>
+        <v>0.514849098877949</v>
       </c>
       <c r="W33" s="53"/>
       <c r="X33" s="55">
-        <v>76.90849210148396</v>
+        <v>72.05127874885005</v>
       </c>
       <c r="Y33" s="55">
         <v>61.5841822414239</v>
       </c>
       <c r="Z33" s="53">
-        <v>0.1549</v>
+        <v>0.151</v>
       </c>
       <c r="AA33" s="56">
         <v>0.174</v>
@@ -11393,54 +11393,54 @@
         <v>94098.32</v>
       </c>
       <c r="I40" s="52">
-        <v>45499.87</v>
+        <v>46289.42</v>
       </c>
       <c r="J40" s="52">
         <v>69042.09000000001</v>
       </c>
       <c r="K40" s="52">
-        <v>35731.93</v>
+        <v>35507.08</v>
       </c>
       <c r="L40" s="52">
-        <v>33310.16000000001</v>
+        <v>33535.01000000001</v>
       </c>
       <c r="M40" s="53">
-        <v>0.4824616404283243</v>
+        <v>0.4857183494879718</v>
       </c>
       <c r="N40" s="53"/>
       <c r="O40" s="52">
         <v>25056.23</v>
       </c>
       <c r="P40" s="52">
-        <v>9767.94</v>
+        <v>10782.34</v>
       </c>
       <c r="Q40" s="52">
-        <v>15288.289999999999</v>
+        <v>14273.89</v>
       </c>
       <c r="R40" s="53">
-        <v>0.6101592298601984</v>
+        <v>0.5696742885901032</v>
       </c>
       <c r="S40" s="54">
         <v>501.83</v>
       </c>
       <c r="T40" s="54">
-        <v>205.75</v>
+        <v>232.25</v>
       </c>
       <c r="U40" s="54">
-        <v>296.08</v>
+        <v>269.58</v>
       </c>
       <c r="V40" s="53">
-        <v>0.5900005978120081</v>
+        <v>0.5371938704342107</v>
       </c>
       <c r="W40" s="53"/>
       <c r="X40" s="55">
-        <v>41.0447630619684</v>
+        <v>32.96193756727664</v>
       </c>
       <c r="Y40" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z40" s="53">
-        <v>0.1565</v>
+        <v>0.1419</v>
       </c>
       <c r="AA40" s="56">
         <v>0.2663</v>
@@ -11758,19 +11758,19 @@
         <v>50582.37</v>
       </c>
       <c r="I47" s="52">
-        <v>25337.26</v>
+        <v>25187.36</v>
       </c>
       <c r="J47" s="52">
         <v>39438.990000000005</v>
       </c>
       <c r="K47" s="52">
-        <v>20582.32</v>
+        <v>20432.420000000002</v>
       </c>
       <c r="L47" s="52">
-        <v>18856.670000000006</v>
+        <v>19006.570000000003</v>
       </c>
       <c r="M47" s="53">
-        <v>0.4781225381278781</v>
+        <v>0.48192334540007237</v>
       </c>
       <c r="N47" s="53"/>
       <c r="O47" s="52">
@@ -11799,13 +11799,13 @@
       </c>
       <c r="W47" s="53"/>
       <c r="X47" s="55">
-        <v>76.63529976019184</v>
+        <v>78.07318944844125</v>
       </c>
       <c r="Y47" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z47" s="53">
-        <v>0.2397</v>
+        <v>0.24420000000000003</v>
       </c>
       <c r="AA47" s="56">
         <v>0.23</v>
@@ -12121,19 +12121,19 @@
         <v>109364.97</v>
       </c>
       <c r="I54" s="52">
-        <v>95642.03</v>
+        <v>95597.19</v>
       </c>
       <c r="J54" s="52">
         <v>75135.01000000001</v>
       </c>
       <c r="K54" s="52">
-        <v>71188.63</v>
+        <v>71143.79000000001</v>
       </c>
       <c r="L54" s="52">
-        <v>3946.3800000000047</v>
+        <v>3991.220000000001</v>
       </c>
       <c r="M54" s="53">
-        <v>0.05252385006669999</v>
+        <v>0.05312064242754477</v>
       </c>
       <c r="N54" s="53"/>
       <c r="O54" s="52">
@@ -12162,13 +12162,13 @@
       </c>
       <c r="W54" s="53"/>
       <c r="X54" s="55">
-        <v>62.138966682761954</v>
+        <v>62.22557218734911</v>
       </c>
       <c r="Y54" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z54" s="53">
-        <v>0.25170000000000003</v>
+        <v>0.2521</v>
       </c>
       <c r="AA54" s="56">
         <v>0.2958</v>
@@ -12841,19 +12841,19 @@
         <v>35572.59</v>
       </c>
       <c r="I68" s="52">
-        <v>9981.43</v>
+        <v>10547.08</v>
       </c>
       <c r="J68" s="52">
         <v>27136.549999999996</v>
       </c>
       <c r="K68" s="52">
-        <v>9832.65</v>
+        <v>10398.3</v>
       </c>
       <c r="L68" s="52">
-        <v>17303.899999999994</v>
+        <v>16738.249999999996</v>
       </c>
       <c r="M68" s="53">
-        <v>0.6376602773749794</v>
+        <v>0.6168156969106242</v>
       </c>
       <c r="N68" s="53"/>
       <c r="O68" s="52">
@@ -12882,13 +12882,13 @@
       </c>
       <c r="W68" s="53"/>
       <c r="X68" s="55">
-        <v>243.27272727272728</v>
+        <v>37.58181818181818</v>
       </c>
       <c r="Y68" s="55">
         <v>72.22475431425701</v>
       </c>
       <c r="Z68" s="53">
-        <v>0.06280000000000001</v>
+        <v>0.0097</v>
       </c>
       <c r="AA68" s="56">
         <v>0.2558</v>
@@ -13916,19 +13916,19 @@
         <v>27002.93</v>
       </c>
       <c r="I89" s="52">
-        <v>26005.99</v>
+        <v>24950.27</v>
       </c>
       <c r="J89" s="52">
         <v>15440.32</v>
       </c>
       <c r="K89" s="52">
-        <v>14988.440000000002</v>
+        <v>13932.720000000001</v>
       </c>
       <c r="L89" s="52">
-        <v>451.8799999999974</v>
+        <v>1507.5999999999985</v>
       </c>
       <c r="M89" s="53">
-        <v>0.029266232824190004</v>
+        <v>0.09764046341008467</v>
       </c>
       <c r="N89" s="53"/>
       <c r="O89" s="52">
@@ -13957,13 +13957,13 @@
       </c>
       <c r="W89" s="53"/>
       <c r="X89" s="55">
-        <v>46.26684503901895</v>
+        <v>50.9746265328874</v>
       </c>
       <c r="Y89" s="55">
         <v>43.49557070636461</v>
       </c>
       <c r="Z89" s="53">
-        <v>0.2852</v>
+        <v>0.31420000000000003</v>
       </c>
       <c r="AA89" s="56">
         <v>0.2718</v>
@@ -14626,30 +14626,74 @@
       <c r="C103" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="D103" s="52"/>
-      <c r="E103" s="69"/>
-      <c r="F103" s="52"/>
-      <c r="G103" s="53"/>
-      <c r="H103" s="52"/>
-      <c r="I103" s="52"/>
-      <c r="J103" s="52"/>
-      <c r="K103" s="52"/>
-      <c r="L103" s="52"/>
-      <c r="M103" s="53"/>
+      <c r="D103" s="52">
+        <v>32473.02</v>
+      </c>
+      <c r="E103" s="69">
+        <v>33188.03</v>
+      </c>
+      <c r="F103" s="52">
+        <v>-715.0099999999984</v>
+      </c>
+      <c r="G103" s="53">
+        <v>-0.022018586506582952</v>
+      </c>
+      <c r="H103" s="52">
+        <v>23075.07</v>
+      </c>
+      <c r="I103" s="52">
+        <v>30925.21</v>
+      </c>
+      <c r="J103" s="52">
+        <v>12691.21</v>
+      </c>
+      <c r="K103" s="52">
+        <v>15184.269999999999</v>
+      </c>
+      <c r="L103" s="52">
+        <v>-2493.0599999999995</v>
+      </c>
+      <c r="M103" s="53">
+        <v>-0.1964398981657383</v>
+      </c>
       <c r="N103" s="53"/>
-      <c r="O103" s="52"/>
-      <c r="P103" s="52"/>
-      <c r="Q103" s="52"/>
-      <c r="R103" s="53"/>
-      <c r="S103" s="54"/>
-      <c r="T103" s="54"/>
-      <c r="U103" s="54"/>
-      <c r="V103" s="53"/>
+      <c r="O103" s="52">
+        <v>10383.86</v>
+      </c>
+      <c r="P103" s="52">
+        <v>15740.94</v>
+      </c>
+      <c r="Q103" s="52">
+        <v>-5357.08</v>
+      </c>
+      <c r="R103" s="53">
+        <v>-0.5159044902377343</v>
+      </c>
+      <c r="S103" s="54">
+        <v>208.2</v>
+      </c>
+      <c r="T103" s="54">
+        <v>317.25</v>
+      </c>
+      <c r="U103" s="54">
+        <v>-109.05000000000001</v>
+      </c>
+      <c r="V103" s="53">
+        <v>-0.5237752161383286</v>
+      </c>
       <c r="W103" s="53"/>
-      <c r="X103" s="55"/>
-      <c r="Y103" s="55"/>
-      <c r="Z103" s="53"/>
-      <c r="AA103" s="56"/>
+      <c r="X103" s="55">
+        <v>7.132608353033885</v>
+      </c>
+      <c r="Y103" s="55">
+        <v>45.139084580403456</v>
+      </c>
+      <c r="Z103" s="53">
+        <v>0.0682</v>
+      </c>
+      <c r="AA103" s="56">
+        <v>0.2894</v>
+      </c>
       <c r="AB103" s="57"/>
       <c r="AD103" s="35" t="s">
         <v>93</v>
@@ -14963,19 +15007,19 @@
         <v>37601.88</v>
       </c>
       <c r="I110" s="52">
-        <v>45837.23</v>
+        <v>45817.77</v>
       </c>
       <c r="J110" s="52">
         <v>21415.85</v>
       </c>
       <c r="K110" s="52">
-        <v>23958.850000000002</v>
+        <v>23939.389999999996</v>
       </c>
       <c r="L110" s="52">
-        <v>-2543.0000000000036</v>
+        <v>-2523.5399999999972</v>
       </c>
       <c r="M110" s="53">
-        <v>-0.11874382758564352</v>
+        <v>-0.11783515480356826</v>
       </c>
       <c r="N110" s="53"/>
       <c r="O110" s="52">
@@ -15004,13 +15048,13 @@
       </c>
       <c r="W110" s="53"/>
       <c r="X110" s="55">
-        <v>48.93201480698043</v>
+        <v>48.973178212585935</v>
       </c>
       <c r="Y110" s="55">
         <v>65.70431400737223</v>
       </c>
       <c r="Z110" s="53">
-        <v>0.3354</v>
+        <v>0.3357</v>
       </c>
       <c r="AA110" s="56">
         <v>0.3616</v>
@@ -15673,19 +15717,19 @@
         <v>82694.87</v>
       </c>
       <c r="I124" s="52">
-        <v>56983.56</v>
+        <v>56763.31</v>
       </c>
       <c r="J124" s="52">
         <v>68214.25</v>
       </c>
       <c r="K124" s="52">
-        <v>52178.049999999996</v>
+        <v>51957.799999999996</v>
       </c>
       <c r="L124" s="52">
-        <v>16036.200000000004</v>
+        <v>16256.450000000004</v>
       </c>
       <c r="M124" s="53">
-        <v>0.23508577753182075</v>
+        <v>0.23831457503380898</v>
       </c>
       <c r="N124" s="53"/>
       <c r="O124" s="52">
@@ -15714,13 +15758,13 @@
       </c>
       <c r="W124" s="53"/>
       <c r="X124" s="55">
-        <v>99.27371428571428</v>
+        <v>101.37133333333333</v>
       </c>
       <c r="Y124" s="55">
         <v>63.04545035767707</v>
       </c>
       <c r="Z124" s="53">
-        <v>0.15460000000000002</v>
+        <v>0.15789999999999998</v>
       </c>
       <c r="AA124" s="56">
         <v>0.1811</v>
@@ -18141,30 +18185,74 @@
       <c r="C173" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="D173" s="52"/>
-      <c r="E173" s="52"/>
-      <c r="F173" s="52"/>
-      <c r="G173" s="53"/>
-      <c r="H173" s="52"/>
-      <c r="I173" s="52"/>
-      <c r="J173" s="52"/>
-      <c r="K173" s="52"/>
-      <c r="L173" s="52"/>
-      <c r="M173" s="53"/>
+      <c r="D173" s="52">
+        <v>146237.11</v>
+      </c>
+      <c r="E173" s="52">
+        <v>125386.21</v>
+      </c>
+      <c r="F173" s="52">
+        <v>20850.89999999998</v>
+      </c>
+      <c r="G173" s="53">
+        <v>0.14258282319720336</v>
+      </c>
+      <c r="H173" s="52">
+        <v>114651.87</v>
+      </c>
+      <c r="I173" s="52">
+        <v>105511.63</v>
+      </c>
+      <c r="J173" s="52">
+        <v>82888.07999999999</v>
+      </c>
+      <c r="K173" s="52">
+        <v>78161.06</v>
+      </c>
+      <c r="L173" s="52">
+        <v>4727.0199999999895</v>
+      </c>
+      <c r="M173" s="53">
+        <v>0.05702894795005495</v>
+      </c>
       <c r="N173" s="53"/>
-      <c r="O173" s="52"/>
-      <c r="P173" s="52"/>
-      <c r="Q173" s="52"/>
-      <c r="R173" s="53"/>
-      <c r="S173" s="54"/>
-      <c r="T173" s="54"/>
-      <c r="U173" s="54"/>
-      <c r="V173" s="53"/>
+      <c r="O173" s="52">
+        <v>31763.79</v>
+      </c>
+      <c r="P173" s="52">
+        <v>27350.57</v>
+      </c>
+      <c r="Q173" s="52">
+        <v>4413.220000000001</v>
+      </c>
+      <c r="R173" s="53">
+        <v>0.13893870976983544</v>
+      </c>
+      <c r="S173" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T173" s="54">
+        <v>548.75</v>
+      </c>
+      <c r="U173" s="54">
+        <v>110.98000000000002</v>
+      </c>
+      <c r="V173" s="53">
+        <v>0.16822033256028984</v>
+      </c>
       <c r="W173" s="53"/>
-      <c r="X173" s="55"/>
-      <c r="Y173" s="55"/>
-      <c r="Z173" s="53"/>
-      <c r="AA173" s="56"/>
+      <c r="X173" s="55">
+        <v>36.21791343963554</v>
+      </c>
+      <c r="Y173" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z173" s="53">
+        <v>0.1585</v>
+      </c>
+      <c r="AA173" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB173" s="57"/>
       <c r="AD173" s="35" t="s">
         <v>93</v>
@@ -18771,30 +18859,74 @@
       <c r="C187" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="D187" s="52"/>
-      <c r="E187" s="52"/>
-      <c r="F187" s="52"/>
-      <c r="G187" s="53"/>
-      <c r="H187" s="52"/>
-      <c r="I187" s="52"/>
-      <c r="J187" s="52"/>
-      <c r="K187" s="52"/>
-      <c r="L187" s="52"/>
-      <c r="M187" s="53"/>
+      <c r="D187" s="52">
+        <v>20992.12</v>
+      </c>
+      <c r="E187" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F187" s="52">
+        <v>6822.439999999999</v>
+      </c>
+      <c r="G187" s="53">
+        <v>0.32500004763692275</v>
+      </c>
+      <c r="H187" s="52">
+        <v>16299.09</v>
+      </c>
+      <c r="I187" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J187" s="52">
+        <v>9784.33</v>
+      </c>
+      <c r="K187" s="52">
+        <v>8137.88</v>
+      </c>
+      <c r="L187" s="52">
+        <v>1646.4499999999998</v>
+      </c>
+      <c r="M187" s="53">
+        <v>0.16827416900288522</v>
+      </c>
       <c r="N187" s="53"/>
-      <c r="O187" s="52"/>
-      <c r="P187" s="52"/>
-      <c r="Q187" s="52"/>
-      <c r="R187" s="53"/>
-      <c r="S187" s="54"/>
-      <c r="T187" s="54"/>
-      <c r="U187" s="54"/>
-      <c r="V187" s="53"/>
+      <c r="O187" s="52">
+        <v>6514.76</v>
+      </c>
+      <c r="P187" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q187" s="52">
+        <v>4953.13</v>
+      </c>
+      <c r="R187" s="53">
+        <v>0.7602935488030257</v>
+      </c>
+      <c r="S187" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T187" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U187" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V187" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W187" s="53"/>
-      <c r="X187" s="55"/>
-      <c r="Y187" s="55"/>
-      <c r="Z187" s="53"/>
-      <c r="AA187" s="56"/>
+      <c r="X187" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y187" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z187" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA187" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB187" s="57"/>
       <c r="AD187" s="35" t="s">
         <v>93</v>
@@ -20023,19 +20155,19 @@
         <v>117394.57</v>
       </c>
       <c r="I215" s="52">
-        <v>26124</v>
+        <v>30594.96</v>
       </c>
       <c r="J215" s="52">
         <v>99479.62000000001</v>
       </c>
       <c r="K215" s="52">
-        <v>26124</v>
+        <v>30594.96</v>
       </c>
       <c r="L215" s="52">
-        <v>73355.62000000001</v>
+        <v>68884.66</v>
       </c>
       <c r="M215" s="53">
-        <v>0.7373934480248316</v>
+        <v>0.692449971159922</v>
       </c>
       <c r="N215" s="53"/>
       <c r="O215" s="52">
@@ -20070,7 +20202,7 @@
         <v>54.93783457863793</v>
       </c>
       <c r="Z215" s="53">
-        <v>0.13419999999999999</v>
+        <v>-0.0139</v>
       </c>
       <c r="AA215" s="56">
         <v>0.1438</v>
@@ -20376,54 +20508,54 @@
         <v>295569.99</v>
       </c>
       <c r="I222" s="52">
-        <v>240067.38</v>
+        <v>241753.24</v>
       </c>
       <c r="J222" s="52">
         <v>178700.37</v>
       </c>
       <c r="K222" s="52">
-        <v>178119.89</v>
+        <v>178956.15</v>
       </c>
       <c r="L222" s="52">
-        <v>580.4799999999814</v>
+        <v>-255.77999999999884</v>
       </c>
       <c r="M222" s="53">
-        <v>0.003248342462861053</v>
+        <v>-0.0014313344734540776</v>
       </c>
       <c r="N222" s="53"/>
       <c r="O222" s="52">
         <v>116869.62</v>
       </c>
       <c r="P222" s="52">
-        <v>61947.49</v>
+        <v>62797.09</v>
       </c>
       <c r="Q222" s="52">
-        <v>54922.13</v>
+        <v>54072.53</v>
       </c>
       <c r="R222" s="53">
-        <v>0.4699436003984611</v>
+        <v>0.4626739609489618</v>
       </c>
       <c r="S222" s="54">
         <v>2344.68</v>
       </c>
       <c r="T222" s="54">
-        <v>1315</v>
+        <v>1335</v>
       </c>
       <c r="U222" s="54">
-        <v>1029.6799999999998</v>
+        <v>1009.6799999999998</v>
       </c>
       <c r="V222" s="53">
-        <v>0.4391558762816247</v>
+        <v>0.4306259276319156</v>
       </c>
       <c r="W222" s="53"/>
       <c r="X222" s="55">
-        <v>50.16819011406844</v>
+        <v>48.153790262172286</v>
       </c>
       <c r="Y222" s="55">
         <v>43.0265399367206</v>
       </c>
       <c r="Z222" s="53">
-        <v>0.21559999999999999</v>
+        <v>0.2101</v>
       </c>
       <c r="AA222" s="56">
         <v>0.2545</v>
@@ -21331,10 +21463,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>972.0499999999884</v>
+        <v>2351.029999999999</v>
       </c>
       <c r="E6" s="52">
-        <v>-972.0499999999884</v>
+        <v>-2351.029999999999</v>
       </c>
       <c r="F6" s="52">
         <v>0</v>
@@ -21358,13 +21490,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-2844.6499999999883</v>
+        <v>-4223.629999999999</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>227.57199999999906</v>
+        <v>337.89039999999994</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>115</v>
@@ -21398,10 +21530,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="52">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E8" s="52">
-        <v>0</v>
+        <v>-300</v>
       </c>
       <c r="F8" s="52"/>
       <c r="G8" s="53">
@@ -21421,13 +21553,13 @@
         <v>0</v>
       </c>
       <c r="M8" s="52">
-        <v>-640</v>
+        <v>-940</v>
       </c>
       <c r="N8" s="54">
         <v>-34.75</v>
       </c>
       <c r="O8" s="58">
-        <v>34.13333333333333</v>
+        <v>50.13333333333333</v>
       </c>
     </row>
     <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21458,10 +21590,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="52">
-        <v>1382.2599999999948</v>
+        <v>1252.699999999997</v>
       </c>
       <c r="E10" s="52">
-        <v>-1382.2599999999948</v>
+        <v>-1252.699999999997</v>
       </c>
       <c r="F10" s="52">
         <v>0</v>
@@ -21485,13 +21617,13 @@
         <v>0</v>
       </c>
       <c r="M10" s="52">
-        <v>-6302.259999999995</v>
+        <v>-6172.699999999997</v>
       </c>
       <c r="N10" s="54">
         <v>-388.25</v>
       </c>
       <c r="O10" s="58">
-        <v>18.522439382806745</v>
+        <v>18.141660543717848</v>
       </c>
     </row>
     <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21522,10 +21654,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>2837.649999999994</v>
+        <v>3843.2399999999907</v>
       </c>
       <c r="E12" s="52">
-        <v>-2837.649999999994</v>
+        <v>-3843.2399999999907</v>
       </c>
       <c r="F12" s="52"/>
       <c r="G12" s="53">
@@ -21547,13 +21679,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-5477.649999999994</v>
+        <v>-6483.239999999991</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-79.38623188405789</v>
+        <v>-93.95999999999987</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>117</v>
@@ -21587,10 +21719,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>3226.1800000000003</v>
+        <v>4015.729999999996</v>
       </c>
       <c r="E14" s="52">
-        <v>-3226.1800000000003</v>
+        <v>-4015.729999999996</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -21614,13 +21746,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-6226.18</v>
+        <v>-7015.729999999996</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>55.59089285714286</v>
+        <v>62.640446428571394</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21651,10 +21783,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>125.67999999999665</v>
+        <v>-24.220000000001164</v>
       </c>
       <c r="E16" s="52">
-        <v>-125.67999999999665</v>
+        <v>24.220000000001164</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -21676,13 +21808,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-3125.6799999999967</v>
+        <v>-2975.779999999999</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>36.030893371757884</v>
+        <v>34.302939481268</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21713,10 +21845,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>321.5200000000041</v>
+        <v>276.68000000000757</v>
       </c>
       <c r="E18" s="52">
-        <v>-321.5200000000041</v>
+        <v>-276.68000000000757</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -21740,13 +21872,13 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-8521.520000000004</v>
+        <v>-8476.680000000008</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>45.087407407407426</v>
+        <v>44.85015873015877</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>118</v>
@@ -21836,10 +21968,10 @@
         <v>0</v>
       </c>
       <c r="D22" s="52">
-        <v>0</v>
+        <v>565.6499999999996</v>
       </c>
       <c r="E22" s="52">
-        <v>0</v>
+        <v>-565.6499999999996</v>
       </c>
       <c r="F22" s="52">
         <v>0</v>
@@ -21859,7 +21991,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="52">
-        <v>0</v>
+        <v>-565.6499999999996</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -22010,10 +22142,10 @@
         <v>0</v>
       </c>
       <c r="D28" s="52">
-        <v>0</v>
+        <v>-1055.7200000000012</v>
       </c>
       <c r="E28" s="52">
-        <v>0</v>
+        <v>1055.7200000000012</v>
       </c>
       <c r="F28" s="52">
         <v>0</v>
@@ -22033,13 +22165,13 @@
         <v>0</v>
       </c>
       <c r="M28" s="52">
-        <v>0</v>
+        <v>1055.7200000000012</v>
       </c>
       <c r="N28" s="54">
         <v>-148.5</v>
       </c>
       <c r="O28" s="58">
-        <v>0</v>
+        <v>-7.109225589225597</v>
       </c>
     </row>
     <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22194,10 +22326,10 @@
         <v>0</v>
       </c>
       <c r="D34" s="52">
-        <v>943.3400000000038</v>
+        <v>923.8799999999974</v>
       </c>
       <c r="E34" s="52">
-        <v>-943.3400000000038</v>
+        <v>-923.8799999999974</v>
       </c>
       <c r="F34" s="52">
         <v>0</v>
@@ -22219,13 +22351,13 @@
         <v>0</v>
       </c>
       <c r="M34" s="52">
-        <v>-943.3400000000038</v>
+        <v>-923.8799999999974</v>
       </c>
       <c r="N34" s="54">
         <v>-204.75</v>
       </c>
       <c r="O34" s="58">
-        <v>4.607277167277186</v>
+        <v>4.512234432234419</v>
       </c>
     </row>
     <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22316,16 +22448,16 @@
         <v>52040.560000000005</v>
       </c>
       <c r="D38" s="52">
-        <v>746.3099999999977</v>
+        <v>526.0599999999977</v>
       </c>
       <c r="E38" s="52">
-        <v>51294.25000000001</v>
+        <v>51514.50000000001</v>
       </c>
       <c r="F38" s="52">
         <v>0</v>
       </c>
       <c r="G38" s="53">
-        <v>0.9856590705403632</v>
+        <v>0.9898913462883566</v>
       </c>
       <c r="H38" s="53">
         <v>0.1750921737769</v>
@@ -22336,10 +22468,10 @@
         <v>0</v>
       </c>
       <c r="L38" s="53">
-        <v>0.9856590705403632</v>
+        <v>0.9898913462883566</v>
       </c>
       <c r="M38" s="52">
-        <v>51294.25000000001</v>
+        <v>51514.50000000001</v>
       </c>
       <c r="N38" s="54"/>
       <c r="O38" s="58">
@@ -22727,10 +22859,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>0</v>
+        <v>2629.5100000000093</v>
       </c>
       <c r="E52" s="99">
-        <v>0</v>
+        <v>-2629.5100000000093</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -22752,13 +22884,13 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-1280</v>
+        <v>-3909.5100000000093</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>4.692942254812099</v>
+        <v>14.333675527039448</v>
       </c>
     </row>
     <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23039,10 +23171,10 @@
         <v>0</v>
       </c>
       <c r="D64" s="99">
-        <v>0</v>
+        <v>4470.959999999999</v>
       </c>
       <c r="E64" s="99">
-        <v>0</v>
+        <v>-4470.959999999999</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
@@ -23062,7 +23194,7 @@
         <v>0</v>
       </c>
       <c r="M64" s="99">
-        <v>-1750</v>
+        <v>-6220.959999999999</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
@@ -23097,14 +23229,14 @@
         <v>34650.399999999965</v>
       </c>
       <c r="D66" s="99">
-        <v>5744.570000000007</v>
+        <v>7430.429999999993</v>
       </c>
       <c r="E66" s="99">
-        <v>28905.829999999958</v>
+        <v>27219.969999999972</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.8342134578533</v>
+        <v>0.7855600512548195</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -23119,16 +23251,16 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.7418624316025207</v>
+        <v>0.6932090250040402</v>
       </c>
       <c r="M66" s="99">
-        <v>25705.829999999958</v>
+        <v>24019.969999999972</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-27.51493711533311</v>
+        <v>-25.71043082686644</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23176,22 +23308,22 @@
         <v>88818.76999999996</v>
       </c>
       <c r="D69" s="104">
-        <v>18681.369999999988</v>
+        <v>29887.739999999983</v>
       </c>
       <c r="E69" s="105">
-        <v>70137.39999999998</v>
+        <v>58931.02999999998</v>
       </c>
       <c r="F69" s="106" t="s">
         <v>122</v>
       </c>
       <c r="G69" s="107">
-        <v>0.7896686702596761</v>
+        <v>0.6634974791927427</v>
       </c>
       <c r="H69" s="108" t="s">
         <v>123</v>
       </c>
       <c r="I69" s="109">
-        <v>0.20609157276102777</v>
+        <v>0.0799203816940944</v>
       </c>
       <c r="J69" s="36"/>
       <c r="K69" s="36"/>
@@ -23799,10 +23931,10 @@
         <v>356.07</v>
       </c>
       <c r="D6" s="54">
-        <v>100.75</v>
+        <v>117.75</v>
       </c>
       <c r="E6" s="54">
-        <v>255.32</v>
+        <v>238.32</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -23962,10 +24094,10 @@
         <v>1120.27</v>
       </c>
       <c r="D12" s="54">
-        <v>522.25</v>
+        <v>543.5</v>
       </c>
       <c r="E12" s="54">
-        <v>598.02</v>
+        <v>576.77</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -24019,10 +24151,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>205.75</v>
+        <v>232.25</v>
       </c>
       <c r="E14" s="54">
-        <v>296.08</v>
+        <v>269.58</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -25011,10 +25143,10 @@
         <v>659.73</v>
       </c>
       <c r="D52" s="54">
-        <v>505.25</v>
+        <v>548.75</v>
       </c>
       <c r="E52" s="54">
-        <v>154.48000000000002</v>
+        <v>110.98000000000002</v>
       </c>
       <c r="F52" s="54"/>
       <c r="G52" s="54"/>
@@ -25358,10 +25490,10 @@
         <v>2344.68</v>
       </c>
       <c r="D66" s="54">
-        <v>1315</v>
+        <v>1335</v>
       </c>
       <c r="E66" s="54">
-        <v>1029.6799999999998</v>
+        <v>1009.6799999999998</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T01:54:13Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16176,7 +16176,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21286,7 +21286,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21300,7 +21300,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21322,7 +21322,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21370,7 +21370,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21388,7 +21388,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21435,7 +21435,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21452,7 +21452,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21502,7 +21502,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21519,7 +21519,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21562,7 +21562,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21579,7 +21579,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21626,7 +21626,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21643,7 +21643,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21659,7 +21659,9 @@
       <c r="E12" s="52">
         <v>-3843.2399999999907</v>
       </c>
-      <c r="F12" s="52"/>
+      <c r="F12" s="52">
+        <v>3</v>
+      </c>
       <c r="G12" s="53">
         <v>0</v>
       </c>
@@ -21691,7 +21693,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21708,7 +21710,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21755,7 +21757,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21772,7 +21774,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21817,7 +21819,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21834,7 +21836,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -21884,7 +21886,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -21901,7 +21903,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -21940,7 +21942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -21957,7 +21959,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -21998,7 +22000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22015,7 +22017,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22052,7 +22054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22069,7 +22071,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22114,7 +22116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22131,7 +22133,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22174,7 +22176,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22191,7 +22193,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22234,7 +22236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22251,7 +22253,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22298,7 +22300,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22315,7 +22317,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22360,7 +22362,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22377,7 +22379,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22420,7 +22422,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22437,7 +22439,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22478,7 +22480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22495,7 +22497,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22540,7 +22542,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22557,7 +22559,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22600,7 +22602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22617,7 +22619,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22654,7 +22656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22671,7 +22673,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22712,7 +22714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22729,7 +22731,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22772,7 +22774,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22789,7 +22791,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22831,7 +22833,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22848,7 +22850,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -22893,7 +22895,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -22910,7 +22912,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -22955,7 +22957,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -22972,7 +22974,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23017,7 +23019,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23034,7 +23036,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23071,7 +23073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23088,7 +23090,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23105,7 +23107,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23122,7 +23124,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23143,7 +23145,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23160,7 +23162,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23201,7 +23203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23218,7 +23220,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23263,7 +23265,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23280,7 +23282,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23297,7 +23299,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23332,7 +23334,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23715,7 +23717,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23726,7 +23728,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23747,7 +23749,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23809,7 +23811,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -23867,7 +23869,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -23901,7 +23903,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -23920,7 +23922,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -23954,7 +23956,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -23973,7 +23975,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24007,7 +24009,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24026,7 +24028,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24064,7 +24066,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24083,7 +24085,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24121,7 +24123,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24140,7 +24142,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24178,7 +24180,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24197,7 +24199,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24230,7 +24232,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24249,7 +24251,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24282,7 +24284,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24301,7 +24303,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24332,7 +24334,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24351,7 +24353,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24386,7 +24388,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24405,7 +24407,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24438,7 +24440,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24457,7 +24459,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24488,7 +24490,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24507,7 +24509,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24539,7 +24541,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24558,7 +24560,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24594,7 +24596,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24613,7 +24615,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24642,7 +24644,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24661,7 +24663,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24692,7 +24694,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24711,7 +24713,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24744,7 +24746,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24763,7 +24765,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24799,7 +24801,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24818,7 +24820,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24853,7 +24855,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -24872,7 +24874,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24902,7 +24904,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -24921,7 +24923,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24961,7 +24963,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -24980,7 +24982,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25009,7 +25011,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25028,7 +25030,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25061,7 +25063,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25080,7 +25082,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25113,7 +25115,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25132,7 +25134,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25168,7 +25170,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25187,7 +25189,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25223,7 +25225,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25242,7 +25244,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25276,7 +25278,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25295,7 +25297,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25330,7 +25332,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25349,7 +25351,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25368,7 +25370,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25387,7 +25389,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25408,7 +25410,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25427,7 +25429,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25460,7 +25462,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25479,7 +25481,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25518,7 +25520,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25537,7 +25539,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25556,7 +25558,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25575,7 +25577,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25620,7 +25622,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25659,7 +25661,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25688,7 +25690,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25733,7 +25735,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25778,7 +25780,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25797,7 +25799,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25844,7 +25846,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -25889,7 +25891,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -25908,7 +25910,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -25931,7 +25933,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -25954,7 +25956,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -25977,7 +25979,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26000,7 +26002,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26023,7 +26025,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26046,7 +26048,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26069,7 +26071,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26092,7 +26094,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26115,7 +26117,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26138,7 +26140,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26161,7 +26163,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26184,7 +26186,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26205,7 +26207,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26226,7 +26228,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26247,7 +26249,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26268,7 +26270,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26289,7 +26291,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26310,7 +26312,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26331,7 +26333,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26354,7 +26356,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26377,7 +26379,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26400,7 +26402,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26423,7 +26425,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26446,7 +26448,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26469,7 +26471,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26492,7 +26494,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26511,7 +26513,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26530,7 +26532,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26549,7 +26551,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26568,7 +26570,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26642,11 +26644,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26678,7 +26679,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26711,7 +26712,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26744,7 +26745,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26777,7 +26778,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26810,7 +26811,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26843,7 +26844,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -26876,7 +26877,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -26909,7 +26910,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -26940,7 +26941,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -26971,7 +26972,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27004,7 +27005,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27037,7 +27038,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27070,7 +27071,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27103,7 +27104,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27136,7 +27137,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27169,7 +27170,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27202,7 +27203,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27235,7 +27236,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27268,7 +27269,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27301,7 +27302,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27334,7 +27335,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27367,7 +27368,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27400,7 +27401,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27433,7 +27434,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27466,7 +27467,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27499,7 +27500,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27531,7 +27532,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27563,7 +27564,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27595,7 +27596,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27627,7 +27628,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27659,7 +27660,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27689,7 +27690,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27719,7 +27720,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27751,7 +27752,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27783,7 +27784,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27815,7 +27816,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27847,7 +27848,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -27879,7 +27880,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -27909,7 +27910,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -27941,7 +27942,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -27973,7 +27974,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28005,7 +28006,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28037,7 +28038,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28067,7 +28068,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28097,7 +28098,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28127,7 +28128,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28157,7 +28158,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28189,7 +28190,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28221,7 +28222,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28251,7 +28252,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28281,7 +28282,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28311,7 +28312,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28341,7 +28342,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28371,7 +28372,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28466,11 +28467,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28502,7 +28502,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28533,7 +28533,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28564,7 +28564,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28595,7 +28595,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28626,7 +28626,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28657,7 +28657,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28688,7 +28688,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28719,7 +28719,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28750,7 +28750,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28781,7 +28781,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28812,7 +28812,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28843,7 +28843,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -28874,7 +28874,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -28905,7 +28905,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -28936,7 +28936,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -28967,7 +28967,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -28998,7 +28998,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29029,7 +29029,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29060,7 +29060,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29091,7 +29091,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29121,7 +29121,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29151,7 +29151,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29181,7 +29181,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29211,7 +29211,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29241,7 +29241,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29271,7 +29271,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29301,7 +29301,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29331,7 +29331,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29361,7 +29361,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29391,7 +29391,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29421,7 +29421,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29451,7 +29451,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29481,7 +29481,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29511,7 +29511,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29541,7 +29541,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29571,7 +29571,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29603,7 +29603,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29635,7 +29635,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29665,7 +29665,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29695,7 +29695,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29725,7 +29725,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29755,7 +29755,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29785,7 +29785,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51528,19 +51528,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51554,7 +51554,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51566,7 +51566,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51577,7 +51577,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51588,7 +51588,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51599,13 +51599,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T01:58:49Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="226">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6757,7 +6757,9 @@
       <c r="R32" s="13"/>
       <c r="S32" s="13"/>
       <c r="T32" s="16"/>
-      <c r="U32" s="1"/>
+      <c r="U32" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
       <c r="X32" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T01:59:30Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="226">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5974,18 +5974,30 @@
       <c r="K12" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="L12" s="13"/>
+      <c r="L12" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="M12" s="13" t="s">
         <v>27</v>
       </c>
       <c r="N12" s="14"/>
       <c r="O12" s="18"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="15"/>
-      <c r="R12" s="13"/>
-      <c r="S12" s="13"/>
+      <c r="P12" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q12" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="T12" s="16"/>
-      <c r="U12" s="1"/>
+      <c r="U12" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
       <c r="X12" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:08:32Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="226">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5798,8 +5798,12 @@
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>28</v>
+      </c>
       <c r="H8" s="13"/>
       <c r="I8" s="13"/>
       <c r="J8" s="13"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:10:58Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -6758,7 +6758,7 @@
         <v>28</v>
       </c>
       <c r="L32" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="14"/>
@@ -21701,13 +21701,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-6483.239999999991</v>
+        <v>-6480.239999999991</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-93.95999999999987</v>
+        <v>-93.9165217391303</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>117</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:12:04Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6760,8 +6760,12 @@
       <c r="L32" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="M32" s="13"/>
-      <c r="N32" s="14"/>
+      <c r="M32" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="N32" s="14" t="s">
+        <v>28</v>
+      </c>
       <c r="O32" s="13" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:13:45Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5824,9 +5824,15 @@
         <v>27</v>
       </c>
       <c r="P8" s="13"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="13"/>
-      <c r="S8" s="13"/>
+      <c r="Q8" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="T8" s="16"/>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:17:00Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5834,7 +5834,9 @@
         <v>27</v>
       </c>
       <c r="T8" s="16"/>
-      <c r="U8" s="1"/>
+      <c r="U8" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
       <c r="X8" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:18:12Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7977,10 +7977,18 @@
       <c r="C64" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="D64" s="29"/>
-      <c r="E64" s="13"/>
-      <c r="F64" s="13"/>
-      <c r="G64" s="14"/>
+      <c r="D64" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E64" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F64" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G64" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="H64" s="13"/>
       <c r="I64" s="13"/>
       <c r="J64" s="13"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:18:55Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7990,9 +7990,15 @@
         <v>27</v>
       </c>
       <c r="H64" s="13"/>
-      <c r="I64" s="13"/>
-      <c r="J64" s="13"/>
-      <c r="K64" s="13"/>
+      <c r="I64" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="J64" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="K64" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="L64" s="13"/>
       <c r="M64" s="13"/>
       <c r="N64" s="14"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:22:34Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -8001,7 +8001,9 @@
       </c>
       <c r="L64" s="13"/>
       <c r="M64" s="13"/>
-      <c r="N64" s="14"/>
+      <c r="N64" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="O64" s="13"/>
       <c r="P64" s="18"/>
       <c r="Q64" s="15"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:23:27Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -8006,7 +8006,9 @@
       </c>
       <c r="O64" s="13"/>
       <c r="P64" s="18"/>
-      <c r="Q64" s="15"/>
+      <c r="Q64" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="R64" s="13"/>
       <c r="S64" s="13"/>
       <c r="T64" s="16"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:30:58Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -8014,7 +8014,9 @@
         <v>27</v>
       </c>
       <c r="R64" s="13"/>
-      <c r="S64" s="13"/>
+      <c r="S64" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="T64" s="16"/>
       <c r="U64" s="1"/>
       <c r="V64" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:32:02Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16244,7 +16244,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21354,7 +21354,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21368,7 +21368,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21390,7 +21390,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21438,7 +21438,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21456,7 +21456,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21503,7 +21503,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21520,7 +21520,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21570,7 +21570,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21587,7 +21587,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21630,7 +21630,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21647,7 +21647,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21694,7 +21694,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21711,7 +21711,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21761,7 +21761,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21778,7 +21778,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21842,7 +21842,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21887,7 +21887,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21904,7 +21904,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -21954,7 +21954,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -21971,7 +21971,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22010,7 +22010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22027,7 +22027,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22068,7 +22068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22085,7 +22085,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22122,7 +22122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22139,7 +22139,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22184,7 +22184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22201,7 +22201,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22244,7 +22244,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22261,7 +22261,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22304,7 +22304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22321,7 +22321,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22368,7 +22368,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22385,7 +22385,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22430,7 +22430,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22447,7 +22447,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22490,7 +22490,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22507,7 +22507,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22548,7 +22548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22565,7 +22565,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22610,7 +22610,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22627,7 +22627,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22670,7 +22670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22687,7 +22687,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22724,7 +22724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22741,7 +22741,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22782,7 +22782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22799,7 +22799,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22842,7 +22842,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22859,7 +22859,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22901,7 +22901,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22918,7 +22918,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -22963,7 +22963,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -22980,7 +22980,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23025,7 +23025,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23042,7 +23042,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23087,7 +23087,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23104,7 +23104,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23141,7 +23141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23158,7 +23158,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23175,7 +23175,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23192,7 +23192,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23213,7 +23213,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23230,7 +23230,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23271,7 +23271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23288,7 +23288,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23333,7 +23333,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23350,7 +23350,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23367,7 +23367,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23402,7 +23402,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23785,7 +23785,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23796,7 +23796,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23817,7 +23817,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23879,7 +23879,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -23937,7 +23937,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -23971,7 +23971,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -23990,7 +23990,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24024,7 +24024,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24043,7 +24043,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24077,7 +24077,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24096,7 +24096,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24134,7 +24134,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24153,7 +24153,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24191,7 +24191,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24210,7 +24210,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24248,7 +24248,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24267,7 +24267,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24300,7 +24300,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24319,7 +24319,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24352,7 +24352,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24371,7 +24371,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24402,7 +24402,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24421,7 +24421,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24456,7 +24456,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24475,7 +24475,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24508,7 +24508,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24527,7 +24527,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24558,7 +24558,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24577,7 +24577,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24609,7 +24609,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24628,7 +24628,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24664,7 +24664,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24683,7 +24683,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24712,7 +24712,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24731,7 +24731,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24762,7 +24762,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24781,7 +24781,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24814,7 +24814,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24833,7 +24833,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24869,7 +24869,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24888,7 +24888,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24923,7 +24923,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -24942,7 +24942,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24972,7 +24972,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -24991,7 +24991,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25031,7 +25031,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25050,7 +25050,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25079,7 +25079,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25098,7 +25098,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25131,7 +25131,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25150,7 +25150,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25183,7 +25183,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25202,7 +25202,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25238,7 +25238,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25257,7 +25257,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25293,7 +25293,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25312,7 +25312,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25346,7 +25346,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25365,7 +25365,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25400,7 +25400,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25419,7 +25419,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25438,7 +25438,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25457,7 +25457,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25478,7 +25478,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25497,7 +25497,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25530,7 +25530,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25549,7 +25549,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25588,7 +25588,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25607,7 +25607,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25626,7 +25626,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25645,7 +25645,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25690,7 +25690,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25729,7 +25729,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25758,7 +25758,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25803,7 +25803,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25848,7 +25848,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25867,7 +25867,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25914,7 +25914,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -25959,7 +25959,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -25978,7 +25978,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -26001,7 +26001,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -26024,7 +26024,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -26047,7 +26047,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26070,7 +26070,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26093,7 +26093,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26116,7 +26116,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26139,7 +26139,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26162,7 +26162,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26185,7 +26185,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26208,7 +26208,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26231,7 +26231,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26254,7 +26254,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26275,7 +26275,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26296,7 +26296,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26317,7 +26317,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26338,7 +26338,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26359,7 +26359,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26380,7 +26380,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26401,7 +26401,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26424,7 +26424,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26447,7 +26447,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26470,7 +26470,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26493,7 +26493,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26516,7 +26516,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26539,7 +26539,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26562,7 +26562,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26581,7 +26581,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26600,7 +26600,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26619,7 +26619,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26638,7 +26638,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26712,10 +26712,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26747,7 +26748,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26780,7 +26781,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26813,7 +26814,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26846,7 +26847,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26879,7 +26880,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26912,7 +26913,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -26945,7 +26946,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -26978,7 +26979,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27009,7 +27010,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27040,7 +27041,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27073,7 +27074,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27106,7 +27107,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27139,7 +27140,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27172,7 +27173,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27205,7 +27206,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27238,7 +27239,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27271,7 +27272,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27304,7 +27305,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27337,7 +27338,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27370,7 +27371,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27403,7 +27404,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27436,7 +27437,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27469,7 +27470,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27502,7 +27503,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27535,7 +27536,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27568,7 +27569,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27600,7 +27601,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27632,7 +27633,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27664,7 +27665,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27696,7 +27697,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27728,7 +27729,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27758,7 +27759,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27788,7 +27789,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27820,7 +27821,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27852,7 +27853,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27884,7 +27885,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27916,7 +27917,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -27948,7 +27949,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -27978,7 +27979,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -28010,7 +28011,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -28042,7 +28043,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28074,7 +28075,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28106,7 +28107,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28136,7 +28137,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28166,7 +28167,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28196,7 +28197,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28226,7 +28227,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28258,7 +28259,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28290,7 +28291,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28320,7 +28321,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28350,7 +28351,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28380,7 +28381,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28410,7 +28411,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28440,7 +28441,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28535,10 +28536,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28570,7 +28572,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28601,7 +28603,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28632,7 +28634,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28663,7 +28665,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28694,7 +28696,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28725,7 +28727,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28756,7 +28758,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28787,7 +28789,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28818,7 +28820,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28849,7 +28851,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28880,7 +28882,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28911,7 +28913,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -28942,7 +28944,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -28973,7 +28975,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29004,7 +29006,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29035,7 +29037,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29066,7 +29068,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29097,7 +29099,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29128,7 +29130,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29159,7 +29161,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29189,7 +29191,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29219,7 +29221,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29249,7 +29251,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29279,7 +29281,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29309,7 +29311,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29339,7 +29341,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29369,7 +29371,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29399,7 +29401,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29429,7 +29431,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29459,7 +29461,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29489,7 +29491,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29519,7 +29521,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29549,7 +29551,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29579,7 +29581,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29609,7 +29611,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29639,7 +29641,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29671,7 +29673,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29703,7 +29705,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29733,7 +29735,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29763,7 +29765,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29793,7 +29795,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29823,7 +29825,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29853,7 +29855,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51596,19 +51598,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51622,7 +51624,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51634,7 +51636,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51645,7 +51647,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51656,7 +51658,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51667,13 +51669,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:33:16Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16244,7 +16244,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21354,7 +21354,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21368,7 +21368,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21390,7 +21390,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21438,7 +21438,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21456,7 +21456,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21503,7 +21503,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21520,7 +21520,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21570,7 +21570,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21587,7 +21587,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21630,7 +21630,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21647,7 +21647,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21694,7 +21694,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21711,7 +21711,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21761,7 +21761,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21778,7 +21778,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21842,7 +21842,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21887,7 +21887,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21904,7 +21904,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -21954,7 +21954,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -21971,7 +21971,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22010,7 +22010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22027,7 +22027,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22068,7 +22068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22085,7 +22085,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22122,7 +22122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22139,7 +22139,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22184,7 +22184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22201,7 +22201,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22244,7 +22244,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22261,7 +22261,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22304,7 +22304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22321,7 +22321,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22368,7 +22368,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22385,7 +22385,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22430,7 +22430,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22447,7 +22447,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22490,7 +22490,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22507,7 +22507,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22548,7 +22548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22565,7 +22565,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22610,7 +22610,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22627,7 +22627,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22670,7 +22670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22687,7 +22687,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22724,7 +22724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22741,7 +22741,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22782,7 +22782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22799,7 +22799,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22842,7 +22842,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22859,7 +22859,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22901,7 +22901,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22918,7 +22918,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -22963,7 +22963,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -22980,7 +22980,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23025,7 +23025,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23042,7 +23042,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23087,7 +23087,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23104,7 +23104,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23141,7 +23141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23158,7 +23158,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23175,7 +23175,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23192,7 +23192,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23213,7 +23213,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23230,7 +23230,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23271,7 +23271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23288,7 +23288,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23333,7 +23333,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23350,7 +23350,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23367,7 +23367,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23402,7 +23402,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23785,7 +23785,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23796,7 +23796,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23817,7 +23817,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23879,7 +23879,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -23937,7 +23937,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -23971,7 +23971,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -23990,7 +23990,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24024,7 +24024,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24043,7 +24043,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24077,7 +24077,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24096,7 +24096,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24134,7 +24134,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24153,7 +24153,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24191,7 +24191,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24210,7 +24210,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24248,7 +24248,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24267,7 +24267,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24300,7 +24300,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24319,7 +24319,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24352,7 +24352,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24371,7 +24371,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24402,7 +24402,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24421,7 +24421,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24456,7 +24456,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24475,7 +24475,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24508,7 +24508,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24527,7 +24527,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24558,7 +24558,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24577,7 +24577,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24609,7 +24609,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24628,7 +24628,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24664,7 +24664,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24683,7 +24683,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24712,7 +24712,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24731,7 +24731,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24762,7 +24762,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24781,7 +24781,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24814,7 +24814,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24833,7 +24833,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24869,7 +24869,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24888,7 +24888,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24923,7 +24923,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -24942,7 +24942,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24972,7 +24972,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -24991,7 +24991,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25031,7 +25031,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25050,7 +25050,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25079,7 +25079,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25098,7 +25098,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25131,7 +25131,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25150,7 +25150,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25183,7 +25183,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25202,7 +25202,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25238,7 +25238,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25257,7 +25257,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25293,7 +25293,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25312,7 +25312,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25346,7 +25346,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25365,7 +25365,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25400,7 +25400,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25419,7 +25419,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25438,7 +25438,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25457,7 +25457,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25478,7 +25478,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25497,7 +25497,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25530,7 +25530,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25549,7 +25549,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25588,7 +25588,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25607,7 +25607,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25626,7 +25626,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25645,7 +25645,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25690,7 +25690,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25729,7 +25729,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25758,7 +25758,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25803,7 +25803,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25848,7 +25848,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25867,7 +25867,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25914,7 +25914,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -25959,7 +25959,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -25978,7 +25978,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -26001,7 +26001,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -26024,7 +26024,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -26047,7 +26047,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26070,7 +26070,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26093,7 +26093,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26116,7 +26116,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26139,7 +26139,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26162,7 +26162,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26185,7 +26185,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26208,7 +26208,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26231,7 +26231,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26254,7 +26254,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26275,7 +26275,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26296,7 +26296,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26317,7 +26317,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26338,7 +26338,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26359,7 +26359,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26380,7 +26380,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26401,7 +26401,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26424,7 +26424,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26447,7 +26447,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26470,7 +26470,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26493,7 +26493,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26516,7 +26516,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26539,7 +26539,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26562,7 +26562,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26581,7 +26581,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26600,7 +26600,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26619,7 +26619,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26638,7 +26638,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26712,11 +26712,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26748,7 +26747,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26781,7 +26780,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26814,7 +26813,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26847,7 +26846,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26880,7 +26879,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26913,7 +26912,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -26946,7 +26945,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -26979,7 +26978,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27010,7 +27009,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27041,7 +27040,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27074,7 +27073,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27107,7 +27106,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27140,7 +27139,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27173,7 +27172,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27206,7 +27205,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27239,7 +27238,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27272,7 +27271,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27305,7 +27304,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27338,7 +27337,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27371,7 +27370,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27404,7 +27403,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27437,7 +27436,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27470,7 +27469,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27503,7 +27502,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27536,7 +27535,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27569,7 +27568,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27601,7 +27600,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27633,7 +27632,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27665,7 +27664,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27697,7 +27696,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27729,7 +27728,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27759,7 +27758,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27789,7 +27788,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27821,7 +27820,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27853,7 +27852,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27885,7 +27884,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27917,7 +27916,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -27949,7 +27948,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -27979,7 +27978,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -28011,7 +28010,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -28043,7 +28042,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28075,7 +28074,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28107,7 +28106,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28137,7 +28136,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28167,7 +28166,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28197,7 +28196,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28227,7 +28226,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28259,7 +28258,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28291,7 +28290,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28321,7 +28320,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28351,7 +28350,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28381,7 +28380,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28411,7 +28410,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28441,7 +28440,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28536,11 +28535,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28572,7 +28570,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28603,7 +28601,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28634,7 +28632,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28665,7 +28663,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28696,7 +28694,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28727,7 +28725,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28758,7 +28756,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28789,7 +28787,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28820,7 +28818,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28851,7 +28849,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28882,7 +28880,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28913,7 +28911,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -28944,7 +28942,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -28975,7 +28973,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29006,7 +29004,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29037,7 +29035,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29068,7 +29066,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29099,7 +29097,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29130,7 +29128,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29161,7 +29159,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29191,7 +29189,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29221,7 +29219,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29251,7 +29249,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29281,7 +29279,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29311,7 +29309,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29341,7 +29339,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29371,7 +29369,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29401,7 +29399,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29431,7 +29429,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29461,7 +29459,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29491,7 +29489,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29521,7 +29519,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29551,7 +29549,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29581,7 +29579,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29611,7 +29609,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29641,7 +29639,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29673,7 +29671,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29705,7 +29703,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29735,7 +29733,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29765,7 +29763,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29795,7 +29793,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29825,7 +29823,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29855,7 +29853,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51598,19 +51596,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51624,7 +51622,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51636,7 +51634,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51647,7 +51645,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51658,7 +51656,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51669,13 +51667,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:34:21Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -8013,12 +8013,16 @@
       <c r="Q64" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="R64" s="13"/>
+      <c r="R64" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="S64" s="13" t="s">
         <v>27</v>
       </c>
       <c r="T64" s="16"/>
-      <c r="U64" s="1"/>
+      <c r="U64" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V64" s="1"/>
       <c r="W64" s="1"/>
       <c r="X64" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:37:38Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6403,7 +6403,9 @@
       <c r="K22" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="L22" s="13"/>
+      <c r="L22" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="M22" s="13"/>
       <c r="N22" s="14"/>
       <c r="O22" s="13"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:40:20Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6406,13 +6406,23 @@
       <c r="L22" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="M22" s="13"/>
-      <c r="N22" s="14"/>
+      <c r="M22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="O22" s="13"/>
       <c r="P22" s="13"/>
-      <c r="Q22" s="15"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="13"/>
+      <c r="Q22" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="R22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="S22" s="13" t="s">
+        <v>28</v>
+      </c>
       <c r="T22" s="16"/>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:42:18Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6424,7 +6424,9 @@
         <v>28</v>
       </c>
       <c r="T22" s="16"/>
-      <c r="U22" s="1"/>
+      <c r="U22" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V22" s="1"/>
       <c r="W22" s="1"/>
       <c r="X22" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:43:04Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6479,7 +6479,9 @@
       <c r="C24" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="13"/>
+      <c r="D24" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="E24" s="13"/>
       <c r="F24" s="13"/>
       <c r="G24" s="14"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:44:47Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6495,9 +6495,15 @@
       <c r="I24" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
+      <c r="J24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L24" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="M24" s="13"/>
       <c r="N24" s="14"/>
       <c r="O24" s="13"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T02:50:00Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1127" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6526,7 +6526,9 @@
         <v>28</v>
       </c>
       <c r="T24" s="16"/>
-      <c r="U24" s="1"/>
+      <c r="U24" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V24" s="1"/>
       <c r="W24" s="1"/>
       <c r="X24" s="1"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-03T03:50:50Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16308,7 +16308,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21418,7 +21418,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21432,7 +21432,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21454,7 +21454,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21502,7 +21502,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21520,7 +21520,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21567,7 +21567,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21584,7 +21584,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21634,7 +21634,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21651,7 +21651,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21694,7 +21694,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21711,7 +21711,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21758,7 +21758,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21775,7 +21775,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21842,7 +21842,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21889,7 +21889,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21906,7 +21906,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21951,7 +21951,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21968,7 +21968,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -22018,7 +22018,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -22035,7 +22035,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22074,7 +22074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22091,7 +22091,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22125,14 +22125,14 @@
         <v>0</v>
       </c>
       <c r="M22" s="52">
-        <v>-565.6499999999996</v>
+        <v>-562.6499999999996</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22149,7 +22149,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22181,14 +22181,14 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>-1528.260000000002</v>
+        <v>-1525.260000000002</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22205,7 +22205,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22250,7 +22250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22267,7 +22267,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22310,7 +22310,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22327,7 +22327,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22370,7 +22370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22387,7 +22387,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22434,7 +22434,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22451,7 +22451,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22496,7 +22496,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22513,7 +22513,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22556,7 +22556,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22573,7 +22573,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22614,7 +22614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22631,7 +22631,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22676,7 +22676,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22693,7 +22693,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22736,7 +22736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22753,7 +22753,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22790,7 +22790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22807,7 +22807,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22848,7 +22848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22865,7 +22865,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22908,7 +22908,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22925,7 +22925,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22967,7 +22967,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22984,7 +22984,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -23029,7 +23029,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -23046,7 +23046,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23091,7 +23091,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23108,7 +23108,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23153,7 +23153,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23170,7 +23170,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23207,7 +23207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23224,7 +23224,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23241,7 +23241,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23258,7 +23258,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23279,7 +23279,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23296,7 +23296,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23337,7 +23337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23354,7 +23354,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23399,7 +23399,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23416,7 +23416,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23433,7 +23433,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23468,7 +23468,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23851,7 +23851,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23862,7 +23862,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23883,7 +23883,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23945,7 +23945,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -24003,7 +24003,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -24037,7 +24037,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -24056,7 +24056,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24090,7 +24090,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24109,7 +24109,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24143,7 +24143,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24162,7 +24162,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24200,7 +24200,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24219,7 +24219,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24257,7 +24257,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24276,7 +24276,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24314,7 +24314,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24333,7 +24333,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24366,7 +24366,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24385,7 +24385,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24418,7 +24418,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24437,7 +24437,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24468,7 +24468,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24487,7 +24487,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24522,7 +24522,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24541,7 +24541,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24574,7 +24574,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24593,7 +24593,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24624,7 +24624,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24643,7 +24643,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24675,7 +24675,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24694,7 +24694,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24730,7 +24730,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24749,7 +24749,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24778,7 +24778,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24797,7 +24797,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24828,7 +24828,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24847,7 +24847,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24880,7 +24880,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24899,7 +24899,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24935,7 +24935,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24954,7 +24954,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24989,7 +24989,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -25008,7 +25008,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25038,7 +25038,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -25057,7 +25057,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25097,7 +25097,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25116,7 +25116,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25145,7 +25145,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25164,7 +25164,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25197,7 +25197,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25216,7 +25216,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25249,7 +25249,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25268,7 +25268,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25304,7 +25304,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25323,7 +25323,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25359,7 +25359,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25378,7 +25378,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25412,7 +25412,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25431,7 +25431,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25466,7 +25466,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25485,7 +25485,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25504,7 +25504,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25523,7 +25523,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25544,7 +25544,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25563,7 +25563,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25596,7 +25596,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25615,7 +25615,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25654,7 +25654,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25673,7 +25673,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25692,7 +25692,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25711,7 +25711,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25756,7 +25756,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25795,7 +25795,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25824,7 +25824,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25869,7 +25869,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25914,7 +25914,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25933,7 +25933,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25980,7 +25980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -26025,7 +26025,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -26044,7 +26044,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -26067,7 +26067,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -26090,7 +26090,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -26113,7 +26113,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26136,7 +26136,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26159,7 +26159,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26182,7 +26182,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26205,7 +26205,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26228,7 +26228,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26251,7 +26251,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26274,7 +26274,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26297,7 +26297,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26320,7 +26320,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26341,7 +26341,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26362,7 +26362,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26383,7 +26383,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26404,7 +26404,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26425,7 +26425,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26446,7 +26446,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26467,7 +26467,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26490,7 +26490,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26513,7 +26513,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26536,7 +26536,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26559,7 +26559,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26582,7 +26582,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26605,7 +26605,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26628,7 +26628,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26647,7 +26647,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26666,7 +26666,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26685,7 +26685,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26704,7 +26704,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26778,10 +26778,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26813,7 +26814,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26846,7 +26847,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26879,7 +26880,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26912,7 +26913,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26945,7 +26946,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26978,7 +26979,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -27011,7 +27012,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -27044,7 +27045,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27075,7 +27076,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27106,7 +27107,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27139,7 +27140,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27172,7 +27173,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27205,7 +27206,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27238,7 +27239,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27271,7 +27272,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27304,7 +27305,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27337,7 +27338,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27370,7 +27371,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27403,7 +27404,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27436,7 +27437,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27469,7 +27470,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27502,7 +27503,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27535,7 +27536,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27568,7 +27569,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27601,7 +27602,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27634,7 +27635,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27666,7 +27667,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27698,7 +27699,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27730,7 +27731,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27762,7 +27763,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27794,7 +27795,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27824,7 +27825,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27854,7 +27855,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27886,7 +27887,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27918,7 +27919,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27950,7 +27951,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27982,7 +27983,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -28014,7 +28015,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -28044,7 +28045,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -28076,7 +28077,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -28108,7 +28109,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28140,7 +28141,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28172,7 +28173,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28202,7 +28203,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28232,7 +28233,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28262,7 +28263,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28292,7 +28293,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28324,7 +28325,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28356,7 +28357,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28386,7 +28387,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28416,7 +28417,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28446,7 +28447,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28476,7 +28477,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28506,7 +28507,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28601,10 +28602,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28636,7 +28638,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28667,7 +28669,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28698,7 +28700,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28729,7 +28731,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28760,7 +28762,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28791,7 +28793,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28822,7 +28824,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28853,7 +28855,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28884,7 +28886,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28915,7 +28917,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28946,7 +28948,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28977,7 +28979,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -29008,7 +29010,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -29039,7 +29041,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29070,7 +29072,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29101,7 +29103,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29132,7 +29134,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29163,7 +29165,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29194,7 +29196,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29225,7 +29227,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29255,7 +29257,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29285,7 +29287,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29315,7 +29317,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29345,7 +29347,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29375,7 +29377,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29405,7 +29407,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29435,7 +29437,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29465,7 +29467,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29495,7 +29497,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29525,7 +29527,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29555,7 +29557,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29585,7 +29587,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29615,7 +29617,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29645,7 +29647,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29675,7 +29677,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29705,7 +29707,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29737,7 +29739,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29769,7 +29771,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29799,7 +29801,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29829,7 +29831,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29859,7 +29861,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29889,7 +29891,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29919,7 +29921,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51662,19 +51664,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51688,7 +51690,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51700,7 +51702,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51711,7 +51713,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51722,7 +51724,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51733,13 +51735,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-06T22:10:46Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16308,7 +16308,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21418,7 +21418,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21432,7 +21432,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21454,7 +21454,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21502,7 +21502,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21520,7 +21520,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21567,7 +21567,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21584,7 +21584,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21634,7 +21634,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21651,7 +21651,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21694,7 +21694,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21711,7 +21711,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21758,7 +21758,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21775,7 +21775,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21842,7 +21842,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21889,7 +21889,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21906,7 +21906,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21951,7 +21951,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21968,7 +21968,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -22018,7 +22018,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -22035,7 +22035,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22074,7 +22074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22091,7 +22091,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22132,7 +22132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22149,7 +22149,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22188,7 +22188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22205,7 +22205,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22250,7 +22250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22267,7 +22267,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22310,7 +22310,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22327,7 +22327,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22370,7 +22370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22387,7 +22387,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22434,7 +22434,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22451,7 +22451,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22496,7 +22496,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22513,7 +22513,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22556,7 +22556,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22573,7 +22573,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22614,7 +22614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22631,7 +22631,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22676,7 +22676,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22693,7 +22693,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22736,7 +22736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22753,7 +22753,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22790,7 +22790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22807,7 +22807,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22848,7 +22848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22865,7 +22865,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22908,7 +22908,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22925,7 +22925,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22967,7 +22967,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22984,7 +22984,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -23029,7 +23029,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -23046,7 +23046,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23091,7 +23091,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23108,7 +23108,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23153,7 +23153,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23170,7 +23170,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23207,7 +23207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23224,7 +23224,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23241,7 +23241,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23258,7 +23258,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23279,7 +23279,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23296,7 +23296,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23337,7 +23337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23354,7 +23354,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23399,7 +23399,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23416,7 +23416,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23433,7 +23433,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23468,7 +23468,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23851,7 +23851,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23862,7 +23862,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23883,7 +23883,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23945,7 +23945,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -24003,7 +24003,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -24037,7 +24037,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -24056,7 +24056,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24090,7 +24090,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24109,7 +24109,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24143,7 +24143,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24162,7 +24162,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24200,7 +24200,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24219,7 +24219,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24257,7 +24257,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24276,7 +24276,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24314,7 +24314,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24333,7 +24333,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24366,7 +24366,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24385,7 +24385,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24418,7 +24418,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24437,7 +24437,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24468,7 +24468,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24487,7 +24487,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24522,7 +24522,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24541,7 +24541,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24574,7 +24574,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24593,7 +24593,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24624,7 +24624,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24643,7 +24643,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24675,7 +24675,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24694,7 +24694,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24730,7 +24730,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24749,7 +24749,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24778,7 +24778,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24797,7 +24797,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24828,7 +24828,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24847,7 +24847,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24880,7 +24880,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24899,7 +24899,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24935,7 +24935,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24954,7 +24954,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24989,7 +24989,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -25008,7 +25008,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25038,7 +25038,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -25057,7 +25057,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25097,7 +25097,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25116,7 +25116,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25145,7 +25145,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25164,7 +25164,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25197,7 +25197,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25216,7 +25216,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25249,7 +25249,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25268,7 +25268,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25304,7 +25304,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25323,7 +25323,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25359,7 +25359,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25378,7 +25378,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25412,7 +25412,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25431,7 +25431,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25466,7 +25466,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25485,7 +25485,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25504,7 +25504,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25523,7 +25523,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25544,7 +25544,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25563,7 +25563,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25596,7 +25596,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25615,7 +25615,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25654,7 +25654,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25673,7 +25673,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25692,7 +25692,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25711,7 +25711,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25756,7 +25756,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25795,7 +25795,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25824,7 +25824,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25869,7 +25869,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25914,7 +25914,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25933,7 +25933,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25980,7 +25980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -26025,7 +26025,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -26044,7 +26044,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -26067,7 +26067,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -26090,7 +26090,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -26113,7 +26113,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26136,7 +26136,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26159,7 +26159,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26182,7 +26182,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26205,7 +26205,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26228,7 +26228,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26251,7 +26251,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26274,7 +26274,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26297,7 +26297,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26320,7 +26320,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26341,7 +26341,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26362,7 +26362,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26383,7 +26383,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26404,7 +26404,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26425,7 +26425,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26446,7 +26446,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26467,7 +26467,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26490,7 +26490,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26513,7 +26513,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26536,7 +26536,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26559,7 +26559,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26582,7 +26582,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26605,7 +26605,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26628,7 +26628,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26647,7 +26647,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26666,7 +26666,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26685,7 +26685,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26704,7 +26704,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26778,11 +26778,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26814,7 +26813,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26847,7 +26846,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26880,7 +26879,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26913,7 +26912,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26946,7 +26945,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26979,7 +26978,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -27012,7 +27011,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -27045,7 +27044,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27076,7 +27075,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27107,7 +27106,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27140,7 +27139,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27173,7 +27172,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27206,7 +27205,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27239,7 +27238,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27272,7 +27271,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27305,7 +27304,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27338,7 +27337,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27371,7 +27370,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27404,7 +27403,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27437,7 +27436,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27470,7 +27469,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27503,7 +27502,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27536,7 +27535,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27569,7 +27568,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27602,7 +27601,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27635,7 +27634,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27667,7 +27666,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27699,7 +27698,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27731,7 +27730,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27763,7 +27762,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27795,7 +27794,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27825,7 +27824,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27855,7 +27854,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27887,7 +27886,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27919,7 +27918,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27951,7 +27950,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27983,7 +27982,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -28015,7 +28014,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -28045,7 +28044,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -28077,7 +28076,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -28109,7 +28108,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28141,7 +28140,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28173,7 +28172,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28203,7 +28202,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28233,7 +28232,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28263,7 +28262,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28293,7 +28292,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28325,7 +28324,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28357,7 +28356,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28387,7 +28386,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28417,7 +28416,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28447,7 +28446,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28477,7 +28476,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28507,7 +28506,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28602,11 +28601,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28638,7 +28636,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28669,7 +28667,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28700,7 +28698,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28731,7 +28729,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28762,7 +28760,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28793,7 +28791,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28824,7 +28822,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28855,7 +28853,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28886,7 +28884,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28917,7 +28915,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28948,7 +28946,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28979,7 +28977,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -29010,7 +29008,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -29041,7 +29039,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29072,7 +29070,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29103,7 +29101,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29134,7 +29132,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29165,7 +29163,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29196,7 +29194,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29227,7 +29225,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29257,7 +29255,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29287,7 +29285,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29317,7 +29315,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29347,7 +29345,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29377,7 +29375,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29407,7 +29405,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29437,7 +29435,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29467,7 +29465,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29497,7 +29495,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29527,7 +29525,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29557,7 +29555,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29587,7 +29585,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29617,7 +29615,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29647,7 +29645,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29677,7 +29675,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29707,7 +29705,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29739,7 +29737,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29771,7 +29769,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29801,7 +29799,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29831,7 +29829,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29861,7 +29859,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29891,7 +29889,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29921,7 +29919,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51664,19 +51662,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51690,7 +51688,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51702,7 +51700,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51713,7 +51711,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51724,7 +51722,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51735,13 +51733,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-07T20:10:37Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -6835,13 +6835,13 @@
         <v>27</v>
       </c>
       <c r="K32" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L32" s="13" t="s">
         <v>27</v>
       </c>
       <c r="M32" s="13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N32" s="14" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-07T20:48:49Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9780,30 +9780,74 @@
       <c r="C5" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="52"/>
-      <c r="L5" s="52"/>
-      <c r="M5" s="53"/>
+      <c r="D5" s="52">
+        <v>245679.5</v>
+      </c>
+      <c r="E5" s="52">
+        <v>216530.08</v>
+      </c>
+      <c r="F5" s="52">
+        <v>29149.420000000013</v>
+      </c>
+      <c r="G5" s="53">
+        <v>0.11864815745717495</v>
+      </c>
+      <c r="H5" s="52">
+        <v>208360.5</v>
+      </c>
+      <c r="I5" s="52">
+        <v>168361.6</v>
+      </c>
+      <c r="J5" s="52">
+        <v>180366.49</v>
+      </c>
+      <c r="K5" s="52">
+        <v>138438.46000000002</v>
+      </c>
+      <c r="L5" s="52">
+        <v>41928.02999999997</v>
+      </c>
+      <c r="M5" s="53">
+        <v>0.23246019812216767</v>
+      </c>
       <c r="N5" s="53"/>
-      <c r="O5" s="52"/>
-      <c r="P5" s="52"/>
-      <c r="Q5" s="52"/>
-      <c r="R5" s="53"/>
-      <c r="S5" s="54"/>
-      <c r="T5" s="54"/>
-      <c r="U5" s="54"/>
-      <c r="V5" s="53"/>
+      <c r="O5" s="52">
+        <v>27994.01</v>
+      </c>
+      <c r="P5" s="52">
+        <v>29923.14</v>
+      </c>
+      <c r="Q5" s="52">
+        <v>-1929.130000000001</v>
+      </c>
+      <c r="R5" s="53">
+        <v>-0.06891224229754869</v>
+      </c>
+      <c r="S5" s="54">
+        <v>565.45</v>
+      </c>
+      <c r="T5" s="54">
+        <v>600.25</v>
+      </c>
+      <c r="U5" s="54">
+        <v>-34.799999999999955</v>
+      </c>
+      <c r="V5" s="53">
+        <v>-0.061543903086037584</v>
+      </c>
       <c r="W5" s="53"/>
-      <c r="X5" s="55"/>
-      <c r="Y5" s="55"/>
-      <c r="Z5" s="53"/>
-      <c r="AA5" s="56"/>
+      <c r="X5" s="55">
+        <v>80.24736359850063</v>
+      </c>
+      <c r="Y5" s="55">
+        <v>65.99877634098505</v>
+      </c>
+      <c r="Z5" s="53">
+        <v>0.2225</v>
+      </c>
+      <c r="AA5" s="56">
+        <v>0.1519</v>
+      </c>
       <c r="AB5" s="57"/>
       <c r="AD5" s="35" t="s">
         <v>95</v>
@@ -10115,54 +10159,54 @@
         <v>101420.72</v>
       </c>
       <c r="I12" s="52">
-        <v>76488.35</v>
+        <v>79791.03</v>
       </c>
       <c r="J12" s="52">
         <v>83645.65</v>
       </c>
       <c r="K12" s="52">
-        <v>70758.46</v>
+        <v>71604.5</v>
       </c>
       <c r="L12" s="52">
-        <v>12887.189999999988</v>
+        <v>12041.149999999994</v>
       </c>
       <c r="M12" s="53">
-        <v>0.1540688607237793</v>
+        <v>0.1439542881189876</v>
       </c>
       <c r="N12" s="53"/>
       <c r="O12" s="52">
         <v>17775.07</v>
       </c>
       <c r="P12" s="52">
-        <v>5729.89</v>
+        <v>8186.53</v>
       </c>
       <c r="Q12" s="52">
-        <v>12045.18</v>
+        <v>9588.54</v>
       </c>
       <c r="R12" s="53">
-        <v>0.6776445887414227</v>
+        <v>0.5394375380800188</v>
       </c>
       <c r="S12" s="54">
         <v>356.07</v>
       </c>
       <c r="T12" s="54">
-        <v>117.75</v>
+        <v>168.25</v>
       </c>
       <c r="U12" s="54">
-        <v>238.32</v>
+        <v>187.82</v>
       </c>
       <c r="V12" s="53">
-        <v>0.6693065970174403</v>
+        <v>0.5274805515769371</v>
       </c>
       <c r="W12" s="53"/>
       <c r="X12" s="55">
-        <v>79.624033970276</v>
+        <v>36.09539375928678</v>
       </c>
       <c r="Y12" s="55">
         <v>77.66490997775718</v>
       </c>
       <c r="Z12" s="53">
-        <v>0.1092</v>
+        <v>0.0707</v>
       </c>
       <c r="AA12" s="56">
         <v>0.2142</v>
@@ -10843,54 +10887,54 @@
         <v>102178.42</v>
       </c>
       <c r="I26" s="52">
-        <v>87101.11</v>
+        <v>89222.05</v>
       </c>
       <c r="J26" s="52">
         <v>62464.86</v>
       </c>
       <c r="K26" s="52">
-        <v>57898.75</v>
+        <v>58984</v>
       </c>
       <c r="L26" s="52">
-        <v>4566.110000000001</v>
+        <v>3480.8600000000006</v>
       </c>
       <c r="M26" s="53">
-        <v>0.07309885910254182</v>
+        <v>0.05572509087509362</v>
       </c>
       <c r="N26" s="53"/>
       <c r="O26" s="52">
         <v>39713.56</v>
       </c>
       <c r="P26" s="52">
-        <v>29202.36</v>
+        <v>30238.05</v>
       </c>
       <c r="Q26" s="52">
-        <v>10511.199999999997</v>
+        <v>9475.509999999998</v>
       </c>
       <c r="R26" s="53">
-        <v>0.26467534011053145</v>
+        <v>0.23859633837913294</v>
       </c>
       <c r="S26" s="54">
         <v>795.22</v>
       </c>
       <c r="T26" s="54">
-        <v>594.5</v>
+        <v>615</v>
       </c>
       <c r="U26" s="54">
-        <v>200.72000000000003</v>
+        <v>180.22000000000003</v>
       </c>
       <c r="V26" s="53">
-        <v>0.25240813862830414</v>
+        <v>0.22662910892583188</v>
       </c>
       <c r="W26" s="53"/>
       <c r="X26" s="55">
-        <v>96.3325315391085</v>
+        <v>89.67276422764228</v>
       </c>
       <c r="Y26" s="55">
         <v>61.20621468124544</v>
       </c>
       <c r="Z26" s="53">
-        <v>0.3967</v>
+        <v>0.382</v>
       </c>
       <c r="AA26" s="56">
         <v>0.3227</v>
@@ -11206,54 +11250,54 @@
         <v>327431.12</v>
       </c>
       <c r="I33" s="65">
-        <v>220187.84</v>
+        <v>223659.54</v>
       </c>
       <c r="J33" s="52">
         <v>271519.78</v>
       </c>
       <c r="K33" s="52">
-        <v>196879.33</v>
+        <v>197370.72</v>
       </c>
       <c r="L33" s="52">
-        <v>74640.45000000004</v>
+        <v>74149.06000000003</v>
       </c>
       <c r="M33" s="53">
-        <v>0.27489875691561044</v>
+        <v>0.27308898084699396</v>
       </c>
       <c r="N33" s="53"/>
       <c r="O33" s="52">
         <v>55911.34</v>
       </c>
       <c r="P33" s="52">
-        <v>23308.51</v>
+        <v>26288.82</v>
       </c>
       <c r="Q33" s="52">
-        <v>32602.829999999998</v>
+        <v>29622.519999999997</v>
       </c>
       <c r="R33" s="53">
-        <v>0.5831165913748445</v>
+        <v>0.5298123779540966</v>
       </c>
       <c r="S33" s="54">
         <v>1120.27</v>
       </c>
       <c r="T33" s="54">
-        <v>543.5</v>
+        <v>607.75</v>
       </c>
       <c r="U33" s="54">
-        <v>576.77</v>
+        <v>512.52</v>
       </c>
       <c r="V33" s="53">
-        <v>0.514849098877949</v>
+        <v>0.4574968534371178</v>
       </c>
       <c r="W33" s="53"/>
       <c r="X33" s="55">
-        <v>72.05127874885005</v>
+        <v>58.721793500617025</v>
       </c>
       <c r="Y33" s="55">
         <v>61.5841822414239</v>
       </c>
       <c r="Z33" s="53">
-        <v>0.151</v>
+        <v>0.1376</v>
       </c>
       <c r="AA33" s="56">
         <v>0.174</v>
@@ -11569,54 +11613,54 @@
         <v>94098.32</v>
       </c>
       <c r="I40" s="52">
-        <v>46289.42</v>
+        <v>49261.61</v>
       </c>
       <c r="J40" s="52">
         <v>69042.09000000001</v>
       </c>
       <c r="K40" s="52">
-        <v>35507.08</v>
+        <v>35683.74</v>
       </c>
       <c r="L40" s="52">
-        <v>33535.01000000001</v>
+        <v>33358.35000000001</v>
       </c>
       <c r="M40" s="53">
-        <v>0.4857183494879718</v>
+        <v>0.4831596204576079</v>
       </c>
       <c r="N40" s="53"/>
       <c r="O40" s="52">
         <v>25056.23</v>
       </c>
       <c r="P40" s="52">
-        <v>10782.34</v>
+        <v>13577.87</v>
       </c>
       <c r="Q40" s="52">
-        <v>14273.89</v>
+        <v>11478.359999999999</v>
       </c>
       <c r="R40" s="53">
-        <v>0.5696742885901032</v>
+        <v>0.45810403241030273</v>
       </c>
       <c r="S40" s="54">
         <v>501.83</v>
       </c>
       <c r="T40" s="54">
-        <v>232.25</v>
+        <v>299.5</v>
       </c>
       <c r="U40" s="54">
-        <v>269.58</v>
+        <v>202.32999999999998</v>
       </c>
       <c r="V40" s="53">
-        <v>0.5371938704342107</v>
+        <v>0.40318434529621583</v>
       </c>
       <c r="W40" s="53"/>
       <c r="X40" s="55">
-        <v>32.96193756727664</v>
+        <v>15.63679465776294</v>
       </c>
       <c r="Y40" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z40" s="53">
-        <v>0.1419</v>
+        <v>0.0868</v>
       </c>
       <c r="AA40" s="56">
         <v>0.2663</v>
@@ -11934,54 +11978,54 @@
         <v>50582.37</v>
       </c>
       <c r="I47" s="52">
-        <v>25187.36</v>
+        <v>25196.36</v>
       </c>
       <c r="J47" s="52">
         <v>39438.990000000005</v>
       </c>
       <c r="K47" s="52">
-        <v>20432.420000000002</v>
+        <v>20036.420000000002</v>
       </c>
       <c r="L47" s="52">
-        <v>19006.570000000003</v>
+        <v>19402.570000000003</v>
       </c>
       <c r="M47" s="53">
-        <v>0.48192334540007237</v>
+        <v>0.49196417048205343</v>
       </c>
       <c r="N47" s="53"/>
       <c r="O47" s="52">
         <v>11143.38</v>
       </c>
       <c r="P47" s="52">
-        <v>4754.94</v>
+        <v>5159.94</v>
       </c>
       <c r="Q47" s="52">
-        <v>6388.44</v>
+        <v>5983.44</v>
       </c>
       <c r="R47" s="53">
-        <v>0.5732946377131535</v>
+        <v>0.5369501892603501</v>
       </c>
       <c r="S47" s="54">
         <v>223.22</v>
       </c>
       <c r="T47" s="54">
-        <v>104.25</v>
+        <v>113.25</v>
       </c>
       <c r="U47" s="54">
-        <v>118.97</v>
+        <v>109.97</v>
       </c>
       <c r="V47" s="53">
-        <v>0.5329719559179285</v>
+        <v>0.49265298808350505</v>
       </c>
       <c r="W47" s="53"/>
       <c r="X47" s="55">
-        <v>78.07318944844125</v>
+        <v>71.78922737306843</v>
       </c>
       <c r="Y47" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z47" s="53">
-        <v>0.24420000000000003</v>
+        <v>0.244</v>
       </c>
       <c r="AA47" s="56">
         <v>0.23</v>
@@ -12297,54 +12341,54 @@
         <v>109364.97</v>
       </c>
       <c r="I54" s="52">
-        <v>95597.19</v>
+        <v>96483.38</v>
       </c>
       <c r="J54" s="52">
         <v>75135.01000000001</v>
       </c>
       <c r="K54" s="52">
-        <v>71143.79000000001</v>
+        <v>71221.34</v>
       </c>
       <c r="L54" s="52">
-        <v>3991.220000000001</v>
+        <v>3913.670000000013</v>
       </c>
       <c r="M54" s="53">
-        <v>0.05312064242754477</v>
+        <v>0.05208850042077604</v>
       </c>
       <c r="N54" s="53"/>
       <c r="O54" s="52">
         <v>34229.96</v>
       </c>
       <c r="P54" s="52">
-        <v>24453.4</v>
+        <v>25262.04</v>
       </c>
       <c r="Q54" s="52">
-        <v>9776.559999999998</v>
+        <v>8967.919999999998</v>
       </c>
       <c r="R54" s="53">
-        <v>0.28561412283274645</v>
+        <v>0.2619903733454552</v>
       </c>
       <c r="S54" s="54">
         <v>685.48</v>
       </c>
       <c r="T54" s="54">
-        <v>517.75</v>
+        <v>533.75</v>
       </c>
       <c r="U54" s="54">
-        <v>167.73000000000002</v>
+        <v>151.73000000000002</v>
       </c>
       <c r="V54" s="53">
-        <v>0.24468985236622515</v>
+        <v>0.22134854408589605</v>
       </c>
       <c r="W54" s="53"/>
       <c r="X54" s="55">
-        <v>62.22557218734911</v>
+        <v>58.699953161592504</v>
       </c>
       <c r="Y54" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z54" s="53">
-        <v>0.2521</v>
+        <v>0.2451</v>
       </c>
       <c r="AA54" s="56">
         <v>0.2958</v>
@@ -13372,19 +13416,19 @@
         <v>54302.66</v>
       </c>
       <c r="I75" s="52">
-        <v>33447.19</v>
+        <v>29696.65</v>
       </c>
       <c r="J75" s="52">
         <v>31383.390000000003</v>
       </c>
       <c r="K75" s="52">
-        <v>27343.140000000003</v>
+        <v>23592.600000000002</v>
       </c>
       <c r="L75" s="52">
-        <v>4040.25</v>
+        <v>7790.790000000001</v>
       </c>
       <c r="M75" s="53">
-        <v>0.128738482362804</v>
+        <v>0.24824564841465502</v>
       </c>
       <c r="N75" s="53"/>
       <c r="O75" s="52">
@@ -13413,13 +13457,13 @@
       </c>
       <c r="W75" s="53"/>
       <c r="X75" s="55">
-        <v>94.11891891891891</v>
+        <v>125.30844074844074</v>
       </c>
       <c r="Y75" s="55">
         <v>48.58165977967362</v>
       </c>
       <c r="Z75" s="53">
-        <v>0.2528</v>
+        <v>0.33659999999999995</v>
       </c>
       <c r="AA75" s="56">
         <v>0.2963</v>
@@ -14092,54 +14136,54 @@
         <v>27002.93</v>
       </c>
       <c r="I89" s="52">
-        <v>24950.27</v>
+        <v>25060.53</v>
       </c>
       <c r="J89" s="52">
         <v>15440.32</v>
       </c>
       <c r="K89" s="52">
-        <v>13932.720000000001</v>
+        <v>13974.73</v>
       </c>
       <c r="L89" s="52">
-        <v>1507.5999999999985</v>
+        <v>1465.5900000000001</v>
       </c>
       <c r="M89" s="53">
-        <v>0.09764046341008467</v>
+        <v>0.09491966487741188</v>
       </c>
       <c r="N89" s="53"/>
       <c r="O89" s="52">
         <v>11562.61</v>
       </c>
       <c r="P89" s="52">
-        <v>11017.55</v>
+        <v>11085.8</v>
       </c>
       <c r="Q89" s="52">
-        <v>545.0600000000013</v>
+        <v>476.8100000000013</v>
       </c>
       <c r="R89" s="53">
-        <v>0.04713987585847843</v>
+        <v>0.041237229310683424</v>
       </c>
       <c r="S89" s="68">
         <v>231.75</v>
       </c>
       <c r="T89" s="68">
-        <v>224.25</v>
+        <v>225.5</v>
       </c>
       <c r="U89" s="54">
-        <v>7.5</v>
+        <v>6.25</v>
       </c>
       <c r="V89" s="53">
-        <v>0.032362459546925564</v>
+        <v>0.02696871628910464</v>
       </c>
       <c r="W89" s="53"/>
       <c r="X89" s="55">
-        <v>50.9746265328874</v>
+        <v>50.20310421286031</v>
       </c>
       <c r="Y89" s="55">
         <v>43.49557070636461</v>
       </c>
       <c r="Z89" s="53">
-        <v>0.31420000000000003</v>
+        <v>0.31120000000000003</v>
       </c>
       <c r="AA89" s="56">
         <v>0.2718</v>
@@ -21872,10 +21916,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="52">
-        <v>0</v>
+        <v>403.9200000000128</v>
       </c>
       <c r="E4" s="52">
-        <v>0</v>
+        <v>-403.9200000000128</v>
       </c>
       <c r="F4" s="52">
         <v>0</v>
@@ -21899,13 +21943,13 @@
         <v>0</v>
       </c>
       <c r="M4" s="52">
-        <v>-7000</v>
+        <v>-7403.920000000013</v>
       </c>
       <c r="N4" s="54">
         <v>20</v>
       </c>
       <c r="O4" s="58">
-        <v>-100</v>
+        <v>-105.77028571428589</v>
       </c>
     </row>
     <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21936,10 +21980,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>2351.029999999999</v>
+        <v>5653.709999999992</v>
       </c>
       <c r="E6" s="52">
-        <v>-2351.029999999999</v>
+        <v>-5653.709999999992</v>
       </c>
       <c r="F6" s="52">
         <v>0</v>
@@ -21963,13 +22007,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-4223.629999999999</v>
+        <v>-7526.309999999992</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>337.89039999999994</v>
+        <v>602.1047999999994</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>117</v>
@@ -22063,10 +22107,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="52">
-        <v>1252.699999999997</v>
+        <v>3373.6399999999994</v>
       </c>
       <c r="E10" s="52">
-        <v>-1252.699999999997</v>
+        <v>-3373.6399999999994</v>
       </c>
       <c r="F10" s="52">
         <v>0</v>
@@ -22090,13 +22134,13 @@
         <v>0</v>
       </c>
       <c r="M10" s="52">
-        <v>-6172.699999999997</v>
+        <v>-8293.64</v>
       </c>
       <c r="N10" s="54">
         <v>-388.25</v>
       </c>
       <c r="O10" s="58">
-        <v>18.141660543717848</v>
+        <v>24.375135929463628</v>
       </c>
     </row>
     <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22127,10 +22171,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>3843.2399999999907</v>
+        <v>7314.940000000002</v>
       </c>
       <c r="E12" s="52">
-        <v>-3843.2399999999907</v>
+        <v>-7314.940000000002</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
@@ -22154,13 +22198,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-6480.239999999991</v>
+        <v>-9951.940000000002</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-93.9165217391303</v>
+        <v>-144.23101449275364</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>119</v>
@@ -22194,10 +22238,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>4015.729999999996</v>
+        <v>6987.919999999998</v>
       </c>
       <c r="E14" s="52">
-        <v>-4015.729999999996</v>
+        <v>-6987.919999999998</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -22221,13 +22265,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-7015.729999999996</v>
+        <v>-9987.919999999998</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>62.640446428571394</v>
+        <v>89.17785714285712</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22258,10 +22302,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>-24.220000000001164</v>
+        <v>-15.220000000001164</v>
       </c>
       <c r="E16" s="52">
-        <v>24.220000000001164</v>
+        <v>15.220000000001164</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -22283,13 +22327,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-2975.779999999999</v>
+        <v>-2984.779999999999</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>34.302939481268</v>
+        <v>34.40668587896252</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22320,10 +22364,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>276.68000000000757</v>
+        <v>1162.87000000001</v>
       </c>
       <c r="E18" s="52">
-        <v>-276.68000000000757</v>
+        <v>-1162.87000000001</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -22347,13 +22391,13 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-8476.680000000008</v>
+        <v>-9362.87000000001</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>44.85015873015877</v>
+        <v>49.538994708994764</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>120</v>
@@ -22501,10 +22545,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>1528.260000000002</v>
+        <v>-2222.279999999999</v>
       </c>
       <c r="E24" s="52">
-        <v>-1528.260000000002</v>
+        <v>2222.279999999999</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -22522,7 +22566,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>-1525.260000000002</v>
+        <v>2225.279999999999</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -22619,10 +22663,10 @@
         <v>0</v>
       </c>
       <c r="D28" s="52">
-        <v>-1055.7200000000012</v>
+        <v>-945.4600000000028</v>
       </c>
       <c r="E28" s="52">
-        <v>1055.7200000000012</v>
+        <v>945.4600000000028</v>
       </c>
       <c r="F28" s="52">
         <v>0</v>
@@ -22642,13 +22686,13 @@
         <v>0</v>
       </c>
       <c r="M28" s="52">
-        <v>1055.7200000000012</v>
+        <v>945.4600000000028</v>
       </c>
       <c r="N28" s="54">
         <v>-148.5</v>
       </c>
       <c r="O28" s="58">
-        <v>-7.109225589225597</v>
+        <v>-6.366734006734025</v>
       </c>
     </row>
     <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23820,22 +23864,22 @@
         <v>88818.76999999996</v>
       </c>
       <c r="D70" s="104">
-        <v>29887.739999999983</v>
+        <v>39414.08000000001</v>
       </c>
       <c r="E70" s="105">
-        <v>58931.02999999998</v>
+        <v>49404.68999999996</v>
       </c>
       <c r="F70" s="106" t="s">
         <v>124</v>
       </c>
       <c r="G70" s="107">
-        <v>0.6634974791927427</v>
+        <v>0.5562415466910877</v>
       </c>
       <c r="H70" s="108" t="s">
         <v>125</v>
       </c>
       <c r="I70" s="109">
-        <v>0.0799203816940944</v>
+        <v>-0.02733555080756062</v>
       </c>
       <c r="J70" s="36"/>
       <c r="K70" s="36"/>
@@ -24390,10 +24434,10 @@
         <v>565.45</v>
       </c>
       <c r="D4" s="54">
-        <v>588.25</v>
+        <v>600.25</v>
       </c>
       <c r="E4" s="54">
-        <v>-22.799999999999955</v>
+        <v>-34.799999999999955</v>
       </c>
       <c r="F4" s="54">
         <v>0</v>
@@ -24445,10 +24489,10 @@
         <v>356.07</v>
       </c>
       <c r="D6" s="54">
-        <v>117.75</v>
+        <v>168.25</v>
       </c>
       <c r="E6" s="54">
-        <v>238.32</v>
+        <v>187.82</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -24551,10 +24595,10 @@
         <v>795.22</v>
       </c>
       <c r="D10" s="54">
-        <v>594.5</v>
+        <v>615</v>
       </c>
       <c r="E10" s="54">
-        <v>200.72000000000003</v>
+        <v>180.22000000000003</v>
       </c>
       <c r="F10" s="54"/>
       <c r="G10" s="54"/>
@@ -24608,10 +24652,10 @@
         <v>1120.27</v>
       </c>
       <c r="D12" s="54">
-        <v>543.5</v>
+        <v>607.75</v>
       </c>
       <c r="E12" s="54">
-        <v>576.77</v>
+        <v>512.52</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -24665,10 +24709,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>232.25</v>
+        <v>299.5</v>
       </c>
       <c r="E14" s="54">
-        <v>269.58</v>
+        <v>202.32999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -24722,10 +24766,10 @@
         <v>223.22</v>
       </c>
       <c r="D16" s="54">
-        <v>104.25</v>
+        <v>113.25</v>
       </c>
       <c r="E16" s="54">
-        <v>118.97</v>
+        <v>109.97</v>
       </c>
       <c r="F16" s="54"/>
       <c r="G16" s="54"/>
@@ -24774,10 +24818,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>517.75</v>
+        <v>533.75</v>
       </c>
       <c r="E18" s="54">
-        <v>167.73000000000002</v>
+        <v>151.73000000000002</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -25032,10 +25076,10 @@
         <v>231.75</v>
       </c>
       <c r="D28" s="54">
-        <v>224.25</v>
+        <v>225.5</v>
       </c>
       <c r="E28" s="54">
-        <v>7.5</v>
+        <v>6.25</v>
       </c>
       <c r="F28" s="54"/>
       <c r="G28" s="54"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-07T20:56:37Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16396,7 +16396,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -18764,30 +18764,74 @@
       <c r="C180" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D180" s="52"/>
-      <c r="E180" s="52"/>
-      <c r="F180" s="52"/>
-      <c r="G180" s="53"/>
-      <c r="H180" s="52"/>
-      <c r="I180" s="52"/>
-      <c r="J180" s="52"/>
-      <c r="K180" s="52"/>
-      <c r="L180" s="52"/>
-      <c r="M180" s="53"/>
+      <c r="D180" s="52">
+        <v>16897.53</v>
+      </c>
+      <c r="E180" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F180" s="52">
+        <v>11405.829999999998</v>
+      </c>
+      <c r="G180" s="53">
+        <v>0.6749998372543206</v>
+      </c>
+      <c r="H180" s="52">
+        <v>9226.27</v>
+      </c>
+      <c r="I180" s="52">
+        <v>3702.78</v>
+      </c>
+      <c r="J180" s="52">
+        <v>2977.1100000000006</v>
+      </c>
+      <c r="K180" s="52">
+        <v>2335.9700000000003</v>
+      </c>
+      <c r="L180" s="52">
+        <v>641.1400000000003</v>
+      </c>
+      <c r="M180" s="53">
+        <v>0.2153565034546927</v>
+      </c>
       <c r="N180" s="53"/>
-      <c r="O180" s="52"/>
-      <c r="P180" s="52"/>
-      <c r="Q180" s="52"/>
-      <c r="R180" s="53"/>
-      <c r="S180" s="54"/>
-      <c r="T180" s="54"/>
-      <c r="U180" s="54"/>
-      <c r="V180" s="53"/>
+      <c r="O180" s="52">
+        <v>6249.16</v>
+      </c>
+      <c r="P180" s="52">
+        <v>1366.81</v>
+      </c>
+      <c r="Q180" s="52">
+        <v>4882.35</v>
+      </c>
+      <c r="R180" s="53">
+        <v>0.7812810041669601</v>
+      </c>
+      <c r="S180" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T180" s="54">
+        <v>23.75</v>
+      </c>
+      <c r="U180" s="54">
+        <v>101.42</v>
+      </c>
+      <c r="V180" s="53">
+        <v>0.8102580490532876</v>
+      </c>
       <c r="W180" s="53"/>
-      <c r="X180" s="55"/>
-      <c r="Y180" s="55"/>
-      <c r="Z180" s="53"/>
-      <c r="AA180" s="56"/>
+      <c r="X180" s="55">
+        <v>75.32294736842105</v>
+      </c>
+      <c r="Y180" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z180" s="53">
+        <v>0.3257</v>
+      </c>
+      <c r="AA180" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB180" s="57"/>
       <c r="AD180" s="35" t="s">
         <v>95</v>
@@ -21061,30 +21105,74 @@
       <c r="C229" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D229" s="52"/>
-      <c r="E229" s="52"/>
-      <c r="F229" s="52"/>
-      <c r="G229" s="53"/>
-      <c r="H229" s="52"/>
-      <c r="I229" s="52"/>
-      <c r="J229" s="52"/>
-      <c r="K229" s="52"/>
-      <c r="L229" s="52"/>
-      <c r="M229" s="53"/>
+      <c r="D229" s="52">
+        <v>8795.03</v>
+      </c>
+      <c r="E229" s="52">
+        <v>0</v>
+      </c>
+      <c r="F229" s="52">
+        <v>8795.03</v>
+      </c>
+      <c r="G229" s="53">
+        <v>1</v>
+      </c>
+      <c r="H229" s="52">
+        <v>6369.12</v>
+      </c>
+      <c r="I229" s="52">
+        <v>0</v>
+      </c>
+      <c r="J229" s="52">
+        <v>4527.889999999999</v>
+      </c>
+      <c r="K229" s="52">
+        <v>0</v>
+      </c>
+      <c r="L229" s="52">
+        <v>4527.889999999999</v>
+      </c>
+      <c r="M229" s="53">
+        <v>1</v>
+      </c>
       <c r="N229" s="53"/>
-      <c r="O229" s="52"/>
-      <c r="P229" s="52"/>
-      <c r="Q229" s="52"/>
-      <c r="R229" s="53"/>
-      <c r="S229" s="54"/>
-      <c r="T229" s="54"/>
-      <c r="U229" s="54"/>
-      <c r="V229" s="53"/>
+      <c r="O229" s="52">
+        <v>1841.23</v>
+      </c>
+      <c r="P229" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q229" s="52">
+        <v>1841.23</v>
+      </c>
+      <c r="R229" s="53">
+        <v>1</v>
+      </c>
+      <c r="S229" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="T229" s="54">
+        <v>0</v>
+      </c>
+      <c r="U229" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="V229" s="53">
+        <v>1</v>
+      </c>
       <c r="W229" s="53"/>
-      <c r="X229" s="55"/>
-      <c r="Y229" s="55"/>
-      <c r="Z229" s="53"/>
-      <c r="AA229" s="56"/>
+      <c r="X229" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y229" s="55">
+        <v>65.70711175027087</v>
+      </c>
+      <c r="Z229" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA229" s="56">
+        <v>0.2758</v>
+      </c>
       <c r="AB229" s="57"/>
       <c r="AD229" s="35"/>
       <c r="AE229" s="36"/>
@@ -21803,7 +21891,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:AD71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21817,7 +21905,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21839,7 +21927,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -21887,7 +21975,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21905,7 +21993,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21952,7 +22040,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21969,7 +22057,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -22019,7 +22107,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -22036,7 +22124,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -22079,7 +22167,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -22096,7 +22184,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -22143,7 +22231,7 @@
         <v>24.375135929463628</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -22160,7 +22248,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -22210,7 +22298,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -22227,7 +22315,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -22274,7 +22362,7 @@
         <v>89.17785714285712</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -22291,7 +22379,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -22336,7 +22424,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -22353,7 +22441,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -22403,7 +22491,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -22420,7 +22508,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22459,7 +22547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22476,7 +22564,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22517,7 +22605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22534,7 +22622,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22573,7 +22661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22590,7 +22678,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22635,7 +22723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22652,7 +22740,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22695,7 +22783,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22712,7 +22800,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22755,7 +22843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22772,7 +22860,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22819,7 +22907,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22836,7 +22924,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22881,7 +22969,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22898,7 +22986,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22941,7 +23029,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22958,7 +23046,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22999,7 +23087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -23016,7 +23104,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -23061,7 +23149,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -23078,7 +23166,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -23121,7 +23209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -23138,7 +23226,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -23175,7 +23263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -23192,7 +23280,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -23233,7 +23321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -23250,7 +23338,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -23293,7 +23381,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -23310,7 +23398,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -23352,7 +23440,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -23369,7 +23457,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -23414,7 +23502,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -23431,7 +23519,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23476,7 +23564,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23493,7 +23581,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23538,7 +23626,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23555,7 +23643,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23592,7 +23680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23609,7 +23697,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23626,7 +23714,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23643,7 +23731,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23664,7 +23752,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23681,7 +23769,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23722,7 +23810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23739,7 +23827,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23784,7 +23872,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -23819,7 +23907,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23836,7 +23924,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -23853,7 +23941,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -23888,7 +23976,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -24271,7 +24359,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB110"/>
+  <dimension ref="A1:AD110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -24282,7 +24370,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -24303,7 +24391,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -24365,7 +24453,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -24423,7 +24511,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -24459,7 +24547,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -24478,7 +24566,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24512,7 +24600,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24531,7 +24619,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24565,7 +24653,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24584,7 +24672,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24622,7 +24710,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24641,7 +24729,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24679,7 +24767,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24698,7 +24786,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24736,7 +24824,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24755,7 +24843,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24788,7 +24876,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24807,7 +24895,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24840,7 +24928,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24859,7 +24947,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24890,7 +24978,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24909,7 +24997,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24944,7 +25032,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24963,7 +25051,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24996,7 +25084,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -25015,7 +25103,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25046,7 +25134,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -25065,7 +25153,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25097,7 +25185,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -25116,7 +25204,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25152,7 +25240,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -25171,7 +25259,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25200,7 +25288,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -25219,7 +25307,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25250,7 +25338,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -25269,7 +25357,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25302,7 +25390,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -25321,7 +25409,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25357,7 +25445,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -25376,7 +25464,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25411,7 +25499,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -25430,7 +25518,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25460,7 +25548,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -25479,7 +25567,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25519,7 +25607,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25538,7 +25626,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25567,7 +25655,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25586,7 +25674,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25619,7 +25707,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25638,7 +25726,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25671,7 +25759,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25690,7 +25778,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25726,7 +25814,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25745,7 +25833,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25781,7 +25869,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25800,7 +25888,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25834,7 +25922,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25853,7 +25941,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25888,7 +25976,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25907,7 +25995,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25926,7 +26014,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25945,7 +26033,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25966,7 +26054,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25985,7 +26073,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -26018,7 +26106,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -26037,7 +26125,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -26076,7 +26164,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -26105,7 +26193,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -26124,7 +26212,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -26143,7 +26231,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -26162,7 +26250,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -26207,7 +26295,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -26246,7 +26334,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -26275,7 +26363,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -26320,7 +26408,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -26365,7 +26453,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -26384,7 +26472,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -26431,7 +26519,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -26476,7 +26564,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -26495,7 +26583,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -26518,7 +26606,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -26541,7 +26629,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -26564,7 +26652,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -26587,7 +26675,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -26610,7 +26698,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -26633,7 +26721,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -26656,7 +26744,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -26679,7 +26767,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -26702,7 +26790,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -26725,7 +26813,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -26748,7 +26836,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -26771,7 +26859,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26792,7 +26880,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26813,7 +26901,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26834,7 +26922,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26855,7 +26943,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26876,7 +26964,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26897,7 +26985,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -26918,7 +27006,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -26941,7 +27029,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -26964,7 +27052,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -26987,7 +27075,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -27010,7 +27098,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -27033,7 +27121,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -27056,7 +27144,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -27079,7 +27167,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -27098,7 +27186,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -27117,7 +27205,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -27136,7 +27224,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -27155,7 +27243,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -27229,10 +27317,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -27264,7 +27353,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -27297,7 +27386,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -27330,7 +27419,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -27363,7 +27452,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -27396,7 +27485,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -27429,7 +27518,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -27462,7 +27551,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -27495,7 +27584,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27526,7 +27615,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27557,7 +27646,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -27590,7 +27679,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -27623,7 +27712,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -27656,7 +27745,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -27689,7 +27778,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -27722,7 +27811,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -27755,7 +27844,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -27788,7 +27877,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -27821,7 +27910,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -27854,7 +27943,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -27887,7 +27976,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -27920,7 +28009,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -27953,7 +28042,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -27986,7 +28075,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -28019,7 +28108,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -28052,7 +28141,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -28085,7 +28174,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -28117,7 +28206,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -28149,7 +28238,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -28181,7 +28270,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -28213,7 +28302,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -28245,7 +28334,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -28275,7 +28364,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -28305,7 +28394,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -28337,7 +28426,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -28369,7 +28458,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -28401,7 +28490,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -28433,7 +28522,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -28465,7 +28554,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -28495,7 +28584,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -28527,7 +28616,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -28559,7 +28648,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -28591,7 +28680,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -28623,7 +28712,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28653,7 +28742,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28683,7 +28772,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28713,7 +28802,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28743,7 +28832,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -28775,7 +28864,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -28807,7 +28896,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28837,7 +28926,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28867,7 +28956,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28897,7 +28986,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28927,7 +29016,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28957,7 +29046,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -29052,10 +29141,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -29087,7 +29177,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -29118,7 +29208,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -29149,7 +29239,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -29180,7 +29270,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -29211,7 +29301,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -29242,7 +29332,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -29273,7 +29363,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -29304,7 +29394,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -29335,7 +29425,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -29366,7 +29456,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -29397,7 +29487,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -29428,7 +29518,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -29459,7 +29549,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -29490,7 +29580,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29521,7 +29611,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29552,7 +29642,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29583,7 +29673,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29614,7 +29704,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29645,7 +29735,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29676,7 +29766,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29706,7 +29796,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29736,7 +29826,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29766,7 +29856,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29796,7 +29886,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29826,7 +29916,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29856,7 +29946,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29886,7 +29976,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29916,7 +30006,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29946,7 +30036,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29976,7 +30066,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -30006,7 +30096,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -30036,7 +30126,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -30066,7 +30156,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -30096,7 +30186,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -30126,7 +30216,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -30156,7 +30246,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -30188,7 +30278,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -30220,7 +30310,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -30250,7 +30340,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -30280,7 +30370,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -30310,7 +30400,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -30340,7 +30430,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -30370,7 +30460,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -52113,19 +52203,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -52139,7 +52229,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -52151,7 +52241,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -52162,7 +52252,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -52173,7 +52263,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -52184,13 +52274,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-07T21:12:10Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9864,30 +9864,74 @@
       <c r="C6" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="52"/>
-      <c r="L6" s="52"/>
-      <c r="M6" s="53"/>
+      <c r="D6" s="52">
+        <v>245679.5</v>
+      </c>
+      <c r="E6" s="52">
+        <v>216530.08</v>
+      </c>
+      <c r="F6" s="52">
+        <v>29149.420000000013</v>
+      </c>
+      <c r="G6" s="53">
+        <v>0.11864815745717495</v>
+      </c>
+      <c r="H6" s="52">
+        <v>208360.5</v>
+      </c>
+      <c r="I6" s="52">
+        <v>168361.6</v>
+      </c>
+      <c r="J6" s="52">
+        <v>180366.49</v>
+      </c>
+      <c r="K6" s="52">
+        <v>138438.46000000002</v>
+      </c>
+      <c r="L6" s="52">
+        <v>41928.02999999997</v>
+      </c>
+      <c r="M6" s="53">
+        <v>0.23246019812216767</v>
+      </c>
       <c r="N6" s="53"/>
-      <c r="O6" s="52"/>
-      <c r="P6" s="52"/>
-      <c r="Q6" s="52"/>
-      <c r="R6" s="53"/>
-      <c r="S6" s="54"/>
-      <c r="T6" s="54"/>
-      <c r="U6" s="54"/>
-      <c r="V6" s="53"/>
+      <c r="O6" s="52">
+        <v>27994.01</v>
+      </c>
+      <c r="P6" s="52">
+        <v>29923.14</v>
+      </c>
+      <c r="Q6" s="52">
+        <v>-1929.130000000001</v>
+      </c>
+      <c r="R6" s="53">
+        <v>-0.06891224229754869</v>
+      </c>
+      <c r="S6" s="54">
+        <v>565.45</v>
+      </c>
+      <c r="T6" s="54">
+        <v>600.25</v>
+      </c>
+      <c r="U6" s="54">
+        <v>-34.799999999999955</v>
+      </c>
+      <c r="V6" s="53">
+        <v>-0.061543903086037584</v>
+      </c>
       <c r="W6" s="53"/>
-      <c r="X6" s="55"/>
-      <c r="Y6" s="55"/>
-      <c r="Z6" s="53"/>
-      <c r="AA6" s="56"/>
+      <c r="X6" s="55">
+        <v>80.24736359850063</v>
+      </c>
+      <c r="Y6" s="55">
+        <v>65.99877634098505</v>
+      </c>
+      <c r="Z6" s="53">
+        <v>0.2225</v>
+      </c>
+      <c r="AA6" s="56">
+        <v>0.1519</v>
+      </c>
       <c r="AB6" s="57"/>
       <c r="AD6" s="35"/>
       <c r="AE6" s="35"/>
@@ -10227,30 +10271,74 @@
       <c r="C13" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="52"/>
-      <c r="E13" s="62"/>
-      <c r="F13" s="52"/>
-      <c r="G13" s="53"/>
-      <c r="H13" s="52"/>
-      <c r="I13" s="52"/>
-      <c r="J13" s="52"/>
-      <c r="K13" s="52"/>
-      <c r="L13" s="52"/>
-      <c r="M13" s="53"/>
+      <c r="D13" s="52">
+        <v>129074.86</v>
+      </c>
+      <c r="E13" s="62">
+        <v>85864.08</v>
+      </c>
+      <c r="F13" s="52">
+        <v>43210.78</v>
+      </c>
+      <c r="G13" s="53">
+        <v>0.3347730146676123</v>
+      </c>
+      <c r="H13" s="52">
+        <v>101420.72</v>
+      </c>
+      <c r="I13" s="52">
+        <v>79791.03</v>
+      </c>
+      <c r="J13" s="52">
+        <v>83645.65</v>
+      </c>
+      <c r="K13" s="52">
+        <v>71604.5</v>
+      </c>
+      <c r="L13" s="52">
+        <v>12041.149999999994</v>
+      </c>
+      <c r="M13" s="53">
+        <v>0.1439542881189876</v>
+      </c>
       <c r="N13" s="53"/>
-      <c r="O13" s="52"/>
-      <c r="P13" s="52"/>
-      <c r="Q13" s="52"/>
-      <c r="R13" s="53"/>
-      <c r="S13" s="54"/>
-      <c r="T13" s="54"/>
-      <c r="U13" s="54"/>
-      <c r="V13" s="53"/>
+      <c r="O13" s="52">
+        <v>17775.07</v>
+      </c>
+      <c r="P13" s="52">
+        <v>8186.53</v>
+      </c>
+      <c r="Q13" s="52">
+        <v>9588.54</v>
+      </c>
+      <c r="R13" s="53">
+        <v>0.5394375380800188</v>
+      </c>
+      <c r="S13" s="54">
+        <v>356.07</v>
+      </c>
+      <c r="T13" s="54">
+        <v>168.25</v>
+      </c>
+      <c r="U13" s="54">
+        <v>187.82</v>
+      </c>
+      <c r="V13" s="53">
+        <v>0.5274805515769371</v>
+      </c>
       <c r="W13" s="53"/>
-      <c r="X13" s="55"/>
-      <c r="Y13" s="55"/>
-      <c r="Z13" s="53"/>
-      <c r="AA13" s="56"/>
+      <c r="X13" s="55">
+        <v>36.09539375928678</v>
+      </c>
+      <c r="Y13" s="55">
+        <v>77.66490997775718</v>
+      </c>
+      <c r="Z13" s="53">
+        <v>0.0707</v>
+      </c>
+      <c r="AA13" s="56">
+        <v>0.2142</v>
+      </c>
       <c r="AB13" s="57"/>
       <c r="AD13" s="35"/>
       <c r="AE13" s="35"/>
@@ -10590,30 +10678,74 @@
       <c r="C20" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D20" s="52"/>
-      <c r="E20" s="52"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="53"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="52"/>
-      <c r="J20" s="52"/>
-      <c r="K20" s="52"/>
-      <c r="L20" s="52"/>
-      <c r="M20" s="53"/>
+      <c r="D20" s="52">
+        <v>27500.32</v>
+      </c>
+      <c r="E20" s="52">
+        <v>11999.08</v>
+      </c>
+      <c r="F20" s="52">
+        <v>15501.24</v>
+      </c>
+      <c r="G20" s="53">
+        <v>0.5636748954193987</v>
+      </c>
+      <c r="H20" s="52">
+        <v>19565.83</v>
+      </c>
+      <c r="I20" s="52">
+        <v>7921.92</v>
+      </c>
+      <c r="J20" s="52">
+        <v>13767.340000000002</v>
+      </c>
+      <c r="K20" s="52">
+        <v>6211.24</v>
+      </c>
+      <c r="L20" s="52">
+        <v>7556.100000000002</v>
+      </c>
+      <c r="M20" s="53">
+        <v>0.5488424052867149</v>
+      </c>
       <c r="N20" s="53"/>
-      <c r="O20" s="52"/>
-      <c r="P20" s="52"/>
-      <c r="Q20" s="52"/>
-      <c r="R20" s="53"/>
-      <c r="S20" s="54"/>
-      <c r="T20" s="54"/>
-      <c r="U20" s="54"/>
-      <c r="V20" s="53"/>
+      <c r="O20" s="52">
+        <v>5798.49</v>
+      </c>
+      <c r="P20" s="52">
+        <v>1710.68</v>
+      </c>
+      <c r="Q20" s="52">
+        <v>4087.8099999999995</v>
+      </c>
+      <c r="R20" s="53">
+        <v>0.7049783650571096</v>
+      </c>
+      <c r="S20" s="54">
+        <v>125.39</v>
+      </c>
+      <c r="T20" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U20" s="54">
+        <v>90.64</v>
+      </c>
+      <c r="V20" s="53">
+        <v>0.7228646622537682</v>
+      </c>
       <c r="W20" s="53"/>
-      <c r="X20" s="55"/>
-      <c r="Y20" s="55"/>
-      <c r="Z20" s="53"/>
-      <c r="AA20" s="56"/>
+      <c r="X20" s="55">
+        <v>117.328345323741</v>
+      </c>
+      <c r="Y20" s="55">
+        <v>63.27846478985563</v>
+      </c>
+      <c r="Z20" s="53">
+        <v>0.3398</v>
+      </c>
+      <c r="AA20" s="56">
+        <v>0.2885</v>
+      </c>
       <c r="AB20" s="57"/>
       <c r="AD20" s="35"/>
       <c r="AE20" s="35"/>
@@ -10955,30 +11087,74 @@
       <c r="C27" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D27" s="55"/>
-      <c r="E27" s="55"/>
-      <c r="F27" s="52"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="52"/>
-      <c r="I27" s="52"/>
-      <c r="J27" s="52"/>
-      <c r="K27" s="52"/>
-      <c r="L27" s="52"/>
-      <c r="M27" s="53"/>
+      <c r="D27" s="55">
+        <v>150850.82</v>
+      </c>
+      <c r="E27" s="55">
+        <v>144370.8</v>
+      </c>
+      <c r="F27" s="52">
+        <v>6480.020000000019</v>
+      </c>
+      <c r="G27" s="53">
+        <v>0.042956478459978</v>
+      </c>
+      <c r="H27" s="52">
+        <v>102178.42</v>
+      </c>
+      <c r="I27" s="52">
+        <v>89222.05</v>
+      </c>
+      <c r="J27" s="52">
+        <v>62464.86</v>
+      </c>
+      <c r="K27" s="52">
+        <v>58984</v>
+      </c>
+      <c r="L27" s="52">
+        <v>3480.8600000000006</v>
+      </c>
+      <c r="M27" s="53">
+        <v>0.05572509087509362</v>
+      </c>
       <c r="N27" s="53"/>
-      <c r="O27" s="52"/>
-      <c r="P27" s="52"/>
-      <c r="Q27" s="52"/>
-      <c r="R27" s="53"/>
-      <c r="S27" s="54"/>
-      <c r="T27" s="54"/>
-      <c r="U27" s="54"/>
-      <c r="V27" s="53"/>
+      <c r="O27" s="52">
+        <v>39713.56</v>
+      </c>
+      <c r="P27" s="52">
+        <v>30238.05</v>
+      </c>
+      <c r="Q27" s="52">
+        <v>9475.509999999998</v>
+      </c>
+      <c r="R27" s="53">
+        <v>0.23859633837913294</v>
+      </c>
+      <c r="S27" s="54">
+        <v>795.22</v>
+      </c>
+      <c r="T27" s="54">
+        <v>615</v>
+      </c>
+      <c r="U27" s="54">
+        <v>180.22000000000003</v>
+      </c>
+      <c r="V27" s="53">
+        <v>0.22662910892583188</v>
+      </c>
       <c r="W27" s="53"/>
-      <c r="X27" s="55"/>
-      <c r="Y27" s="55"/>
-      <c r="Z27" s="53"/>
-      <c r="AA27" s="56"/>
+      <c r="X27" s="55">
+        <v>89.67276422764228</v>
+      </c>
+      <c r="Y27" s="55">
+        <v>61.20621468124544</v>
+      </c>
+      <c r="Z27" s="53">
+        <v>0.382</v>
+      </c>
+      <c r="AA27" s="56">
+        <v>0.3227</v>
+      </c>
       <c r="AB27" s="57"/>
       <c r="AD27" s="35"/>
       <c r="AE27" s="35"/>
@@ -11318,30 +11494,74 @@
       <c r="C34" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="53"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="65"/>
-      <c r="J34" s="52"/>
-      <c r="K34" s="52"/>
-      <c r="L34" s="52"/>
-      <c r="M34" s="53"/>
+      <c r="D34" s="52">
+        <v>396422.03</v>
+      </c>
+      <c r="E34" s="52">
+        <v>259347.71</v>
+      </c>
+      <c r="F34" s="52">
+        <v>137074.32000000004</v>
+      </c>
+      <c r="G34" s="53">
+        <v>0.3457787651205964</v>
+      </c>
+      <c r="H34" s="52">
+        <v>327431.12</v>
+      </c>
+      <c r="I34" s="65">
+        <v>223659.54</v>
+      </c>
+      <c r="J34" s="52">
+        <v>271519.78</v>
+      </c>
+      <c r="K34" s="52">
+        <v>197370.72</v>
+      </c>
+      <c r="L34" s="52">
+        <v>74149.06000000003</v>
+      </c>
+      <c r="M34" s="53">
+        <v>0.27308898084699396</v>
+      </c>
       <c r="N34" s="53"/>
-      <c r="O34" s="52"/>
-      <c r="P34" s="52"/>
-      <c r="Q34" s="52"/>
-      <c r="R34" s="53"/>
-      <c r="S34" s="54"/>
-      <c r="T34" s="54"/>
-      <c r="U34" s="54"/>
-      <c r="V34" s="53"/>
+      <c r="O34" s="52">
+        <v>55911.34</v>
+      </c>
+      <c r="P34" s="52">
+        <v>26288.82</v>
+      </c>
+      <c r="Q34" s="52">
+        <v>29622.519999999997</v>
+      </c>
+      <c r="R34" s="53">
+        <v>0.5298123779540966</v>
+      </c>
+      <c r="S34" s="54">
+        <v>1120.27</v>
+      </c>
+      <c r="T34" s="54">
+        <v>607.75</v>
+      </c>
+      <c r="U34" s="54">
+        <v>512.52</v>
+      </c>
+      <c r="V34" s="53">
+        <v>0.4574968534371178</v>
+      </c>
       <c r="W34" s="53"/>
-      <c r="X34" s="55"/>
-      <c r="Y34" s="55"/>
-      <c r="Z34" s="53"/>
-      <c r="AA34" s="56"/>
+      <c r="X34" s="55">
+        <v>58.721793500617025</v>
+      </c>
+      <c r="Y34" s="55">
+        <v>61.5841822414239</v>
+      </c>
+      <c r="Z34" s="53">
+        <v>0.1376</v>
+      </c>
+      <c r="AA34" s="56">
+        <v>0.174</v>
+      </c>
       <c r="AB34" s="57"/>
       <c r="AD34" s="35"/>
       <c r="AE34" s="35"/>
@@ -11681,30 +11901,74 @@
       <c r="C41" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="53"/>
-      <c r="H41" s="52"/>
-      <c r="I41" s="52"/>
-      <c r="J41" s="52"/>
-      <c r="K41" s="52"/>
-      <c r="L41" s="52"/>
-      <c r="M41" s="53"/>
+      <c r="D41" s="52">
+        <v>128258.5</v>
+      </c>
+      <c r="E41" s="52">
+        <v>53944.83</v>
+      </c>
+      <c r="F41" s="52">
+        <v>74313.67</v>
+      </c>
+      <c r="G41" s="53">
+        <v>0.5794054195238522</v>
+      </c>
+      <c r="H41" s="52">
+        <v>94098.32</v>
+      </c>
+      <c r="I41" s="52">
+        <v>49261.61</v>
+      </c>
+      <c r="J41" s="52">
+        <v>69042.09000000001</v>
+      </c>
+      <c r="K41" s="52">
+        <v>35683.74</v>
+      </c>
+      <c r="L41" s="52">
+        <v>33358.35000000001</v>
+      </c>
+      <c r="M41" s="53">
+        <v>0.4831596204576079</v>
+      </c>
       <c r="N41" s="53"/>
-      <c r="O41" s="52"/>
-      <c r="P41" s="52"/>
-      <c r="Q41" s="52"/>
-      <c r="R41" s="53"/>
-      <c r="S41" s="54"/>
-      <c r="T41" s="54"/>
-      <c r="U41" s="54"/>
-      <c r="V41" s="53"/>
+      <c r="O41" s="52">
+        <v>25056.23</v>
+      </c>
+      <c r="P41" s="52">
+        <v>13577.87</v>
+      </c>
+      <c r="Q41" s="52">
+        <v>11478.359999999999</v>
+      </c>
+      <c r="R41" s="53">
+        <v>0.45810403241030273</v>
+      </c>
+      <c r="S41" s="54">
+        <v>501.83</v>
+      </c>
+      <c r="T41" s="54">
+        <v>299.5</v>
+      </c>
+      <c r="U41" s="54">
+        <v>202.32999999999998</v>
+      </c>
+      <c r="V41" s="53">
+        <v>0.40318434529621583</v>
+      </c>
       <c r="W41" s="53"/>
-      <c r="X41" s="55"/>
-      <c r="Y41" s="55"/>
-      <c r="Z41" s="53"/>
-      <c r="AA41" s="56"/>
+      <c r="X41" s="55">
+        <v>15.63679465776294</v>
+      </c>
+      <c r="Y41" s="55">
+        <v>68.07122423898531</v>
+      </c>
+      <c r="Z41" s="53">
+        <v>0.0868</v>
+      </c>
+      <c r="AA41" s="56">
+        <v>0.2663</v>
+      </c>
       <c r="AB41" s="57"/>
       <c r="AD41" s="35"/>
       <c r="AE41" s="35"/>
@@ -12046,30 +12310,74 @@
       <c r="C48" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D48" s="52"/>
-      <c r="E48" s="52"/>
-      <c r="F48" s="52"/>
-      <c r="G48" s="53"/>
-      <c r="H48" s="52"/>
-      <c r="I48" s="52"/>
-      <c r="J48" s="52"/>
-      <c r="K48" s="52"/>
-      <c r="L48" s="52"/>
-      <c r="M48" s="53"/>
+      <c r="D48" s="52">
+        <v>65693.36</v>
+      </c>
+      <c r="E48" s="52">
+        <v>33326.49</v>
+      </c>
+      <c r="F48" s="52">
+        <v>32366.870000000003</v>
+      </c>
+      <c r="G48" s="53">
+        <v>0.49269621769993194</v>
+      </c>
+      <c r="H48" s="52">
+        <v>50582.37</v>
+      </c>
+      <c r="I48" s="52">
+        <v>25196.36</v>
+      </c>
+      <c r="J48" s="52">
+        <v>39438.990000000005</v>
+      </c>
+      <c r="K48" s="52">
+        <v>20036.420000000002</v>
+      </c>
+      <c r="L48" s="52">
+        <v>19402.570000000003</v>
+      </c>
+      <c r="M48" s="53">
+        <v>0.49196417048205343</v>
+      </c>
       <c r="N48" s="53"/>
-      <c r="O48" s="52"/>
-      <c r="P48" s="52"/>
-      <c r="Q48" s="52"/>
-      <c r="R48" s="53"/>
-      <c r="S48" s="54"/>
-      <c r="T48" s="54"/>
-      <c r="U48" s="54"/>
-      <c r="V48" s="53"/>
+      <c r="O48" s="52">
+        <v>11143.38</v>
+      </c>
+      <c r="P48" s="52">
+        <v>5159.94</v>
+      </c>
+      <c r="Q48" s="52">
+        <v>5983.44</v>
+      </c>
+      <c r="R48" s="53">
+        <v>0.5369501892603501</v>
+      </c>
+      <c r="S48" s="54">
+        <v>223.22</v>
+      </c>
+      <c r="T48" s="54">
+        <v>113.25</v>
+      </c>
+      <c r="U48" s="54">
+        <v>109.97</v>
+      </c>
+      <c r="V48" s="53">
+        <v>0.49265298808350505</v>
+      </c>
       <c r="W48" s="53"/>
-      <c r="X48" s="55"/>
-      <c r="Y48" s="55"/>
-      <c r="Z48" s="53"/>
-      <c r="AA48" s="56"/>
+      <c r="X48" s="55">
+        <v>71.78922737306843</v>
+      </c>
+      <c r="Y48" s="55">
+        <v>67.69550512136009</v>
+      </c>
+      <c r="Z48" s="53">
+        <v>0.244</v>
+      </c>
+      <c r="AA48" s="56">
+        <v>0.23</v>
+      </c>
       <c r="AB48" s="57"/>
       <c r="AD48" s="35"/>
       <c r="AE48" s="35"/>
@@ -12409,30 +12717,74 @@
       <c r="C55" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="53"/>
-      <c r="H55" s="52"/>
-      <c r="I55" s="52"/>
-      <c r="J55" s="52"/>
-      <c r="K55" s="52"/>
-      <c r="L55" s="52"/>
-      <c r="M55" s="53"/>
+      <c r="D55" s="52">
+        <v>155296.79</v>
+      </c>
+      <c r="E55" s="52">
+        <v>127814.48</v>
+      </c>
+      <c r="F55" s="52">
+        <v>27482.310000000012</v>
+      </c>
+      <c r="G55" s="53">
+        <v>0.176966375158173</v>
+      </c>
+      <c r="H55" s="52">
+        <v>109364.97</v>
+      </c>
+      <c r="I55" s="52">
+        <v>96483.38</v>
+      </c>
+      <c r="J55" s="52">
+        <v>75135.01000000001</v>
+      </c>
+      <c r="K55" s="52">
+        <v>71221.34</v>
+      </c>
+      <c r="L55" s="52">
+        <v>3913.670000000013</v>
+      </c>
+      <c r="M55" s="53">
+        <v>0.05208850042077604</v>
+      </c>
       <c r="N55" s="53"/>
-      <c r="O55" s="52"/>
-      <c r="P55" s="52"/>
-      <c r="Q55" s="52"/>
-      <c r="R55" s="53"/>
-      <c r="S55" s="54"/>
-      <c r="T55" s="54"/>
-      <c r="U55" s="54"/>
-      <c r="V55" s="53"/>
+      <c r="O55" s="52">
+        <v>34229.96</v>
+      </c>
+      <c r="P55" s="52">
+        <v>25262.04</v>
+      </c>
+      <c r="Q55" s="52">
+        <v>8967.919999999998</v>
+      </c>
+      <c r="R55" s="53">
+        <v>0.2619903733454552</v>
+      </c>
+      <c r="S55" s="54">
+        <v>685.48</v>
+      </c>
+      <c r="T55" s="54">
+        <v>533.75</v>
+      </c>
+      <c r="U55" s="54">
+        <v>151.73000000000002</v>
+      </c>
+      <c r="V55" s="53">
+        <v>0.22134854408589605</v>
+      </c>
       <c r="W55" s="53"/>
-      <c r="X55" s="55"/>
-      <c r="Y55" s="55"/>
-      <c r="Z55" s="53"/>
-      <c r="AA55" s="56"/>
+      <c r="X55" s="55">
+        <v>58.699953161592504</v>
+      </c>
+      <c r="Y55" s="55">
+        <v>67.00679527854935</v>
+      </c>
+      <c r="Z55" s="53">
+        <v>0.2451</v>
+      </c>
+      <c r="AA55" s="56">
+        <v>0.2958</v>
+      </c>
       <c r="AB55" s="57"/>
       <c r="AD55" s="35"/>
       <c r="AE55" s="35"/>
@@ -12772,30 +13124,74 @@
       <c r="C62" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D62" s="52"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="53"/>
-      <c r="H62" s="52"/>
-      <c r="I62" s="52"/>
-      <c r="J62" s="52"/>
-      <c r="K62" s="52"/>
-      <c r="L62" s="52"/>
-      <c r="M62" s="53"/>
+      <c r="D62" s="52">
+        <v>20420.56</v>
+      </c>
+      <c r="E62" s="52">
+        <v>20420.56</v>
+      </c>
+      <c r="F62" s="52">
+        <v>0</v>
+      </c>
+      <c r="G62" s="53">
+        <v>0</v>
+      </c>
+      <c r="H62" s="52">
+        <v>15859.68</v>
+      </c>
+      <c r="I62" s="52">
+        <v>13435.12</v>
+      </c>
+      <c r="J62" s="52">
+        <v>12689.1</v>
+      </c>
+      <c r="K62" s="52">
+        <v>11478.25</v>
+      </c>
+      <c r="L62" s="52">
+        <v>1210.8500000000004</v>
+      </c>
+      <c r="M62" s="53">
+        <v>0.09542441938356545</v>
+      </c>
       <c r="N62" s="53"/>
-      <c r="O62" s="52"/>
-      <c r="P62" s="52"/>
-      <c r="Q62" s="52"/>
-      <c r="R62" s="53"/>
-      <c r="S62" s="54"/>
-      <c r="T62" s="54"/>
-      <c r="U62" s="54"/>
-      <c r="V62" s="53"/>
+      <c r="O62" s="52">
+        <v>3170.58</v>
+      </c>
+      <c r="P62" s="52">
+        <v>1956.87</v>
+      </c>
+      <c r="Q62" s="52">
+        <v>1213.71</v>
+      </c>
+      <c r="R62" s="53">
+        <v>0.38280377722687964</v>
+      </c>
+      <c r="S62" s="54">
+        <v>63.5</v>
+      </c>
+      <c r="T62" s="54">
+        <v>48.25</v>
+      </c>
+      <c r="U62" s="54">
+        <v>15.25</v>
+      </c>
+      <c r="V62" s="53">
+        <v>0.24015748031496062</v>
+      </c>
       <c r="W62" s="53"/>
-      <c r="X62" s="55"/>
-      <c r="Y62" s="55"/>
-      <c r="Z62" s="53"/>
-      <c r="AA62" s="56"/>
+      <c r="X62" s="55">
+        <v>144.7759585492228</v>
+      </c>
+      <c r="Y62" s="55">
+        <v>71.82495570677168</v>
+      </c>
+      <c r="Z62" s="53">
+        <v>0.3421</v>
+      </c>
+      <c r="AA62" s="56">
+        <v>0.2233</v>
+      </c>
       <c r="AB62" s="57"/>
       <c r="AD62" s="35"/>
       <c r="AE62" s="35"/>
@@ -13129,30 +13525,74 @@
       <c r="C69" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D69" s="52"/>
-      <c r="E69" s="52"/>
-      <c r="F69" s="52"/>
-      <c r="G69" s="53"/>
-      <c r="H69" s="52"/>
-      <c r="I69" s="52"/>
-      <c r="J69" s="52"/>
-      <c r="K69" s="52"/>
-      <c r="L69" s="52"/>
-      <c r="M69" s="53"/>
+      <c r="D69" s="52">
+        <v>47801.68</v>
+      </c>
+      <c r="E69" s="52">
+        <v>10650.43</v>
+      </c>
+      <c r="F69" s="52">
+        <v>37151.25</v>
+      </c>
+      <c r="G69" s="53">
+        <v>0.7771954876899724</v>
+      </c>
+      <c r="H69" s="52">
+        <v>35572.59</v>
+      </c>
+      <c r="I69" s="52">
+        <v>10547.08</v>
+      </c>
+      <c r="J69" s="52">
+        <v>27136.549999999996</v>
+      </c>
+      <c r="K69" s="52">
+        <v>10398.3</v>
+      </c>
+      <c r="L69" s="52">
+        <v>16738.249999999996</v>
+      </c>
+      <c r="M69" s="53">
+        <v>0.6168156969106242</v>
+      </c>
       <c r="N69" s="53"/>
-      <c r="O69" s="52"/>
-      <c r="P69" s="52"/>
-      <c r="Q69" s="52"/>
-      <c r="R69" s="53"/>
-      <c r="S69" s="54"/>
-      <c r="T69" s="54"/>
-      <c r="U69" s="54"/>
-      <c r="V69" s="53"/>
+      <c r="O69" s="52">
+        <v>8436.04</v>
+      </c>
+      <c r="P69" s="52">
+        <v>148.78</v>
+      </c>
+      <c r="Q69" s="52">
+        <v>8287.26</v>
+      </c>
+      <c r="R69" s="53">
+        <v>0.9823637630926358</v>
+      </c>
+      <c r="S69" s="54">
+        <v>169.32</v>
+      </c>
+      <c r="T69" s="54">
+        <v>2.75</v>
+      </c>
+      <c r="U69" s="54">
+        <v>166.57</v>
+      </c>
+      <c r="V69" s="53">
+        <v>0.9837585636664304</v>
+      </c>
       <c r="W69" s="53"/>
-      <c r="X69" s="55"/>
-      <c r="Y69" s="55"/>
-      <c r="Z69" s="53"/>
-      <c r="AA69" s="56"/>
+      <c r="X69" s="55">
+        <v>37.58181818181818</v>
+      </c>
+      <c r="Y69" s="55">
+        <v>72.22475431425701</v>
+      </c>
+      <c r="Z69" s="53">
+        <v>0.0097</v>
+      </c>
+      <c r="AA69" s="56">
+        <v>0.2558</v>
+      </c>
       <c r="AB69" s="57"/>
       <c r="AD69" s="35"/>
       <c r="AE69" s="35"/>
@@ -13482,30 +13922,74 @@
       <c r="C76" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D76" s="52"/>
-      <c r="E76" s="52"/>
-      <c r="F76" s="52"/>
-      <c r="G76" s="53"/>
-      <c r="H76" s="52"/>
-      <c r="I76" s="52"/>
-      <c r="J76" s="52"/>
-      <c r="K76" s="52"/>
-      <c r="L76" s="52"/>
-      <c r="M76" s="53"/>
+      <c r="D76" s="52">
+        <v>77166.16</v>
+      </c>
+      <c r="E76" s="52">
+        <v>44764.99</v>
+      </c>
+      <c r="F76" s="52">
+        <v>32401.170000000006</v>
+      </c>
+      <c r="G76" s="53">
+        <v>0.41988832928838243</v>
+      </c>
+      <c r="H76" s="52">
+        <v>54302.66</v>
+      </c>
+      <c r="I76" s="52">
+        <v>29696.65</v>
+      </c>
+      <c r="J76" s="52">
+        <v>31383.390000000003</v>
+      </c>
+      <c r="K76" s="52">
+        <v>23592.600000000002</v>
+      </c>
+      <c r="L76" s="52">
+        <v>7790.790000000001</v>
+      </c>
+      <c r="M76" s="53">
+        <v>0.24824564841465502</v>
+      </c>
       <c r="N76" s="53"/>
-      <c r="O76" s="52"/>
-      <c r="P76" s="52"/>
-      <c r="Q76" s="52"/>
-      <c r="R76" s="53"/>
-      <c r="S76" s="54"/>
-      <c r="T76" s="54"/>
-      <c r="U76" s="54"/>
-      <c r="V76" s="53"/>
+      <c r="O76" s="52">
+        <v>22919.27</v>
+      </c>
+      <c r="P76" s="52">
+        <v>6104.05</v>
+      </c>
+      <c r="Q76" s="52">
+        <v>16815.22</v>
+      </c>
+      <c r="R76" s="53">
+        <v>0.7336717094392623</v>
+      </c>
+      <c r="S76" s="54">
+        <v>470.62</v>
+      </c>
+      <c r="T76" s="54">
+        <v>120.25</v>
+      </c>
+      <c r="U76" s="54">
+        <v>350.37</v>
+      </c>
+      <c r="V76" s="53">
+        <v>0.7444859971951894</v>
+      </c>
       <c r="W76" s="53"/>
-      <c r="X76" s="55"/>
-      <c r="Y76" s="55"/>
-      <c r="Z76" s="53"/>
-      <c r="AA76" s="56"/>
+      <c r="X76" s="55">
+        <v>125.30844074844074</v>
+      </c>
+      <c r="Y76" s="55">
+        <v>48.58165977967362</v>
+      </c>
+      <c r="Z76" s="53">
+        <v>0.33659999999999995</v>
+      </c>
+      <c r="AA76" s="56">
+        <v>0.2963</v>
+      </c>
       <c r="AB76" s="57"/>
       <c r="AD76" s="35"/>
       <c r="AE76" s="35"/>
@@ -13841,30 +14325,74 @@
       <c r="C83" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D83" s="52"/>
-      <c r="E83" s="52"/>
-      <c r="F83" s="52"/>
-      <c r="G83" s="53"/>
-      <c r="H83" s="52"/>
-      <c r="I83" s="52"/>
-      <c r="J83" s="52"/>
-      <c r="K83" s="52"/>
-      <c r="L83" s="52"/>
-      <c r="M83" s="53"/>
+      <c r="D83" s="52">
+        <v>25467.84</v>
+      </c>
+      <c r="E83" s="52">
+        <v>19598.41</v>
+      </c>
+      <c r="F83" s="52">
+        <v>5869.43</v>
+      </c>
+      <c r="G83" s="53">
+        <v>0.2304643817457625</v>
+      </c>
+      <c r="H83" s="52">
+        <v>16606.83</v>
+      </c>
+      <c r="I83" s="52">
+        <v>12958.24</v>
+      </c>
+      <c r="J83" s="52">
+        <v>9659.990000000002</v>
+      </c>
+      <c r="K83" s="52">
+        <v>5354.12</v>
+      </c>
+      <c r="L83" s="52">
+        <v>4305.870000000002</v>
+      </c>
+      <c r="M83" s="53">
+        <v>0.44574269745620865</v>
+      </c>
       <c r="N83" s="53"/>
-      <c r="O83" s="52"/>
-      <c r="P83" s="52"/>
-      <c r="Q83" s="52"/>
-      <c r="R83" s="53"/>
-      <c r="S83" s="54"/>
-      <c r="T83" s="54"/>
-      <c r="U83" s="54"/>
-      <c r="V83" s="53"/>
+      <c r="O83" s="52">
+        <v>6946.84</v>
+      </c>
+      <c r="P83" s="52">
+        <v>7604.12</v>
+      </c>
+      <c r="Q83" s="52">
+        <v>-657.2799999999997</v>
+      </c>
+      <c r="R83" s="53">
+        <v>-0.09461568137455299</v>
+      </c>
+      <c r="S83" s="54">
+        <v>139.07</v>
+      </c>
+      <c r="T83" s="54">
+        <v>147.75</v>
+      </c>
+      <c r="U83" s="54">
+        <v>-8.680000000000007</v>
+      </c>
+      <c r="V83" s="53">
+        <v>-0.06241461134680382</v>
+      </c>
       <c r="W83" s="53"/>
-      <c r="X83" s="55"/>
-      <c r="Y83" s="55"/>
-      <c r="Z83" s="53"/>
-      <c r="AA83" s="56"/>
+      <c r="X83" s="55">
+        <v>44.94192893401015</v>
+      </c>
+      <c r="Y83" s="55">
+        <v>63.7162162306752</v>
+      </c>
+      <c r="Z83" s="53">
+        <v>0.33880000000000005</v>
+      </c>
+      <c r="AA83" s="56">
+        <v>0.3479</v>
+      </c>
       <c r="AB83" s="57"/>
       <c r="AD83" s="35"/>
       <c r="AE83" s="35"/>
@@ -14204,30 +14732,74 @@
       <c r="C90" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D90" s="67"/>
-      <c r="E90" s="67"/>
-      <c r="F90" s="52"/>
-      <c r="G90" s="53"/>
-      <c r="H90" s="52"/>
-      <c r="I90" s="52"/>
-      <c r="J90" s="52"/>
-      <c r="K90" s="52"/>
-      <c r="L90" s="52"/>
-      <c r="M90" s="53"/>
+      <c r="D90" s="67">
+        <v>37083.03</v>
+      </c>
+      <c r="E90" s="67">
+        <v>36381.33</v>
+      </c>
+      <c r="F90" s="52">
+        <v>701.6999999999971</v>
+      </c>
+      <c r="G90" s="53">
+        <v>0.018922401972007064</v>
+      </c>
+      <c r="H90" s="52">
+        <v>27002.93</v>
+      </c>
+      <c r="I90" s="52">
+        <v>25060.53</v>
+      </c>
+      <c r="J90" s="52">
+        <v>15440.32</v>
+      </c>
+      <c r="K90" s="52">
+        <v>13974.73</v>
+      </c>
+      <c r="L90" s="52">
+        <v>1465.5900000000001</v>
+      </c>
+      <c r="M90" s="53">
+        <v>0.09491966487741188</v>
+      </c>
       <c r="N90" s="53"/>
-      <c r="O90" s="52"/>
-      <c r="P90" s="52"/>
-      <c r="Q90" s="52"/>
-      <c r="R90" s="53"/>
-      <c r="S90" s="68"/>
-      <c r="T90" s="68"/>
-      <c r="U90" s="54"/>
-      <c r="V90" s="53"/>
+      <c r="O90" s="52">
+        <v>11562.61</v>
+      </c>
+      <c r="P90" s="52">
+        <v>11085.8</v>
+      </c>
+      <c r="Q90" s="52">
+        <v>476.8100000000013</v>
+      </c>
+      <c r="R90" s="53">
+        <v>0.041237229310683424</v>
+      </c>
+      <c r="S90" s="68">
+        <v>231.75</v>
+      </c>
+      <c r="T90" s="68">
+        <v>225.5</v>
+      </c>
+      <c r="U90" s="54">
+        <v>6.25</v>
+      </c>
+      <c r="V90" s="53">
+        <v>0.02696871628910464</v>
+      </c>
       <c r="W90" s="53"/>
-      <c r="X90" s="55"/>
-      <c r="Y90" s="55"/>
-      <c r="Z90" s="53"/>
-      <c r="AA90" s="56"/>
+      <c r="X90" s="55">
+        <v>50.20310421286031</v>
+      </c>
+      <c r="Y90" s="55">
+        <v>43.49557070636461</v>
+      </c>
+      <c r="Z90" s="53">
+        <v>0.31120000000000003</v>
+      </c>
+      <c r="AA90" s="56">
+        <v>0.2718</v>
+      </c>
       <c r="AB90" s="57"/>
       <c r="AD90" s="35"/>
       <c r="AE90" s="35"/>
@@ -14567,30 +15139,74 @@
       <c r="C97" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D97" s="52"/>
-      <c r="E97" s="52"/>
-      <c r="F97" s="52"/>
-      <c r="G97" s="53"/>
-      <c r="H97" s="52"/>
-      <c r="I97" s="52"/>
-      <c r="J97" s="52"/>
-      <c r="K97" s="52"/>
-      <c r="L97" s="52"/>
-      <c r="M97" s="53"/>
+      <c r="D97" s="52">
+        <v>26186.14</v>
+      </c>
+      <c r="E97" s="52">
+        <v>5762.27</v>
+      </c>
+      <c r="F97" s="52">
+        <v>20423.87</v>
+      </c>
+      <c r="G97" s="53">
+        <v>0.7799496222047235</v>
+      </c>
+      <c r="H97" s="52">
+        <v>19428.98</v>
+      </c>
+      <c r="I97" s="52">
+        <v>7925.81</v>
+      </c>
+      <c r="J97" s="52">
+        <v>12051.32</v>
+      </c>
+      <c r="K97" s="52">
+        <v>7679.910000000001</v>
+      </c>
+      <c r="L97" s="52">
+        <v>4371.409999999999</v>
+      </c>
+      <c r="M97" s="53">
+        <v>0.36273287905391266</v>
+      </c>
       <c r="N97" s="53"/>
-      <c r="O97" s="52"/>
-      <c r="P97" s="52"/>
-      <c r="Q97" s="52"/>
-      <c r="R97" s="53"/>
-      <c r="S97" s="54"/>
-      <c r="T97" s="54"/>
-      <c r="U97" s="54"/>
-      <c r="V97" s="53"/>
+      <c r="O97" s="52">
+        <v>7377.66</v>
+      </c>
+      <c r="P97" s="52">
+        <v>245.9</v>
+      </c>
+      <c r="Q97" s="52">
+        <v>7131.76</v>
+      </c>
+      <c r="R97" s="53">
+        <v>0.9666696486419813</v>
+      </c>
+      <c r="S97" s="54">
+        <v>147.9</v>
+      </c>
+      <c r="T97" s="54">
+        <v>5</v>
+      </c>
+      <c r="U97" s="54">
+        <v>142.9</v>
+      </c>
+      <c r="V97" s="53">
+        <v>0.9661933739012847</v>
+      </c>
       <c r="W97" s="53"/>
-      <c r="X97" s="55"/>
-      <c r="Y97" s="55"/>
-      <c r="Z97" s="53"/>
-      <c r="AA97" s="56"/>
+      <c r="X97" s="55">
+        <v>-432.70799999999997</v>
+      </c>
+      <c r="Y97" s="55">
+        <v>45.687352144692355</v>
+      </c>
+      <c r="Z97" s="53">
+        <v>-0.37549999999999994</v>
+      </c>
+      <c r="AA97" s="56">
+        <v>0.258</v>
+      </c>
       <c r="AB97" s="57"/>
       <c r="AD97" s="35"/>
       <c r="AE97" s="35"/>
@@ -14930,30 +15546,74 @@
       <c r="C104" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D104" s="52"/>
-      <c r="E104" s="69"/>
-      <c r="F104" s="52"/>
-      <c r="G104" s="53"/>
-      <c r="H104" s="52"/>
-      <c r="I104" s="52"/>
-      <c r="J104" s="52"/>
-      <c r="K104" s="52"/>
-      <c r="L104" s="52"/>
-      <c r="M104" s="53"/>
+      <c r="D104" s="52">
+        <v>32473.02</v>
+      </c>
+      <c r="E104" s="69">
+        <v>33188.03</v>
+      </c>
+      <c r="F104" s="52">
+        <v>-715.0099999999984</v>
+      </c>
+      <c r="G104" s="53">
+        <v>-0.022018586506582952</v>
+      </c>
+      <c r="H104" s="52">
+        <v>23075.07</v>
+      </c>
+      <c r="I104" s="52">
+        <v>30925.21</v>
+      </c>
+      <c r="J104" s="52">
+        <v>12691.21</v>
+      </c>
+      <c r="K104" s="52">
+        <v>15184.269999999999</v>
+      </c>
+      <c r="L104" s="52">
+        <v>-2493.0599999999995</v>
+      </c>
+      <c r="M104" s="53">
+        <v>-0.1964398981657383</v>
+      </c>
       <c r="N104" s="53"/>
-      <c r="O104" s="52"/>
-      <c r="P104" s="52"/>
-      <c r="Q104" s="52"/>
-      <c r="R104" s="53"/>
-      <c r="S104" s="54"/>
-      <c r="T104" s="54"/>
-      <c r="U104" s="54"/>
-      <c r="V104" s="53"/>
+      <c r="O104" s="52">
+        <v>10383.86</v>
+      </c>
+      <c r="P104" s="52">
+        <v>15740.94</v>
+      </c>
+      <c r="Q104" s="52">
+        <v>-5357.08</v>
+      </c>
+      <c r="R104" s="53">
+        <v>-0.5159044902377343</v>
+      </c>
+      <c r="S104" s="54">
+        <v>208.2</v>
+      </c>
+      <c r="T104" s="54">
+        <v>317.25</v>
+      </c>
+      <c r="U104" s="54">
+        <v>-109.05000000000001</v>
+      </c>
+      <c r="V104" s="53">
+        <v>-0.5237752161383286</v>
+      </c>
       <c r="W104" s="53"/>
-      <c r="X104" s="55"/>
-      <c r="Y104" s="55"/>
-      <c r="Z104" s="53"/>
-      <c r="AA104" s="56"/>
+      <c r="X104" s="55">
+        <v>7.132608353033885</v>
+      </c>
+      <c r="Y104" s="55">
+        <v>45.139084580403456</v>
+      </c>
+      <c r="Z104" s="53">
+        <v>0.0682</v>
+      </c>
+      <c r="AA104" s="56">
+        <v>0.2894</v>
+      </c>
       <c r="AB104" s="57"/>
       <c r="AD104" s="35"/>
       <c r="AE104" s="35"/>
@@ -15295,30 +15955,74 @@
       <c r="C111" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D111" s="52"/>
-      <c r="E111" s="52"/>
-      <c r="F111" s="52"/>
-      <c r="G111" s="53"/>
-      <c r="H111" s="52"/>
-      <c r="I111" s="52"/>
-      <c r="J111" s="52"/>
-      <c r="K111" s="52"/>
-      <c r="L111" s="52"/>
-      <c r="M111" s="53"/>
+      <c r="D111" s="52">
+        <v>58902.56</v>
+      </c>
+      <c r="E111" s="52">
+        <v>0</v>
+      </c>
+      <c r="F111" s="52">
+        <v>58902.56</v>
+      </c>
+      <c r="G111" s="53">
+        <v>1</v>
+      </c>
+      <c r="H111" s="52">
+        <v>37601.88</v>
+      </c>
+      <c r="I111" s="52">
+        <v>45817.77</v>
+      </c>
+      <c r="J111" s="52">
+        <v>21415.85</v>
+      </c>
+      <c r="K111" s="52">
+        <v>23939.389999999996</v>
+      </c>
+      <c r="L111" s="52">
+        <v>-2523.5399999999972</v>
+      </c>
+      <c r="M111" s="53">
+        <v>-0.11783515480356826</v>
+      </c>
       <c r="N111" s="53"/>
-      <c r="O111" s="52"/>
-      <c r="P111" s="52"/>
-      <c r="Q111" s="52"/>
-      <c r="R111" s="53"/>
-      <c r="S111" s="54"/>
-      <c r="T111" s="54"/>
-      <c r="U111" s="54"/>
-      <c r="V111" s="53"/>
+      <c r="O111" s="52">
+        <v>16186.03</v>
+      </c>
+      <c r="P111" s="52">
+        <v>21878.38</v>
+      </c>
+      <c r="Q111" s="52">
+        <v>-5692.35</v>
+      </c>
+      <c r="R111" s="53">
+        <v>-0.3516829018604315</v>
+      </c>
+      <c r="S111" s="54">
+        <v>324.19</v>
+      </c>
+      <c r="T111" s="54">
+        <v>472.75</v>
+      </c>
+      <c r="U111" s="54">
+        <v>-148.56</v>
+      </c>
+      <c r="V111" s="53">
+        <v>-0.45824979178876585</v>
+      </c>
       <c r="W111" s="53"/>
-      <c r="X111" s="55"/>
-      <c r="Y111" s="55"/>
-      <c r="Z111" s="53"/>
-      <c r="AA111" s="56"/>
+      <c r="X111" s="55">
+        <v>48.973178212585935</v>
+      </c>
+      <c r="Y111" s="55">
+        <v>65.70431400737223</v>
+      </c>
+      <c r="Z111" s="53">
+        <v>0.3357</v>
+      </c>
+      <c r="AA111" s="56">
+        <v>0.3616</v>
+      </c>
       <c r="AB111" s="57"/>
       <c r="AD111" s="35"/>
       <c r="AE111" s="35"/>
@@ -18848,30 +19552,74 @@
       <c r="C181" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D181" s="52"/>
-      <c r="E181" s="52"/>
-      <c r="F181" s="52"/>
-      <c r="G181" s="53"/>
-      <c r="H181" s="52"/>
-      <c r="I181" s="52"/>
-      <c r="J181" s="52"/>
-      <c r="K181" s="52"/>
-      <c r="L181" s="52"/>
-      <c r="M181" s="53"/>
+      <c r="D181" s="52">
+        <v>16897.53</v>
+      </c>
+      <c r="E181" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F181" s="52">
+        <v>11405.829999999998</v>
+      </c>
+      <c r="G181" s="53">
+        <v>0.6749998372543206</v>
+      </c>
+      <c r="H181" s="52">
+        <v>9226.27</v>
+      </c>
+      <c r="I181" s="52">
+        <v>3702.78</v>
+      </c>
+      <c r="J181" s="52">
+        <v>2977.1100000000006</v>
+      </c>
+      <c r="K181" s="52">
+        <v>2335.9700000000003</v>
+      </c>
+      <c r="L181" s="52">
+        <v>641.1400000000003</v>
+      </c>
+      <c r="M181" s="53">
+        <v>0.2153565034546927</v>
+      </c>
       <c r="N181" s="53"/>
-      <c r="O181" s="52"/>
-      <c r="P181" s="52"/>
-      <c r="Q181" s="52"/>
-      <c r="R181" s="53"/>
-      <c r="S181" s="54"/>
-      <c r="T181" s="54"/>
-      <c r="U181" s="54"/>
-      <c r="V181" s="53"/>
+      <c r="O181" s="52">
+        <v>6249.16</v>
+      </c>
+      <c r="P181" s="52">
+        <v>1366.81</v>
+      </c>
+      <c r="Q181" s="52">
+        <v>4882.35</v>
+      </c>
+      <c r="R181" s="53">
+        <v>0.7812810041669601</v>
+      </c>
+      <c r="S181" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T181" s="54">
+        <v>23.75</v>
+      </c>
+      <c r="U181" s="54">
+        <v>101.42</v>
+      </c>
+      <c r="V181" s="53">
+        <v>0.8102580490532876</v>
+      </c>
       <c r="W181" s="53"/>
-      <c r="X181" s="55"/>
-      <c r="Y181" s="55"/>
-      <c r="Z181" s="53"/>
-      <c r="AA181" s="56"/>
+      <c r="X181" s="55">
+        <v>75.32294736842105</v>
+      </c>
+      <c r="Y181" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z181" s="53">
+        <v>0.3257</v>
+      </c>
+      <c r="AA181" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB181" s="57"/>
       <c r="AD181" s="35"/>
       <c r="AE181" s="35"/>
@@ -21185,30 +21933,74 @@
       <c r="C230" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D230" s="52"/>
-      <c r="E230" s="52"/>
-      <c r="F230" s="52"/>
-      <c r="G230" s="53"/>
-      <c r="H230" s="52"/>
-      <c r="I230" s="52"/>
-      <c r="J230" s="52"/>
-      <c r="K230" s="52"/>
-      <c r="L230" s="52"/>
-      <c r="M230" s="53"/>
+      <c r="D230" s="52">
+        <v>8795.03</v>
+      </c>
+      <c r="E230" s="52">
+        <v>0</v>
+      </c>
+      <c r="F230" s="52">
+        <v>8795.03</v>
+      </c>
+      <c r="G230" s="53">
+        <v>1</v>
+      </c>
+      <c r="H230" s="52">
+        <v>6369.12</v>
+      </c>
+      <c r="I230" s="52">
+        <v>0</v>
+      </c>
+      <c r="J230" s="52">
+        <v>4527.889999999999</v>
+      </c>
+      <c r="K230" s="52">
+        <v>0</v>
+      </c>
+      <c r="L230" s="52">
+        <v>4527.889999999999</v>
+      </c>
+      <c r="M230" s="53">
+        <v>1</v>
+      </c>
       <c r="N230" s="53"/>
-      <c r="O230" s="52"/>
-      <c r="P230" s="52"/>
-      <c r="Q230" s="52"/>
-      <c r="R230" s="53"/>
-      <c r="S230" s="54"/>
-      <c r="T230" s="54"/>
-      <c r="U230" s="54"/>
-      <c r="V230" s="53"/>
+      <c r="O230" s="52">
+        <v>1841.23</v>
+      </c>
+      <c r="P230" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q230" s="52">
+        <v>1841.23</v>
+      </c>
+      <c r="R230" s="53">
+        <v>1</v>
+      </c>
+      <c r="S230" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="T230" s="54">
+        <v>0</v>
+      </c>
+      <c r="U230" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="V230" s="53">
+        <v>1</v>
+      </c>
       <c r="W230" s="53"/>
-      <c r="X230" s="55"/>
-      <c r="Y230" s="55"/>
-      <c r="Z230" s="53"/>
-      <c r="AA230" s="56"/>
+      <c r="X230" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y230" s="55">
+        <v>65.70711175027087</v>
+      </c>
+      <c r="Z230" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA230" s="56">
+        <v>0.2758</v>
+      </c>
       <c r="AB230" s="57"/>
       <c r="AD230" s="35"/>
       <c r="AE230" s="35"/>

</xml_diff>

<commit_message>
Sync data files (2026-09-07T21:15:40Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17100,7 +17100,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -22683,7 +22683,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD71"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -22697,7 +22697,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -22719,7 +22719,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -22767,7 +22767,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -22785,7 +22785,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -22832,7 +22832,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -22849,7 +22849,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -22899,7 +22899,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -22916,7 +22916,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -22959,7 +22959,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -22976,7 +22976,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23023,7 +23023,7 @@
         <v>24.375135929463628</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23040,7 +23040,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23090,7 +23090,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23107,7 +23107,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23154,7 +23154,7 @@
         <v>89.17785714285712</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23171,7 +23171,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23216,7 +23216,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23233,7 +23233,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23283,7 +23283,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23300,7 +23300,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23339,7 +23339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23356,7 +23356,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23397,7 +23397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23414,7 +23414,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -23453,7 +23453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -23470,7 +23470,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -23515,7 +23515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -23532,7 +23532,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -23575,7 +23575,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -23592,7 +23592,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -23635,7 +23635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -23652,7 +23652,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -23699,7 +23699,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -23716,7 +23716,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -23761,7 +23761,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -23778,7 +23778,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -23821,7 +23821,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -23838,7 +23838,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -23879,7 +23879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -23896,7 +23896,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -23941,7 +23941,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -23958,7 +23958,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24001,7 +24001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24018,7 +24018,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24055,7 +24055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24072,7 +24072,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24113,7 +24113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24130,7 +24130,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24173,7 +24173,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24190,7 +24190,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24232,7 +24232,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24249,7 +24249,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24294,7 +24294,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24311,7 +24311,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24356,7 +24356,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24373,7 +24373,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24418,7 +24418,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -24435,7 +24435,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -24472,7 +24472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -24489,7 +24489,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -24506,7 +24506,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -24523,7 +24523,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -24544,7 +24544,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -24561,7 +24561,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -24602,7 +24602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -24619,7 +24619,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -24664,7 +24664,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -24699,7 +24699,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -24716,7 +24716,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -24733,7 +24733,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -24768,7 +24768,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25151,7 +25151,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD110"/>
+  <dimension ref="A1:AB110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25162,7 +25162,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25183,7 +25183,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25245,7 +25245,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25303,7 +25303,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25339,7 +25339,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25358,7 +25358,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25392,7 +25392,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25411,7 +25411,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -25445,7 +25445,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -25464,7 +25464,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -25502,7 +25502,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -25521,7 +25521,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -25559,7 +25559,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -25578,7 +25578,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -25616,7 +25616,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -25635,7 +25635,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -25668,7 +25668,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -25687,7 +25687,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -25720,7 +25720,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -25739,7 +25739,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -25770,7 +25770,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -25789,7 +25789,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -25824,7 +25824,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -25843,7 +25843,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -25876,7 +25876,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -25895,7 +25895,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25926,7 +25926,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -25945,7 +25945,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25977,7 +25977,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -25996,7 +25996,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26032,7 +26032,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26051,7 +26051,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26080,7 +26080,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26099,7 +26099,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26130,7 +26130,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26149,7 +26149,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26182,7 +26182,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26201,7 +26201,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26237,7 +26237,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26256,7 +26256,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26291,7 +26291,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26310,7 +26310,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26340,7 +26340,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26359,7 +26359,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26399,7 +26399,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26418,7 +26418,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -26447,7 +26447,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -26466,7 +26466,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -26499,7 +26499,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -26518,7 +26518,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -26551,7 +26551,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -26570,7 +26570,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -26606,7 +26606,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -26625,7 +26625,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -26661,7 +26661,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -26680,7 +26680,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -26714,7 +26714,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -26733,7 +26733,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -26768,7 +26768,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -26787,7 +26787,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -26806,7 +26806,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -26825,7 +26825,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -26846,7 +26846,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -26865,7 +26865,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -26898,7 +26898,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -26917,7 +26917,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -26956,7 +26956,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -26985,7 +26985,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27004,7 +27004,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27023,7 +27023,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27042,7 +27042,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27087,7 +27087,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27126,7 +27126,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27155,7 +27155,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27200,7 +27200,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27245,7 +27245,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27264,7 +27264,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27311,7 +27311,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27356,7 +27356,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27375,7 +27375,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27398,7 +27398,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -27421,7 +27421,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -27444,7 +27444,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -27467,7 +27467,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -27490,7 +27490,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -27513,7 +27513,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -27536,7 +27536,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -27559,7 +27559,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -27582,7 +27582,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -27605,7 +27605,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -27628,7 +27628,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -27651,7 +27651,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -27672,7 +27672,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -27693,7 +27693,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -27714,7 +27714,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -27735,7 +27735,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -27756,7 +27756,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -27777,7 +27777,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -27798,7 +27798,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -27821,7 +27821,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -27844,7 +27844,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -27867,7 +27867,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -27890,7 +27890,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -27913,7 +27913,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -27936,7 +27936,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -27959,7 +27959,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -27978,7 +27978,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -27997,7 +27997,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28016,7 +28016,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28035,7 +28035,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28109,11 +28109,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28145,7 +28144,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28178,7 +28177,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28211,7 +28210,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28244,7 +28243,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28277,7 +28276,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28310,7 +28309,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28343,7 +28342,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28376,7 +28375,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28407,7 +28406,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -28438,7 +28437,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -28471,7 +28470,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -28504,7 +28503,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -28537,7 +28536,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -28570,7 +28569,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -28603,7 +28602,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -28636,7 +28635,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -28669,7 +28668,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -28702,7 +28701,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -28735,7 +28734,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -28768,7 +28767,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -28801,7 +28800,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -28834,7 +28833,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -28867,7 +28866,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -28900,7 +28899,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -28933,7 +28932,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -28966,7 +28965,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -28998,7 +28997,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29030,7 +29029,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29062,7 +29061,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29094,7 +29093,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29126,7 +29125,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29156,7 +29155,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29186,7 +29185,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29218,7 +29217,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29250,7 +29249,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29282,7 +29281,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29314,7 +29313,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29346,7 +29345,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29376,7 +29375,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29408,7 +29407,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -29440,7 +29439,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -29472,7 +29471,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -29504,7 +29503,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -29534,7 +29533,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -29564,7 +29563,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -29594,7 +29593,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -29624,7 +29623,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -29656,7 +29655,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -29688,7 +29687,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -29718,7 +29717,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -29748,7 +29747,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -29778,7 +29777,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -29808,7 +29807,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -29838,7 +29837,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -29933,11 +29932,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -29969,7 +29967,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30000,7 +29998,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30031,7 +30029,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30062,7 +30060,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30093,7 +30091,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30124,7 +30122,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30155,7 +30153,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30186,7 +30184,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30217,7 +30215,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30248,7 +30246,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30279,7 +30277,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30310,7 +30308,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30341,7 +30339,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30372,7 +30370,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30403,7 +30401,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -30434,7 +30432,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -30465,7 +30463,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -30496,7 +30494,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -30527,7 +30525,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -30558,7 +30556,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -30588,7 +30586,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -30618,7 +30616,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -30648,7 +30646,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -30678,7 +30676,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -30708,7 +30706,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -30738,7 +30736,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -30768,7 +30766,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -30798,7 +30796,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -30828,7 +30826,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -30858,7 +30856,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -30888,7 +30886,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -30918,7 +30916,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -30948,7 +30946,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -30978,7 +30976,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31008,7 +31006,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31038,7 +31036,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -31070,7 +31068,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -31102,7 +31100,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31132,7 +31130,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31162,7 +31160,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31192,7 +31190,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31222,7 +31220,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31252,7 +31250,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -52995,19 +52993,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53021,7 +53019,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -53033,7 +53031,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -53044,7 +53042,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -53055,7 +53053,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -53066,13 +53064,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Sync data files (2026-09-07T21:23:05Z)
</commit_message>
<xml_diff>
--- a/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17100,7 +17100,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -17432,30 +17432,74 @@
       <c r="C139" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D139" s="52"/>
-      <c r="E139" s="52"/>
-      <c r="F139" s="52"/>
-      <c r="G139" s="53"/>
-      <c r="H139" s="52"/>
-      <c r="I139" s="52"/>
-      <c r="J139" s="52"/>
-      <c r="K139" s="52"/>
-      <c r="L139" s="52"/>
-      <c r="M139" s="53"/>
+      <c r="D139" s="52">
+        <v>30749.24</v>
+      </c>
+      <c r="E139" s="52">
+        <v>30749.24</v>
+      </c>
+      <c r="F139" s="52">
+        <v>0</v>
+      </c>
+      <c r="G139" s="53">
+        <v>0</v>
+      </c>
+      <c r="H139" s="52">
+        <v>22587.89</v>
+      </c>
+      <c r="I139" s="52">
+        <v>25905.23</v>
+      </c>
+      <c r="J139" s="52">
+        <v>12565.06</v>
+      </c>
+      <c r="K139" s="52">
+        <v>11805.46</v>
+      </c>
+      <c r="L139" s="52">
+        <v>759.6000000000004</v>
+      </c>
+      <c r="M139" s="53">
+        <v>0.06045335239147289</v>
+      </c>
       <c r="N139" s="53"/>
-      <c r="O139" s="52"/>
-      <c r="P139" s="52"/>
-      <c r="Q139" s="52"/>
-      <c r="R139" s="53"/>
-      <c r="S139" s="54"/>
-      <c r="T139" s="54"/>
-      <c r="U139" s="54"/>
-      <c r="V139" s="53"/>
+      <c r="O139" s="52">
+        <v>10022.83</v>
+      </c>
+      <c r="P139" s="52">
+        <v>14099.77</v>
+      </c>
+      <c r="Q139" s="52">
+        <v>-4076.9400000000005</v>
+      </c>
+      <c r="R139" s="53">
+        <v>-0.40676535469523084</v>
+      </c>
+      <c r="S139" s="54">
+        <v>200.82</v>
+      </c>
+      <c r="T139" s="54">
+        <v>283.75</v>
+      </c>
+      <c r="U139" s="54">
+        <v>-82.93</v>
+      </c>
+      <c r="V139" s="53">
+        <v>-0.4129568768050991</v>
+      </c>
       <c r="W139" s="53"/>
-      <c r="X139" s="55"/>
-      <c r="Y139" s="55"/>
-      <c r="Z139" s="53"/>
-      <c r="AA139" s="56"/>
+      <c r="X139" s="55">
+        <v>17.07140088105727</v>
+      </c>
+      <c r="Y139" s="55">
+        <v>40.64013272149188</v>
+      </c>
+      <c r="Z139" s="53">
+        <v>0.1575</v>
+      </c>
+      <c r="AA139" s="56">
+        <v>0.2654</v>
+      </c>
       <c r="AB139" s="57"/>
       <c r="AD139" s="35"/>
       <c r="AE139" s="35"/>
@@ -17785,30 +17829,74 @@
       <c r="C146" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D146" s="52"/>
-      <c r="E146" s="52"/>
-      <c r="F146" s="52"/>
-      <c r="G146" s="53"/>
-      <c r="H146" s="52"/>
-      <c r="I146" s="52"/>
-      <c r="J146" s="52"/>
-      <c r="K146" s="52"/>
-      <c r="L146" s="52"/>
-      <c r="M146" s="53"/>
+      <c r="D146" s="52">
+        <v>268228.26</v>
+      </c>
+      <c r="E146" s="52">
+        <v>9034.53</v>
+      </c>
+      <c r="F146" s="52">
+        <v>259193.73</v>
+      </c>
+      <c r="G146" s="53">
+        <v>0.9663177548853353</v>
+      </c>
+      <c r="H146" s="52">
+        <v>238611.58</v>
+      </c>
+      <c r="I146" s="52">
+        <v>6362.08</v>
+      </c>
+      <c r="J146" s="52">
+        <v>214154.25</v>
+      </c>
+      <c r="K146" s="52">
+        <v>3465.35</v>
+      </c>
+      <c r="L146" s="52">
+        <v>210688.9</v>
+      </c>
+      <c r="M146" s="53">
+        <v>0.9838184392791645</v>
+      </c>
       <c r="N146" s="53"/>
-      <c r="O146" s="52"/>
-      <c r="P146" s="52"/>
-      <c r="Q146" s="52"/>
-      <c r="R146" s="53"/>
-      <c r="S146" s="54"/>
-      <c r="T146" s="54"/>
-      <c r="U146" s="54"/>
-      <c r="V146" s="53"/>
+      <c r="O146" s="52">
+        <v>24457.33</v>
+      </c>
+      <c r="P146" s="52">
+        <v>2896.73</v>
+      </c>
+      <c r="Q146" s="52">
+        <v>21560.600000000002</v>
+      </c>
+      <c r="R146" s="53">
+        <v>0.8815598432044708</v>
+      </c>
+      <c r="S146" s="54">
+        <v>497.55</v>
+      </c>
+      <c r="T146" s="54">
+        <v>58.25</v>
+      </c>
+      <c r="U146" s="54">
+        <v>439.3</v>
+      </c>
+      <c r="V146" s="53">
+        <v>0.8829263390614008</v>
+      </c>
       <c r="W146" s="53"/>
-      <c r="X146" s="55"/>
-      <c r="Y146" s="55"/>
-      <c r="Z146" s="53"/>
-      <c r="AA146" s="56"/>
+      <c r="X146" s="55">
+        <v>45.878969957081544</v>
+      </c>
+      <c r="Y146" s="55">
+        <v>59.525035875791396</v>
+      </c>
+      <c r="Z146" s="53">
+        <v>0.2958</v>
+      </c>
+      <c r="AA146" s="56">
+        <v>0.1104</v>
+      </c>
       <c r="AB146" s="57"/>
       <c r="AD146" s="35"/>
       <c r="AE146" s="35"/>
@@ -18142,30 +18230,74 @@
       <c r="C153" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D153" s="52"/>
-      <c r="E153" s="52"/>
-      <c r="F153" s="52"/>
-      <c r="G153" s="53"/>
-      <c r="H153" s="52"/>
-      <c r="I153" s="52"/>
-      <c r="J153" s="52"/>
-      <c r="K153" s="52"/>
-      <c r="L153" s="52"/>
-      <c r="M153" s="53"/>
+      <c r="D153" s="52">
+        <v>32773.41</v>
+      </c>
+      <c r="E153" s="52">
+        <v>32773.41</v>
+      </c>
+      <c r="F153" s="52">
+        <v>0</v>
+      </c>
+      <c r="G153" s="53">
+        <v>0</v>
+      </c>
+      <c r="H153" s="52">
+        <v>22750.99</v>
+      </c>
+      <c r="I153" s="52">
+        <v>22254.11</v>
+      </c>
+      <c r="J153" s="52">
+        <v>12243.410000000002</v>
+      </c>
+      <c r="K153" s="52">
+        <v>9324.41</v>
+      </c>
+      <c r="L153" s="52">
+        <v>2919.000000000002</v>
+      </c>
+      <c r="M153" s="53">
+        <v>0.23841397127107575</v>
+      </c>
       <c r="N153" s="53"/>
-      <c r="O153" s="52"/>
-      <c r="P153" s="52"/>
-      <c r="Q153" s="52"/>
-      <c r="R153" s="53"/>
-      <c r="S153" s="54"/>
-      <c r="T153" s="54"/>
-      <c r="U153" s="54"/>
-      <c r="V153" s="53"/>
+      <c r="O153" s="52">
+        <v>10507.58</v>
+      </c>
+      <c r="P153" s="52">
+        <v>12929.7</v>
+      </c>
+      <c r="Q153" s="52">
+        <v>-2422.120000000001</v>
+      </c>
+      <c r="R153" s="53">
+        <v>-0.23051168775303169</v>
+      </c>
+      <c r="S153" s="54">
+        <v>210.6</v>
+      </c>
+      <c r="T153" s="54">
+        <v>260.75</v>
+      </c>
+      <c r="U153" s="54">
+        <v>-50.150000000000006</v>
+      </c>
+      <c r="V153" s="53">
+        <v>-0.2381291547958215</v>
+      </c>
       <c r="W153" s="53"/>
-      <c r="X153" s="55"/>
-      <c r="Y153" s="55"/>
-      <c r="Z153" s="53"/>
-      <c r="AA153" s="56"/>
+      <c r="X153" s="55">
+        <v>40.342473633748796</v>
+      </c>
+      <c r="Y153" s="55">
+        <v>47.58984852136751</v>
+      </c>
+      <c r="Z153" s="53">
+        <v>0.321</v>
+      </c>
+      <c r="AA153" s="56">
+        <v>0.3058</v>
+      </c>
       <c r="AB153" s="57"/>
       <c r="AD153" s="35"/>
       <c r="AE153" s="35"/>
@@ -18499,30 +18631,74 @@
       <c r="C160" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D160" s="52"/>
-      <c r="E160" s="52"/>
-      <c r="F160" s="52"/>
-      <c r="G160" s="53"/>
-      <c r="H160" s="52"/>
-      <c r="I160" s="52"/>
-      <c r="J160" s="52"/>
-      <c r="K160" s="52"/>
-      <c r="L160" s="52"/>
-      <c r="M160" s="53"/>
+      <c r="D160" s="52">
+        <v>17899.33</v>
+      </c>
+      <c r="E160" s="52">
+        <v>13424.5</v>
+      </c>
+      <c r="F160" s="52">
+        <v>4474.830000000002</v>
+      </c>
+      <c r="G160" s="53">
+        <v>0.24999986032996774</v>
+      </c>
+      <c r="H160" s="52">
+        <v>13919.4</v>
+      </c>
+      <c r="I160" s="52">
+        <v>10402.37</v>
+      </c>
+      <c r="J160" s="52">
+        <v>8410.93</v>
+      </c>
+      <c r="K160" s="52">
+        <v>7278.380000000001</v>
+      </c>
+      <c r="L160" s="52">
+        <v>1132.5499999999993</v>
+      </c>
+      <c r="M160" s="53">
+        <v>0.13465217282749936</v>
+      </c>
       <c r="N160" s="53"/>
-      <c r="O160" s="52"/>
-      <c r="P160" s="52"/>
-      <c r="Q160" s="52"/>
-      <c r="R160" s="53"/>
-      <c r="S160" s="54"/>
-      <c r="T160" s="54"/>
-      <c r="U160" s="54"/>
-      <c r="V160" s="53"/>
+      <c r="O160" s="52">
+        <v>5508.47</v>
+      </c>
+      <c r="P160" s="52">
+        <v>3123.99</v>
+      </c>
+      <c r="Q160" s="52">
+        <v>2384.4800000000005</v>
+      </c>
+      <c r="R160" s="53">
+        <v>0.43287519038861977</v>
+      </c>
+      <c r="S160" s="54">
+        <v>110.44</v>
+      </c>
+      <c r="T160" s="54">
+        <v>60.75</v>
+      </c>
+      <c r="U160" s="54">
+        <v>49.69</v>
+      </c>
+      <c r="V160" s="53">
+        <v>0.44992756247736326</v>
+      </c>
       <c r="W160" s="53"/>
-      <c r="X160" s="55"/>
-      <c r="Y160" s="55"/>
-      <c r="Z160" s="53"/>
-      <c r="AA160" s="56"/>
+      <c r="X160" s="55">
+        <v>49.74699588477367</v>
+      </c>
+      <c r="Y160" s="55">
+        <v>36.03704967040926</v>
+      </c>
+      <c r="Z160" s="53">
+        <v>0.22510000000000002</v>
+      </c>
+      <c r="AA160" s="56">
+        <v>0.2224</v>
+      </c>
       <c r="AB160" s="57"/>
       <c r="AD160" s="35"/>
       <c r="AE160" s="35"/>
@@ -18838,30 +19014,74 @@
       <c r="C167" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D167" s="52"/>
-      <c r="E167" s="52"/>
-      <c r="F167" s="52"/>
-      <c r="G167" s="53"/>
-      <c r="H167" s="52"/>
-      <c r="I167" s="52"/>
-      <c r="J167" s="52"/>
-      <c r="K167" s="52"/>
-      <c r="L167" s="52"/>
-      <c r="M167" s="53"/>
+      <c r="D167" s="52">
+        <v>10827.2</v>
+      </c>
+      <c r="E167" s="52">
+        <v>0</v>
+      </c>
+      <c r="F167" s="52">
+        <v>10827.2</v>
+      </c>
+      <c r="G167" s="53">
+        <v>1</v>
+      </c>
+      <c r="H167" s="52">
+        <v>7687.77</v>
+      </c>
+      <c r="I167" s="52">
+        <v>2116.21</v>
+      </c>
+      <c r="J167" s="52">
+        <v>4437.14</v>
+      </c>
+      <c r="K167" s="52">
+        <v>1029.51</v>
+      </c>
+      <c r="L167" s="52">
+        <v>3407.63</v>
+      </c>
+      <c r="M167" s="53">
+        <v>0.7679789233605431</v>
+      </c>
       <c r="N167" s="53"/>
-      <c r="O167" s="52"/>
-      <c r="P167" s="52"/>
-      <c r="Q167" s="52"/>
-      <c r="R167" s="53"/>
-      <c r="S167" s="54"/>
-      <c r="T167" s="54"/>
-      <c r="U167" s="54"/>
-      <c r="V167" s="53"/>
+      <c r="O167" s="52">
+        <v>3250.63</v>
+      </c>
+      <c r="P167" s="52">
+        <v>1086.7</v>
+      </c>
+      <c r="Q167" s="52">
+        <v>2163.9300000000003</v>
+      </c>
+      <c r="R167" s="53">
+        <v>0.6656955728581845</v>
+      </c>
+      <c r="S167" s="54">
+        <v>65.13</v>
+      </c>
+      <c r="T167" s="54">
+        <v>24.33</v>
+      </c>
+      <c r="U167" s="54">
+        <v>40.8</v>
+      </c>
+      <c r="V167" s="53">
+        <v>0.6264394288346384</v>
+      </c>
       <c r="W167" s="53"/>
-      <c r="X167" s="55"/>
-      <c r="Y167" s="55"/>
-      <c r="Z167" s="53"/>
-      <c r="AA167" s="56"/>
+      <c r="X167" s="55">
+        <v>-86.97944923962187</v>
+      </c>
+      <c r="Y167" s="55">
+        <v>48.202633430830645</v>
+      </c>
+      <c r="Z167" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA167" s="56">
+        <v>0.29</v>
+      </c>
       <c r="AB167" s="57"/>
       <c r="AD167" s="35"/>
       <c r="AE167" s="35"/>
@@ -19191,30 +19411,74 @@
       <c r="C174" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D174" s="52"/>
-      <c r="E174" s="52"/>
-      <c r="F174" s="52"/>
-      <c r="G174" s="53"/>
-      <c r="H174" s="52"/>
-      <c r="I174" s="52"/>
-      <c r="J174" s="52"/>
-      <c r="K174" s="52"/>
-      <c r="L174" s="52"/>
-      <c r="M174" s="53"/>
+      <c r="D174" s="52">
+        <v>146237.11</v>
+      </c>
+      <c r="E174" s="52">
+        <v>125386.21</v>
+      </c>
+      <c r="F174" s="52">
+        <v>20850.89999999998</v>
+      </c>
+      <c r="G174" s="53">
+        <v>0.14258282319720336</v>
+      </c>
+      <c r="H174" s="52">
+        <v>114651.87</v>
+      </c>
+      <c r="I174" s="52">
+        <v>105118.87</v>
+      </c>
+      <c r="J174" s="52">
+        <v>82888.07999999999</v>
+      </c>
+      <c r="K174" s="52">
+        <v>77768.29999999999</v>
+      </c>
+      <c r="L174" s="52">
+        <v>5119.779999999999</v>
+      </c>
+      <c r="M174" s="53">
+        <v>0.06176738561202044</v>
+      </c>
       <c r="N174" s="53"/>
-      <c r="O174" s="52"/>
-      <c r="P174" s="52"/>
-      <c r="Q174" s="52"/>
-      <c r="R174" s="53"/>
-      <c r="S174" s="54"/>
-      <c r="T174" s="54"/>
-      <c r="U174" s="54"/>
-      <c r="V174" s="53"/>
+      <c r="O174" s="52">
+        <v>31763.79</v>
+      </c>
+      <c r="P174" s="52">
+        <v>27350.57</v>
+      </c>
+      <c r="Q174" s="52">
+        <v>4413.220000000001</v>
+      </c>
+      <c r="R174" s="53">
+        <v>0.13893870976983544</v>
+      </c>
+      <c r="S174" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T174" s="54">
+        <v>548.75</v>
+      </c>
+      <c r="U174" s="54">
+        <v>110.98000000000002</v>
+      </c>
+      <c r="V174" s="53">
+        <v>0.16822033256028984</v>
+      </c>
       <c r="W174" s="53"/>
-      <c r="X174" s="55"/>
-      <c r="Y174" s="55"/>
-      <c r="Z174" s="53"/>
-      <c r="AA174" s="56"/>
+      <c r="X174" s="55">
+        <v>36.933649202733484</v>
+      </c>
+      <c r="Y174" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z174" s="53">
+        <v>0.1616</v>
+      </c>
+      <c r="AA174" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB174" s="57"/>
       <c r="AD174" s="35"/>
       <c r="AE174" s="35"/>
@@ -19953,30 +20217,74 @@
       <c r="C188" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D188" s="52"/>
-      <c r="E188" s="52"/>
-      <c r="F188" s="52"/>
-      <c r="G188" s="53"/>
-      <c r="H188" s="52"/>
-      <c r="I188" s="52"/>
-      <c r="J188" s="52"/>
-      <c r="K188" s="52"/>
-      <c r="L188" s="52"/>
-      <c r="M188" s="53"/>
+      <c r="D188" s="52">
+        <v>20992.12</v>
+      </c>
+      <c r="E188" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F188" s="52">
+        <v>6822.439999999999</v>
+      </c>
+      <c r="G188" s="53">
+        <v>0.32500004763692275</v>
+      </c>
+      <c r="H188" s="52">
+        <v>16299.09</v>
+      </c>
+      <c r="I188" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J188" s="52">
+        <v>9784.33</v>
+      </c>
+      <c r="K188" s="52">
+        <v>8137.88</v>
+      </c>
+      <c r="L188" s="52">
+        <v>1646.4499999999998</v>
+      </c>
+      <c r="M188" s="53">
+        <v>0.16827416900288522</v>
+      </c>
       <c r="N188" s="53"/>
-      <c r="O188" s="52"/>
-      <c r="P188" s="52"/>
-      <c r="Q188" s="52"/>
-      <c r="R188" s="53"/>
-      <c r="S188" s="54"/>
-      <c r="T188" s="54"/>
-      <c r="U188" s="54"/>
-      <c r="V188" s="53"/>
+      <c r="O188" s="52">
+        <v>6514.76</v>
+      </c>
+      <c r="P188" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q188" s="52">
+        <v>4953.13</v>
+      </c>
+      <c r="R188" s="53">
+        <v>0.7602935488030257</v>
+      </c>
+      <c r="S188" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T188" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U188" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V188" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W188" s="53"/>
-      <c r="X188" s="55"/>
-      <c r="Y188" s="55"/>
-      <c r="Z188" s="53"/>
-      <c r="AA188" s="56"/>
+      <c r="X188" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y188" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z188" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA188" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB188" s="57"/>
       <c r="AD188" s="35"/>
       <c r="AE188" s="35"/>
@@ -20304,30 +20612,74 @@
       <c r="C195" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D195" s="52"/>
-      <c r="E195" s="52"/>
-      <c r="F195" s="52"/>
-      <c r="G195" s="53"/>
-      <c r="H195" s="52"/>
-      <c r="I195" s="52"/>
-      <c r="J195" s="52"/>
-      <c r="K195" s="52"/>
-      <c r="L195" s="52"/>
-      <c r="M195" s="53"/>
+      <c r="D195" s="52">
+        <v>23770.95</v>
+      </c>
+      <c r="E195" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F195" s="52">
+        <v>13566.41</v>
+      </c>
+      <c r="G195" s="53">
+        <v>0.5707138334816235</v>
+      </c>
+      <c r="H195" s="52">
+        <v>14310.96</v>
+      </c>
+      <c r="I195" s="52">
+        <v>6935.96</v>
+      </c>
+      <c r="J195" s="52">
+        <v>7389.339999999999</v>
+      </c>
+      <c r="K195" s="52">
+        <v>6605.05</v>
+      </c>
+      <c r="L195" s="52">
+        <v>784.289999999999</v>
+      </c>
+      <c r="M195" s="53">
+        <v>0.1061380312720756</v>
+      </c>
       <c r="N195" s="53"/>
-      <c r="O195" s="52"/>
-      <c r="P195" s="52"/>
-      <c r="Q195" s="52"/>
-      <c r="R195" s="53"/>
-      <c r="S195" s="54"/>
-      <c r="T195" s="54"/>
-      <c r="U195" s="54"/>
-      <c r="V195" s="53"/>
+      <c r="O195" s="52">
+        <v>6921.62</v>
+      </c>
+      <c r="P195" s="52">
+        <v>330.91</v>
+      </c>
+      <c r="Q195" s="52">
+        <v>6590.71</v>
+      </c>
+      <c r="R195" s="53">
+        <v>0.9521918279246766</v>
+      </c>
+      <c r="S195" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T195" s="54">
+        <v>5.75</v>
+      </c>
+      <c r="U195" s="54">
+        <v>134.4</v>
+      </c>
+      <c r="V195" s="53">
+        <v>0.9589725294327506</v>
+      </c>
       <c r="W195" s="53"/>
-      <c r="X195" s="55"/>
-      <c r="Y195" s="55"/>
-      <c r="Z195" s="53"/>
-      <c r="AA195" s="56"/>
+      <c r="X195" s="55">
+        <v>568.4486956521739</v>
+      </c>
+      <c r="Y195" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z195" s="53">
+        <v>0.32030000000000003</v>
+      </c>
+      <c r="AA195" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB195" s="57"/>
       <c r="AD195" s="35"/>
       <c r="AE195" s="35"/>
@@ -21233,30 +21585,74 @@
       <c r="C216" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D216" s="52"/>
-      <c r="E216" s="52"/>
-      <c r="F216" s="52"/>
-      <c r="G216" s="53"/>
-      <c r="H216" s="52"/>
-      <c r="I216" s="52"/>
-      <c r="J216" s="52"/>
-      <c r="K216" s="52"/>
-      <c r="L216" s="52"/>
-      <c r="M216" s="53"/>
+      <c r="D216" s="52">
+        <v>137109.56</v>
+      </c>
+      <c r="E216" s="52">
+        <v>30174.75</v>
+      </c>
+      <c r="F216" s="52">
+        <v>106934.81</v>
+      </c>
+      <c r="G216" s="53">
+        <v>0.7799223482301307</v>
+      </c>
+      <c r="H216" s="52">
+        <v>117394.57</v>
+      </c>
+      <c r="I216" s="52">
+        <v>30594.96</v>
+      </c>
+      <c r="J216" s="52">
+        <v>99479.62000000001</v>
+      </c>
+      <c r="K216" s="52">
+        <v>30594.96</v>
+      </c>
+      <c r="L216" s="52">
+        <v>68884.66</v>
+      </c>
+      <c r="M216" s="53">
+        <v>0.692449971159922</v>
+      </c>
       <c r="N216" s="53"/>
-      <c r="O216" s="52"/>
-      <c r="P216" s="52"/>
-      <c r="Q216" s="52"/>
-      <c r="R216" s="53"/>
-      <c r="S216" s="54"/>
-      <c r="T216" s="54"/>
-      <c r="U216" s="54"/>
-      <c r="V216" s="53"/>
+      <c r="O216" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="P216" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q216" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="R216" s="53">
+        <v>1</v>
+      </c>
+      <c r="S216" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T216" s="54">
+        <v>0</v>
+      </c>
+      <c r="U216" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V216" s="53">
+        <v>1</v>
+      </c>
       <c r="W216" s="53"/>
-      <c r="X216" s="55"/>
-      <c r="Y216" s="55"/>
-      <c r="Z216" s="53"/>
-      <c r="AA216" s="56"/>
+      <c r="X216" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y216" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z216" s="53">
+        <v>-0.0139</v>
+      </c>
+      <c r="AA216" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB216" s="57"/>
       <c r="AD216" s="35"/>
       <c r="AE216" s="35"/>
@@ -21586,30 +21982,74 @@
       <c r="C223" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D223" s="52"/>
-      <c r="E223" s="52"/>
-      <c r="F223" s="52"/>
-      <c r="G223" s="53"/>
-      <c r="H223" s="52"/>
-      <c r="I223" s="52"/>
-      <c r="J223" s="52"/>
-      <c r="K223" s="52"/>
-      <c r="L223" s="52"/>
-      <c r="M223" s="53"/>
+      <c r="D223" s="52">
+        <v>396453.46</v>
+      </c>
+      <c r="E223" s="52">
+        <v>306038.55</v>
+      </c>
+      <c r="F223" s="52">
+        <v>90414.91000000003</v>
+      </c>
+      <c r="G223" s="53">
+        <v>0.2280593288301735</v>
+      </c>
+      <c r="H223" s="52">
+        <v>295569.99</v>
+      </c>
+      <c r="I223" s="52">
+        <v>245307.56</v>
+      </c>
+      <c r="J223" s="52">
+        <v>178700.37</v>
+      </c>
+      <c r="K223" s="52">
+        <v>180550.95</v>
+      </c>
+      <c r="L223" s="52">
+        <v>-1850.5800000000163</v>
+      </c>
+      <c r="M223" s="53">
+        <v>-0.010355770388164369</v>
+      </c>
       <c r="N223" s="53"/>
-      <c r="O223" s="52"/>
-      <c r="P223" s="52"/>
-      <c r="Q223" s="52"/>
-      <c r="R223" s="53"/>
-      <c r="S223" s="54"/>
-      <c r="T223" s="54"/>
-      <c r="U223" s="54"/>
-      <c r="V223" s="53"/>
+      <c r="O223" s="52">
+        <v>116869.62</v>
+      </c>
+      <c r="P223" s="52">
+        <v>64756.61</v>
+      </c>
+      <c r="Q223" s="52">
+        <v>52113.009999999995</v>
+      </c>
+      <c r="R223" s="53">
+        <v>0.4459072426178848</v>
+      </c>
+      <c r="S223" s="54">
+        <v>2344.68</v>
+      </c>
+      <c r="T223" s="54">
+        <v>1377.92</v>
+      </c>
+      <c r="U223" s="54">
+        <v>966.7599999999998</v>
+      </c>
+      <c r="V223" s="53">
+        <v>0.4123206578296398</v>
+      </c>
       <c r="W223" s="53"/>
-      <c r="X223" s="55"/>
-      <c r="Y223" s="55"/>
-      <c r="Z223" s="53"/>
-      <c r="AA223" s="56"/>
+      <c r="X223" s="55">
+        <v>44.07439473989781</v>
+      </c>
+      <c r="Y223" s="55">
+        <v>43.0265399367206</v>
+      </c>
+      <c r="Z223" s="53">
+        <v>0.1984</v>
+      </c>
+      <c r="AA223" s="56">
+        <v>0.2545</v>
+      </c>
       <c r="AB223" s="57"/>
       <c r="AD223" s="35"/>
       <c r="AE223" s="35"/>
@@ -22683,7 +23123,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:AD71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -22697,7 +23137,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -22719,7 +23159,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -22767,7 +23207,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -22785,7 +23225,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -22832,7 +23272,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -22849,7 +23289,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -22899,7 +23339,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -22916,7 +23356,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -22959,7 +23399,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -22976,7 +23416,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23023,7 +23463,7 @@
         <v>24.375135929463628</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23040,7 +23480,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23090,7 +23530,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23107,7 +23547,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23154,7 +23594,7 @@
         <v>89.17785714285712</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23171,7 +23611,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23216,7 +23656,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23233,7 +23673,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23283,7 +23723,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23300,7 +23740,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23339,7 +23779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23356,7 +23796,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23397,7 +23837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23414,7 +23854,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -23453,7 +23893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -23470,7 +23910,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -23515,7 +23955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -23532,7 +23972,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -23575,7 +24015,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -23592,7 +24032,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -23635,7 +24075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -23652,7 +24092,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -23699,7 +24139,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -23716,7 +24156,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -23761,7 +24201,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -23778,7 +24218,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -23821,7 +24261,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -23838,7 +24278,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -23879,7 +24319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -23896,7 +24336,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -23941,7 +24381,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -23958,7 +24398,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24001,7 +24441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24018,7 +24458,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24055,7 +24495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24072,7 +24512,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24113,7 +24553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24130,7 +24570,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24173,7 +24613,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24190,7 +24630,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24201,10 +24641,10 @@
         <v>0</v>
       </c>
       <c r="D50" s="99">
-        <v>853.55</v>
+        <v>2116.21</v>
       </c>
       <c r="E50" s="99">
-        <v>-853.55</v>
+        <v>-2116.21</v>
       </c>
       <c r="F50" s="99"/>
       <c r="G50" s="100">
@@ -24222,7 +24662,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="99">
-        <v>-853.55</v>
+        <v>-2116.21</v>
       </c>
       <c r="N50" s="98"/>
       <c r="O50" s="60">
@@ -24232,7 +24672,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24249,7 +24689,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24260,10 +24700,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>2629.5100000000093</v>
+        <v>2236.75</v>
       </c>
       <c r="E52" s="99">
-        <v>-2629.5100000000093</v>
+        <v>-2236.75</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -24285,16 +24725,16 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-3909.5100000000093</v>
+        <v>-3516.75</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>14.333675527039448</v>
-      </c>
-    </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>12.893675527039413</v>
+      </c>
+    </row>
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24311,7 +24751,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24356,7 +24796,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24373,7 +24813,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24418,7 +24858,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -24435,7 +24875,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -24472,7 +24912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -24489,7 +24929,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -24506,7 +24946,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -24523,7 +24963,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -24544,7 +24984,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -24561,7 +25001,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -24602,7 +25042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -24619,7 +25059,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -24630,14 +25070,14 @@
         <v>34650.399999999965</v>
       </c>
       <c r="D66" s="99">
-        <v>7430.429999999993</v>
+        <v>10984.75</v>
       </c>
       <c r="E66" s="99">
-        <v>27219.969999999972</v>
+        <v>23665.649999999965</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.7855600512548195</v>
+        <v>0.6829834576224225</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -24652,19 +25092,19 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.6932090250040402</v>
+        <v>0.5906324313716432</v>
       </c>
       <c r="M66" s="99">
-        <v>24019.969999999972</v>
+        <v>20465.649999999965</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-25.71043082686644</v>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-21.90596735349207</v>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -24699,7 +25139,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -24716,7 +25156,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -24733,7 +25173,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -24744,22 +25184,22 @@
         <v>88818.76999999996</v>
       </c>
       <c r="D70" s="104">
-        <v>39414.08000000001</v>
+        <v>43838.3</v>
       </c>
       <c r="E70" s="105">
-        <v>49404.68999999996</v>
+        <v>44980.469999999965</v>
       </c>
       <c r="F70" s="106" t="s">
         <v>124</v>
       </c>
       <c r="G70" s="107">
-        <v>0.5562415466910877</v>
+        <v>0.5064297783002397</v>
       </c>
       <c r="H70" s="108" t="s">
         <v>125</v>
       </c>
       <c r="I70" s="109">
-        <v>-0.02733555080756062</v>
+        <v>-0.07714731919840859</v>
       </c>
       <c r="J70" s="36"/>
       <c r="K70" s="36"/>
@@ -24768,7 +25208,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25151,7 +25591,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB110"/>
+  <dimension ref="A1:AD110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25162,7 +25602,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25183,7 +25623,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25245,7 +25685,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25303,7 +25743,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25339,7 +25779,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25358,7 +25798,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25392,7 +25832,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25411,7 +25851,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -25445,7 +25885,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -25464,7 +25904,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -25502,7 +25942,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -25521,7 +25961,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -25559,7 +25999,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -25578,7 +26018,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -25616,7 +26056,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -25635,7 +26075,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -25668,7 +26108,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -25687,7 +26127,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -25720,7 +26160,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -25739,7 +26179,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -25770,7 +26210,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -25789,7 +26229,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -25824,7 +26264,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -25843,7 +26283,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -25876,7 +26316,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -25895,7 +26335,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25926,7 +26366,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -25945,7 +26385,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25977,7 +26417,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -25996,7 +26436,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26032,7 +26472,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26051,7 +26491,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26080,7 +26520,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26099,7 +26539,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26130,7 +26570,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26149,7 +26589,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26182,7 +26622,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26201,7 +26641,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26237,7 +26677,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26256,7 +26696,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26291,7 +26731,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26310,7 +26750,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26340,7 +26780,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26359,7 +26799,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26399,7 +26839,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26418,7 +26858,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -26447,7 +26887,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -26466,7 +26906,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -26499,7 +26939,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -26518,7 +26958,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -26529,10 +26969,10 @@
         <v>65.13</v>
       </c>
       <c r="D50" s="54">
-        <v>0</v>
+        <v>24.33</v>
       </c>
       <c r="E50" s="54">
-        <v>65.13</v>
+        <v>40.8</v>
       </c>
       <c r="F50" s="54"/>
       <c r="G50" s="54"/>
@@ -26551,7 +26991,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -26570,7 +27010,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -26606,7 +27046,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -26625,7 +27065,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -26661,7 +27101,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -26680,7 +27120,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -26714,7 +27154,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -26733,7 +27173,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -26768,7 +27208,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -26787,7 +27227,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -26806,7 +27246,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -26825,7 +27265,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -26846,7 +27286,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -26865,7 +27305,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -26898,7 +27338,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -26917,7 +27357,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -26928,10 +27368,10 @@
         <v>2344.68</v>
       </c>
       <c r="D66" s="54">
-        <v>1335</v>
+        <v>1377.92</v>
       </c>
       <c r="E66" s="54">
-        <v>1009.6799999999998</v>
+        <v>966.7599999999998</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>
@@ -26956,7 +27396,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -26985,7 +27425,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27004,7 +27444,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27023,7 +27463,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27042,7 +27482,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27087,7 +27527,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27126,7 +27566,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27155,7 +27595,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27200,7 +27640,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27245,7 +27685,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27264,7 +27704,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27311,7 +27751,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27356,7 +27796,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27375,7 +27815,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27398,7 +27838,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -27421,7 +27861,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -27444,7 +27884,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -27467,7 +27907,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -27490,7 +27930,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -27513,7 +27953,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -27536,7 +27976,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -27559,7 +27999,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -27582,7 +28022,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -27605,7 +28045,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -27628,7 +28068,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -27651,7 +28091,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -27672,7 +28112,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -27693,7 +28133,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -27714,7 +28154,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -27735,7 +28175,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -27756,7 +28196,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -27777,7 +28217,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -27798,7 +28238,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -27821,7 +28261,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -27844,7 +28284,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -27867,7 +28307,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -27890,7 +28330,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -27913,7 +28353,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -27936,7 +28376,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -27959,7 +28399,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -27978,7 +28418,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -27997,7 +28437,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28016,7 +28456,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28035,7 +28475,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28109,10 +28549,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28144,7 +28585,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28177,7 +28618,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28210,7 +28651,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28243,7 +28684,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28276,7 +28717,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28309,7 +28750,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28342,7 +28783,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28375,7 +28816,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28406,7 +28847,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -28437,7 +28878,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -28470,7 +28911,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -28503,7 +28944,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -28536,7 +28977,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -28569,7 +29010,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -28602,7 +29043,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -28635,7 +29076,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -28668,7 +29109,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -28701,7 +29142,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -28734,7 +29175,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -28767,7 +29208,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -28800,7 +29241,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -28833,7 +29274,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -28866,7 +29307,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -28899,7 +29340,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -28932,7 +29373,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -28965,7 +29406,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -28997,7 +29438,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29029,7 +29470,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29061,7 +29502,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29093,7 +29534,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29125,7 +29566,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29155,7 +29596,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29185,7 +29626,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29217,7 +29658,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29249,7 +29690,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29281,7 +29722,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29313,7 +29754,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29345,7 +29786,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29375,7 +29816,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29407,7 +29848,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -29439,7 +29880,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -29471,7 +29912,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -29503,7 +29944,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -29533,7 +29974,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -29563,7 +30004,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -29593,7 +30034,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -29623,7 +30064,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -29655,7 +30096,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -29687,7 +30128,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -29717,7 +30158,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -29747,7 +30188,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -29777,7 +30218,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -29807,7 +30248,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -29837,7 +30278,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -29932,10 +30373,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -29967,7 +30409,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -29998,7 +30440,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30029,7 +30471,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30060,7 +30502,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30091,7 +30533,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30122,7 +30564,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30153,7 +30595,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30184,7 +30626,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30215,7 +30657,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="1